<commit_message>
chore: actualizar reporte FT buffer [2026-09-14]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/11/2026 at 1:07 PM ET)</t>
+          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>279 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>279 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>249 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
     </row>
@@ -2326,117 +2326,117 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.73 / 5.44%</t>
+          <t>$47.66 / 5.27%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.66 / 0.22%</t>
+          <t>$57.51 / -0.04%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.78 / 9.36%</t>
+          <t>$55.73 / 9.26%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.44 / 7.81%</t>
+          <t>$62.33 / 7.62%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.45 / 8.00%</t>
+          <t>$56.35 / 7.80%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.19 / 2.24%</t>
+          <t>$61.04 / 1.99%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.14 / 2.11%</t>
+          <t>$60.96 / 1.81%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.44 / 10.61%</t>
+          <t>$53.41 / 10.54%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.36 / 3.23%</t>
+          <t>$57.21 / 2.96%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.94 / 12.57%</t>
+          <t>$59.87 / 12.43%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.80 / 12.38%</t>
+          <t>$53.71 / 12.20%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.84 / 12.76%</t>
+          <t>$56.81 / 12.70%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.48 / 4.52%</t>
+          <t>$42.41 / 4.35%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.07 / 0.13%</t>
+          <t>$42.00 / -0.03%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.68 / 7.94%</t>
+          <t>$40.62 / 7.78%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.90 / 6.34%</t>
+          <t>$44.87 / 6.26%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.96 / 6.76%</t>
+          <t>$45.92 / 6.65%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.51 / 1.97%</t>
+          <t>$44.43 / 1.80%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.91 / 1.85%</t>
+          <t>$41.85 / 1.69%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.09 / 8.56%</t>
+          <t>$45.06 / 8.49%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.88 / 2.91%</t>
+          <t>$43.79 / 2.70%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.71 / 10.30%</t>
+          <t>$42.68 / 10.23%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.50 / 10.19%</t>
+          <t>$42.48 / 10.14%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$765.66 / 7.82%</t>
+          <t>$762.37 / 7.35%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$765.66 / -0.01%</t>
+          <t>$762.37 / -0.44%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$765.66 / 12.50%</t>
+          <t>$762.37 / 12.02%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$765.66 / 11.06%</t>
+          <t>$762.37 / 10.58%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$765.66 / 10.70%</t>
+          <t>$762.37 / 10.22%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$765.66 / 3.01%</t>
+          <t>$762.37 / 2.57%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$765.66 / 2.53%</t>
+          <t>$762.37 / 2.09%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$765.66 / 18.05%</t>
+          <t>$762.37 / 17.55%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$765.66 / 3.58%</t>
+          <t>$762.37 / 3.14%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$765.66 / 16.18%</t>
+          <t>$762.37 / 15.68%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$765.66 / 15.24%</t>
+          <t>$762.37 / 14.75%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$765.66 / 15.36%</t>
+          <t>$762.37 / 14.87%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$765.66 / 7.82%</t>
+          <t>$762.34 / 7.35%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$765.66 / -0.01%</t>
+          <t>$762.34 / -0.44%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$765.66 / 12.50%</t>
+          <t>$762.34 / 12.01%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$765.66 / 11.06%</t>
+          <t>$762.34 / 10.57%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$765.66 / 10.70%</t>
+          <t>$762.34 / 10.22%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$765.66 / 3.01%</t>
+          <t>$762.34 / 2.56%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$765.66 / 2.53%</t>
+          <t>$762.34 / 2.09%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$765.66 / 18.05%</t>
+          <t>$762.34 / 17.54%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$765.66 / 3.58%</t>
+          <t>$762.34 / 3.13%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$765.66 / 16.18%</t>
+          <t>$762.34 / 15.68%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$765.66 / 15.24%</t>
+          <t>$762.34 / 14.74%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$765.66 / 15.36%</t>
+          <t>$762.34 / 14.86%</t>
         </is>
       </c>
     </row>
@@ -2580,117 +2580,117 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.89% (8.42%)</t>
+          <t>9.06% (8.59%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.86% (16.06%)</t>
+          <t>17.16% (16.36%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.37% (4.16%)</t>
+          <t>4.45% (4.25%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.24% (5.90%)</t>
+          <t>6.42% (6.07%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.53% (5.26%)</t>
+          <t>5.72% (5.45%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.13% (13.43%)</t>
+          <t>14.41% (13.71%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.85% (13.21%)</t>
+          <t>14.18% (13.55%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.56% (5.17%)</t>
+          <t>5.63% (5.24%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.15% (12.59%)</t>
+          <t>13.44% (12.88%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.99% (2.85%)</t>
+          <t>3.11% (2.97%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.73% (1.66%)</t>
+          <t>1.89% (1.82%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.36% (0.35%)</t>
+          <t>0.41% (0.40%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.16% (6.67%)</t>
+          <t>7.33% (6.85%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.55% (12.76%)</t>
+          <t>13.74% (12.94%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.27% (3.05%)</t>
+          <t>3.41% (3.21%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.93% (4.58%)</t>
+          <t>5.00% (4.65%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.22% (3.94%)</t>
+          <t>4.31% (4.04%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.50% (10.80%)</t>
+          <t>11.68% (10.98%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.10% (10.46%)</t>
+          <t>11.27% (10.63%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.73% (4.32%)</t>
+          <t>4.79% (4.39%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.34% (9.77%)</t>
+          <t>10.56% (10.00%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.05% (1.91%)</t>
+          <t>2.12% (1.98%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.08% (1.01%)</t>
+          <t>1.12% (1.05%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.81%</t>
+          <t>7.27%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.18%</t>
+          <t>17.68%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>14.06%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>-0.32%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>13.53%</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0.30%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>-0.75%</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>13.04%</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0.38%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>-0.13%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>-1.18%</t>
-        </is>
-      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.37%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.35%</t>
+          <t>-2.92%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.37%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.52%</t>
+          <t>-2.09%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.69%</t>
+          <t>-2.26%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-3.36%</t>
+          <t>-2.94%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.04% (10.56%)</t>
+          <t>10.82% (10.35%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.72% (8.92%)</t>
+          <t>9.58% (8.79%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.88% (10.67%)</t>
+          <t>10.61% (10.40%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.28% (10.93%)</t>
+          <t>11.08% (10.74%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.77% (10.50%)</t>
+          <t>10.59% (10.32%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.31% (9.61%)</t>
+          <t>10.17% (9.47%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.96% (9.33%)</t>
+          <t>9.87% (9.23%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.80% (13.41%)</t>
+          <t>13.53% (13.14%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.71% (9.14%)</t>
+          <t>9.59% (9.02%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.76% (10.62%)</t>
+          <t>10.52% (10.39%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.21% (10.13%)</t>
+          <t>10.00% (9.94%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.93% (9.92%)</t>
+          <t>9.64% (9.63%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.51% (16.03%)</t>
+          <t>16.32% (15.84%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.81% (14.01%)</t>
+          <t>14.60% (13.81%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.51% (16.30%)</t>
+          <t>16.31% (16.11%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.06% (16.71%)</t>
+          <t>16.78% (16.44%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.36% (16.09%)</t>
+          <t>16.11% (15.85%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.43% (14.72%)</t>
+          <t>15.22% (14.53%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.09% (14.45%)</t>
+          <t>14.87% (14.24%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.74% (19.33%)</t>
+          <t>19.48% (19.08%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.84% (14.27%)</t>
+          <t>14.68% (14.11%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.88% (16.73%)</t>
+          <t>16.61% (16.47%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.30% (16.23%)</t>
+          <t>16.02% (15.95%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>16.05% (16.04%)</t>
+          <t>15.72% (15.72%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.48% (-5.96%)</t>
+          <t>-5.34% (-5.82%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.27% (-1.07%)</t>
+          <t>-0.02% (-0.81%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.12% (-9.33%)</t>
+          <t>-9.05% (-9.25%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.68% (-8.03%)</t>
+          <t>-7.53% (-7.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.92% (-8.20%)</t>
+          <t>-7.76% (-8.02%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.32% (-3.02%)</t>
+          <t>-2.08% (-2.78%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.26% (-2.90%)</t>
+          <t>-1.98% (-2.61%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.96% (-10.36%)</t>
+          <t>-9.91% (-10.30%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.40% (-3.97%)</t>
+          <t>-3.15% (-3.72%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.77% (-11.92%)</t>
+          <t>-11.67% (-11.81%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.70% (-11.77%)</t>
+          <t>-11.56% (-11.63%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-12.05% (-12.07%)</t>
+          <t>-12.01% (-12.02%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.65% (-5.13%)</t>
+          <t>-4.50% (-4.98%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.18% (-0.98%)</t>
+          <t>-0.02% (-0.81%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.93% (-8.14%)</t>
+          <t>-7.80% (-8.00%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.40% (-6.75%)</t>
+          <t>-6.34% (-6.69%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.85% (-7.12%)</t>
+          <t>-6.76% (-7.03%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.05% (-2.76%)</t>
+          <t>-1.90% (-2.59%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.01% (-2.65%)</t>
+          <t>-1.86% (-2.49%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.26% (-8.66%)</t>
+          <t>-8.20% (-8.60%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.09% (-3.67%)</t>
+          <t>-2.90% (-3.47%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.96% (-10.11%)</t>
+          <t>-9.90% (-10.04%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.94% (-10.01%)</t>
+          <t>-9.90% (-9.97%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.26% (-10.28%)</t>
+          <t>-10.27% (-10.28%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.53%</t>
+          <t>-16.17%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.99%</t>
+          <t>-9.60%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.00%</t>
+          <t>-19.65%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.96%</t>
+          <t>-18.61%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.70%</t>
+          <t>-18.35%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.63%</t>
+          <t>-12.25%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.22%</t>
+          <t>-11.84%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.76%</t>
+          <t>-23.43%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.11%</t>
+          <t>-12.74%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.53%</t>
+          <t>-22.20%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.90%</t>
+          <t>-21.57%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-21.98%</t>
+          <t>-21.65%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.16%</t>
+          <t>-20.82%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.99%</t>
+          <t>-14.62%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.44%</t>
+          <t>-24.11%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.46%</t>
+          <t>-23.13%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-22.88%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.48%</t>
+          <t>-17.12%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.10%</t>
+          <t>-16.74%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.00%</t>
+          <t>-27.68%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.94%</t>
+          <t>-17.58%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.83%</t>
+          <t>-26.52%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.24%</t>
+          <t>-25.92%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-26.32%</t>
+          <t>-25.99%</t>
         </is>
       </c>
     </row>
@@ -3215,117 +3215,117 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.93% (1.45%)</t>
+          <t>1.64% (1.17%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.27% (-1.07%)</t>
+          <t>-0.02% (-0.81%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.31% (2.10%)</t>
+          <t>1.95% (1.75%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.58% (2.23%)</t>
+          <t>2.30% (1.96%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.98% (1.71%)</t>
+          <t>1.72% (1.46%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.63% (-0.08%)</t>
+          <t>0.43% (-0.26%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.22% (-0.42%)</t>
+          <t>0.08% (-0.55%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.56% (5.17%)</t>
+          <t>5.63% (5.24%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.07% (-0.50%)</t>
+          <t>-0.11% (-0.67%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.60% (2.46%)</t>
+          <t>2.27% (2.13%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.73% (1.66%)</t>
+          <t>1.58% (1.51%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.36% (0.35%)</t>
+          <t>0.41% (0.40%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.83% (2.34%)</t>
+          <t>2.54% (2.07%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.18% (-0.98%)</t>
+          <t>-0.02% (-0.81%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.27% (3.05%)</t>
+          <t>3.34% (3.14%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.00% (3.64%)</t>
+          <t>3.61% (3.26%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.17% (2.90%)</t>
+          <t>2.82% (2.55%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.89% (0.19%)</t>
+          <t>0.62% (-0.08%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.48% (-0.16%)</t>
+          <t>0.19% (-0.44%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.73% (4.32%)</t>
+          <t>4.79% (4.39%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.38% (-0.19%)</t>
+          <t>0.15% (-0.42%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.05% (1.91%)</t>
+          <t>2.12% (1.98%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.08% (1.01%)</t>
+          <t>1.12% (1.05%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 11/9/2026</t>
+          <t>As of 14/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>5.45%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>7.80%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.20%</t>
+          <t>-8.02%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.90%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.81%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.06%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.03%</t>
+          <t>-7.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.14%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.05%</t>
+          <t>17.55%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.36%</t>
+          <t>-10.30%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.42%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.27%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.35%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.81%</t>
+          <t>7.27%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.96%</t>
+          <t>-5.82%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.14%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.23%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.14%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>13.53%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.97%</t>
+          <t>-3.72%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.55%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.11%</t>
+          <t>1.81%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>14.06%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-2.61%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.43%</t>
+          <t>13.71%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.24%</t>
+          <t>1.99%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.57%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.02%</t>
+          <t>-2.78%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.18%</t>
+          <t>17.68%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-0.81%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.70%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.36%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-12.07%</t>
+          <t>-12.02%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.13%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.66%</t>
+          <t>1.82%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.20%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>14.75%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.77%</t>
+          <t>-11.63%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.85%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.57%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.18%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.38%</t>
+          <t>0.81%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.92%</t>
+          <t>-11.81%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.40%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.16%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>9.26%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>12.02%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.33%</t>
+          <t>-9.25%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 11/9/2026</t>
+          <t>As of 14/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.09%</t>
+          <t>15.85%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.76%</t>
+          <t>6.65%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.70%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.12%</t>
+          <t>-7.03%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>16.44%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.58%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.34%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.06%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.75%</t>
+          <t>-6.69%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.33%</t>
+          <t>19.08%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>8.49%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.05%</t>
+          <t>17.54%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.35%</t>
+          <t>-2.92%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.66%</t>
+          <t>-8.60%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.03%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.67%</t>
+          <t>6.85%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.35%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.13%</t>
+          <t>-4.98%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.11%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>2.70%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.37%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.67%</t>
+          <t>-3.47%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.45%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.46%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.69%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.65%</t>
+          <t>-2.49%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.72%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.80%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>1.80%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-2.59%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>13.81%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-0.81%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>15.72%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15.36%</t>
+          <t>14.86%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-3.36%</t>
+          <t>-2.94%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>15.95%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>10.14%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>14.74%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.69%</t>
+          <t>-2.26%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.01%</t>
+          <t>-9.97%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.73%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.98%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.18%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.52%</t>
+          <t>-2.09%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.11%</t>
+          <t>-10.04%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.30%</t>
+          <t>16.11%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.94%</t>
+          <t>7.78%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.37%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.14%</t>
+          <t>-8.00%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-15]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:40 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/14/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>249 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.66 / 5.27%</t>
+          <t>$47.46 / 4.84%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.51 / -0.04%</t>
+          <t>$57.26 / -0.48%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.73 / 9.26%</t>
+          <t>$55.50 / 8.80%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.33 / 7.62%</t>
+          <t>$62.12 / 7.26%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.35 / 7.80%</t>
+          <t>$56.15 / 7.42%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.04 / 1.99%</t>
+          <t>$60.79 / 1.57%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.96 / 1.81%</t>
+          <t>$60.73 / 1.43%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.41 / 10.54%</t>
+          <t>$53.28 / 10.27%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.21 / 2.96%</t>
+          <t>$56.95 / 2.49%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.87 / 12.43%</t>
+          <t>$59.68 / 12.09%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.71 / 12.20%</t>
+          <t>$53.52 / 11.80%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.81 / 12.70%</t>
+          <t>$56.66 / 12.40%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.41 / 4.35%</t>
+          <t>$42.31 / 4.09%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.00 / -0.03%</t>
+          <t>$41.84 / -0.40%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.62 / 7.78%</t>
+          <t>$40.55 / 7.58%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.87 / 6.26%</t>
+          <t>$44.76 / 6.00%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.92 / 6.65%</t>
+          <t>$45.80 / 6.38%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.43 / 1.80%</t>
+          <t>$44.28 / 1.44%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.85 / 1.69%</t>
+          <t>$41.70 / 1.34%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.06 / 8.49%</t>
+          <t>$45.00 / 8.34%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.79 / 2.70%</t>
+          <t>$43.63 / 2.31%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.68 / 10.23%</t>
+          <t>$42.60 / 10.01%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.48 / 10.14%</t>
+          <t>$42.40 / 9.93%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.97 / 10.52%</t>
+          <t>$41.96 / 10.48%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$762.37 / 7.35%</t>
+          <t>$757.19 / 6.62%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$762.37 / -0.44%</t>
+          <t>$757.19 / -1.11%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$762.37 / 12.02%</t>
+          <t>$757.19 / 11.25%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$762.37 / 10.58%</t>
+          <t>$757.19 / 9.83%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$762.37 / 10.22%</t>
+          <t>$757.19 / 9.47%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$762.37 / 2.57%</t>
+          <t>$757.19 / 1.87%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$762.37 / 2.09%</t>
+          <t>$757.19 / 1.40%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$762.37 / 17.55%</t>
+          <t>$757.19 / 16.75%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$762.37 / 3.14%</t>
+          <t>$757.19 / 2.44%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$762.37 / 15.68%</t>
+          <t>$757.19 / 14.89%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$762.37 / 14.75%</t>
+          <t>$757.19 / 13.97%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$762.37 / 14.87%</t>
+          <t>$757.19 / 14.09%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$762.34 / 7.35%</t>
+          <t>$757.19 / 6.62%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$762.34 / -0.44%</t>
+          <t>$757.19 / -1.11%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$762.34 / 12.01%</t>
+          <t>$757.19 / 11.25%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$762.34 / 10.57%</t>
+          <t>$757.19 / 9.83%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$762.34 / 10.22%</t>
+          <t>$757.19 / 9.47%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$762.34 / 2.56%</t>
+          <t>$757.19 / 1.87%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$762.34 / 2.09%</t>
+          <t>$757.19 / 1.40%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$762.34 / 17.54%</t>
+          <t>$757.19 / 16.75%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$762.34 / 3.13%</t>
+          <t>$757.19 / 2.44%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$762.34 / 15.68%</t>
+          <t>$757.19 / 14.89%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$762.34 / 14.74%</t>
+          <t>$757.19 / 13.97%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$762.34 / 14.86%</t>
+          <t>$757.19 / 14.09%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.06% (8.59%)</t>
+          <t>9.51% (9.03%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17.16% (16.36%)</t>
+          <t>17.68% (16.88%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.45% (4.25%)</t>
+          <t>4.89% (4.69%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.42% (6.07%)</t>
+          <t>6.77% (6.43%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.72% (5.45%)</t>
+          <t>6.09% (5.83%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.41% (13.71%)</t>
+          <t>14.88% (14.18%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.18% (13.55%)</t>
+          <t>14.61% (13.98%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.63% (5.24%)</t>
+          <t>5.88% (5.49%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.44% (12.88%)</t>
+          <t>13.97% (13.41%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.11% (2.97%)</t>
+          <t>3.42% (3.29%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.89% (1.82%)</t>
+          <t>2.25% (2.18%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.41% (0.40%)</t>
+          <t>0.67% (0.67%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.33% (6.85%)</t>
+          <t>7.59% (7.12%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.74% (12.94%)</t>
+          <t>14.15% (13.36%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.41% (3.21%)</t>
+          <t>3.60% (3.40%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.00% (4.65%)</t>
+          <t>5.25% (4.91%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.31% (4.04%)</t>
+          <t>4.58% (4.32%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.68% (10.98%)</t>
+          <t>12.07% (11.37%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.27% (10.63%)</t>
+          <t>11.65% (11.02%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.79% (4.39%)</t>
+          <t>4.93% (4.53%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.56% (10.00%)</t>
+          <t>10.98% (10.42%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.12% (1.98%)</t>
+          <t>2.32% (2.18%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.12% (1.05%)</t>
+          <t>1.31% (1.24%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.12% (0.11%)</t>
+          <t>0.15% (0.14%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.27%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.68%</t>
+          <t>18.49%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>3.14%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.72%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.62%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.06%</t>
+          <t>14.84%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.99%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>5.36%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>15.04%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.79%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-2.26%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>11.12%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.26%</t>
+          <t>-1.60%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-2.28%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.82% (10.35%)</t>
+          <t>10.64% (10.16%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.58% (8.79%)</t>
+          <t>9.41% (8.62%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.61% (10.40%)</t>
+          <t>10.44% (10.24%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.08% (10.74%)</t>
+          <t>10.83% (10.49%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.59% (10.32%)</t>
+          <t>10.36% (10.09%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.17% (9.47%)</t>
+          <t>9.97% (9.27%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.87% (9.23%)</t>
+          <t>9.63% (9.00%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.53% (13.14%)</t>
+          <t>13.22% (12.83%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.59% (9.02%)</t>
+          <t>9.44% (8.87%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.52% (10.39%)</t>
+          <t>10.26% (10.13%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.00% (9.94%)</t>
+          <t>9.78% (9.71%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.64% (9.63%)</t>
+          <t>9.33% (9.32%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.32% (15.84%)</t>
+          <t>16.02% (15.54%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.60% (13.81%)</t>
+          <t>14.39% (13.60%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.31% (16.11%)</t>
+          <t>15.97% (15.76%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.78% (16.44%)</t>
+          <t>16.49% (16.14%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.11% (15.85%)</t>
+          <t>15.83% (15.57%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.22% (14.53%)</t>
+          <t>15.00% (14.30%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.87% (14.24%)</t>
+          <t>14.65% (14.01%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.48% (19.08%)</t>
+          <t>19.11% (18.71%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.68% (14.11%)</t>
+          <t>14.48% (13.92%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.61% (16.47%)</t>
+          <t>16.29% (16.15%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.02% (15.95%)</t>
+          <t>15.68% (15.61%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.72% (15.72%)</t>
+          <t>15.25% (15.24%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.34% (-5.82%)</t>
+          <t>-4.95% (-5.43%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.02% (-0.81%)</t>
+          <t>0.00% (-0.37%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.05% (-9.25%)</t>
+          <t>-8.66% (-8.87%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.53% (-7.87%)</t>
+          <t>-7.22% (-7.56%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.76% (-8.02%)</t>
+          <t>-7.43% (-7.70%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.08% (-2.78%)</t>
+          <t>-1.68% (-2.38%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-1.98% (-2.61%)</t>
+          <t>-1.61% (-2.24%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.91% (-10.30%)</t>
+          <t>-9.69% (-10.08%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.15% (-3.72%)</t>
+          <t>-2.71% (-3.27%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.67% (-11.81%)</t>
+          <t>-11.40% (-11.54%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.56% (-11.63%)</t>
+          <t>-11.25% (-11.32%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-12.01% (-12.02%)</t>
+          <t>-11.78% (-11.79%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.50% (-4.98%)</t>
+          <t>-4.26% (-4.74%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.02% (-0.81%)</t>
+          <t>0.00% (-0.44%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.80% (-8.00%)</t>
+          <t>-7.63% (-7.83%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.34% (-6.69%)</t>
+          <t>-6.12% (-6.46%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.76% (-7.03%)</t>
+          <t>-6.52% (-6.79%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.90% (-2.59%)</t>
+          <t>-1.55% (-2.25%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.86% (-2.49%)</t>
+          <t>-1.52% (-2.16%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.20% (-8.60%)</t>
+          <t>-8.08% (-8.48%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.90% (-3.47%)</t>
+          <t>-2.54% (-3.10%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.90% (-10.04%)</t>
+          <t>-9.72% (-9.86%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.90% (-9.97%)</t>
+          <t>-9.73% (-9.80%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.27% (-10.28%)</t>
+          <t>-10.24% (-10.25%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>-15.59%</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-8.99%</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-19.10%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-18.05%</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-17.79%</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-11.65%</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-11.24%</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-22.91%</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>-12.14%</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-21.67%</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-21.03%</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>-21.11%</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>-20.28%</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-14.04%</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-23.60%</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-22.60%</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-22.35%</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>-16.56%</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
           <t>-16.17%</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>-9.60%</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>-19.65%</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>-18.61%</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>-18.35%</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>-12.25%</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>-11.84%</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>-23.43%</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>-12.74%</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>-22.20%</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>-21.57%</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>-21.65%</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>-20.82%</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>-14.62%</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-24.11%</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-23.13%</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-22.88%</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>-17.12%</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>-16.74%</t>
-        </is>
-      </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.68%</t>
+          <t>-27.19%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.58%</t>
+          <t>-17.02%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.52%</t>
+          <t>-26.02%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.92%</t>
+          <t>-25.41%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.99%</t>
+          <t>-25.49%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.64% (1.17%)</t>
+          <t>1.36% (0.89%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.81%)</t>
+          <t>0.42% (-0.37%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.95% (1.75%)</t>
+          <t>1.68% (1.48%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.30% (1.96%)</t>
+          <t>1.94% (1.60%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.72% (1.46%)</t>
+          <t>1.39% (1.12%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.43% (-0.26%)</t>
+          <t>0.16% (-0.54%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.08% (-0.55%)</t>
+          <t>-0.23% (-0.86%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.63% (5.24%)</t>
+          <t>5.50% (5.11%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.11% (-0.67%)</t>
+          <t>-0.33% (-0.89%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.27% (2.13%)</t>
+          <t>1.89% (1.75%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.58% (1.51%)</t>
+          <t>1.24% (1.18%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.41% (0.40%)</t>
+          <t>0.67% (0.67%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.54% (2.07%)</t>
+          <t>2.10% (1.62%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.81%)</t>
+          <t>0.35% (-0.44%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.34% (3.14%)</t>
+          <t>2.83% (2.63%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.61% (3.26%)</t>
+          <t>3.15% (2.81%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.82% (2.55%)</t>
+          <t>2.38% (2.12%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.62% (-0.08%)</t>
+          <t>0.29% (-0.41%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.19% (-0.44%)</t>
+          <t>-0.15% (-0.78%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.79% (4.39%)</t>
+          <t>4.93% (4.53%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.15% (-0.42%)</t>
+          <t>-0.16% (-0.72%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.12% (1.98%)</t>
+          <t>2.32% (2.18%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.12% (1.05%)</t>
+          <t>1.31% (1.24%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.12% (0.11%)</t>
+          <t>0.15% (0.14%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/9/2026</t>
+          <t>As of 15/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.45%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.80%</t>
+          <t>7.42%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.62%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.02%</t>
+          <t>-7.70%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.49%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>7.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>9.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.72%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.87%</t>
+          <t>-7.56%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.14%</t>
+          <t>12.83%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.55%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.30%</t>
+          <t>-10.08%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>9.03%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.27%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.35%</t>
+          <t>6.62%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.27%</t>
+          <t>8.01%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.82%</t>
+          <t>-5.43%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>8.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.14%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.72%</t>
+          <t>-3.27%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.55%</t>
+          <t>13.98%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.81%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.06%</t>
+          <t>14.84%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.61%</t>
+          <t>-2.24%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>9.27%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.71%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.99%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.57%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.78%</t>
+          <t>-2.38%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.62%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>16.88%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.44%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.68%</t>
+          <t>18.49%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-0.37%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.70%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-12.02%</t>
+          <t>-11.79%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>9.71%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.82%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.20%</t>
+          <t>11.80%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.75%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.99%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.63%</t>
+          <t>-11.32%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.39%</t>
+          <t>10.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>12.09%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>14.89%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.81%</t>
+          <t>-11.54%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.40%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>4.69%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.02%</t>
+          <t>11.25%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>3.14%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.25%</t>
+          <t>-8.87%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/9/2026</t>
+          <t>As of 15/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.85%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.65%</t>
+          <t>6.38%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>9.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.03%</t>
+          <t>-6.79%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.44%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.91%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>9.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.69%</t>
+          <t>-6.46%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.08%</t>
+          <t>18.71%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.49%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.54%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-2.26%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.60%</t>
+          <t>-8.48%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>15.54%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.85%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.35%</t>
+          <t>6.62%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>5.36%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.98%</t>
+          <t>-4.74%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.11%</t>
+          <t>13.92%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.70%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>11.12%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.10%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>11.02%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.69%</t>
+          <t>1.34%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.79%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.49%</t>
+          <t>-2.16%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.80%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.59%</t>
+          <t>-2.25%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.81%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>13.36%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>-1.11%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>15.04%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>-0.44%</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>14.26%</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>-0.81%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.24%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.86%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-2.28%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.28%</t>
+          <t>-10.25%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.95%</t>
+          <t>15.61%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.14%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.74%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.26%</t>
+          <t>-1.60%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.97%</t>
+          <t>-9.80%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.15%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.98%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.01%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>14.89%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.04%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.11%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>3.40%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.78%</t>
+          <t>7.58%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>11.25%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.00%</t>
+          <t>-7.83%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-16]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/15/2026 at 1:33 PM ET)</t>
+          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.46 / 4.84%</t>
+          <t>$47.57 / 5.09%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.26 / -0.48%</t>
+          <t>$57.42 / -0.20%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.50 / 8.80%</t>
+          <t>$55.60 / 9.00%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.12 / 7.26%</t>
+          <t>$62.24 / 7.47%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.15 / 7.42%</t>
+          <t>$56.28 / 7.68%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.79 / 1.57%</t>
+          <t>$60.95 / 1.84%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.73 / 1.43%</t>
+          <t>$60.84 / 1.61%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.28 / 10.27%</t>
+          <t>$53.36 / 10.43%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$56.95 / 2.49%</t>
+          <t>$57.10 / 2.77%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.68 / 12.09%</t>
+          <t>$59.80 / 12.30%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.52 / 11.80%</t>
+          <t>$53.67 / 12.11%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.66 / 12.40%</t>
+          <t>$56.79 / 12.65%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.31 / 4.09%</t>
+          <t>$42.37 / 4.24%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.84 / -0.40%</t>
+          <t>$41.91 / -0.24%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.55 / 7.58%</t>
+          <t>$40.60 / 7.71%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.76 / 6.00%</t>
+          <t>$44.84 / 6.19%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.80 / 6.38%</t>
+          <t>$45.85 / 6.50%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.28 / 1.44%</t>
+          <t>$44.36 / 1.62%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.70 / 1.34%</t>
+          <t>$41.76 / 1.48%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.00 / 8.34%</t>
+          <t>$45.04 / 8.44%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.63 / 2.31%</t>
+          <t>$43.71 / 2.51%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.60 / 10.01%</t>
+          <t>$42.65 / 10.14%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.40 / 9.93%</t>
+          <t>$42.47 / 10.12%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$41.96 / 10.48%</t>
+          <t>$42.01 / 10.61%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$757.19 / 6.62%</t>
+          <t>$759.86 / 7.00%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$757.19 / -1.11%</t>
+          <t>$759.86 / -0.77%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$757.19 / 11.25%</t>
+          <t>$759.86 / 11.65%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$757.19 / 9.83%</t>
+          <t>$759.86 / 10.22%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$757.19 / 9.47%</t>
+          <t>$759.86 / 9.86%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$757.19 / 1.87%</t>
+          <t>$759.86 / 2.23%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$757.19 / 1.40%</t>
+          <t>$759.86 / 1.76%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$757.19 / 16.75%</t>
+          <t>$759.86 / 17.16%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$757.19 / 2.44%</t>
+          <t>$759.86 / 2.80%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$757.19 / 14.89%</t>
+          <t>$759.86 / 15.30%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$757.19 / 13.97%</t>
+          <t>$759.86 / 14.37%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$757.19 / 14.09%</t>
+          <t>$759.86 / 14.49%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$757.19 / 6.62%</t>
+          <t>$759.86 / 7.00%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$757.19 / -1.11%</t>
+          <t>$759.86 / -0.77%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$757.19 / 11.25%</t>
+          <t>$759.86 / 11.65%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$757.19 / 9.83%</t>
+          <t>$759.86 / 10.22%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$757.19 / 9.47%</t>
+          <t>$759.86 / 9.86%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$757.19 / 1.87%</t>
+          <t>$759.86 / 2.23%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$757.19 / 1.40%</t>
+          <t>$759.86 / 1.76%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$757.19 / 16.75%</t>
+          <t>$759.86 / 17.16%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$757.19 / 2.44%</t>
+          <t>$759.86 / 2.80%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$757.19 / 14.89%</t>
+          <t>$759.86 / 15.30%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$757.19 / 13.97%</t>
+          <t>$759.86 / 14.37%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$757.19 / 14.09%</t>
+          <t>$759.86 / 14.49%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.51% (9.03%)</t>
+          <t>9.25% (8.78%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17.68% (16.88%)</t>
+          <t>17.35% (16.56%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.89% (4.69%)</t>
+          <t>4.69% (4.49%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.77% (6.43%)</t>
+          <t>6.57% (6.23%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6.09% (5.83%)</t>
+          <t>5.84% (5.58%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.88% (14.18%)</t>
+          <t>14.57% (13.88%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.61% (13.98%)</t>
+          <t>14.40% (13.77%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.88% (5.49%)</t>
+          <t>5.72% (5.33%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.97% (13.41%)</t>
+          <t>13.66% (13.10%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.42% (3.29%)</t>
+          <t>3.22% (3.09%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2.25% (2.18%)</t>
+          <t>1.97% (1.90%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.67% (0.67%)</t>
+          <t>0.45% (0.45%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.59% (7.12%)</t>
+          <t>7.44% (6.96%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>14.15% (13.36%)</t>
+          <t>13.96% (13.17%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.60% (3.40%)</t>
+          <t>3.47% (3.27%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.25% (4.91%)</t>
+          <t>5.06% (4.72%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.58% (4.32%)</t>
+          <t>4.45% (4.19%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>12.07% (11.37%)</t>
+          <t>11.86% (11.17%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.65% (11.02%)</t>
+          <t>11.49% (10.86%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.93% (4.53%)</t>
+          <t>4.84% (4.44%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.98% (10.42%)</t>
+          <t>10.76% (10.20%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.32% (2.18%)</t>
+          <t>2.20% (2.06%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.31% (1.24%)</t>
+          <t>1.13% (1.06%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.15% (0.14%)</t>
+          <t>0.03% (0.03%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>7.63%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>18.49%</t>
+          <t>18.07%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.14%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.72%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.62%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.84%</t>
+          <t>14.44%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.36%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.14%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.99%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>-0.43%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.36%</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>15.04%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.75%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.14%</t>
+          <t>1.78%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.79%</t>
+          <t>11.40%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.26%</t>
+          <t>-2.61%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>11.12%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-1.95%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.28%</t>
+          <t>-2.63%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.64% (10.16%)</t>
+          <t>10.71% (10.24%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.41% (8.62%)</t>
+          <t>9.45% (8.66%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.44% (10.24%)</t>
+          <t>10.55% (10.35%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.83% (10.49%)</t>
+          <t>10.94% (10.60%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.36% (10.09%)</t>
+          <t>10.42% (10.16%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.97% (9.27%)</t>
+          <t>10.02% (9.33%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.63% (9.00%)</t>
+          <t>9.76% (9.14%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.22% (12.83%)</t>
+          <t>13.36% (12.97%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.44% (8.87%)</t>
+          <t>9.48% (8.92%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.26% (10.13%)</t>
+          <t>10.37% (10.23%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.78% (9.71%)</t>
+          <t>9.81% (9.75%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.33% (9.32%)</t>
+          <t>9.41% (9.41%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.02% (15.54%)</t>
+          <t>16.16% (15.68%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.39% (13.60%)</t>
+          <t>14.52% (13.73%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.97% (15.76%)</t>
+          <t>16.12% (15.92%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.49% (16.14%)</t>
+          <t>16.59% (16.25%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.83% (15.57%)</t>
+          <t>15.99% (15.73%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.00% (14.30%)</t>
+          <t>15.12% (14.42%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.65% (14.01%)</t>
+          <t>14.80% (14.17%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.11% (18.71%)</t>
+          <t>19.28% (18.89%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.48% (13.92%)</t>
+          <t>14.58% (14.02%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.29% (16.15%)</t>
+          <t>16.44% (16.31%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.68% (15.61%)</t>
+          <t>15.78% (15.72%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.25% (15.24%)</t>
+          <t>15.40% (15.40%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-4.95% (-5.43%)</t>
+          <t>-5.18% (-5.65%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.00% (-0.37%)</t>
+          <t>0.00% (-0.65%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.66% (-8.87%)</t>
+          <t>-8.84% (-9.04%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.22% (-7.56%)</t>
+          <t>-7.40% (-7.74%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.43% (-7.70%)</t>
+          <t>-7.66% (-7.92%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-1.68% (-2.38%)</t>
+          <t>-1.94% (-2.64%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-1.61% (-2.24%)</t>
+          <t>-1.79% (-2.42%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.69% (-10.08%)</t>
+          <t>-9.83% (-10.21%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-2.71% (-3.27%)</t>
+          <t>-2.97% (-3.53%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.40% (-11.54%)</t>
+          <t>-11.58% (-11.71%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.25% (-11.32%)</t>
+          <t>-11.49% (-11.56%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.78% (-11.79%)</t>
+          <t>-11.98% (-11.98%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.26% (-4.74%)</t>
+          <t>-4.40% (-4.87%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.00% (-0.44%)</t>
+          <t>0.00% (-0.61%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.63% (-7.83%)</t>
+          <t>-7.74% (-7.95%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.12% (-6.46%)</t>
+          <t>-6.29% (-6.63%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.52% (-6.79%)</t>
+          <t>-6.64% (-6.90%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.55% (-2.25%)</t>
+          <t>-1.73% (-2.43%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.52% (-2.16%)</t>
+          <t>-1.67% (-2.30%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.08% (-8.48%)</t>
+          <t>-8.17% (-8.56%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.54% (-3.10%)</t>
+          <t>-2.73% (-3.29%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.72% (-9.86%)</t>
+          <t>-9.83% (-9.97%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.73% (-9.80%)</t>
+          <t>-9.90% (-9.96%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.24% (-10.25%)</t>
+          <t>-10.35% (-10.35%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.59%</t>
+          <t>-15.89%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-8.99%</t>
+          <t>-9.31%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.10%</t>
+          <t>-19.39%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-18.34%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-17.79%</t>
+          <t>-18.08%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-11.65%</t>
+          <t>-11.96%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.24%</t>
+          <t>-11.55%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-22.91%</t>
+          <t>-23.18%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.14%</t>
+          <t>-12.45%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.67%</t>
+          <t>-21.94%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.03%</t>
+          <t>-21.31%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-21.11%</t>
+          <t>-21.39%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.28%</t>
+          <t>-20.56%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.04%</t>
+          <t>-14.34%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.60%</t>
+          <t>-23.86%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.60%</t>
+          <t>-22.88%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.35%</t>
+          <t>-22.63%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-16.56%</t>
+          <t>-16.85%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.17%</t>
+          <t>-16.46%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.19%</t>
+          <t>-27.45%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.02%</t>
+          <t>-17.31%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.02%</t>
+          <t>-26.28%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.41%</t>
+          <t>-25.68%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.49%</t>
+          <t>-25.75%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.36% (0.89%)</t>
+          <t>1.49% (1.02%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.42% (-0.37%)</t>
+          <t>0.14% (-0.65%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.68% (1.48%)</t>
+          <t>1.85% (1.65%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.94% (1.60%)</t>
+          <t>2.10% (1.77%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.39% (1.12%)</t>
+          <t>1.50% (1.24%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.16% (-0.54%)</t>
+          <t>0.24% (-0.45%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.23% (-0.86%)</t>
+          <t>-0.06% (-0.69%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.50% (5.11%)</t>
+          <t>5.71% (5.32%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.33% (-0.89%)</t>
+          <t>-0.25% (-0.81%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.89% (1.75%)</t>
+          <t>2.05% (1.91%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.24% (1.18%)</t>
+          <t>1.32% (1.26%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.67% (0.67%)</t>
+          <t>0.45% (0.45%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.10% (1.62%)</t>
+          <t>2.31% (1.84%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.35% (-0.44%)</t>
+          <t>0.18% (-0.61%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.83% (2.63%)</t>
+          <t>3.07% (2.86%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.15% (2.81%)</t>
+          <t>3.33% (2.99%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.38% (2.12%)</t>
+          <t>2.62% (2.36%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.29% (-0.41%)</t>
+          <t>0.46% (-0.24%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.15% (-0.78%)</t>
+          <t>0.06% (-0.57%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.93% (4.53%)</t>
+          <t>4.84% (4.44%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.16% (-0.72%)</t>
+          <t>0.00% (-0.56%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.32% (2.18%)</t>
+          <t>2.20% (2.06%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.31% (1.24%)</t>
+          <t>1.13% (1.06%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.15% (0.14%)</t>
+          <t>0.03% (0.03%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/9/2026</t>
+          <t>As of 16/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.83%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.42%</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>9.86%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.62%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.70%</t>
+          <t>-7.92%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.49%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>6.23%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.26%</t>
+          <t>7.47%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.83%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.72%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.56%</t>
+          <t>-7.74%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.83%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.33%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>17.16%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.36%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.08%</t>
+          <t>-10.21%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9.03%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>5.09%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>7.00%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>7.63%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.43%</t>
+          <t>-5.65%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.87%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.49%</t>
+          <t>2.77%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.27%</t>
+          <t>-3.53%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>9.14%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.98%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.40%</t>
+          <t>1.76%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.84%</t>
+          <t>14.44%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.24%</t>
+          <t>-2.42%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.27%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>13.88%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.57%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.38%</t>
+          <t>-2.64%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.62%</t>
+          <t>8.66%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.88%</t>
+          <t>16.56%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18.49%</t>
+          <t>18.07%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.37%</t>
+          <t>-0.65%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>12.65%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>-0.43%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.79%</t>
+          <t>-11.98%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.71%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.80%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.37%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.99%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.32%</t>
+          <t>-11.56%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.13%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.09%</t>
+          <t>12.30%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.89%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.14%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.54%</t>
+          <t>-11.71%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.69%</t>
+          <t>4.49%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.25%</t>
+          <t>11.65%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.14%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.87%</t>
+          <t>-9.04%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/9/2026</t>
+          <t>As of 16/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>15.73%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.38%</t>
+          <t>6.50%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.47%</t>
+          <t>9.86%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.14%</t>
+          <t>1.78%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.79%</t>
+          <t>-6.90%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.91%</t>
+          <t>4.72%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>6.19%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9.83%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.46%</t>
+          <t>-6.63%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.71%</t>
+          <t>18.89%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.44%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.44%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>17.16%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.26%</t>
+          <t>-2.61%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.48%</t>
+          <t>-8.56%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.54%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.96%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>7.00%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.36%</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.74%</t>
+          <t>-4.87%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.92%</t>
+          <t>14.02%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.12%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.10%</t>
+          <t>-3.29%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.02%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.40%</t>
+          <t>1.76%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.79%</t>
+          <t>11.40%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.16%</t>
+          <t>-2.30%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.37%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.25%</t>
+          <t>-2.43%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13.36%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-1.11%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.04%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.44%</t>
+          <t>-0.61%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.24%</t>
+          <t>15.40%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.14%</t>
+          <t>0.03%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.28%</t>
+          <t>-2.63%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.25%</t>
+          <t>-10.35%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.61%</t>
+          <t>15.72%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.37%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-1.95%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.80%</t>
+          <t>-9.96%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.15%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>2.06%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>10.14%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.89%</t>
+          <t>15.30%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.97%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.40%</t>
+          <t>3.27%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.58%</t>
+          <t>7.71%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.25%</t>
+          <t>11.65%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.75%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.83%</t>
+          <t>-7.95%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-17]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/16/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.57 / 5.09%</t>
+          <t>$47.66 / 5.27%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.42 / -0.20%</t>
+          <t>$57.48 / -0.09%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.60 / 9.00%</t>
+          <t>$55.72 / 9.24%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.24 / 7.47%</t>
+          <t>$62.35 / 7.65%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.28 / 7.68%</t>
+          <t>$56.38 / 7.87%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.95 / 1.84%</t>
+          <t>$61.03 / 1.97%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.84 / 1.61%</t>
+          <t>$60.97 / 1.83%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.36 / 10.43%</t>
+          <t>$53.42 / 10.57%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.10 / 2.77%</t>
+          <t>$57.20 / 2.94%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.80 / 12.30%</t>
+          <t>$59.92 / 12.54%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.67 / 12.11%</t>
+          <t>$53.79 / 12.37%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.79 / 12.65%</t>
+          <t>$56.98 / 13.04%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.37 / 4.24%</t>
+          <t>$42.43 / 4.40%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.91 / -0.24%</t>
+          <t>$41.98 / -0.07%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.60 / 7.71%</t>
+          <t>$40.65 / 7.86%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.84 / 6.19%</t>
+          <t>$44.89 / 6.31%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.85 / 6.50%</t>
+          <t>$45.93 / 6.68%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.36 / 1.62%</t>
+          <t>$44.41 / 1.75%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.76 / 1.48%</t>
+          <t>$41.83 / 1.64%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.04 / 8.44%</t>
+          <t>$45.08 / 8.54%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.71 / 2.51%</t>
+          <t>$43.78 / 2.66%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.65 / 10.14%</t>
+          <t>$42.71 / 10.29%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.47 / 10.12%</t>
+          <t>$42.53 / 10.28%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.01 / 10.61%</t>
+          <t>$42.03 / 10.67%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$759.86 / 7.00%</t>
+          <t>$761.94 / 7.29%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$759.86 / -0.77%</t>
+          <t>$761.94 / -0.49%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$759.86 / 11.65%</t>
+          <t>$761.94 / 11.95%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$759.86 / 10.22%</t>
+          <t>$761.94 / 10.52%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$759.86 / 9.86%</t>
+          <t>$761.94 / 10.16%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$759.86 / 2.23%</t>
+          <t>$761.94 / 2.51%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$759.86 / 1.76%</t>
+          <t>$761.94 / 2.04%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$759.86 / 17.16%</t>
+          <t>$761.94 / 17.48%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$759.86 / 2.80%</t>
+          <t>$761.94 / 3.08%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$759.86 / 15.30%</t>
+          <t>$761.94 / 15.62%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$759.86 / 14.37%</t>
+          <t>$761.94 / 14.68%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$759.86 / 14.49%</t>
+          <t>$761.94 / 14.80%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$759.86 / 7.00%</t>
+          <t>$761.94 / 7.29%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$759.86 / -0.77%</t>
+          <t>$761.94 / -0.49%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$759.86 / 11.65%</t>
+          <t>$761.94 / 11.95%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$759.86 / 10.22%</t>
+          <t>$761.94 / 10.52%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$759.86 / 9.86%</t>
+          <t>$761.94 / 10.16%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$759.86 / 2.23%</t>
+          <t>$761.94 / 2.51%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$759.86 / 1.76%</t>
+          <t>$761.94 / 2.04%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$759.86 / 17.16%</t>
+          <t>$761.94 / 17.48%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$759.86 / 2.80%</t>
+          <t>$761.94 / 3.08%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$759.86 / 15.30%</t>
+          <t>$761.94 / 15.62%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$759.86 / 14.37%</t>
+          <t>$761.94 / 14.68%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$759.86 / 14.49%</t>
+          <t>$761.94 / 14.80%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.25% (8.78%)</t>
+          <t>9.05% (8.59%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17.35% (16.56%)</t>
+          <t>17.21% (16.42%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.69% (4.49%)</t>
+          <t>4.47% (4.27%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.57% (6.23%)</t>
+          <t>6.38% (6.05%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.84% (5.58%)</t>
+          <t>5.65% (5.39%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.57% (13.88%)</t>
+          <t>14.42% (13.73%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.40% (13.77%)</t>
+          <t>14.15% (13.53%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.72% (5.33%)</t>
+          <t>5.59% (5.21%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.66% (13.10%)</t>
+          <t>13.47% (12.91%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.22% (3.09%)</t>
+          <t>3.01% (2.87%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.97% (1.90%)</t>
+          <t>1.73% (1.67%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.45% (0.45%)</t>
+          <t>0.10% (0.10%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.44% (6.96%)</t>
+          <t>7.27% (6.80%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.96% (13.17%)</t>
+          <t>13.77% (12.98%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.47% (3.27%)</t>
+          <t>3.33% (3.13%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>5.06% (4.72%)</t>
+          <t>4.94% (4.60%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.45% (4.19%)</t>
+          <t>4.28% (4.02%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.86% (11.17%)</t>
+          <t>11.72% (11.03%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.49% (10.86%)</t>
+          <t>11.31% (10.69%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.84% (4.44%)</t>
+          <t>4.74% (4.35%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.76% (10.20%)</t>
+          <t>10.60% (10.04%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.20% (2.06%)</t>
+          <t>2.05% (1.92%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>1.13% (1.06%)</t>
+          <t>0.98% (0.92%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.03% (0.03%)</t>
+          <t>-0.03% (-0.03%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.63%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>18.07%</t>
+          <t>17.75%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>13.96%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.44%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.14%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>14.32%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>11.09%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.61%</t>
+          <t>-2.87%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.95%</t>
+          <t>-2.21%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.63%</t>
+          <t>-2.89%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.71% (10.24%)</t>
+          <t>10.77% (10.30%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.45% (8.66%)</t>
+          <t>9.58% (8.79%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.55% (10.35%)</t>
+          <t>10.57% (10.38%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.94% (10.60%)</t>
+          <t>11.01% (10.67%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.42% (10.16%)</t>
+          <t>10.48% (10.22%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.02% (9.33%)</t>
+          <t>10.13% (9.44%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.76% (9.14%)</t>
+          <t>9.79% (9.17%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.36% (12.97%)</t>
+          <t>13.45% (13.07%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.48% (8.92%)</t>
+          <t>9.55% (9.00%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.37% (10.23%)</t>
+          <t>10.39% (10.26%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.81% (9.75%)</t>
+          <t>9.82% (9.76%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.41% (9.41%)</t>
+          <t>9.32% (9.32%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.16% (15.68%)</t>
+          <t>16.23% (15.76%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.52% (13.73%)</t>
+          <t>14.59% (13.80%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.12% (15.92%)</t>
+          <t>16.20% (16.00%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.59% (16.25%)</t>
+          <t>16.69% (16.35%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.99% (15.73%)</t>
+          <t>16.05% (15.79%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.12% (14.42%)</t>
+          <t>15.22% (14.53%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.80% (14.17%)</t>
+          <t>14.87% (14.25%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.28% (18.89%)</t>
+          <t>19.39% (19.00%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.58% (14.02%)</t>
+          <t>14.66% (14.10%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.44% (16.31%)</t>
+          <t>16.52% (16.38%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.78% (15.72%)</t>
+          <t>15.85% (15.79%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.40% (15.40%)</t>
+          <t>15.55% (15.55%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.18% (-5.65%)</t>
+          <t>-5.35% (-5.82%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.00% (-0.65%)</t>
+          <t>0.00% (-0.76%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.84% (-9.04%)</t>
+          <t>-9.04% (-9.23%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.40% (-7.74%)</t>
+          <t>-7.56% (-7.89%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.66% (-7.92%)</t>
+          <t>-7.82% (-8.08%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-1.94% (-2.64%)</t>
+          <t>-2.08% (-2.76%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-1.79% (-2.42%)</t>
+          <t>-2.00% (-2.63%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.83% (-10.21%)</t>
+          <t>-9.94% (-10.32%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-2.97% (-3.53%)</t>
+          <t>-3.14% (-3.69%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.58% (-11.71%)</t>
+          <t>-11.76% (-11.89%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.49% (-11.56%)</t>
+          <t>-11.70% (-11.76%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-11.98% (-11.98%)</t>
+          <t>-12.28% (-12.28%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.40% (-4.87%)</t>
+          <t>-4.55% (-5.02%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.00% (-0.61%)</t>
+          <t>0.00% (-0.78%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.74% (-7.95%)</t>
+          <t>-7.87% (-8.07%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.29% (-6.63%)</t>
+          <t>-6.39% (-6.73%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.64% (-6.90%)</t>
+          <t>-6.79% (-7.05%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.73% (-2.43%)</t>
+          <t>-1.86% (-2.55%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.67% (-2.30%)</t>
+          <t>-1.82% (-2.45%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.17% (-8.56%)</t>
+          <t>-8.25% (-8.64%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.73% (-3.29%)</t>
+          <t>-2.88% (-3.43%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.83% (-9.97%)</t>
+          <t>-9.96% (-10.10%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-9.90% (-9.96%)</t>
+          <t>-10.03% (-10.09%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.35% (-10.35%)</t>
+          <t>-10.40% (-10.41%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.89%</t>
+          <t>-16.12%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.31%</t>
+          <t>-9.55%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.39%</t>
+          <t>-19.61%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.34%</t>
+          <t>-18.56%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.08%</t>
+          <t>-18.30%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-11.96%</t>
+          <t>-12.20%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.55%</t>
+          <t>-11.79%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.18%</t>
+          <t>-23.39%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.45%</t>
+          <t>-12.69%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.94%</t>
+          <t>-22.16%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.31%</t>
+          <t>-21.52%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-21.39%</t>
+          <t>-21.60%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.56%</t>
+          <t>-20.78%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.34%</t>
+          <t>-14.58%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.86%</t>
+          <t>-24.07%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.88%</t>
+          <t>-23.09%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.63%</t>
+          <t>-22.84%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-16.85%</t>
+          <t>-17.08%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.46%</t>
+          <t>-16.69%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.45%</t>
+          <t>-27.65%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.31%</t>
+          <t>-17.54%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.28%</t>
+          <t>-26.48%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.68%</t>
+          <t>-25.88%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.75%</t>
+          <t>-25.96%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.49% (1.02%)</t>
+          <t>1.58% (1.11%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.14% (-0.65%)</t>
+          <t>0.03% (-0.76%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.85% (1.65%)</t>
+          <t>1.90% (1.71%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.10% (1.77%)</t>
+          <t>2.21% (1.88%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.50% (1.24%)</t>
+          <t>1.60% (1.34%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.24% (-0.45%)</t>
+          <t>0.39% (-0.30%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.69%)</t>
+          <t>0.00% (-0.63%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.71% (5.32%)</t>
+          <t>5.59% (5.21%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.25% (-0.81%)</t>
+          <t>-0.14% (-0.70%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.05% (1.91%)</t>
+          <t>2.11% (1.98%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.32% (1.26%)</t>
+          <t>1.36% (1.30%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.45% (0.45%)</t>
+          <t>0.10% (0.10%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.31% (1.84%)</t>
+          <t>2.44% (1.96%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.18% (-0.61%)</t>
+          <t>0.01% (-0.78%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.07% (2.86%)</t>
+          <t>3.21% (3.01%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.33% (2.99%)</t>
+          <t>3.50% (3.16%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.62% (2.36%)</t>
+          <t>2.73% (2.47%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.46% (-0.24%)</t>
+          <t>0.60% (-0.09%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.06% (-0.57%)</t>
+          <t>0.18% (-0.45%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.84% (4.44%)</t>
+          <t>4.74% (4.35%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.00% (-0.56%)</t>
+          <t>0.12% (-0.44%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.20% (2.06%)</t>
+          <t>2.05% (1.92%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>1.13% (1.06%)</t>
+          <t>0.98% (0.92%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.03% (0.03%)</t>
+          <t>-0.03% (-0.03%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/9/2026</t>
+          <t>As of 17/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>10.22%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5.39%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7.87%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>10.16%</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>5.58%</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>7.68%</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>9.86%</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.92%</t>
+          <t>-8.08%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.23%</t>
+          <t>6.05%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.47%</t>
+          <t>7.65%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.74%</t>
+          <t>-7.89%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>13.07%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.33%</t>
+          <t>5.21%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.16%</t>
+          <t>17.48%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.26%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.21%</t>
+          <t>-10.32%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>5.27%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.00%</t>
+          <t>7.29%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.63%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.82%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>12.91%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.77%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-3.69%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.14%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>13.53%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.83%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.76%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.44%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.42%</t>
+          <t>-2.63%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.88%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>13.96%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.64%</t>
+          <t>-2.76%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.66%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18.07%</t>
+          <t>17.75%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.76%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>12.65%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>14.80%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-11.98%</t>
+          <t>-12.28%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.90%</t>
+          <t>1.67%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.37%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.56%</t>
+          <t>-11.76%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.09%</t>
+          <t>2.87%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.30%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.30%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.14%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.71%</t>
+          <t>-11.89%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.38%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.49%</t>
+          <t>4.27%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.65%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-9.23%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/9/2026</t>
+          <t>As of 17/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.73%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.50%</t>
+          <t>6.68%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.86%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-6.90%</t>
+          <t>-7.05%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>16.35%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.72%</t>
+          <t>4.60%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.19%</t>
+          <t>6.31%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.63%</t>
+          <t>-6.73%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.89%</t>
+          <t>19.00%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.44%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.44%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.16%</t>
+          <t>17.48%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.61%</t>
+          <t>-2.87%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.56%</t>
+          <t>-8.64%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.96%</t>
+          <t>6.80%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>4.40%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.00%</t>
+          <t>7.29%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.87%</t>
+          <t>-5.02%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.02%</t>
+          <t>14.10%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.43%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.43%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>14.25%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.76%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>11.09%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.30%</t>
+          <t>-2.45%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.43%</t>
+          <t>-2.55%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.80%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>14.32%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>-0.78%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.40%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.03%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>14.80%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.63%</t>
+          <t>-2.89%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.35%</t>
+          <t>-10.41%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.37%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.95%</t>
+          <t>-2.21%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-9.96%</t>
+          <t>-10.09%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.31%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>1.92%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.14%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.30%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-9.97%</t>
+          <t>-10.10%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.27%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.71%</t>
+          <t>7.86%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.65%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-7.95%</t>
+          <t>-8.07%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-18]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/17/2026 at 1:31 PM ET)</t>
+          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>272 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>272 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
     </row>
@@ -2326,107 +2326,107 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.66 / 5.27%</t>
+          <t>$47.61 / 5.16%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.48 / -0.09%</t>
+          <t>$57.43 / -0.18%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.72 / 9.24%</t>
+          <t>$55.69 / 9.18%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.35 / 7.65%</t>
+          <t>$62.33 / 7.62%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.38 / 7.87%</t>
+          <t>$56.36 / 7.82%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.03 / 1.97%</t>
+          <t>$60.99 / 1.90%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.97 / 1.83%</t>
+          <t>$60.92 / 1.75%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.42 / 10.57%</t>
+          <t>$53.42 / 10.56%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.20 / 2.94%</t>
+          <t>$57.16 / 2.87%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.92 / 12.54%</t>
+          <t>$59.90 / 12.50%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.79 / 12.37%</t>
+          <t>$53.78 / 12.35%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$56.98 / 13.04%</t>
+          <t>$57.08 / 13.24%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.43 / 4.40%</t>
+          <t>$42.41 / 4.33%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.98 / -0.07%</t>
+          <t>$41.93 / -0.19%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.65 / 7.86%</t>
+          <t>$40.64 / 7.83%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.89 / 6.31%</t>
+          <t>$44.87 / 6.26%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.93 / 6.68%</t>
+          <t>$45.91 / 6.63%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.41 / 1.75%</t>
+          <t>$44.37 / 1.66%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.83 / 1.64%</t>
+          <t>$41.80 / 1.57%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.08 / 8.54%</t>
+          <t>$45.07 / 8.51%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.78 / 2.66%</t>
+          <t>$43.75 / 2.59%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2436,12 +2436,12 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.53 / 10.28%</t>
+          <t>$42.55 / 10.32%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.03 / 10.67%</t>
+          <t>$42.07 / 10.77%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$761.94 / 7.29%</t>
+          <t>$759.41 / 6.94%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$761.94 / -0.49%</t>
+          <t>$759.41 / -0.82%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$761.94 / 11.95%</t>
+          <t>$759.38 / 11.58%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$761.94 / 10.52%</t>
+          <t>$759.41 / 10.15%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$761.94 / 10.16%</t>
+          <t>$759.41 / 9.80%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$761.94 / 2.51%</t>
+          <t>$759.41 / 2.17%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$761.94 / 2.04%</t>
+          <t>$759.41 / 1.70%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$761.94 / 17.48%</t>
+          <t>$759.41 / 17.09%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$761.94 / 3.08%</t>
+          <t>$759.41 / 2.74%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$761.94 / 15.62%</t>
+          <t>$759.38 / 15.23%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$761.94 / 14.68%</t>
+          <t>$759.38 / 14.30%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$761.94 / 14.80%</t>
+          <t>$759.41 / 14.42%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$761.94 / 7.29%</t>
+          <t>$759.38 / 6.93%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$761.94 / -0.49%</t>
+          <t>$759.38 / -0.83%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$761.94 / 11.95%</t>
+          <t>$759.38 / 11.58%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$761.94 / 10.52%</t>
+          <t>$759.38 / 10.15%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$761.94 / 10.16%</t>
+          <t>$759.38 / 9.79%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$761.94 / 2.51%</t>
+          <t>$759.38 / 2.16%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$761.94 / 2.04%</t>
+          <t>$759.38 / 1.69%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$761.94 / 17.48%</t>
+          <t>$759.38 / 17.09%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$761.94 / 3.08%</t>
+          <t>$759.38 / 2.73%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$761.94 / 15.62%</t>
+          <t>$759.38 / 15.23%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$761.94 / 14.68%</t>
+          <t>$759.38 / 14.30%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$761.94 / 14.80%</t>
+          <t>$759.38 / 14.42%</t>
         </is>
       </c>
     </row>
@@ -2580,107 +2580,107 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.05% (8.59%)</t>
+          <t>9.16% (8.70%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17.21% (16.42%)</t>
+          <t>17.31% (16.53%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.47% (4.27%)</t>
+          <t>4.52% (4.33%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.38% (6.05%)</t>
+          <t>6.41% (6.07%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.65% (5.39%)</t>
+          <t>5.69% (5.44%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.42% (13.73%)</t>
+          <t>14.49% (13.80%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.15% (13.53%)</t>
+          <t>14.24% (13.61%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.59% (5.21%)</t>
+          <t>5.60% (5.22%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.47% (12.91%)</t>
+          <t>13.53% (12.98%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.01% (2.87%)</t>
+          <t>3.04% (2.91%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.73% (1.67%)</t>
+          <t>1.74% (1.69%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.10% (0.10%)</t>
+          <t>-0.07% (-0.07%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.27% (6.80%)</t>
+          <t>7.33% (6.86%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.77% (12.98%)</t>
+          <t>13.90% (13.12%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.33% (3.13%)</t>
+          <t>3.35% (3.16%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.94% (4.60%)</t>
+          <t>4.99% (4.65%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.28% (4.02%)</t>
+          <t>4.32% (4.07%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.72% (11.03%)</t>
+          <t>11.82% (11.13%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.31% (10.69%)</t>
+          <t>11.39% (10.77%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.74% (4.35%)</t>
+          <t>4.76% (4.37%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.60% (10.04%)</t>
+          <t>10.67% (10.11%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2690,12 +2690,12 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.98% (0.92%)</t>
+          <t>0.95% (0.89%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>-0.03% (-0.03%)</t>
+          <t>-0.12% (-0.12%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.69%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.75%</t>
+          <t>18.14%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.96%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>14.51%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>1.21%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.36%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.37%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.32%</t>
+          <t>14.70%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.09%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.87%</t>
+          <t>-2.55%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.80%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-1.71%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>-1.88%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.89%</t>
+          <t>-2.56%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.77% (10.30%)</t>
+          <t>10.59% (10.12%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.58% (8.79%)</t>
+          <t>9.36% (8.58%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.57% (10.38%)</t>
+          <t>10.35% (10.15%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.01% (10.67%)</t>
+          <t>10.75% (10.42%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.48% (10.22%)</t>
+          <t>10.25% (9.99%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.13% (9.44%)</t>
+          <t>9.90% (9.21%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.79% (9.17%)</t>
+          <t>9.57% (8.95%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.45% (13.07%)</t>
+          <t>13.21% (12.82%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.55% (9.00%)</t>
+          <t>9.32% (8.77%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.39% (10.26%)</t>
+          <t>10.16% (10.03%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.82% (9.76%)</t>
+          <t>9.57% (9.51%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.32% (9.32%)</t>
+          <t>8.91% (8.91%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.23% (15.76%)</t>
+          <t>16.01% (15.54%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.59% (13.80%)</t>
+          <t>14.41% (13.63%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.20% (16.00%)</t>
+          <t>15.97% (15.77%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.69% (16.35%)</t>
+          <t>16.47% (16.14%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.05% (15.79%)</t>
+          <t>15.83% (15.57%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.22% (14.53%)</t>
+          <t>15.03% (14.34%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.87% (14.25%)</t>
+          <t>14.66% (14.03%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.39% (19.00%)</t>
+          <t>19.17% (18.78%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.66% (14.10%)</t>
+          <t>14.45% (13.89%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.52% (16.38%)</t>
+          <t>16.27% (16.13%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.85% (15.79%)</t>
+          <t>15.57% (15.51%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.55% (15.55%)</t>
+          <t>15.22% (15.22%)</t>
         </is>
       </c>
     </row>
@@ -2961,107 +2961,107 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.35% (-5.82%)</t>
+          <t>-5.25% (-5.72%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.00% (-0.76%)</t>
+          <t>0.00% (-0.67%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.04% (-9.23%)</t>
+          <t>-8.99% (-9.18%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.56% (-7.89%)</t>
+          <t>-7.54% (-7.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.82% (-8.08%)</t>
+          <t>-7.78% (-8.04%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.08% (-2.76%)</t>
+          <t>-2.01% (-2.70%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.00% (-2.63%)</t>
+          <t>-1.93% (-2.55%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.94% (-10.32%)</t>
+          <t>-9.93% (-10.31%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.14% (-3.69%)</t>
+          <t>-3.08% (-3.63%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.76% (-11.89%)</t>
+          <t>-11.73% (-11.86%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.70% (-11.76%)</t>
+          <t>-11.69% (-11.75%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-12.28% (-12.28%)</t>
+          <t>-12.44% (-12.44%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.55% (-5.02%)</t>
+          <t>-4.50% (-4.96%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.00% (-0.78%)</t>
+          <t>0.00% (-0.66%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.87% (-8.07%)</t>
+          <t>-7.85% (-8.05%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.39% (-6.73%)</t>
+          <t>-6.35% (-6.69%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.79% (-7.05%)</t>
+          <t>-6.75% (-7.01%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.86% (-2.55%)</t>
+          <t>-1.77% (-2.46%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.82% (-2.45%)</t>
+          <t>-1.75% (-2.38%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.25% (-8.64%)</t>
+          <t>-8.23% (-8.62%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.88% (-3.43%)</t>
+          <t>-2.81% (-3.37%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -3071,12 +3071,12 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.03% (-10.09%)</t>
+          <t>-10.06% (-10.12%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.40% (-10.41%)</t>
+          <t>-10.48% (-10.48%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.12%</t>
+          <t>-15.84%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.55%</t>
+          <t>-9.25%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.61%</t>
+          <t>-19.34%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.56%</t>
+          <t>-18.29%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.30%</t>
+          <t>-18.03%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.20%</t>
+          <t>-11.91%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.79%</t>
+          <t>-11.50%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.39%</t>
+          <t>-23.14%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.69%</t>
+          <t>-12.40%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.16%</t>
+          <t>-21.89%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.52%</t>
+          <t>-21.26%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-21.60%</t>
+          <t>-21.34%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.78%</t>
+          <t>-20.51%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.58%</t>
+          <t>-14.29%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.07%</t>
+          <t>-23.82%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.09%</t>
+          <t>-22.83%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.84%</t>
+          <t>-22.58%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.08%</t>
+          <t>-16.80%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.69%</t>
+          <t>-16.41%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.65%</t>
+          <t>-27.40%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.54%</t>
+          <t>-17.26%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.48%</t>
+          <t>-26.23%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.88%</t>
+          <t>-25.63%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.96%</t>
+          <t>-25.71%</t>
         </is>
       </c>
     </row>
@@ -3215,107 +3215,107 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.58% (1.11%)</t>
+          <t>1.35% (0.88%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.03% (-0.76%)</t>
+          <t>0.11% (-0.67%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.90% (1.71%)</t>
+          <t>1.61% (1.42%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.21% (1.88%)</t>
+          <t>1.89% (1.56%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.60% (1.34%)</t>
+          <t>1.30% (1.04%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.39% (-0.30%)</t>
+          <t>0.11% (-0.57%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.00% (-0.63%)</t>
+          <t>-0.26% (-0.89%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.59% (5.21%)</t>
+          <t>5.53% (5.14%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.14% (-0.70%)</t>
+          <t>-0.42% (-0.97%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.11% (1.98%)</t>
+          <t>1.80% (1.67%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.36% (1.30%)</t>
+          <t>1.04% (0.98%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.10% (0.10%)</t>
+          <t>-0.07% (-0.07%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.44% (1.96%)</t>
+          <t>2.15% (1.68%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.01% (-0.78%)</t>
+          <t>0.13% (-0.66%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.21% (3.01%)</t>
+          <t>2.88% (2.69%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.50% (3.16%)</t>
+          <t>3.19% (2.86%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.73% (2.47%)</t>
+          <t>2.43% (2.17%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.60% (-0.09%)</t>
+          <t>0.35% (-0.34%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.18% (-0.45%)</t>
+          <t>-0.09% (-0.71%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.74% (4.35%)</t>
+          <t>4.76% (4.37%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.12% (-0.44%)</t>
+          <t>-0.15% (-0.71%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -3325,12 +3325,12 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.98% (0.92%)</t>
+          <t>0.95% (0.89%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.03%)</t>
+          <t>-0.12% (-0.12%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/9/2026</t>
+          <t>As of 18/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>9.99%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.39%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>7.82%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.08%</t>
+          <t>-8.04%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.05%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.65%</t>
+          <t>7.62%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.89%</t>
+          <t>-7.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.07%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.21%</t>
+          <t>5.22%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.48%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.32%</t>
+          <t>-10.31%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.27%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.69%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.82%</t>
+          <t>-5.72%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.91%</t>
+          <t>12.98%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.87%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.69%</t>
+          <t>-3.63%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.53%</t>
+          <t>13.61%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.83%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>14.51%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.63%</t>
+          <t>-2.55%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.80%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.96%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-2.70%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.53%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.75%</t>
+          <t>18.14%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.67%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>13.24%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.80%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.37%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-12.28%</t>
+          <t>-12.44%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.67%</t>
+          <t>1.69%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.36%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.76%</t>
+          <t>-11.75%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.03%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.87%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>15.23%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>1.21%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.89%</t>
+          <t>-11.86%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.38%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.27%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.58%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.23%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 17/9/2026</t>
+          <t>As of 18/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.68%</t>
+          <t>6.63%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.05%</t>
+          <t>-7.01%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.60%</t>
+          <t>4.65%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>6.26%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.73%</t>
+          <t>-6.69%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.00%</t>
+          <t>18.78%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.48%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.87%</t>
+          <t>-2.55%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.64%</t>
+          <t>-8.62%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.54%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.80%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.40%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>6.93%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.02%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.10%</t>
+          <t>13.89%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.59%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.73%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.43%</t>
+          <t>10.80%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-3.37%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.25%</t>
+          <t>14.03%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>1.69%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.09%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.45%</t>
+          <t>-2.38%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.16%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.55%</t>
+          <t>-2.46%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>13.12%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.32%</t>
+          <t>14.70%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.78%</t>
+          <t>-0.66%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.80%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.89%</t>
+          <t>-2.56%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.41%</t>
+          <t>-10.48%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>-1.88%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.09%</t>
+          <t>-10.12%</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4310,12 +4310,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>15.23%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-1.71%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>3.16%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.86%</t>
+          <t>7.83%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.58%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.07%</t>
+          <t>-8.05%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-21]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:04 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/18/2026 at 1:05 PM ET)</t>
+          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>9/22/2025 - 9/18/2026</t>
+          <t>9/21/2026 - 9/17/2027</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>9/22/2025 - 9/18/2026</t>
+          <t>9/21/2026 - 9/17/2027</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>14.00% (13.15%)</t>
+          <t>16.68% (15.83%)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>11.48% (10.63%)</t>
+          <t>14.09% (13.24%)</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>15.00% (14.15%)</t>
+          <t>15.02% (14.17%)</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>$50.41</t>
+          <t>$57.08</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>$37.98</t>
+          <t>$42.04</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>$57.04</t>
+          <t>$66.11</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>$42.01</t>
+          <t>$47.61</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>$663.70</t>
+          <t>$761.69</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>$663.70</t>
+          <t>$761.69</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>$756.62</t>
+          <t>$888.74</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>$739.91</t>
+          <t>$869.01</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.00% / $663.70</t>
+          <t>0.00% / $761.69</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>0.00% / $663.72</t>
+          <t>0.02% / $761.84</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>-10.00% / $597.33</t>
+          <t>-10.00% / $685.52</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>-15.00% / $564.17</t>
+          <t>-15.00% / $647.44</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>272 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>272 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>242 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.61 / 5.16%</t>
+          <t>$48.06 / 6.16%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.43 / -0.18%</t>
+          <t>$58.09 / 0.96%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$55.69 / 9.18%</t>
+          <t>$56.17 / 10.12%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.33 / 7.62%</t>
+          <t>$62.85 / 8.51%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.36 / 7.82%</t>
+          <t>$56.88 / 8.82%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$60.99 / 1.90%</t>
+          <t>$61.66 / 3.03%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$60.92 / 1.75%</t>
+          <t>$61.61 / 2.90%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.42 / 10.56%</t>
+          <t>$53.73 / 11.20%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.16 / 2.87%</t>
+          <t>$57.83 / 4.07%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$59.90 / 12.50%</t>
+          <t>$60.35 / 13.34%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$53.78 / 12.35%</t>
+          <t>$54.19 / 13.19%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.08 / 13.24%</t>
+          <t>$57.54 / 0.81%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.41 / 4.33%</t>
+          <t>$42.69 / 5.04%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$41.93 / -0.19%</t>
+          <t>$42.32 / 0.74%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.64 / 7.83%</t>
+          <t>$40.88 / 8.47%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$44.87 / 6.26%</t>
+          <t>$45.12 / 6.87%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$45.91 / 6.63%</t>
+          <t>$46.19 / 7.29%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.37 / 1.66%</t>
+          <t>$44.76 / 2.54%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.80 / 1.57%</t>
+          <t>$42.17 / 2.48%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.07 / 8.51%</t>
+          <t>$45.26 / 8.98%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.75 / 2.59%</t>
+          <t>$44.13 / 3.49%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.71 / 10.29%</t>
+          <t>$42.90 / 10.78%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.55 / 10.32%</t>
+          <t>$42.68 / 10.67%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.07 / 10.77%</t>
+          <t>$42.33 / 0.69%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$759.41 / 6.94%</t>
+          <t>$773.97 / 8.99%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$759.41 / -0.82%</t>
+          <t>$773.97 / 1.08%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$759.38 / 11.58%</t>
+          <t>$773.97 / 13.72%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$759.41 / 10.15%</t>
+          <t>$773.97 / 12.26%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$759.41 / 9.80%</t>
+          <t>$773.97 / 11.90%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$759.41 / 2.17%</t>
+          <t>$773.97 / 4.13%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$759.41 / 1.70%</t>
+          <t>$773.97 / 3.65%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$759.41 / 17.09%</t>
+          <t>$773.97 / 19.33%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$759.41 / 2.74%</t>
+          <t>$773.97 / 4.71%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$759.38 / 15.23%</t>
+          <t>$773.97 / 17.44%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$759.38 / 14.30%</t>
+          <t>$773.97 / 16.49%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$759.41 / 14.42%</t>
+          <t>$773.97 / 1.61%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$759.38 / 6.93%</t>
+          <t>$773.97 / 8.99%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$759.38 / -0.83%</t>
+          <t>$773.97 / 1.08%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$759.38 / 11.58%</t>
+          <t>$773.97 / 13.72%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$759.38 / 10.15%</t>
+          <t>$773.97 / 12.26%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$759.38 / 9.79%</t>
+          <t>$773.97 / 11.90%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$759.38 / 2.16%</t>
+          <t>$773.97 / 4.13%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$759.38 / 1.69%</t>
+          <t>$773.97 / 3.65%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$759.38 / 17.09%</t>
+          <t>$773.97 / 19.33%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$759.38 / 2.73%</t>
+          <t>$773.97 / 4.71%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$759.38 / 15.23%</t>
+          <t>$773.97 / 17.44%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$759.38 / 14.30%</t>
+          <t>$773.97 / 16.49%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$759.38 / 14.42%</t>
+          <t>$773.97 / 1.61%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9.16% (8.70%)</t>
+          <t>8.14% (7.68%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17.31% (16.53%)</t>
+          <t>15.98% (15.21%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.52% (4.33%)</t>
+          <t>3.62% (3.43%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6.41% (6.07%)</t>
+          <t>5.53% (5.20%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.69% (5.44%)</t>
+          <t>4.72% (4.47%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.49% (13.80%)</t>
+          <t>13.23% (12.56%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14.24% (13.61%)</t>
+          <t>12.96% (12.35%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.60% (5.22%)</t>
+          <t>4.98% (4.61%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.53% (12.98%)</t>
+          <t>12.22% (11.68%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.04% (2.91%)</t>
+          <t>2.27% (2.15%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.74% (1.69%)</t>
+          <t>0.98% (0.93%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>-0.07% (-0.07%)</t>
+          <t>15.73% (14.90%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>7.33% (6.86%)</t>
+          <t>6.61% (6.15%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.90% (13.12%)</t>
+          <t>12.85% (12.08%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.35% (3.16%)</t>
+          <t>2.74% (2.55%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.99% (4.65%)</t>
+          <t>4.39% (4.06%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4.32% (4.07%)</t>
+          <t>3.67% (3.42%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.82% (11.13%)</t>
+          <t>10.85% (10.18%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.39% (10.77%)</t>
+          <t>10.39% (9.78%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.76% (4.37%)</t>
+          <t>4.30% (3.92%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.67% (10.11%)</t>
+          <t>9.71% (9.16%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2.05% (1.92%)</t>
+          <t>1.59% (1.47%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.95% (0.89%)</t>
+          <t>0.62% (0.57%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>-0.12% (-0.12%)</t>
+          <t>13.31% (12.47%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.69%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>18.14%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.51%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>-1.81%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-1.20%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>-0.37%</t>
+          <t>14.83%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.70%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.73%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.55%</t>
+          <t>-4.38%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.80%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-1.71%</t>
+          <t>-3.57%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-1.88%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>12.28%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.59% (10.12%)</t>
+          <t>11.28% (10.82%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.36% (8.58%)</t>
+          <t>9.93% (9.16%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.35% (10.15%)</t>
+          <t>11.08% (10.90%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.75% (10.42%)</t>
+          <t>11.53% (11.20%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.25% (9.99%)</t>
+          <t>10.94% (10.69%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.90% (9.21%)</t>
+          <t>10.47% (9.80%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.57% (8.95%)</t>
+          <t>10.14% (9.53%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.21% (12.82%)</t>
+          <t>14.12% (13.75%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.32% (8.77%)</t>
+          <t>9.85% (9.31%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.16% (10.03%)</t>
+          <t>10.97% (10.85%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.57% (9.51%)</t>
+          <t>10.39% (10.34%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>8.91% (8.91%)</t>
+          <t>10.62% (9.78%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.01% (15.54%)</t>
+          <t>16.87% (16.41%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.41% (13.63%)</t>
+          <t>15.10% (14.33%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.97% (15.77%)</t>
+          <t>16.85% (16.66%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.47% (16.14%)</t>
+          <t>17.39% (17.06%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.83% (15.57%)</t>
+          <t>16.70% (16.45%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.03% (14.34%)</t>
+          <t>15.74% (15.06%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.66% (14.03%)</t>
+          <t>15.35% (14.74%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.17% (18.78%)</t>
+          <t>20.14% (19.75%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.45% (13.89%)</t>
+          <t>15.16% (14.62%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.27% (16.13%)</t>
+          <t>17.25% (17.13%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.57% (15.51%)</t>
+          <t>16.68% (16.63%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.22% (15.22%)</t>
+          <t>15.68% (14.84%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.25% (-5.72%)</t>
+          <t>-6.14% (-6.60%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.00% (-0.67%)</t>
+          <t>-1.03% (-1.79%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-8.99% (-9.18%)</t>
+          <t>-9.77% (-9.96%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.54% (-7.87%)</t>
+          <t>-8.30% (-8.63%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-7.78% (-8.04%)</t>
+          <t>-8.63% (-8.88%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.01% (-2.70%)</t>
+          <t>-3.09% (-3.77%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-1.93% (-2.55%)</t>
+          <t>-3.03% (-3.64%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-9.93% (-10.31%)</t>
+          <t>-10.46% (-10.83%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.08% (-3.63%)</t>
+          <t>-4.20% (-4.74%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-11.73% (-11.86%)</t>
+          <t>-12.39% (-12.51%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-11.69% (-11.75%)</t>
+          <t>-12.35% (-12.40%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-12.44% (-12.44%)</t>
+          <t>-0.81% (-1.65%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.50% (-4.96%)</t>
+          <t>-5.14% (-5.60%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.00% (-0.66%)</t>
+          <t>-0.80% (-1.57%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-7.85% (-8.05%)</t>
+          <t>-8.40% (-8.59%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.35% (-6.69%)</t>
+          <t>-6.89% (-7.22%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-6.75% (-7.01%)</t>
+          <t>-7.33% (-7.58%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-1.77% (-2.46%)</t>
+          <t>-2.62% (-3.30%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-1.75% (-2.38%)</t>
+          <t>-2.63% (-3.25%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.23% (-8.62%)</t>
+          <t>-8.63% (-9.02%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-2.81% (-3.37%)</t>
+          <t>-3.66% (-4.20%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-9.96% (-10.10%)</t>
+          <t>-10.37% (-10.49%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.06% (-10.12%)</t>
+          <t>-10.35% (-10.40%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-10.48% (-10.48%)</t>
+          <t>-0.67% (-1.50%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.84%</t>
+          <t>-17.42%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.25%</t>
+          <t>-10.96%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.34%</t>
+          <t>-20.86%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.29%</t>
+          <t>-19.83%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.03%</t>
+          <t>-19.57%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-11.91%</t>
+          <t>-13.57%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.50%</t>
+          <t>-13.17%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.14%</t>
+          <t>-24.58%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.40%</t>
+          <t>-14.05%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-21.89%</t>
+          <t>-23.36%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.26%</t>
+          <t>-22.74%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-21.34%</t>
+          <t>-11.43%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.51%</t>
+          <t>-22.01%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.29%</t>
+          <t>-15.90%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.82%</t>
+          <t>-25.25%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.83%</t>
+          <t>-24.28%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.58%</t>
+          <t>-24.04%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-16.80%</t>
+          <t>-18.37%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.41%</t>
+          <t>-17.99%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.40%</t>
+          <t>-28.77%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.26%</t>
+          <t>-18.82%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.23%</t>
+          <t>-27.62%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-25.63%</t>
+          <t>-27.03%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-25.71%</t>
+          <t>-16.35%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.35% (0.88%)</t>
+          <t>2.32% (1.87%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.11% (-0.67%)</t>
+          <t>0.04% (-0.73%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.61% (1.42%)</t>
+          <t>2.68% (2.50%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.89% (1.56%)</t>
+          <t>3.00% (2.67%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.30% (1.04%)</t>
+          <t>2.30% (2.05%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.11% (-0.57%)</t>
+          <t>0.91% (0.24%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.89%)</t>
+          <t>0.51% (-0.09%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.53% (5.14%)</t>
+          <t>4.98% (4.61%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.42% (-0.97%)</t>
+          <t>0.32% (-0.22%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.80% (1.67%)</t>
+          <t>2.27% (2.15%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.04% (0.98%)</t>
+          <t>0.98% (0.93%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>-0.07% (-0.07%)</t>
+          <t>0.79% (-0.05%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.15% (1.68%)</t>
+          <t>3.41% (2.96%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.13% (-0.66%)</t>
+          <t>0.26% (-0.51%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.88% (2.69%)</t>
+          <t>2.74% (2.55%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.19% (2.86%)</t>
+          <t>4.39% (4.06%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.43% (2.17%)</t>
+          <t>3.67% (3.42%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.35% (-0.34%)</t>
+          <t>1.40% (0.72%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.71%)</t>
+          <t>0.92% (0.31%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.76% (4.37%)</t>
+          <t>4.30% (3.92%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.15% (-0.71%)</t>
+          <t>0.89% (0.35%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2.05% (1.92%)</t>
+          <t>1.59% (1.47%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.95% (0.89%)</t>
+          <t>0.62% (0.57%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.12% (-0.12%)</t>
+          <t>0.91% (0.08%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 18/9/2026</t>
+          <t>As of 21/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.99%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>4.47%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>11.90%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.04%</t>
+          <t>-8.88%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.62%</t>
+          <t>8.51%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.87%</t>
+          <t>-8.63%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>13.75%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.22%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>19.33%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.07%</t>
+          <t>-1.81%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.31%</t>
+          <t>-10.83%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.16%</t>
+          <t>6.16%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.69%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.72%</t>
+          <t>-6.60%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.98%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.87%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.63%</t>
+          <t>-4.74%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.53%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.61%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>2.90%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.51%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.55%</t>
+          <t>-3.64%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.80%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.90%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>4.13%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.70%</t>
+          <t>-3.77%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.53%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18.14%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.67%</t>
+          <t>-1.79%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>13.24%</t>
+          <t>0.81%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.37%</t>
+          <t>14.83%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-12.44%</t>
+          <t>-1.65%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>10.34%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.69%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>13.19%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-1.20%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.75%</t>
+          <t>-12.40%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.03%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>2.15%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>13.34%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.23%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.86%</t>
+          <t>-12.51%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>10.90%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.58%</t>
+          <t>13.72%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.96%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 18/9/2026</t>
+          <t>As of 21/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>16.45%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.63%</t>
+          <t>7.29%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>11.90%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.84%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.01%</t>
+          <t>-7.58%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>17.06%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.65%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.26%</t>
+          <t>6.87%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.73%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-6.69%</t>
+          <t>-7.22%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.78%</t>
+          <t>19.75%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>3.92%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>19.33%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.55%</t>
+          <t>-4.38%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.62%</t>
+          <t>-9.02%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.54%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.86%</t>
+          <t>6.15%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.33%</t>
+          <t>5.04%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6.93%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-4.96%</t>
+          <t>-5.60%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.89%</t>
+          <t>14.62%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.59%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.73%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.80%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-4.20%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.03%</t>
+          <t>14.74%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.57%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.69%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.38%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>15.06%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.66%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.16%</t>
+          <t>4.13%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.46%</t>
+          <t>-3.30%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13.12%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>0.74%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.70%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-1.57%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>14.84%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>12.47%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>12.28%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-10.48%</t>
+          <t>-1.50%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>16.63%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.88%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.12%</t>
+          <t>-10.40%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>17.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.92%</t>
+          <t>1.47%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.23%</t>
+          <t>17.44%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.71%</t>
+          <t>-3.57%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.10%</t>
+          <t>-10.49%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>16.66%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.16%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.58%</t>
+          <t>13.72%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.05%</t>
+          <t>-8.59%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-22]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/21/2026 at 2:42 PM ET)</t>
+          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>242 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
     </row>
@@ -2336,107 +2336,107 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.17 / 10.12%</t>
+          <t>$56.23 / 10.24%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.85 / 8.51%</t>
+          <t>$62.86 / 8.54%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.88 / 8.82%</t>
+          <t>$56.88 / 8.83%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.66 / 3.03%</t>
+          <t>$61.64 / 3.00%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.61 / 2.90%</t>
+          <t>$61.59 / 2.86%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.73 / 11.20%</t>
+          <t>$53.72 / 11.19%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.83 / 4.07%</t>
+          <t>$57.80 / 4.02%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.35 / 13.34%</t>
+          <t>$60.39 / 13.42%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.19 / 13.19%</t>
+          <t>$54.24 / 13.30%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.54 / 0.81%</t>
+          <t>$57.55 / 0.83%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.69 / 5.04%</t>
+          <t>$42.71 / 5.08%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.32 / 0.74%</t>
+          <t>$42.31 / 0.70%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.88 / 8.47%</t>
+          <t>$40.92 / 8.58%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.12 / 6.87%</t>
+          <t>$45.14 / 6.90%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.19 / 7.29%</t>
+          <t>$46.21 / 7.33%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.76 / 2.54%</t>
+          <t>$44.75 / 2.52%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.17 / 2.48%</t>
+          <t>$42.16 / 2.46%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.26 / 8.98%</t>
+          <t>$45.30 / 9.07%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.13 / 3.49%</t>
+          <t>$44.14 / 3.52%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.90 / 10.78%</t>
+          <t>$42.92 / 10.83%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.68 / 10.67%</t>
+          <t>$42.73 / 10.80%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$773.97 / 8.99%</t>
+          <t>$773.44 / 8.91%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$773.97 / 1.08%</t>
+          <t>$773.44 / 1.01%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$773.97 / 13.72%</t>
+          <t>$773.44 / 13.64%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$773.97 / 12.26%</t>
+          <t>$773.44 / 12.18%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$773.97 / 11.90%</t>
+          <t>$773.44 / 11.82%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$773.97 / 4.13%</t>
+          <t>$773.44 / 4.06%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$773.97 / 3.65%</t>
+          <t>$773.44 / 3.57%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$773.97 / 19.33%</t>
+          <t>$773.44 / 19.25%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$773.97 / 4.71%</t>
+          <t>$773.44 / 4.64%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$773.97 / 17.44%</t>
+          <t>$773.44 / 17.36%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$773.97 / 16.49%</t>
+          <t>$773.44 / 16.41%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$773.97 / 1.61%</t>
+          <t>$773.44 / 1.54%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$773.97 / 8.99%</t>
+          <t>$773.44 / 8.91%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$773.97 / 1.08%</t>
+          <t>$773.44 / 1.01%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$773.97 / 13.72%</t>
+          <t>$773.44 / 13.64%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$773.97 / 12.26%</t>
+          <t>$773.44 / 12.18%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$773.97 / 11.90%</t>
+          <t>$773.44 / 11.82%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$773.97 / 4.13%</t>
+          <t>$773.44 / 4.06%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$773.97 / 3.65%</t>
+          <t>$773.44 / 3.57%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$773.97 / 19.33%</t>
+          <t>$773.44 / 19.25%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$773.97 / 4.71%</t>
+          <t>$773.44 / 4.64%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$773.97 / 17.44%</t>
+          <t>$773.44 / 17.36%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$773.97 / 16.49%</t>
+          <t>$773.44 / 16.41%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$773.97 / 1.61%</t>
+          <t>$773.44 / 1.54%</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.14% (7.68%)</t>
+          <t>8.13% (7.68%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2590,112 +2590,112 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.62% (3.43%)</t>
+          <t>3.51% (3.32%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.53% (5.20%)</t>
+          <t>5.50% (5.18%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.72% (4.47%)</t>
+          <t>4.71% (4.46%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.23% (12.56%)</t>
+          <t>13.27% (12.59%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.96% (12.35%)</t>
+          <t>12.99% (12.39%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.98% (4.61%)</t>
+          <t>4.99% (4.62%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.22% (11.68%)</t>
+          <t>12.27% (11.73%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.27% (2.15%)</t>
+          <t>2.19% (2.07%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.98% (0.93%)</t>
+          <t>0.88% (0.83%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.73% (14.90%)</t>
+          <t>15.71% (14.88%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.61% (6.15%)</t>
+          <t>6.56% (6.10%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.85% (12.08%)</t>
+          <t>12.88% (12.12%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.74% (2.55%)</t>
+          <t>2.64% (2.45%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.39% (4.06%)</t>
+          <t>4.35% (4.02%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.67% (3.42%)</t>
+          <t>3.64% (3.39%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.85% (10.18%)</t>
+          <t>10.88% (10.20%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.39% (9.78%)</t>
+          <t>10.42% (9.81%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.30% (3.92%)</t>
+          <t>4.22% (3.84%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.71% (9.16%)</t>
+          <t>9.67% (9.13%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.59% (1.47%)</t>
+          <t>1.54% (1.42%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.62% (0.57%)</t>
+          <t>0.50% (0.45%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.31% (12.47%)</t>
+          <t>13.30% (12.47%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.74%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.98%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.35%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>12.27%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.81%</t>
+          <t>-1.75%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.90%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.20%</t>
+          <t>-1.14%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.83%</t>
+          <t>14.91%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.38%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.50%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-3.67%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.28%</t>
+          <t>12.36%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.28% (10.82%)</t>
+          <t>11.22% (10.77%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.93% (9.16%)</t>
+          <t>9.87% (9.10%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.08% (10.90%)</t>
+          <t>10.93% (10.75%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.53% (11.20%)</t>
+          <t>11.45% (11.13%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.94% (10.69%)</t>
+          <t>10.87% (10.63%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.47% (9.80%)</t>
+          <t>10.44% (9.77%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.14% (9.53%)</t>
+          <t>10.11% (9.50%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.12% (13.75%)</t>
+          <t>14.08% (13.71%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.85% (9.31%)</t>
+          <t>9.83% (9.29%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.97% (10.85%)</t>
+          <t>10.85% (10.73%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.39% (10.34%)</t>
+          <t>10.25% (10.20%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.62% (9.78%)</t>
+          <t>10.54% (9.70%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.87% (16.41%)</t>
+          <t>16.77% (16.31%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.10% (14.33%)</t>
+          <t>15.08% (14.31%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.85% (16.66%)</t>
+          <t>16.71% (16.52%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.39% (17.06%)</t>
+          <t>17.31% (16.98%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.70% (16.45%)</t>
+          <t>16.62% (16.37%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.74% (15.06%)</t>
+          <t>15.71% (15.03%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.35% (14.74%)</t>
+          <t>15.32% (14.71%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.14% (19.75%)</t>
+          <t>20.01% (19.63%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.16% (14.62%)</t>
+          <t>15.07% (14.53%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.25% (17.13%)</t>
+          <t>17.16% (17.03%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.68% (16.63%)</t>
+          <t>16.52% (16.47%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.68% (14.84%)</t>
+          <t>15.62% (14.79%)</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.14% (-6.60%)</t>
+          <t>-6.15% (-6.60%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2971,107 +2971,107 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.77% (-9.96%)</t>
+          <t>-9.87% (-10.06%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.30% (-8.63%)</t>
+          <t>-8.33% (-8.65%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.63% (-8.88%)</t>
+          <t>-8.64% (-8.89%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.09% (-3.77%)</t>
+          <t>-3.06% (-3.74%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.03% (-3.64%)</t>
+          <t>-3.00% (-3.61%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.46% (-10.83%)</t>
+          <t>-10.45% (-10.82%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.20% (-4.74%)</t>
+          <t>-4.16% (-4.70%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.39% (-12.51%)</t>
+          <t>-12.46% (-12.58%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.35% (-12.40%)</t>
+          <t>-12.44% (-12.49%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.81% (-1.65%)</t>
+          <t>-0.83% (-1.66%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.14% (-5.60%)</t>
+          <t>-5.19% (-5.64%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.80% (-1.57%)</t>
+          <t>-0.77% (-1.54%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.40% (-8.59%)</t>
+          <t>-8.49% (-8.68%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.89% (-7.22%)</t>
+          <t>-6.92% (-7.25%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.33% (-7.58%)</t>
+          <t>-7.37% (-7.61%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.62% (-3.30%)</t>
+          <t>-2.60% (-3.28%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.63% (-3.25%)</t>
+          <t>-2.61% (-3.22%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.63% (-9.02%)</t>
+          <t>-8.71% (-9.09%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.66% (-4.20%)</t>
+          <t>-3.69% (-4.23%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.37% (-10.49%)</t>
+          <t>-10.41% (-10.54%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.35% (-10.40%)</t>
+          <t>-10.46% (-10.51%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.42%</t>
+          <t>-17.36%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.96%</t>
+          <t>-10.90%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.86%</t>
+          <t>-20.80%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.83%</t>
+          <t>-19.77%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.57%</t>
+          <t>-19.52%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.57%</t>
+          <t>-13.51%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.17%</t>
+          <t>-13.11%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.58%</t>
+          <t>-24.53%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.05%</t>
+          <t>-13.99%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.36%</t>
+          <t>-23.31%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.74%</t>
+          <t>-22.69%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.43%</t>
+          <t>-11.37%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.01%</t>
+          <t>-21.95%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.90%</t>
+          <t>-15.85%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.25%</t>
+          <t>-25.20%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.28%</t>
+          <t>-24.23%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.04%</t>
+          <t>-23.98%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.37%</t>
+          <t>-18.31%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.99%</t>
+          <t>-17.93%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.77%</t>
+          <t>-28.72%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.82%</t>
+          <t>-18.76%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.62%</t>
+          <t>-27.57%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.03%</t>
+          <t>-26.98%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.35%</t>
+          <t>-16.29%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.32% (1.87%)</t>
+          <t>2.25% (1.80%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.04% (-0.73%)</t>
+          <t>-0.03% (-0.80%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.68% (2.50%)</t>
+          <t>2.50% (2.32%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.00% (2.67%)</t>
+          <t>2.90% (2.58%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.30% (2.05%)</t>
+          <t>2.22% (1.97%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.91% (0.24%)</t>
+          <t>0.87% (0.20%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.51% (-0.09%)</t>
+          <t>0.48% (-0.13%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.98% (4.61%)</t>
+          <t>4.99% (4.62%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.32% (-0.22%)</t>
+          <t>0.30% (-0.24%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.27% (2.15%)</t>
+          <t>2.19% (2.07%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.98% (0.93%)</t>
+          <t>0.88% (0.83%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.79% (-0.05%)</t>
+          <t>0.70% (-0.13%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.41% (2.96%)</t>
+          <t>3.29% (2.84%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.26% (-0.51%)</t>
+          <t>0.23% (-0.54%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.74% (2.55%)</t>
+          <t>2.64% (2.45%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.39% (4.06%)</t>
+          <t>4.35% (4.02%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.67% (3.42%)</t>
+          <t>3.64% (3.39%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.40% (0.72%)</t>
+          <t>1.35% (0.67%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.92% (0.31%)</t>
+          <t>0.87% (0.26%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.30% (3.92%)</t>
+          <t>4.22% (3.84%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.89% (0.35%)</t>
+          <t>0.79% (0.24%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.59% (1.47%)</t>
+          <t>1.54% (1.42%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.62% (0.57%)</t>
+          <t>0.50% (0.45%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.91% (0.08%)</t>
+          <t>0.84% (0.01%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/9/2026</t>
+          <t>As of 22/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.47%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.90%</t>
+          <t>11.82%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.35%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.88%</t>
+          <t>-8.89%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>5.18%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.51%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.63%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.75%</t>
+          <t>13.71%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.62%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.33%</t>
+          <t>19.25%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.81%</t>
+          <t>-1.75%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.83%</t>
+          <t>-10.82%</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3536,12 +3536,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.74%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>11.73%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.64%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.90%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.74%</t>
+          <t>-4.70%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.53%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.90%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.64%</t>
+          <t>-3.61%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>12.27%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.77%</t>
+          <t>-3.74%</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.16%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>14.88%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.83%</t>
+          <t>14.91%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.65%</t>
+          <t>-1.66%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.34%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.19%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.20%</t>
+          <t>-1.14%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.40%</t>
+          <t>-12.49%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.07%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.34%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.44%</t>
+          <t>17.36%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.51%</t>
+          <t>-12.58%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.90%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.72%</t>
+          <t>13.64%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.98%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.96%</t>
+          <t>-10.06%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/9/2026</t>
+          <t>As of 22/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.45%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.90%</t>
+          <t>11.82%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.58%</t>
+          <t>-7.61%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.06%</t>
+          <t>16.98%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.87%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.26%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.19%</t>
+          <t>-0.12%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.22%</t>
+          <t>-7.25%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.75%</t>
+          <t>19.63%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.92%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.33%</t>
+          <t>19.25%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.38%</t>
+          <t>-4.32%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.02%</t>
+          <t>-9.09%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.15%</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.04%</t>
+          <t>5.08%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.60%</t>
+          <t>-5.64%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.62%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.16%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>4.64%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.20%</t>
+          <t>-4.23%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.74%</t>
+          <t>14.71%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.46%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-3.22%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.06%</t>
+          <t>15.03%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>2.52%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.13%</t>
+          <t>4.06%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.30%</t>
+          <t>-3.28%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.31%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>12.12%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.74%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.57%</t>
+          <t>-1.54%</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.84%</t>
+          <t>14.79%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.28%</t>
+          <t>12.36%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.63%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.80%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-3.67%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.40%</t>
+          <t>-10.51%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.13%</t>
+          <t>17.03%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.78%</t>
+          <t>10.83%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.44%</t>
+          <t>17.36%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.50%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.49%</t>
+          <t>-10.54%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.66%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.55%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.72%</t>
+          <t>13.64%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-1.37%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.59%</t>
+          <t>-8.68%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-23]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/22/2026 at 1:32 PM ET)</t>
+          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>14.09% (13.24%)</t>
+          <t>14.07% (13.22%)</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>15.02% (14.17%)</t>
+          <t>15.00% (14.15%)</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>$47.61</t>
+          <t>$47.60</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.06 / 6.16%</t>
+          <t>$47.93 / 5.88%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.09 / 0.96%</t>
+          <t>$57.87 / 0.59%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.23 / 10.24%</t>
+          <t>$56.06 / 9.90%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.86 / 8.54%</t>
+          <t>$62.71 / 8.27%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.88 / 8.83%</t>
+          <t>$56.74 / 8.56%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.64 / 3.00%</t>
+          <t>$61.44 / 2.66%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.59 / 2.86%</t>
+          <t>$61.36 / 2.48%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.72 / 11.19%</t>
+          <t>$53.63 / 10.99%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.80 / 4.02%</t>
+          <t>$57.61 / 3.68%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.39 / 13.42%</t>
+          <t>$60.24 / 13.13%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.24 / 13.30%</t>
+          <t>$54.11 / 13.04%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.55 / 0.83%</t>
+          <t>$57.34 / 0.45%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.71 / 5.08%</t>
+          <t>$42.64 / 4.90%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.31 / 0.70%</t>
+          <t>$42.21 / 0.47%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.92 / 8.58%</t>
+          <t>$40.84 / 8.35%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.14 / 6.90%</t>
+          <t>$45.06 / 6.73%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.21 / 7.33%</t>
+          <t>$46.13 / 7.14%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.75 / 2.52%</t>
+          <t>$44.63 / 2.25%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.16 / 2.46%</t>
+          <t>$42.05 / 2.19%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.30 / 9.07%</t>
+          <t>$45.24 / 8.93%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.14 / 3.52%</t>
+          <t>$44.03 / 3.25%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.92 / 10.83%</t>
+          <t>$42.86 / 10.69%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.73 / 10.80%</t>
+          <t>$42.69 / 10.68%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.33 / 0.69%</t>
+          <t>$42.23 / 0.45%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$773.44 / 8.91%</t>
+          <t>$768.68 / 8.24%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$773.44 / 1.01%</t>
+          <t>$768.68 / 0.39%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$773.44 / 13.64%</t>
+          <t>$768.68 / 12.94%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$773.44 / 12.18%</t>
+          <t>$768.68 / 11.49%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$773.44 / 11.82%</t>
+          <t>$768.68 / 11.13%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$773.44 / 4.06%</t>
+          <t>$768.68 / 3.42%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$773.44 / 3.57%</t>
+          <t>$768.68 / 2.94%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$773.44 / 19.25%</t>
+          <t>$768.68 / 18.52%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$773.44 / 4.64%</t>
+          <t>$768.68 / 3.99%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$773.44 / 17.36%</t>
+          <t>$768.68 / 16.64%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$773.44 / 16.41%</t>
+          <t>$768.68 / 15.70%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$773.44 / 1.54%</t>
+          <t>$768.68 / 0.92%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$773.44 / 8.91%</t>
+          <t>$768.68 / 8.24%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$773.44 / 1.01%</t>
+          <t>$768.68 / 0.39%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$773.44 / 13.64%</t>
+          <t>$768.68 / 12.94%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$773.44 / 12.18%</t>
+          <t>$768.68 / 11.49%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$773.44 / 11.82%</t>
+          <t>$768.68 / 11.13%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$773.44 / 4.06%</t>
+          <t>$768.68 / 3.42%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$773.44 / 3.57%</t>
+          <t>$768.68 / 2.94%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$773.44 / 19.25%</t>
+          <t>$768.68 / 18.52%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$773.44 / 4.64%</t>
+          <t>$768.68 / 3.99%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$773.44 / 17.36%</t>
+          <t>$768.68 / 16.64%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$773.44 / 16.41%</t>
+          <t>$768.68 / 15.70%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$773.44 / 1.54%</t>
+          <t>$768.68 / 0.92%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.13% (7.68%)</t>
+          <t>8.41% (7.96%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.98% (15.21%)</t>
+          <t>16.41% (15.64%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.51% (3.32%)</t>
+          <t>3.83% (3.65%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.50% (5.18%)</t>
+          <t>5.76% (5.44%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.71% (4.46%)</t>
+          <t>4.96% (4.72%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.27% (12.59%)</t>
+          <t>13.64% (12.97%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.99% (12.39%)</t>
+          <t>13.41% (12.81%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.99% (4.62%)</t>
+          <t>5.18% (4.80%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.27% (11.73%)</t>
+          <t>12.64% (12.10%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.19% (2.07%)</t>
+          <t>2.46% (2.34%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.88% (0.83%)</t>
+          <t>1.11% (1.07%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.71% (14.88%)</t>
+          <t>16.14% (15.31%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.56% (6.10%)</t>
+          <t>6.74% (6.29%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.88% (12.12%)</t>
+          <t>13.15% (12.38%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.64% (2.45%)</t>
+          <t>2.85% (2.66%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.35% (4.02%)</t>
+          <t>4.52% (4.20%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.64% (3.39%)</t>
+          <t>3.82% (3.57%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.88% (10.20%)</t>
+          <t>11.16% (10.49%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.42% (9.81%)</t>
+          <t>10.70% (10.09%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.22% (3.84%)</t>
+          <t>4.35% (3.97%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.67% (9.13%)</t>
+          <t>9.95% (9.41%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.54% (1.42%)</t>
+          <t>1.67% (1.55%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.50% (0.45%)</t>
+          <t>0.60% (0.56%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.30% (12.47%)</t>
+          <t>13.55% (12.72%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.74%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>16.72%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.98%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-1.14%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.90%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.91%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.32%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-2.90%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.67%</t>
+          <t>-3.07%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>13.05%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.22% (10.77%)</t>
+          <t>10.95% (10.50%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.87% (9.10%)</t>
+          <t>9.68% (8.92%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.93% (10.75%)</t>
+          <t>10.72% (10.54%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.45% (11.13%)</t>
+          <t>11.18% (10.85%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.87% (10.63%)</t>
+          <t>10.60% (10.35%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.44% (9.77%)</t>
+          <t>10.23% (9.56%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.11% (9.50%)</t>
+          <t>9.93% (9.32%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.08% (13.71%)</t>
+          <t>13.77% (13.40%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.83% (9.29%)</t>
+          <t>9.61% (9.07%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.85% (10.73%)</t>
+          <t>10.60% (10.48%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.25% (10.20%)</t>
+          <t>9.97% (9.93%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.54% (9.70%)</t>
+          <t>10.36% (9.52%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.77% (16.31%)</t>
+          <t>16.45% (15.99%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.08% (14.31%)</t>
+          <t>14.79% (14.02%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.71% (16.52%)</t>
+          <t>16.44% (16.25%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.31% (16.98%)</t>
+          <t>16.99% (16.67%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.62% (16.37%)</t>
+          <t>16.31% (16.06%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.71% (15.03%)</t>
+          <t>15.45% (14.77%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.32% (14.71%)</t>
+          <t>15.06% (14.45%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.01% (19.63%)</t>
+          <t>19.68% (19.30%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.07% (14.53%)</t>
+          <t>14.82% (14.28%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.16% (17.03%)</t>
+          <t>16.82% (16.70%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.52% (16.47%)</t>
+          <t>16.16% (16.12%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.62% (14.79%)</t>
+          <t>15.31% (14.48%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.15% (-6.60%)</t>
+          <t>-5.90% (-6.36%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.03% (-1.79%)</t>
+          <t>-0.66% (-1.43%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.87% (-10.06%)</t>
+          <t>-9.59% (-9.78%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.33% (-8.65%)</t>
+          <t>-8.10% (-8.42%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.64% (-8.89%)</t>
+          <t>-8.42% (-8.66%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.06% (-3.74%)</t>
+          <t>-2.74% (-3.41%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.00% (-3.61%)</t>
+          <t>-2.64% (-3.25%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.45% (-10.82%)</t>
+          <t>-10.29% (-10.67%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.16% (-4.70%)</t>
+          <t>-3.85% (-4.39%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.46% (-12.58%)</t>
+          <t>-12.24% (-12.35%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.44% (-12.49%)</t>
+          <t>-12.24% (-12.28%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.83% (-1.66%)</t>
+          <t>-0.46% (-1.29%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.19% (-5.64%)</t>
+          <t>-5.02% (-5.48%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.77% (-1.54%)</t>
+          <t>-0.54% (-1.30%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.49% (-8.68%)</t>
+          <t>-8.30% (-8.49%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.92% (-7.25%)</t>
+          <t>-6.77% (-7.09%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.37% (-7.61%)</t>
+          <t>-7.21% (-7.45%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.60% (-3.28%)</t>
+          <t>-2.36% (-3.03%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.61% (-3.22%)</t>
+          <t>-2.36% (-2.97%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.71% (-9.09%)</t>
+          <t>-8.60% (-8.98%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.69% (-4.23%)</t>
+          <t>-3.44% (-3.98%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.41% (-10.54%)</t>
+          <t>-10.30% (-10.42%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.46% (-10.51%)</t>
+          <t>-10.36% (-10.41%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.67% (-1.50%)</t>
+          <t>-0.46% (-1.29%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.36%</t>
+          <t>-16.85%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.90%</t>
+          <t>-10.35%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.80%</t>
+          <t>-20.31%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.77%</t>
+          <t>-19.28%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.52%</t>
+          <t>-19.02%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.51%</t>
+          <t>-12.97%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.11%</t>
+          <t>-12.57%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.53%</t>
+          <t>-24.06%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.99%</t>
+          <t>-13.45%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.31%</t>
+          <t>-22.84%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.69%</t>
+          <t>-22.21%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.37%</t>
+          <t>-10.82%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.95%</t>
+          <t>-21.47%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.85%</t>
+          <t>-15.32%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.20%</t>
+          <t>-24.74%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.23%</t>
+          <t>-23.76%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.98%</t>
+          <t>-23.51%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.31%</t>
+          <t>-17.80%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.93%</t>
+          <t>-17.42%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.72%</t>
+          <t>-28.28%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.76%</t>
+          <t>-18.26%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.57%</t>
+          <t>-27.12%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.98%</t>
+          <t>-26.53%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.29%</t>
+          <t>-15.77%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.25% (1.80%)</t>
+          <t>1.88% (1.43%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.80%)</t>
+          <t>-0.28% (-1.05%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.50% (2.32%)</t>
+          <t>2.18% (2.00%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.90% (2.58%)</t>
+          <t>2.51% (2.19%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.22% (1.97%)</t>
+          <t>1.84% (1.59%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.87% (0.20%)</t>
+          <t>0.58% (-0.09%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.48% (-0.13%)</t>
+          <t>0.23% (-0.38%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.99% (4.62%)</t>
+          <t>5.18% (4.80%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.30% (-0.24%)</t>
+          <t>0.00% (-0.54%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.19% (2.07%)</t>
+          <t>2.46% (2.34%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.88% (0.83%)</t>
+          <t>1.11% (1.07%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.70% (-0.13%)</t>
+          <t>0.45% (-0.38%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.29% (2.84%)</t>
+          <t>2.83% (2.38%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.23% (-0.54%)</t>
+          <t>-0.16% (-0.92%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.64% (2.45%)</t>
+          <t>2.85% (2.66%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.35% (4.02%)</t>
+          <t>4.00% (3.67%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.64% (3.39%)</t>
+          <t>3.18% (2.94%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.35% (0.67%)</t>
+          <t>0.98% (0.31%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.87% (0.26%)</t>
+          <t>0.51% (-0.10%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.22% (3.84%)</t>
+          <t>4.35% (3.97%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.79% (0.24%)</t>
+          <t>0.42% (-0.12%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.54% (1.42%)</t>
+          <t>1.67% (1.55%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.50% (0.45%)</t>
+          <t>0.60% (0.56%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.84% (0.01%)</t>
+          <t>0.44% (-0.40%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/9/2026</t>
+          <t>As of 23/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.72%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>8.56%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.89%</t>
+          <t>-8.66%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.18%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.42%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.71%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.62%</t>
+          <t>4.80%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.25%</t>
+          <t>18.52%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-1.14%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.82%</t>
+          <t>-10.67%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>10.50%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>7.96%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.16%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.74%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.60%</t>
+          <t>-6.36%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.73%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.64%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.90%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.70%</t>
+          <t>-4.39%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-3.41%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>15.64%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>0.59%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>16.72%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.43%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.52%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.88%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.91%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-1.29%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>15.70%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-0.52%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.49%</t>
+          <t>-12.28%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.07%</t>
+          <t>2.34%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.36%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.58%</t>
+          <t>-12.35%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.64%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.98%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.06%</t>
+          <t>-9.78%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/9/2026</t>
+          <t>As of 23/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.61%</t>
+          <t>-7.45%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.98%</t>
+          <t>16.67%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>6.73%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>11.49%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.12%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.25%</t>
+          <t>-7.09%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.63%</t>
+          <t>19.30%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.25%</t>
+          <t>18.52%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-3.73%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.09%</t>
+          <t>-8.98%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.31%</t>
+          <t>15.99%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.08%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>8.24%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.64%</t>
+          <t>-5.48%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.28%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.64%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-3.98%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.71%</t>
+          <t>14.45%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.46%</t>
+          <t>2.19%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.22%</t>
+          <t>-2.97%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.03%</t>
+          <t>14.77%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.49%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.52%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.06%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-3.03%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.31%</t>
+          <t>14.02%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.12%</t>
+          <t>12.38%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.70%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.32%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.54%</t>
+          <t>-1.30%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.79%</t>
+          <t>14.48%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.47%</t>
+          <t>12.72%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.50%</t>
+          <t>-1.29%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.56%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.80%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>15.70%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.67%</t>
+          <t>-3.07%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.51%</t>
+          <t>-10.41%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.03%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.42%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.83%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.36%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-2.90%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.54%</t>
+          <t>-10.42%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.45%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>8.35%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.64%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.68%</t>
+          <t>-8.49%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-24]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/23/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>14.07% (13.22%)</t>
+          <t>14.09% (13.24%)</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>15.00% (14.15%)</t>
+          <t>15.02% (14.17%)</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>$47.60</t>
+          <t>$47.61</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
     </row>
@@ -2326,77 +2326,77 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.93 / 5.88%</t>
+          <t>$47.87 / 5.74%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.87 / 0.59%</t>
+          <t>$57.77 / 0.42%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.06 / 9.90%</t>
+          <t>$56.01 / 9.80%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.71 / 8.27%</t>
+          <t>$62.63 / 8.13%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.74 / 8.56%</t>
+          <t>$56.65 / 8.39%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.44 / 2.66%</t>
+          <t>$61.35 / 2.51%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.36 / 2.48%</t>
+          <t>$61.31 / 2.39%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.63 / 10.99%</t>
+          <t>$53.64 / 11.01%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.61 / 3.68%</t>
+          <t>$57.49 / 3.47%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.24 / 13.13%</t>
+          <t>$60.23 / 13.11%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.11 / 13.04%</t>
+          <t>$54.08 / 12.96%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.34 / 0.45%</t>
+          <t>$57.24 / 0.28%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.64 / 4.90%</t>
+          <t>$42.58 / 4.75%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.21 / 0.47%</t>
+          <t>$42.15 / 0.34%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.84 / 8.35%</t>
+          <t>$40.79 / 8.23%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2406,42 +2406,42 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.13 / 7.14%</t>
+          <t>$46.12 / 7.12%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.63 / 2.25%</t>
+          <t>$44.57 / 2.10%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.05 / 2.19%</t>
+          <t>$42.01 / 2.08%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.24 / 8.93%</t>
+          <t>$45.21 / 8.86%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.03 / 3.25%</t>
+          <t>$43.97 / 3.11%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.86 / 10.69%</t>
+          <t>$42.85 / 10.65%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.69 / 10.68%</t>
+          <t>$42.69 / 10.69%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.23 / 0.45%</t>
+          <t>$42.18 / 0.33%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$768.68 / 8.24%</t>
+          <t>$766.19 / 7.89%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$768.68 / 0.39%</t>
+          <t>$766.19 / 0.06%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$768.68 / 12.94%</t>
+          <t>$766.19 / 12.58%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$768.68 / 11.49%</t>
+          <t>$766.19 / 11.13%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$768.68 / 11.13%</t>
+          <t>$766.19 / 10.77%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$768.68 / 3.42%</t>
+          <t>$766.19 / 3.08%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$768.68 / 2.94%</t>
+          <t>$766.19 / 2.60%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$768.68 / 18.52%</t>
+          <t>$766.19 / 18.13%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$768.68 / 3.99%</t>
+          <t>$766.19 / 3.65%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$768.68 / 16.64%</t>
+          <t>$766.19 / 16.26%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$768.68 / 15.70%</t>
+          <t>$766.19 / 15.32%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$768.68 / 0.92%</t>
+          <t>$766.19 / 0.59%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$768.68 / 8.24%</t>
+          <t>$766.19 / 7.89%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$768.68 / 0.39%</t>
+          <t>$766.19 / 0.06%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$768.68 / 12.94%</t>
+          <t>$766.19 / 12.58%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$768.68 / 11.49%</t>
+          <t>$766.19 / 11.13%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$768.68 / 11.13%</t>
+          <t>$766.19 / 10.77%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$768.68 / 3.42%</t>
+          <t>$766.19 / 3.08%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$768.68 / 2.94%</t>
+          <t>$766.19 / 2.60%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$768.68 / 18.52%</t>
+          <t>$766.19 / 18.13%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$768.68 / 3.99%</t>
+          <t>$766.19 / 3.65%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$768.68 / 16.64%</t>
+          <t>$766.19 / 16.26%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$768.68 / 15.70%</t>
+          <t>$766.19 / 15.32%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$768.68 / 0.92%</t>
+          <t>$766.19 / 0.59%</t>
         </is>
       </c>
     </row>
@@ -2580,77 +2580,77 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.41% (7.96%)</t>
+          <t>8.56% (8.11%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.41% (15.64%)</t>
+          <t>16.61% (15.84%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.83% (3.65%)</t>
+          <t>3.92% (3.74%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.76% (5.44%)</t>
+          <t>5.89% (5.57%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.96% (4.72%)</t>
+          <t>5.13% (4.89%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.64% (12.97%)</t>
+          <t>13.80% (13.13%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.41% (12.81%)</t>
+          <t>13.50% (12.90%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.18% (4.80%)</t>
+          <t>5.15% (4.78%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.64% (12.10%)</t>
+          <t>12.87% (12.33%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.46% (2.34%)</t>
+          <t>2.47% (2.35%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.11% (1.07%)</t>
+          <t>1.18% (1.13%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.14% (15.31%)</t>
+          <t>16.34% (15.51%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.74% (6.29%)</t>
+          <t>6.89% (6.44%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.15% (12.38%)</t>
+          <t>13.29% (12.53%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.85% (2.66%)</t>
+          <t>2.96% (2.78%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2660,42 +2660,42 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.82% (3.57%)</t>
+          <t>3.84% (3.59%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.16% (10.49%)</t>
+          <t>11.32% (10.65%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.70% (10.09%)</t>
+          <t>10.82% (10.21%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.35% (3.97%)</t>
+          <t>4.41% (4.04%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.95% (9.41%)</t>
+          <t>10.10% (9.56%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.67% (1.55%)</t>
+          <t>1.70% (1.58%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.60% (0.56%)</t>
+          <t>0.59% (0.54%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.55% (12.72%)</t>
+          <t>13.70% (12.87%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.74%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.72%</t>
+          <t>17.10%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>13.33%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>13.49%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>-0.82%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>12.96%</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>13.13%</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>-1.14%</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>12.60%</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>4.12%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.32%</t>
+          <t>13.68%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-3.41%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.82%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-2.59%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.07%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.42%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.95% (10.50%)</t>
+          <t>10.80% (10.35%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.68% (8.92%)</t>
+          <t>9.56% (8.80%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.72% (10.54%)</t>
+          <t>10.54% (10.36%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.18% (10.85%)</t>
+          <t>11.03% (10.71%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.60% (10.35%)</t>
+          <t>10.48% (10.24%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.23% (9.56%)</t>
+          <t>10.08% (9.41%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.93% (9.32%)</t>
+          <t>9.72% (9.12%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.77% (13.40%)</t>
+          <t>13.50% (13.13%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.61% (9.07%)</t>
+          <t>9.53% (8.99%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.60% (10.48%)</t>
+          <t>10.36% (10.25%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.97% (9.93%)</t>
+          <t>9.78% (9.73%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.36% (9.52%)</t>
+          <t>10.24% (9.41%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.45% (15.99%)</t>
+          <t>16.32% (15.87%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.79% (14.02%)</t>
+          <t>14.64% (13.87%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.44% (16.25%)</t>
+          <t>16.29% (16.11%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.99% (16.67%)</t>
+          <t>16.74% (16.42%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.31% (16.06%)</t>
+          <t>16.08% (15.83%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.45% (14.77%)</t>
+          <t>15.32% (14.65%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.06% (14.45%)</t>
+          <t>14.90% (14.29%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.68% (19.30%)</t>
+          <t>19.51% (19.13%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.82% (14.28%)</t>
+          <t>14.68% (14.14%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.82% (16.70%)</t>
+          <t>16.61% (16.49%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.16% (16.12%)</t>
+          <t>15.91% (15.87%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.31% (14.48%)</t>
+          <t>15.18% (14.35%)</t>
         </is>
       </c>
     </row>
@@ -2961,77 +2961,77 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.90% (-6.36%)</t>
+          <t>-5.78% (-6.23%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.66% (-1.43%)</t>
+          <t>-0.49% (-1.26%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.59% (-9.78%)</t>
+          <t>-9.52% (-9.70%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.10% (-8.42%)</t>
+          <t>-7.99% (-8.31%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.42% (-8.66%)</t>
+          <t>-8.28% (-8.52%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.74% (-3.41%)</t>
+          <t>-2.61% (-3.28%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.64% (-3.25%)</t>
+          <t>-2.56% (-3.17%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.29% (-10.67%)</t>
+          <t>-10.31% (-10.68%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.85% (-4.39%)</t>
+          <t>-3.65% (-4.19%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.24% (-12.35%)</t>
+          <t>-12.22% (-12.34%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.24% (-12.28%)</t>
+          <t>-12.18% (-12.23%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.46% (-1.29%)</t>
+          <t>-0.29% (-1.12%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.02% (-5.48%)</t>
+          <t>-4.89% (-5.34%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.54% (-1.30%)</t>
+          <t>-0.41% (-1.18%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.30% (-8.49%)</t>
+          <t>-8.20% (-8.39%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3041,42 +3041,42 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.21% (-7.45%)</t>
+          <t>-7.19% (-7.43%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.36% (-3.03%)</t>
+          <t>-2.22% (-2.89%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.36% (-2.97%)</t>
+          <t>-2.26% (-2.87%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.60% (-8.98%)</t>
+          <t>-8.54% (-8.92%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.44% (-3.98%)</t>
+          <t>-3.31% (-3.85%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.30% (-10.42%)</t>
+          <t>-10.27% (-10.39%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.36% (-10.41%)</t>
+          <t>-10.38% (-10.42%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.46% (-1.29%)</t>
+          <t>-0.32% (-1.15%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.85%</t>
+          <t>-16.58%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.35%</t>
+          <t>-10.05%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.31%</t>
+          <t>-20.05%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.28%</t>
+          <t>-19.02%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.02%</t>
+          <t>-18.75%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.97%</t>
+          <t>-12.69%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.57%</t>
+          <t>-12.28%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.06%</t>
+          <t>-23.82%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.45%</t>
+          <t>-13.17%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.84%</t>
+          <t>-22.59%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.21%</t>
+          <t>-21.96%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.82%</t>
+          <t>-10.53%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.47%</t>
+          <t>-21.21%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.32%</t>
+          <t>-15.05%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.74%</t>
+          <t>-24.49%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.76%</t>
+          <t>-23.51%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.51%</t>
+          <t>-23.27%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.80%</t>
+          <t>-17.54%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.42%</t>
+          <t>-17.15%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.28%</t>
+          <t>-28.05%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.26%</t>
+          <t>-18.00%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.12%</t>
+          <t>-26.88%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.53%</t>
+          <t>-26.29%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.77%</t>
+          <t>-15.50%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.88% (1.43%)</t>
+          <t>1.68% (1.24%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.28% (-1.05%)</t>
+          <t>-0.43% (-1.20%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.18% (2.00%)</t>
+          <t>1.94% (1.76%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.51% (2.19%)</t>
+          <t>2.31% (1.99%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.84% (1.59%)</t>
+          <t>1.66% (1.42%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.58% (-0.09%)</t>
+          <t>0.39% (-0.28%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.23% (-0.38%)</t>
+          <t>-0.02% (-0.62%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.18% (4.80%)</t>
+          <t>5.15% (4.78%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.00% (-0.54%)</t>
+          <t>-0.12% (-0.65%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.46% (2.34%)</t>
+          <t>2.15% (2.03%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.11% (1.07%)</t>
+          <t>1.18% (1.13%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.45% (-0.38%)</t>
+          <t>0.30% (-0.53%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.83% (2.38%)</t>
+          <t>2.64% (2.19%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.16% (-0.92%)</t>
+          <t>-0.35% (-1.12%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.85% (2.66%)</t>
+          <t>2.96% (2.78%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.00% (3.67%)</t>
+          <t>3.66% (3.34%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.18% (2.94%)</t>
+          <t>2.87% (2.62%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.98% (0.31%)</t>
+          <t>0.80% (0.13%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.51% (-0.10%)</t>
+          <t>0.29% (-0.32%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.35% (3.97%)</t>
+          <t>4.41% (4.04%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.42% (-0.12%)</t>
+          <t>0.23% (-0.31%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.67% (1.55%)</t>
+          <t>1.70% (1.58%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.60% (0.56%)</t>
+          <t>0.59% (0.54%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.44% (-0.40%)</t>
+          <t>0.25% (-0.58%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/9/2026</t>
+          <t>As of 24/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.72%</t>
+          <t>4.89%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.56%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.66%</t>
+          <t>-8.52%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.27%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.42%</t>
+          <t>-8.31%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.40%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.80%</t>
+          <t>4.78%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.99%</t>
+          <t>11.01%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.52%</t>
+          <t>18.13%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.67%</t>
+          <t>-10.68%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.96%</t>
+          <t>8.11%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>5.74%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>7.89%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.74%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.36%</t>
+          <t>-6.23%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.68%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.39%</t>
+          <t>-4.19%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>12.90%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.60%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.96%</t>
+          <t>13.33%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-3.28%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.64%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.72%</t>
+          <t>17.10%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>-1.26%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.52%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.59%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>16.00%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>-1.12%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>1.13%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.70%</t>
+          <t>15.32%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.28%</t>
+          <t>-12.23%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>10.25%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.34%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.11%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.35%</t>
+          <t>-12.34%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.36%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.93%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.78%</t>
+          <t>-9.70%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/9/2026</t>
+          <t>As of 24/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.45%</t>
+          <t>-7.43%</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>16.42%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.49%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.30%</t>
+          <t>19.13%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>8.86%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.52%</t>
+          <t>18.13%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-3.41%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.98%</t>
+          <t>-8.92%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.99%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>6.44%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>7.89%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>4.12%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.48%</t>
+          <t>-5.34%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.28%</t>
+          <t>14.14%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.82%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.98%</t>
+          <t>-3.85%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.45%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.21%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.19%</t>
+          <t>2.08%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.60%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.48%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.97%</t>
+          <t>-2.87%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.77%</t>
+          <t>14.65%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.49%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.03%</t>
+          <t>-2.89%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.02%</t>
+          <t>13.87%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.38%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.32%</t>
+          <t>13.68%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>-1.18%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.48%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.72%</t>
+          <t>12.87%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.59%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.56%</t>
+          <t>0.54%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.70%</t>
+          <t>15.32%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.07%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.41%</t>
+          <t>-10.42%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.90%</t>
+          <t>-2.59%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.42%</t>
+          <t>-10.39%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>16.11%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.35%</t>
+          <t>8.23%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.49%</t>
+          <t>-8.39%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-25]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/24/2026 at 1:46 PM ET)</t>
+          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>265 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>265 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.87 / 5.74%</t>
+          <t>$48.04 / 6.11%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.77 / 0.42%</t>
+          <t>$58.01 / 0.82%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.01 / 9.80%</t>
+          <t>$56.15 / 10.08%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.63 / 8.13%</t>
+          <t>$62.83 / 8.48%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.65 / 8.39%</t>
+          <t>$56.85 / 8.77%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.35 / 2.51%</t>
+          <t>$61.57 / 2.87%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.31 / 2.39%</t>
+          <t>$61.52 / 2.75%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.64 / 11.01%</t>
+          <t>$53.73 / 11.20%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.49 / 3.47%</t>
+          <t>$57.72 / 3.88%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.23 / 13.11%</t>
+          <t>$60.37 / 13.37%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.08 / 12.96%</t>
+          <t>$54.20 / 13.23%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.24 / 0.28%</t>
+          <t>$57.46 / 0.67%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.58 / 4.75%</t>
+          <t>$42.71 / 5.07%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.15 / 0.34%</t>
+          <t>$42.28 / 0.64%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.79 / 8.23%</t>
+          <t>$40.90 / 8.52%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.06 / 6.73%</t>
+          <t>$45.14 / 6.92%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.12 / 7.12%</t>
+          <t>$46.21 / 7.34%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.57 / 2.10%</t>
+          <t>$44.73 / 2.48%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.01 / 2.08%</t>
+          <t>$42.14 / 2.40%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.21 / 8.86%</t>
+          <t>$45.29 / 9.05%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.97 / 3.11%</t>
+          <t>$44.12 / 3.46%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.85 / 10.65%</t>
+          <t>$42.91 / 10.81%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.69 / 10.69%</t>
+          <t>$42.72 / 10.77%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.18 / 0.33%</t>
+          <t>$42.31 / 0.64%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$766.19 / 7.89%</t>
+          <t>$771.02 / 8.57%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$766.19 / 0.06%</t>
+          <t>$771.02 / 0.69%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$766.19 / 12.58%</t>
+          <t>$771.02 / 13.29%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$766.19 / 11.13%</t>
+          <t>$771.02 / 11.83%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$766.19 / 10.77%</t>
+          <t>$771.02 / 11.47%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$766.19 / 3.08%</t>
+          <t>$771.02 / 3.73%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$766.19 / 2.60%</t>
+          <t>$771.02 / 3.25%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$766.19 / 18.13%</t>
+          <t>$771.02 / 18.88%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$766.19 / 3.65%</t>
+          <t>$771.02 / 4.31%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$766.19 / 16.26%</t>
+          <t>$771.02 / 16.99%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$766.19 / 15.32%</t>
+          <t>$771.02 / 16.05%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$766.19 / 0.59%</t>
+          <t>$771.02 / 1.22%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$766.19 / 7.89%</t>
+          <t>$771.02 / 8.57%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$766.19 / 0.06%</t>
+          <t>$771.02 / 0.69%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$766.19 / 12.58%</t>
+          <t>$771.02 / 13.29%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$766.19 / 11.13%</t>
+          <t>$771.02 / 11.83%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$766.19 / 10.77%</t>
+          <t>$771.02 / 11.47%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$766.19 / 3.08%</t>
+          <t>$771.02 / 3.73%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$766.19 / 2.60%</t>
+          <t>$771.02 / 3.25%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$766.19 / 18.13%</t>
+          <t>$771.02 / 18.88%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$766.19 / 3.65%</t>
+          <t>$771.02 / 4.31%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$766.19 / 16.26%</t>
+          <t>$771.02 / 16.99%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$766.19 / 15.32%</t>
+          <t>$771.02 / 16.05%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$766.19 / 0.59%</t>
+          <t>$771.02 / 1.22%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.56% (8.11%)</t>
+          <t>8.17% (7.73%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.61% (15.84%)</t>
+          <t>16.13% (15.37%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.92% (3.74%)</t>
+          <t>3.65% (3.47%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.89% (5.57%)</t>
+          <t>5.55% (5.24%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.13% (4.89%)</t>
+          <t>4.76% (4.52%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.80% (13.13%)</t>
+          <t>13.40% (12.73%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.50% (12.90%)</t>
+          <t>13.11% (12.51%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.15% (4.78%)</t>
+          <t>4.98% (4.61%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.87% (12.33%)</t>
+          <t>12.42% (11.88%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.47% (2.35%)</t>
+          <t>2.23% (2.12%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.18% (1.13%)</t>
+          <t>0.94% (0.90%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.34% (15.51%)</t>
+          <t>15.89% (15.06%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.89% (6.44%)</t>
+          <t>6.56% (6.11%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.29% (12.53%)</t>
+          <t>12.94% (12.18%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.96% (2.78%)</t>
+          <t>2.68% (2.50%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.52% (4.20%)</t>
+          <t>4.33% (4.01%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.84% (3.59%)</t>
+          <t>3.62% (3.38%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.32% (10.65%)</t>
+          <t>10.91% (10.24%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.82% (10.21%)</t>
+          <t>10.47% (9.87%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.41% (4.04%)</t>
+          <t>4.23% (3.85%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.10% (9.56%)</t>
+          <t>9.73% (9.19%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.70% (1.58%)</t>
+          <t>1.56% (1.44%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.59% (0.54%)</t>
+          <t>0.52% (0.47%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.70% (12.87%)</t>
+          <t>13.35% (12.52%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.74%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.10%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.33%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.96%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>15.27%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.68%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.44%</t>
+          <t>-1.06%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-4.02%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.82%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.59%</t>
+          <t>-3.20%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-3.37%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>12.71%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.80% (10.35%)</t>
+          <t>10.99% (10.55%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.56% (8.80%)</t>
+          <t>9.72% (8.96%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.54% (10.36%)</t>
+          <t>10.80% (10.63%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.03% (10.71%)</t>
+          <t>11.24% (10.93%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.48% (10.24%)</t>
+          <t>10.66% (10.42%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.08% (9.41%)</t>
+          <t>10.28% (9.62%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.72% (9.12%)</t>
+          <t>9.94% (9.34%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.50% (13.13%)</t>
+          <t>13.83% (13.46%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.53% (8.99%)</t>
+          <t>9.68% (9.15%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.36% (10.25%)</t>
+          <t>10.64% (10.53%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.78% (9.73%)</t>
+          <t>10.06% (10.02%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.24% (9.41%)</t>
+          <t>10.41% (9.58%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.32% (15.87%)</t>
+          <t>16.53% (16.08%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.64% (13.87%)</t>
+          <t>14.86% (14.10%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.29% (16.11%)</t>
+          <t>16.51% (16.33%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.74% (16.42%)</t>
+          <t>17.05% (16.73%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.08% (15.83%)</t>
+          <t>16.36% (16.12%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.32% (14.65%)</t>
+          <t>15.48% (14.81%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.90% (14.29%)</t>
+          <t>15.11% (14.51%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.51% (19.13%)</t>
+          <t>19.79% (19.42%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.68% (14.14%)</t>
+          <t>14.87% (14.33%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.61% (16.49%)</t>
+          <t>16.95% (16.83%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.91% (15.87%)</t>
+          <t>16.31% (16.27%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.18% (14.35%)</t>
+          <t>15.40% (14.57%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.23%)</t>
+          <t>-6.11% (-6.56%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.49% (-1.26%)</t>
+          <t>-0.90% (-1.66%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.52% (-9.70%)</t>
+          <t>-9.75% (-9.93%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-7.99% (-8.31%)</t>
+          <t>-8.28% (-8.60%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.28% (-8.52%)</t>
+          <t>-8.60% (-8.84%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.61% (-3.28%)</t>
+          <t>-2.95% (-3.62%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>-2.90% (-3.50%)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-10.47% (-10.83%)</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>-4.03% (-4.57%)</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>-12.43% (-12.54%)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>-12.39% (-12.43%)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>-0.68% (-1.51%)</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>-5.18% (-5.63%)</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-0.72% (-1.48%)</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-8.45% (-8.63%)</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-6.94% (-7.26%)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-7.38% (-7.62%)</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>-2.58% (-3.25%)</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
           <t>-2.56% (-3.17%)</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>-10.31% (-10.68%)</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>-3.65% (-4.19%)</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>-12.22% (-12.34%)</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>-12.18% (-12.23%)</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>-0.29% (-1.12%)</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>-4.89% (-5.34%)</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>-0.41% (-1.18%)</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>-8.20% (-8.39%)</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-6.77% (-7.09%)</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>-7.19% (-7.43%)</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>-2.22% (-2.89%)</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>-2.26% (-2.87%)</t>
-        </is>
-      </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.54% (-8.92%)</t>
+          <t>-8.70% (-9.08%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.31% (-3.85%)</t>
+          <t>-3.64% (-4.18%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.27% (-10.39%)</t>
+          <t>-10.40% (-10.52%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.38% (-10.42%)</t>
+          <t>-10.44% (-10.49%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.32% (-1.15%)</t>
+          <t>-0.63% (-1.46%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.58%</t>
+          <t>-17.11%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.05%</t>
+          <t>-10.62%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.05%</t>
+          <t>-20.56%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.02%</t>
+          <t>-19.52%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.75%</t>
+          <t>-19.26%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.69%</t>
+          <t>-13.24%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.28%</t>
+          <t>-12.83%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.82%</t>
+          <t>-24.29%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.17%</t>
+          <t>-13.72%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.59%</t>
+          <t>-23.07%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.96%</t>
+          <t>-22.45%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.53%</t>
+          <t>-11.09%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.21%</t>
+          <t>-21.71%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.05%</t>
+          <t>-15.58%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.49%</t>
+          <t>-24.97%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.51%</t>
+          <t>-23.99%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.27%</t>
+          <t>-23.75%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.54%</t>
+          <t>-18.05%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.15%</t>
+          <t>-17.67%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.05%</t>
+          <t>-28.50%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.00%</t>
+          <t>-18.51%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.88%</t>
+          <t>-27.34%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.29%</t>
+          <t>-26.75%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.50%</t>
+          <t>-16.03%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.68% (1.24%)</t>
+          <t>1.96% (1.52%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.43% (-1.20%)</t>
+          <t>-0.21% (-0.97%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.94% (1.76%)</t>
+          <t>2.32% (2.14%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.31% (1.99%)</t>
+          <t>2.63% (2.31%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.66% (1.42%)</t>
+          <t>1.95% (1.71%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.39% (-0.28%)</t>
+          <t>0.67% (0.01%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.62%)</t>
+          <t>0.27% (-0.33%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.15% (4.78%)</t>
+          <t>4.98% (4.61%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.12% (-0.65%)</t>
+          <t>0.11% (-0.42%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.15% (2.03%)</t>
+          <t>2.23% (2.12%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.18% (1.13%)</t>
+          <t>0.94% (0.90%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.30% (-0.53%)</t>
+          <t>0.53% (-0.29%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.64% (2.19%)</t>
+          <t>2.97% (2.52%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.35% (-1.12%)</t>
+          <t>-0.03% (-0.79%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.96% (2.78%)</t>
+          <t>2.68% (2.50%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.66% (3.34%)</t>
+          <t>4.13% (3.81%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.87% (2.62%)</t>
+          <t>3.30% (3.06%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.80% (0.13%)</t>
+          <t>1.06% (0.39%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.29% (-0.32%)</t>
+          <t>0.61% (0.01%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.41% (4.04%)</t>
+          <t>4.23% (3.85%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.23% (-0.31%)</t>
+          <t>0.52% (-0.02%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.70% (1.58%)</t>
+          <t>1.56% (1.44%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.59% (0.54%)</t>
+          <t>0.52% (0.47%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.25% (-0.58%)</t>
+          <t>0.57% (-0.26%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 24/9/2026</t>
+          <t>As of 25/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.89%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.39%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-8.84%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>5.24%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.31%</t>
+          <t>-8.60%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.46%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.78%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.01%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.13%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.68%</t>
+          <t>-10.83%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.11%</t>
+          <t>7.73%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.74%</t>
+          <t>6.11%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.89%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.74%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.23%</t>
+          <t>-6.56%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>11.88%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.96%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-4.57%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.34%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.90%</t>
+          <t>12.51%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.60%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-3.50%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.73%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.87%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.33%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-3.62%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.96%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>15.37%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.10%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.66%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>15.06%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.00%</t>
+          <t>15.27%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-1.51%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.13%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.96%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.32%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.23%</t>
+          <t>-12.43%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>10.53%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.35%</t>
+          <t>2.12%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.11%</t>
+          <t>13.37%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.34%</t>
+          <t>-12.54%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.36%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.70%</t>
+          <t>-9.93%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 24/9/2026</t>
+          <t>As of 25/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>7.34%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.43%</t>
+          <t>-7.62%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.42%</t>
+          <t>16.73%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.73%</t>
+          <t>6.92%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.09%</t>
+          <t>-7.26%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.13%</t>
+          <t>19.42%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.86%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.13%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-4.02%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.92%</t>
+          <t>-9.08%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.44%</t>
+          <t>6.11%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>5.07%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.89%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.34%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.14%</t>
+          <t>14.33%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.82%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-4.18%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>14.51%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.21%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.08%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.60%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.48%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.87%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.65%</t>
+          <t>14.81%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.89%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.87%</t>
+          <t>14.10%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.06%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.68%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.48%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>14.57%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.87%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.59%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.46%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.32%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-3.37%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.42%</t>
+          <t>-10.49%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.81%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.59%</t>
+          <t>-3.20%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.39%</t>
+          <t>-10.52%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.11%</t>
+          <t>16.33%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.23%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.58%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.44%</t>
+          <t>-1.06%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.39%</t>
+          <t>-8.63%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-28]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/25/2026 at 1:52 PM ET)</t>
+          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>203 days</t>
+          <t>200 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>326 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>112 days</t>
+          <t>109 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>294 days</t>
+          <t>291 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>265 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>235 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>18 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>203 days</t>
+          <t>200 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>326 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>112 days</t>
+          <t>109 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>294 days</t>
+          <t>291 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>265 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>235 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>18 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.04 / 6.11%</t>
+          <t>$47.89 / 5.78%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.01 / 0.82%</t>
+          <t>$57.73 / 0.35%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.15 / 10.08%</t>
+          <t>$56.05 / 9.89%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.83 / 8.48%</t>
+          <t>$62.65 / 8.18%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.85 / 8.77%</t>
+          <t>$56.68 / 8.44%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.57 / 2.87%</t>
+          <t>$61.33 / 2.47%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.52 / 2.75%</t>
+          <t>$61.24 / 2.28%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.73 / 11.20%</t>
+          <t>$53.65 / 11.03%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.72 / 3.88%</t>
+          <t>$57.47 / 3.43%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.37 / 13.37%</t>
+          <t>$60.23 / 13.11%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.20 / 13.23%</t>
+          <t>$54.10 / 13.01%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.46 / 0.67%</t>
+          <t>$57.24 / 0.28%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.71 / 5.07%</t>
+          <t>$42.60 / 4.80%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.28 / 0.64%</t>
+          <t>$42.16 / 0.35%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.90 / 8.52%</t>
+          <t>$40.83 / 8.32%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.14 / 6.92%</t>
+          <t>$45.05 / 6.70%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.21 / 7.34%</t>
+          <t>$46.13 / 7.15%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.73 / 2.48%</t>
+          <t>$44.58 / 2.13%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.14 / 2.40%</t>
+          <t>$41.99 / 2.03%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.29 / 9.05%</t>
+          <t>$45.23 / 8.91%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.12 / 3.46%</t>
+          <t>$43.97 / 3.11%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.91 / 10.81%</t>
+          <t>$42.89 / 10.77%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.72 / 10.77%</t>
+          <t>$42.72 / 10.76%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.31 / 0.64%</t>
+          <t>$42.18 / 0.32%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$771.02 / 8.57%</t>
+          <t>$765.52 / 7.80%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$771.02 / 0.69%</t>
+          <t>$765.52 / -0.03%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$771.02 / 13.29%</t>
+          <t>$765.52 / 12.48%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$771.02 / 11.83%</t>
+          <t>$765.52 / 11.04%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$771.02 / 11.47%</t>
+          <t>$765.52 / 10.68%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$771.02 / 3.73%</t>
+          <t>$765.52 / 2.99%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$771.02 / 3.25%</t>
+          <t>$765.52 / 2.51%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$771.02 / 18.88%</t>
+          <t>$765.52 / 18.03%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$771.02 / 4.31%</t>
+          <t>$765.52 / 3.56%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$771.02 / 16.99%</t>
+          <t>$765.52 / 16.16%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$771.02 / 16.05%</t>
+          <t>$765.52 / 15.22%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$771.02 / 1.22%</t>
+          <t>$765.52 / 0.50%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$771.02 / 8.57%</t>
+          <t>$765.52 / 7.80%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$771.02 / 0.69%</t>
+          <t>$765.52 / -0.03%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$771.02 / 13.29%</t>
+          <t>$765.52 / 12.48%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$771.02 / 11.83%</t>
+          <t>$765.52 / 11.04%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$771.02 / 11.47%</t>
+          <t>$765.52 / 10.68%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$771.02 / 3.73%</t>
+          <t>$765.52 / 2.99%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$771.02 / 3.25%</t>
+          <t>$765.52 / 2.51%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$771.02 / 18.88%</t>
+          <t>$765.52 / 18.03%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$771.02 / 4.31%</t>
+          <t>$765.52 / 3.56%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$771.02 / 16.99%</t>
+          <t>$765.52 / 16.16%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$771.02 / 16.05%</t>
+          <t>$765.52 / 15.22%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$771.02 / 1.22%</t>
+          <t>$765.52 / 0.50%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.17% (7.73%)</t>
+          <t>8.50% (8.06%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.13% (15.37%)</t>
+          <t>16.68% (15.92%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.65% (3.47%)</t>
+          <t>3.83% (3.66%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.55% (5.24%)</t>
+          <t>5.84% (5.53%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.76% (4.52%)</t>
+          <t>5.07% (4.83%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.40% (12.73%)</t>
+          <t>13.83% (13.17%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.11% (12.51%)</t>
+          <t>13.63% (13.03%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.98% (4.61%)</t>
+          <t>5.13% (4.76%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.42% (11.88%)</t>
+          <t>12.90% (12.37%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.23% (2.12%)</t>
+          <t>2.46% (2.35%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.94% (0.90%)</t>
+          <t>1.13% (1.09%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.89% (15.06%)</t>
+          <t>16.33% (15.51%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.56% (6.11%)</t>
+          <t>6.83% (6.39%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.94% (12.18%)</t>
+          <t>13.27% (12.52%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.68% (2.50%)</t>
+          <t>2.86% (2.69%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.33% (4.01%)</t>
+          <t>4.53% (4.22%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.62% (3.38%)</t>
+          <t>3.79% (3.56%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.91% (10.24%)</t>
+          <t>11.28% (10.62%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.47% (9.87%)</t>
+          <t>10.86% (10.26%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.23% (3.85%)</t>
+          <t>4.36% (3.99%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.73% (9.19%)</t>
+          <t>10.09% (9.56%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.56% (1.44%)</t>
+          <t>1.59% (1.48%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.52% (0.47%)</t>
+          <t>0.52% (0.49%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.35% (12.52%)</t>
+          <t>13.71% (12.88%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.27%</t>
+          <t>16.10%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>13.78%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.02%</t>
+          <t>-3.33%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.20%</t>
+          <t>-2.50%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-2.67%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>13.52%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.99% (10.55%)</t>
+          <t>10.68% (10.24%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.72% (8.96%)</t>
+          <t>9.54% (8.79%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.80% (10.63%)</t>
+          <t>10.39% (10.22%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.24% (10.93%)</t>
+          <t>10.91% (10.60%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.66% (10.42%)</t>
+          <t>10.35% (10.12%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.28% (9.62%)</t>
+          <t>10.03% (9.37%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.94% (9.34%)</t>
+          <t>9.75% (9.15%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.83% (13.46%)</t>
+          <t>13.41% (13.05%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.68% (9.15%)</t>
+          <t>9.47% (8.95%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.64% (10.53%)</t>
+          <t>10.29% (10.18%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.06% (10.02%)</t>
+          <t>9.67% (9.63%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.41% (9.58%)</t>
+          <t>10.15% (9.33%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.53% (16.08%)</t>
+          <t>16.20% (15.76%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.86% (14.10%)</t>
+          <t>14.54% (13.79%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.51% (16.33%)</t>
+          <t>16.14% (15.96%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.05% (16.73%)</t>
+          <t>16.69% (16.37%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.36% (16.12%)</t>
+          <t>15.97% (15.73%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.48% (14.81%)</t>
+          <t>15.22% (14.55%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.11% (14.51%)</t>
+          <t>14.86% (14.26%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.79% (19.42%)</t>
+          <t>19.39% (19.03%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.87% (14.33%)</t>
+          <t>14.60% (14.07%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.95% (16.83%)</t>
+          <t>16.45% (16.34%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.31% (16.27%)</t>
+          <t>15.79% (15.75%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.40% (14.57%)</t>
+          <t>15.10% (14.28%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.11% (-6.56%)</t>
+          <t>-5.83% (-6.27%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.90% (-1.66%)</t>
+          <t>-0.43% (-1.19%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.75% (-9.93%)</t>
+          <t>-9.60% (-9.77%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.28% (-8.60%)</t>
+          <t>-8.03% (-8.34%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.60% (-8.84%)</t>
+          <t>-8.33% (-8.57%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.95% (-3.62%)</t>
+          <t>-2.58% (-3.24%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.90% (-3.50%)</t>
+          <t>-2.46% (-3.06%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.47% (-10.83%)</t>
+          <t>-10.34% (-10.70%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.03% (-4.57%)</t>
+          <t>-3.62% (-4.15%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.43% (-12.54%)</t>
+          <t>-12.23% (-12.34%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.39% (-12.43%)</t>
+          <t>-12.22% (-12.26%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.68% (-1.51%)</t>
+          <t>-0.30% (-1.12%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.18% (-5.63%)</t>
+          <t>-4.94% (-5.39%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.72% (-1.48%)</t>
+          <t>-0.43% (-1.19%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.45% (-8.63%)</t>
+          <t>-8.29% (-8.46%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.94% (-7.26%)</t>
+          <t>-6.76% (-7.07%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.38% (-7.62%)</t>
+          <t>-7.23% (-7.46%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.58% (-3.25%)</t>
+          <t>-2.25% (-2.91%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.56% (-3.17%)</t>
+          <t>-2.22% (-2.82%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.70% (-9.08%)</t>
+          <t>-8.59% (-8.96%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.64% (-4.18%)</t>
+          <t>-3.32% (-3.85%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.40% (-10.52%)</t>
+          <t>-10.37% (-10.48%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.44% (-10.49%)</t>
+          <t>-10.44% (-10.48%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.63% (-1.46%)</t>
+          <t>-0.32% (-1.14%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.11%</t>
+          <t>-16.51%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.62%</t>
+          <t>-9.98%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.56%</t>
+          <t>-19.98%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.52%</t>
+          <t>-18.94%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.26%</t>
+          <t>-18.68%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.24%</t>
+          <t>-12.61%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.83%</t>
+          <t>-12.21%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.29%</t>
+          <t>-23.75%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.72%</t>
+          <t>-13.10%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.07%</t>
+          <t>-22.52%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.45%</t>
+          <t>-21.89%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.09%</t>
+          <t>-10.45%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.71%</t>
+          <t>-21.15%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.58%</t>
+          <t>-14.97%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.97%</t>
+          <t>-24.43%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.99%</t>
+          <t>-23.45%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.75%</t>
+          <t>-23.20%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-17.46%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.67%</t>
+          <t>-17.08%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.50%</t>
+          <t>-27.98%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.51%</t>
+          <t>-17.92%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.34%</t>
+          <t>-26.82%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.75%</t>
+          <t>-26.23%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.03%</t>
+          <t>-15.42%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.96% (1.52%)</t>
+          <t>1.54% (1.10%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.21% (-0.97%)</t>
+          <t>-0.43% (-1.19%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.32% (2.14%)</t>
+          <t>1.76% (1.59%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.63% (2.31%)</t>
+          <t>2.17% (1.86%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.95% (1.71%)</t>
+          <t>1.51% (1.28%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.67% (0.01%)</t>
+          <t>0.34% (-0.32%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.27% (-0.33%)</t>
+          <t>0.00% (-0.60%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.98% (4.61%)</t>
+          <t>5.13% (4.76%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.11% (-0.42%)</t>
+          <t>-0.18% (-0.71%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.23% (2.12%)</t>
+          <t>2.05% (1.94%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.94% (0.90%)</t>
+          <t>1.13% (1.09%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.53% (-0.29%)</t>
+          <t>0.20% (-0.62%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.97% (2.52%)</t>
+          <t>2.49% (2.05%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.79%)</t>
+          <t>-0.43% (-1.19%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.68% (2.50%)</t>
+          <t>2.86% (2.69%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.13% (3.81%)</t>
+          <t>3.58% (3.27%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.30% (3.06%)</t>
+          <t>2.73% (2.50%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.06% (0.39%)</t>
+          <t>0.68% (0.01%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.61% (0.01%)</t>
+          <t>0.24% (-0.36%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.23% (3.85%)</t>
+          <t>4.36% (3.99%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.52% (-0.02%)</t>
+          <t>0.13% (-0.40%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.56% (1.44%)</t>
+          <t>1.59% (1.48%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.52% (0.47%)</t>
+          <t>0.52% (0.49%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.57% (-0.26%)</t>
+          <t>0.16% (-0.66%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 25/9/2026</t>
+          <t>As of 28/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>4.83%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>8.44%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>3.48%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.84%</t>
+          <t>-8.57%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.60%</t>
+          <t>-8.34%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.46%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.76%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>18.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.83%</t>
+          <t>-10.70%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.73%</t>
+          <t>8.06%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.11%</t>
+          <t>5.78%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>7.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.56%</t>
+          <t>-6.27%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.88%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.57%</t>
+          <t>-4.15%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.34%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.51%</t>
+          <t>13.03%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.50%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.73%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.87%</t>
+          <t>2.47%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.99%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.62%</t>
+          <t>-3.24%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.96%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.37%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>17.20%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-1.19%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.06%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.27%</t>
+          <t>16.10%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-1.12%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.23%</t>
+          <t>13.01%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.43%</t>
+          <t>-12.26%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.53%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.12%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.37%</t>
+          <t>13.11%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.16%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.54%</t>
+          <t>-12.34%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.89%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.93%</t>
+          <t>-9.77%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 25/9/2026</t>
+          <t>As of 28/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>15.73%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.34%</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.62%</t>
+          <t>-7.46%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.73%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.92%</t>
+          <t>6.70%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.04%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.26%</t>
+          <t>-7.07%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.42%</t>
+          <t>19.03%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.85%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>18.03%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.02%</t>
+          <t>-3.33%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.08%</t>
+          <t>-8.96%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.11%</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.07%</t>
+          <t>4.80%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>7.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.39%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.33%</t>
+          <t>14.07%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.18%</t>
+          <t>-3.85%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.51%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-2.82%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.81%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.99%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-2.91%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.10%</t>
+          <t>13.79%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>13.78%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.48%</t>
+          <t>-1.19%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.57%</t>
+          <t>14.28%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.46%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.49%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-2.67%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.49%</t>
+          <t>-10.48%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.83%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.44%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>10.77%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.16%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.20%</t>
+          <t>-2.50%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.52%</t>
+          <t>-10.48%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.33%</t>
+          <t>15.96%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.63%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-29]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/28/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>200 days</t>
+          <t>199 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>109 days</t>
+          <t>108 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>291 days</t>
+          <t>290 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>235 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>18 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
     </row>
@@ -2326,42 +2326,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.89 / 5.78%</t>
+          <t>$47.86 / 5.73%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.73 / 0.35%</t>
+          <t>$57.76 / 0.40%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.05 / 9.89%</t>
+          <t>$56.00 / 9.79%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.65 / 8.18%</t>
+          <t>$62.63 / 8.13%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.68 / 8.44%</t>
+          <t>$56.68 / 8.43%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.33 / 2.47%</t>
+          <t>$61.31 / 2.44%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.24 / 2.28%</t>
+          <t>$61.23 / 2.27%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.65 / 11.03%</t>
+          <t>$53.64 / 11.02%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.23 / 13.11%</t>
+          <t>$60.21 / 13.07%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2381,22 +2381,22 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.24 / 0.28%</t>
+          <t>$57.22 / 0.24%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.60 / 4.80%</t>
+          <t>$42.60 / 4.81%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.16 / 0.35%</t>
+          <t>$42.13 / 0.28%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.83 / 8.32%</t>
+          <t>$40.83 / 8.34%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.13 / 7.15%</t>
+          <t>$46.11 / 7.10%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2416,32 +2416,32 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.99 / 2.03%</t>
+          <t>$41.98 / 2.02%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.23 / 8.91%</t>
+          <t>$45.25 / 8.95%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.97 / 3.11%</t>
+          <t>$43.95 / 3.06%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.89 / 10.77%</t>
+          <t>$42.88 / 10.74%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.72 / 10.76%</t>
+          <t>$42.70 / 10.71%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.18 / 0.32%</t>
+          <t>$42.15 / 0.26%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$765.52 / 7.80%</t>
+          <t>$765.24 / 7.76%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$765.52 / -0.03%</t>
+          <t>$765.24 / -0.06%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$765.52 / 12.48%</t>
+          <t>$765.24 / 12.44%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$765.52 / 11.04%</t>
+          <t>$765.24 / 11.00%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$765.52 / 10.68%</t>
+          <t>$765.24 / 10.64%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$765.52 / 2.99%</t>
+          <t>$765.24 / 2.95%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$765.52 / 2.51%</t>
+          <t>$765.24 / 2.48%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$765.52 / 18.03%</t>
+          <t>$765.24 / 17.99%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$765.52 / 3.56%</t>
+          <t>$765.24 / 3.53%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$765.52 / 16.16%</t>
+          <t>$765.24 / 16.12%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$765.52 / 15.22%</t>
+          <t>$765.24 / 15.18%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$765.52 / 0.50%</t>
+          <t>$765.24 / 0.47%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$765.52 / 7.80%</t>
+          <t>$765.24 / 7.76%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$765.52 / -0.03%</t>
+          <t>$765.24 / -0.06%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$765.52 / 12.48%</t>
+          <t>$765.24 / 12.44%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$765.52 / 11.04%</t>
+          <t>$765.24 / 11.00%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$765.52 / 10.68%</t>
+          <t>$765.24 / 10.64%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$765.52 / 2.99%</t>
+          <t>$765.24 / 2.95%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$765.52 / 2.51%</t>
+          <t>$765.24 / 2.48%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$765.52 / 18.03%</t>
+          <t>$765.24 / 17.99%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$765.52 / 3.56%</t>
+          <t>$765.24 / 3.53%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$765.52 / 16.16%</t>
+          <t>$765.24 / 16.12%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$765.52 / 15.22%</t>
+          <t>$765.24 / 15.18%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$765.52 / 0.50%</t>
+          <t>$765.24 / 0.47%</t>
         </is>
       </c>
     </row>
@@ -2580,42 +2580,42 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.50% (8.06%)</t>
+          <t>8.56% (8.12%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.68% (15.92%)</t>
+          <t>16.61% (15.86%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.83% (3.66%)</t>
+          <t>3.92% (3.75%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.84% (5.53%)</t>
+          <t>5.88% (5.57%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.07% (4.83%)</t>
+          <t>5.07% (4.84%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.83% (13.17%)</t>
+          <t>13.87% (13.21%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.63% (13.03%)</t>
+          <t>13.63% (13.04%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.13% (4.76%)</t>
+          <t>5.13% (4.77%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.46% (2.35%)</t>
+          <t>2.49% (2.39%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.33% (15.51%)</t>
+          <t>16.37% (15.55%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.83% (6.39%)</t>
+          <t>6.82% (6.37%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.27% (12.52%)</t>
+          <t>13.35% (12.60%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.86% (2.69%)</t>
+          <t>2.85% (2.68%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.79% (3.56%)</t>
+          <t>3.85% (3.61%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2670,32 +2670,32 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.86% (10.26%)</t>
+          <t>10.87% (10.28%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.36% (3.99%)</t>
+          <t>4.32% (3.96%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.09% (9.56%)</t>
+          <t>10.14% (9.61%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.59% (1.48%)</t>
+          <t>1.61% (1.50%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.52% (0.49%)</t>
+          <t>0.57% (0.53%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.71% (12.88%)</t>
+          <t>13.77% (12.95%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.83%</t>
+          <t>6.87%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.02%</t>
+          <t>2.06%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.43%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.10%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.78%</t>
+          <t>13.82%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>-0.31%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.50%</t>
+          <t>-2.47%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-2.64%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.56%</t>
         </is>
       </c>
     </row>
@@ -2834,27 +2834,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.68% (10.24%)</t>
+          <t>10.70% (10.26%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.54% (8.79%)</t>
+          <t>9.46% (8.70%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.39% (10.22%)</t>
+          <t>10.44% (10.27%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.91% (10.60%)</t>
+          <t>10.92% (10.61%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.35% (10.12%)</t>
+          <t>10.33% (10.09%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2864,17 +2864,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.75% (9.15%)</t>
+          <t>9.72% (9.13%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.41% (13.05%)</t>
+          <t>13.39% (13.03%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.47% (8.95%)</t>
+          <t>9.44% (8.91%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.67% (9.63%)</t>
+          <t>9.64% (9.60%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2894,62 +2894,62 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.20% (15.76%)</t>
+          <t>16.16% (15.72%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.54% (13.79%)</t>
+          <t>14.58% (13.83%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.14% (15.96%)</t>
+          <t>16.10% (15.92%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.69% (16.37%)</t>
+          <t>16.66% (16.34%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.97% (15.73%)</t>
+          <t>15.99% (15.76%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.22% (14.55%)</t>
+          <t>15.19% (14.52%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.86% (14.26%)</t>
+          <t>14.84% (14.24%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.39% (19.03%)</t>
+          <t>19.34% (18.97%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.60% (14.07%)</t>
+          <t>14.61% (14.09%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.45% (16.34%)</t>
+          <t>16.44% (16.33%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.79% (15.75%)</t>
+          <t>15.80% (15.77%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.10% (14.28%)</t>
+          <t>15.13% (14.31%)</t>
         </is>
       </c>
     </row>
@@ -2961,52 +2961,52 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.83% (-6.27%)</t>
+          <t>-5.78% (-6.22%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.43% (-1.19%)</t>
+          <t>-0.49% (-1.24%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.60% (-9.77%)</t>
+          <t>-9.52% (-9.69%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.03% (-8.34%)</t>
+          <t>-8.00% (-8.31%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.33% (-8.57%)</t>
+          <t>-8.33% (-8.56%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.58% (-3.24%)</t>
+          <t>-2.55% (-3.21%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.46% (-3.06%)</t>
+          <t>-2.45% (-3.05%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.34% (-10.70%)</t>
+          <t>-10.33% (-10.69%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.62% (-4.15%)</t>
+          <t>-3.63% (-4.15%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.23% (-12.34%)</t>
+          <t>-12.20% (-12.31%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -3016,22 +3016,22 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.30% (-1.12%)</t>
+          <t>-0.27% (-1.09%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.94% (-5.39%)</t>
+          <t>-4.96% (-5.40%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.43% (-1.19%)</t>
+          <t>-0.36% (-1.12%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.29% (-8.46%)</t>
+          <t>-8.30% (-8.48%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.23% (-7.46%)</t>
+          <t>-7.18% (-7.41%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -3051,32 +3051,32 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.22% (-2.82%)</t>
+          <t>-2.21% (-2.81%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.59% (-8.96%)</t>
+          <t>-8.62% (-8.99%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.32% (-3.85%)</t>
+          <t>-3.28% (-3.81%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.37% (-10.48%)</t>
+          <t>-10.35% (-10.46%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.44% (-10.48%)</t>
+          <t>-10.40% (-10.43%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.32% (-1.14%)</t>
+          <t>-0.26% (-1.08%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.51%</t>
+          <t>-16.48%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.98%</t>
+          <t>-9.94%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.98%</t>
+          <t>-19.96%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.94%</t>
+          <t>-18.92%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.68%</t>
+          <t>-18.65%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.61%</t>
+          <t>-12.58%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.21%</t>
+          <t>-12.18%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.75%</t>
+          <t>-23.72%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.10%</t>
+          <t>-13.07%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.52%</t>
+          <t>-22.49%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.89%</t>
+          <t>-21.86%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.45%</t>
+          <t>-10.42%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.15%</t>
+          <t>-21.12%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.97%</t>
+          <t>-14.94%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.43%</t>
+          <t>-24.40%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.45%</t>
+          <t>-23.42%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.20%</t>
+          <t>-23.17%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.46%</t>
+          <t>-17.44%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.08%</t>
+          <t>-17.05%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.98%</t>
+          <t>-27.96%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.92%</t>
+          <t>-17.89%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.82%</t>
+          <t>-26.79%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.23%</t>
+          <t>-26.20%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.42%</t>
+          <t>-15.39%</t>
         </is>
       </c>
     </row>
@@ -3215,17 +3215,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.54% (1.10%)</t>
+          <t>1.56% (1.12%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.43% (-1.19%)</t>
+          <t>-0.49% (-1.24%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.76% (1.59%)</t>
+          <t>1.81% (1.64%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -3235,27 +3235,27 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.51% (1.28%)</t>
+          <t>1.48% (1.25%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.34% (-0.32%)</t>
+          <t>0.33% (-0.33%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.00% (-0.60%)</t>
+          <t>-0.03% (-0.63%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.13% (4.76%)</t>
+          <t>5.13% (4.77%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.18% (-0.71%)</t>
+          <t>-0.22% (-0.74%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3275,62 +3275,62 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.49% (2.05%)</t>
+          <t>2.44% (2.00%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.43% (-1.19%)</t>
+          <t>-0.36% (-1.12%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.86% (2.69%)</t>
+          <t>2.85% (2.68%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.58% (3.27%)</t>
+          <t>3.54% (3.23%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.73% (2.50%)</t>
+          <t>2.75% (2.52%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.68% (0.01%)</t>
+          <t>0.64% (-0.02%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.24% (-0.36%)</t>
+          <t>0.21% (-0.38%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.36% (3.99%)</t>
+          <t>4.32% (3.96%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.13% (-0.40%)</t>
+          <t>0.14% (-0.39%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.59% (1.48%)</t>
+          <t>1.61% (1.50%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.52% (0.49%)</t>
+          <t>0.57% (0.53%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.16% (-0.66%)</t>
+          <t>0.18% (-0.64%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/9/2026</t>
+          <t>As of 29/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.83%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.44%</t>
+          <t>8.43%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.48%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.57%</t>
+          <t>-8.56%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.57%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.18%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.34%</t>
+          <t>-8.31%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.03%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.76%</t>
+          <t>4.77%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.02%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.03%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.70%</t>
+          <t>-10.69%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.06%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.78%</t>
+          <t>5.73%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.80%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.83%</t>
+          <t>6.87%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.27%</t>
+          <t>-6.22%</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3573,12 +3573,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.03%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.59%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-3.05%</t>
         </is>
       </c>
     </row>
@@ -3637,27 +3637,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>2.95%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.43%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.24%</t>
+          <t>-3.21%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>15.86%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.20%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-1.24%</t>
         </is>
       </c>
     </row>
@@ -3711,27 +3711,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.10%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-1.09%</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.60%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3785,27 +3785,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.35%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.11%</t>
+          <t>13.07%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.16%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.34%</t>
+          <t>-12.31%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.89%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>12.44%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.02%</t>
+          <t>2.06%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.77%</t>
+          <t>-9.69%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/9/2026</t>
+          <t>As of 29/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.73%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.61%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.46%</t>
+          <t>-7.41%</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.04%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.03%</t>
+          <t>18.97%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>3.96%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.03%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.33%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.96%</t>
+          <t>-8.99%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.72%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.37%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.80%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.80%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>4.25%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.39%</t>
+          <t>-5.40%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.07%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-3.81%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.82%</t>
+          <t>-2.81%</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>14.52%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4162,12 +4162,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>2.95%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.79%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.78%</t>
+          <t>13.82%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-1.12%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.28%</t>
+          <t>14.31%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>12.95%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.47%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.56%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-1.08%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.49%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-2.64%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.48%</t>
+          <t>-10.43%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>16.33%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.77%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.16%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.50%</t>
+          <t>-2.47%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.48%</t>
+          <t>-10.46%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.96%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>2.68%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>12.44%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>-0.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.48%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-09-30]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/29/2026 at 2:41 PM ET)</t>
+          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>199 days</t>
+          <t>198 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>108 days</t>
+          <t>107 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>290 days</t>
+          <t>289 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.86 / 5.73%</t>
+          <t>$47.95 / 5.91%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.76 / 0.40%</t>
+          <t>$57.85 / 0.55%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.00 / 9.79%</t>
+          <t>$56.10 / 9.98%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.63 / 8.13%</t>
+          <t>$62.72 / 8.30%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.68 / 8.43%</t>
+          <t>$56.75 / 8.58%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.31 / 2.44%</t>
+          <t>$61.41 / 2.62%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.23 / 2.27%</t>
+          <t>$61.38 / 2.51%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.64 / 11.02%</t>
+          <t>$53.69 / 11.13%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.47 / 3.43%</t>
+          <t>$57.56 / 3.59%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.21 / 13.07%</t>
+          <t>$60.30 / 13.24%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.10 / 13.01%</t>
+          <t>$54.19 / 13.19%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.22 / 0.24%</t>
+          <t>$57.32 / 0.42%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.60 / 4.81%</t>
+          <t>$42.65 / 4.94%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.13 / 0.28%</t>
+          <t>$42.19 / 0.43%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.83 / 8.34%</t>
+          <t>$40.86 / 8.40%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.05 / 6.70%</t>
+          <t>$45.11 / 6.84%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.11 / 7.10%</t>
+          <t>$46.16 / 7.21%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.58 / 2.13%</t>
+          <t>$44.65 / 2.29%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.98 / 2.02%</t>
+          <t>$42.07 / 2.23%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.25 / 8.95%</t>
+          <t>$45.28 / 9.03%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.95 / 3.06%</t>
+          <t>$44.02 / 3.24%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.88 / 10.74%</t>
+          <t>$42.92 / 10.85%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.70 / 10.71%</t>
+          <t>$42.74 / 10.82%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.15 / 0.26%</t>
+          <t>$42.23 / 0.44%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$765.24 / 7.76%</t>
+          <t>$766.72 / 7.97%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$765.24 / -0.06%</t>
+          <t>$766.72 / 0.13%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$765.24 / 12.44%</t>
+          <t>$766.72 / 12.65%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$765.24 / 11.00%</t>
+          <t>$766.72 / 11.21%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$765.24 / 10.64%</t>
+          <t>$766.72 / 10.85%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$765.24 / 2.95%</t>
+          <t>$766.72 / 3.15%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$765.24 / 2.48%</t>
+          <t>$766.72 / 2.67%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$765.24 / 17.99%</t>
+          <t>$766.72 / 18.22%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$765.24 / 3.53%</t>
+          <t>$766.72 / 3.73%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$765.24 / 16.12%</t>
+          <t>$766.72 / 16.34%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$765.24 / 15.18%</t>
+          <t>$766.72 / 15.40%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$765.24 / 0.47%</t>
+          <t>$766.72 / 0.66%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$765.24 / 7.76%</t>
+          <t>$766.72 / 7.97%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$765.24 / -0.06%</t>
+          <t>$766.72 / 0.13%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$765.24 / 12.44%</t>
+          <t>$766.72 / 12.65%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$765.24 / 11.00%</t>
+          <t>$766.72 / 11.21%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$765.24 / 10.64%</t>
+          <t>$766.72 / 10.85%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$765.24 / 2.95%</t>
+          <t>$766.72 / 3.15%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$765.24 / 2.48%</t>
+          <t>$766.72 / 2.67%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$765.24 / 17.99%</t>
+          <t>$766.72 / 18.22%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$765.24 / 3.53%</t>
+          <t>$766.72 / 3.73%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$765.24 / 16.12%</t>
+          <t>$766.72 / 16.34%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$765.24 / 15.18%</t>
+          <t>$766.72 / 15.40%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$765.24 / 0.47%</t>
+          <t>$766.72 / 0.66%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.56% (8.12%)</t>
+          <t>8.36% (7.93%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.61% (15.86%)</t>
+          <t>16.43% (15.68%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.92% (3.75%)</t>
+          <t>3.73% (3.56%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.88% (5.57%)</t>
+          <t>5.72% (5.41%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.07% (4.84%)</t>
+          <t>4.93% (4.70%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.87% (13.21%)</t>
+          <t>13.67% (13.02%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.63% (13.04%)</t>
+          <t>13.36% (12.77%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.13% (4.77%)</t>
+          <t>5.03% (4.68%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.90% (12.37%)</t>
+          <t>12.72% (12.19%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.49% (2.39%)</t>
+          <t>2.34% (2.23%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.13% (1.09%)</t>
+          <t>0.96% (0.93%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.37% (15.55%)</t>
+          <t>16.17% (15.35%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.82% (6.37%)</t>
+          <t>6.69% (6.25%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.35% (12.60%)</t>
+          <t>13.17% (12.42%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.85% (2.68%)</t>
+          <t>2.78% (2.61%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.53% (4.22%)</t>
+          <t>4.39% (4.08%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.85% (3.61%)</t>
+          <t>3.73% (3.50%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.28% (10.62%)</t>
+          <t>11.11% (10.45%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.87% (10.28%)</t>
+          <t>10.65% (10.06%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.32% (3.96%)</t>
+          <t>4.24% (3.88%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.14% (9.61%)</t>
+          <t>9.95% (9.43%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.61% (1.50%)</t>
+          <t>1.51% (1.41%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.57% (0.53%)</t>
+          <t>0.46% (0.43%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.77% (12.95%)</t>
+          <t>13.57% (12.75%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.87%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>17.02%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.47%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.69%</t>
+          <t>-0.88%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>-0.27%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.82%</t>
+          <t>13.61%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.31%</t>
+          <t>-0.51%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.34%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.40%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.48%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.47%</t>
+          <t>-2.65%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.64%</t>
+          <t>-2.82%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.56%</t>
+          <t>13.34%</t>
         </is>
       </c>
     </row>
@@ -2834,57 +2834,57 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.70% (10.26%)</t>
+          <t>10.69% (10.26%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.46% (8.70%)</t>
+          <t>9.47% (8.72%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.44% (10.27%)</t>
+          <t>10.43% (10.26%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.92% (10.61%)</t>
+          <t>10.93% (10.63%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.33% (10.09%)</t>
+          <t>10.36% (10.13%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.03% (9.37%)</t>
+          <t>10.03% (9.38%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.72% (9.13%)</t>
+          <t>9.66% (9.07%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.39% (13.03%)</t>
+          <t>13.45% (13.09%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.44% (8.91%)</t>
+          <t>9.46% (8.93%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.29% (10.18%)</t>
+          <t>10.30% (10.20%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.64% (9.60%)</t>
+          <t>9.64% (9.61%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2894,62 +2894,62 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.16% (15.72%)</t>
+          <t>16.20% (15.76%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.58% (13.83%)</t>
+          <t>14.59% (13.84%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.10% (15.92%)</t>
+          <t>16.18% (16.01%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.66% (16.34%)</t>
+          <t>16.68% (16.37%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.99% (15.76%)</t>
+          <t>16.04% (15.80%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.19% (14.52%)</t>
+          <t>15.19% (14.53%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.84% (14.24%)</t>
+          <t>14.80% (14.21%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.34% (18.97%)</t>
+          <t>19.40% (19.04%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.61% (14.09%)</t>
+          <t>14.61% (14.08%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.44% (16.33%)</t>
+          <t>16.50% (16.39%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.80% (15.77%)</t>
+          <t>15.85% (15.81%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.13% (14.31%)</t>
+          <t>15.11% (14.30%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.22%)</t>
+          <t>-5.95% (-6.38%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.49% (-1.24%)</t>
+          <t>-0.64% (-1.39%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.52% (-9.69%)</t>
+          <t>-9.68% (-9.85%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.00% (-8.31%)</t>
+          <t>-8.14% (-8.45%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.33% (-8.56%)</t>
+          <t>-8.45% (-8.68%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.55% (-3.21%)</t>
+          <t>-2.72% (-3.37%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.45% (-3.05%)</t>
+          <t>-2.69% (-3.28%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.33% (-10.69%)</t>
+          <t>-10.42% (-10.77%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.63% (-4.15%)</t>
+          <t>-3.78% (-4.30%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.20% (-12.31%)</t>
+          <t>-12.34% (-12.44%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.22% (-12.26%)</t>
+          <t>-12.37% (-12.40%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.27% (-1.09%)</t>
+          <t>-0.44% (-1.26%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.96% (-5.40%)</t>
+          <t>-5.07% (-5.51%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.36% (-1.12%)</t>
+          <t>-0.52% (-1.27%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.30% (-8.48%)</t>
+          <t>-8.36% (-8.53%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.76% (-7.07%)</t>
+          <t>-6.89% (-7.20%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.18% (-7.41%)</t>
+          <t>-7.28% (-7.51%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.25% (-2.91%)</t>
+          <t>-2.40% (-3.06%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.21% (-2.81%)</t>
+          <t>-2.41% (-3.00%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.62% (-8.99%)</t>
+          <t>-8.69% (-9.06%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.28% (-3.81%)</t>
+          <t>-3.45% (-3.97%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.35% (-10.46%)</t>
+          <t>-10.44% (-10.55%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.40% (-10.43%)</t>
+          <t>-10.49% (-10.53%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.26% (-1.08%)</t>
+          <t>-0.44% (-1.26%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.48%</t>
+          <t>-16.64%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.94%</t>
+          <t>-10.12%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.96%</t>
+          <t>-20.11%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.92%</t>
+          <t>-19.07%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.65%</t>
+          <t>-18.81%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.58%</t>
+          <t>-12.75%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.18%</t>
+          <t>-12.34%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.72%</t>
+          <t>-23.87%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.07%</t>
+          <t>-13.23%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.49%</t>
+          <t>-22.64%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.86%</t>
+          <t>-22.01%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.42%</t>
+          <t>-10.59%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.12%</t>
+          <t>-21.27%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.94%</t>
+          <t>-15.11%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.40%</t>
+          <t>-24.55%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.42%</t>
+          <t>-23.56%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.17%</t>
+          <t>-23.32%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.44%</t>
+          <t>-17.59%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.05%</t>
+          <t>-17.21%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.96%</t>
+          <t>-28.10%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.89%</t>
+          <t>-18.05%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.79%</t>
+          <t>-26.94%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.20%</t>
+          <t>-26.34%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.39%</t>
+          <t>-15.56%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.56% (1.12%)</t>
+          <t>1.57% (1.14%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.49% (-1.24%)</t>
+          <t>-0.52% (-1.27%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.81% (1.64%)</t>
+          <t>1.82% (1.66%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.17% (1.86%)</t>
+          <t>2.21% (1.91%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.48% (1.25%)</t>
+          <t>1.54% (1.31%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.33% (-0.33%)</t>
+          <t>0.35% (-0.30%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.63%)</t>
+          <t>-0.08% (-0.67%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.13% (4.77%)</t>
+          <t>5.03% (4.68%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.22% (-0.74%)</t>
+          <t>-0.18% (-0.71%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.05% (1.94%)</t>
+          <t>2.09% (1.99%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.13% (1.09%)</t>
+          <t>0.96% (0.93%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
+          <t>0.21% (-0.60%)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2.52% (2.08%)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>-0.39% (-1.14%)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2.78% (2.61%)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>3.60% (3.29%)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>2.84% (2.60%)</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>0.67% (0.02%)</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>0.20% (-0.39%)</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>4.24% (3.88%)</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0.16% (-0.36%)</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>1.51% (1.41%)</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>0.46% (0.43%)</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
           <t>0.20% (-0.62%)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>2.44% (2.00%)</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>-0.36% (-1.12%)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>2.85% (2.68%)</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>3.54% (3.23%)</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>2.75% (2.52%)</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>0.64% (-0.02%)</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>0.21% (-0.38%)</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>4.32% (3.96%)</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>0.14% (-0.39%)</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>1.61% (1.50%)</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>0.57% (0.53%)</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>0.18% (-0.64%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/9/2026</t>
+          <t>As of 30/9/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.13%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.43%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.56%</t>
+          <t>-8.68%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.30%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.31%</t>
+          <t>-8.45%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.03%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.77%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.02%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>18.22%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.69%</t>
+          <t>-0.88%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.69%</t>
+          <t>-10.77%</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>7.93%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.73%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>7.97%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.87%</t>
+          <t>6.66%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.22%</t>
+          <t>-6.38%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.53%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.15%</t>
+          <t>-4.30%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.05%</t>
+          <t>-3.28%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.38%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.02%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.47%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.21%</t>
+          <t>-3.37%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.86%</t>
+          <t>15.68%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>17.02%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-1.39%</t>
         </is>
       </c>
     </row>
@@ -3711,27 +3711,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.66%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-1.26%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.60%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.01%</t>
+          <t>13.19%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.40%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>-0.27%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.26%</t>
+          <t>-12.40%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.07%</t>
+          <t>13.24%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.31%</t>
+          <t>-12.44%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.79%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.44%</t>
+          <t>12.65%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>1.86%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.69%</t>
+          <t>-9.85%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/9/2026</t>
+          <t>As of 30/9/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.80%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.61%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>7.21%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.41%</t>
+          <t>-7.51%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>4.08%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.70%</t>
+          <t>6.84%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.07%</t>
+          <t>-7.20%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.97%</t>
+          <t>19.04%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.96%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.03%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>18.22%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.48%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.99%</t>
+          <t>-9.06%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.37%</t>
+          <t>6.25%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>7.97%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.25%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.40%</t>
+          <t>-5.51%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.08%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.53%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-3.97%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.02%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.40%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.81%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.52%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.13%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.34%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.91%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>13.84%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.42%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.82%</t>
+          <t>13.61%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-1.27%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.31%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.95%</t>
+          <t>12.75%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.66%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.56%</t>
+          <t>13.34%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.08%</t>
+          <t>-1.26%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>15.40%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.64%</t>
+          <t>-2.82%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.43%</t>
+          <t>-10.53%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.33%</t>
+          <t>16.39%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.41%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.47%</t>
+          <t>-2.65%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.46%</t>
+          <t>-10.55%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.40%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.44%</t>
+          <t>12.65%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.31%</t>
+          <t>-0.51%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.48%</t>
+          <t>-8.53%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-01]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 9/30/2026 at 2:23 PM ET)</t>
+          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>198 days</t>
+          <t>197 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>107 days</t>
+          <t>106 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>289 days</t>
+          <t>288 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>15 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
     </row>
@@ -2326,112 +2326,112 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.95 / 5.91%</t>
+          <t>$47.86 / 5.73%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.85 / 0.55%</t>
+          <t>$57.71 / 0.30%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.10 / 9.98%</t>
+          <t>$56.01 / 9.80%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.72 / 8.30%</t>
+          <t>$62.64 / 8.16%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.75 / 8.58%</t>
+          <t>$56.62 / 8.32%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.41 / 2.62%</t>
+          <t>$61.29 / 2.41%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.38 / 2.51%</t>
+          <t>$61.22 / 2.25%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.69 / 11.13%</t>
+          <t>$53.63 / 10.99%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.56 / 3.59%</t>
+          <t>$57.43 / 3.35%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.30 / 13.24%</t>
+          <t>$60.21 / 13.07%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.19 / 13.19%</t>
+          <t>$54.14 / 13.09%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.32 / 0.42%</t>
+          <t>$57.19 / 0.19%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.65 / 4.94%</t>
+          <t>$42.60 / 4.81%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.19 / 0.43%</t>
+          <t>$42.13 / 0.28%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.86 / 8.40%</t>
+          <t>$40.82 / 8.31%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.11 / 6.84%</t>
+          <t>$45.04 / 6.68%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.16 / 7.21%</t>
+          <t>$46.12 / 7.12%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.65 / 2.29%</t>
+          <t>$44.58 / 2.14%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.07 / 2.23%</t>
+          <t>$41.99 / 2.03%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.28 / 9.03%</t>
+          <t>$45.24 / 8.92%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.02 / 3.24%</t>
+          <t>$43.95 / 3.06%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.92 / 10.85%</t>
+          <t>$42.88 / 10.74%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.23 / 0.44%</t>
+          <t>$42.17 / 0.30%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$766.72 / 7.97%</t>
+          <t>$764.38 / 7.64%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$766.72 / 0.13%</t>
+          <t>$764.38 / -0.18%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$766.72 / 12.65%</t>
+          <t>$764.38 / 12.31%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$766.72 / 11.21%</t>
+          <t>$764.38 / 10.87%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$766.72 / 10.85%</t>
+          <t>$764.38 / 10.51%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$766.72 / 3.15%</t>
+          <t>$764.38 / 2.84%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$766.72 / 2.67%</t>
+          <t>$764.38 / 2.36%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$766.72 / 18.22%</t>
+          <t>$764.38 / 17.86%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$766.72 / 3.73%</t>
+          <t>$764.38 / 3.41%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$766.72 / 16.34%</t>
+          <t>$764.38 / 15.98%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$766.72 / 15.40%</t>
+          <t>$764.38 / 15.05%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$766.72 / 0.66%</t>
+          <t>$764.38 / 0.35%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$766.72 / 7.97%</t>
+          <t>$764.38 / 7.64%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$766.72 / 0.13%</t>
+          <t>$764.38 / -0.18%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$766.72 / 12.65%</t>
+          <t>$764.38 / 12.31%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$766.72 / 11.21%</t>
+          <t>$764.38 / 10.87%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$766.72 / 10.85%</t>
+          <t>$764.38 / 10.51%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$766.72 / 3.15%</t>
+          <t>$764.38 / 2.84%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$766.72 / 2.67%</t>
+          <t>$764.38 / 2.36%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$766.72 / 18.22%</t>
+          <t>$764.38 / 17.86%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$766.72 / 3.73%</t>
+          <t>$764.38 / 3.41%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$766.72 / 16.34%</t>
+          <t>$764.38 / 15.98%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$766.72 / 15.40%</t>
+          <t>$764.38 / 15.05%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$766.72 / 0.66%</t>
+          <t>$764.38 / 0.35%</t>
         </is>
       </c>
     </row>
@@ -2580,112 +2580,112 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.36% (7.93%)</t>
+          <t>8.55% (8.12%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.43% (15.68%)</t>
+          <t>16.72% (15.97%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.73% (3.56%)</t>
+          <t>3.90% (3.74%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.72% (5.41%)</t>
+          <t>5.85% (5.55%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.93% (4.70%)</t>
+          <t>5.18% (4.95%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.67% (13.02%)</t>
+          <t>13.90% (13.25%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.36% (12.77%)</t>
+          <t>13.65% (13.06%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.03% (4.68%)</t>
+          <t>5.16% (4.80%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.72% (12.19%)</t>
+          <t>12.98% (12.46%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.34% (2.23%)</t>
+          <t>2.49% (2.39%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.96% (0.93%)</t>
+          <t>1.05% (1.02%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.17% (15.35%)</t>
+          <t>16.43% (15.61%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.69% (6.25%)</t>
+          <t>6.81% (6.37%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.17% (12.42%)</t>
+          <t>13.35% (12.60%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.78% (2.61%)</t>
+          <t>2.87% (2.70%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.39% (4.08%)</t>
+          <t>4.55% (4.24%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.73% (3.50%)</t>
+          <t>3.82% (3.59%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.11% (10.45%)</t>
+          <t>11.27% (10.61%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.65% (10.06%)</t>
+          <t>10.86% (10.26%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.24% (3.88%)</t>
+          <t>4.34% (3.98%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.95% (9.43%)</t>
+          <t>10.14% (9.61%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.51% (1.41%)</t>
+          <t>1.61% (1.50%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.57% (12.75%)</t>
+          <t>13.71% (12.90%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.02%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.76%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.88%</t>
+          <t>-0.58%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.61%</t>
+          <t>13.95%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.51%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>1.18%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.34%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.40%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.48%</t>
+          <t>-3.18%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.65%</t>
+          <t>-2.36%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.82%</t>
+          <t>-2.53%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.34%</t>
+          <t>13.69%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.69% (10.26%)</t>
+          <t>10.60% (10.17%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.47% (8.72%)</t>
+          <t>9.44% (8.69%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.43% (10.26%)</t>
+          <t>10.34% (10.17%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.93% (10.63%)</t>
+          <t>10.80% (10.50%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.36% (10.13%)</t>
+          <t>10.33% (10.10%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.03% (9.38%)</t>
+          <t>9.96% (9.31%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.66% (9.07%)</t>
+          <t>9.63% (9.04%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.45% (13.09%)</t>
+          <t>13.32% (12.97%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.46% (8.93%)</t>
+          <t>9.41% (8.89%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.30% (10.20%)</t>
+          <t>10.20% (10.09%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.64% (9.61%)</t>
+          <t>9.48% (9.45%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.15% (9.33%)</t>
+          <t>10.10% (9.28%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.20% (15.76%)</t>
+          <t>16.07% (15.63%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.59% (13.84%)</t>
+          <t>14.48% (13.73%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.18% (16.01%)</t>
+          <t>16.03% (15.86%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.68% (16.37%)</t>
+          <t>16.59% (16.28%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.04% (15.80%)</t>
+          <t>15.88% (15.65%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.19% (14.53%)</t>
+          <t>15.08% (14.42%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.80% (14.21%)</t>
+          <t>14.73% (14.14%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.40% (19.04%)</t>
+          <t>19.27% (18.91%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.61% (14.08%)</t>
+          <t>14.52% (13.99%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.50% (16.39%)</t>
+          <t>16.35% (16.25%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.85% (15.81%)</t>
+          <t>15.62% (15.59%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.11% (14.30%)</t>
+          <t>14.98% (14.17%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.95% (-6.38%)</t>
+          <t>-5.78% (-6.22%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.64% (-1.39%)</t>
+          <t>-0.40% (-1.15%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.68% (-9.85%)</t>
+          <t>-9.53% (-9.70%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.14% (-8.45%)</t>
+          <t>-8.02% (-8.33%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.45% (-8.68%)</t>
+          <t>-8.23% (-8.46%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.72% (-3.37%)</t>
+          <t>-2.52% (-3.18%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.69% (-3.28%)</t>
+          <t>-2.44% (-3.03%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.42% (-10.77%)</t>
+          <t>-10.31% (-10.67%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.78% (-4.30%)</t>
+          <t>-3.55% (-4.08%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.34% (-12.44%)</t>
+          <t>-12.21% (-12.31%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.37% (-12.40%)</t>
+          <t>-12.29% (-12.32%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.44% (-1.26%)</t>
+          <t>-0.22% (-1.04%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.07% (-5.51%)</t>
+          <t>-4.96% (-5.40%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.52% (-1.27%)</t>
+          <t>-0.37% (-1.12%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.36% (-8.53%)</t>
+          <t>-8.29% (-8.45%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.89% (-7.20%)</t>
+          <t>-6.74% (-7.05%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.28% (-7.51%)</t>
+          <t>-7.20% (-7.43%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.40% (-3.06%)</t>
+          <t>-2.26% (-2.92%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.41% (-3.00%)</t>
+          <t>-2.23% (-2.82%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.69% (-9.06%)</t>
+          <t>-8.61% (-8.97%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.45% (-3.97%)</t>
+          <t>-3.28% (-3.81%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.44% (-10.55%)</t>
+          <t>-10.36% (-10.46%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.49% (-10.53%)</t>
+          <t>-10.50% (-10.53%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.44% (-1.26%)</t>
+          <t>-0.31% (-1.13%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.64%</t>
+          <t>-16.39%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.12%</t>
+          <t>-9.84%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.11%</t>
+          <t>-19.87%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.07%</t>
+          <t>-18.82%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.81%</t>
+          <t>-18.56%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.75%</t>
+          <t>-12.48%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.34%</t>
+          <t>-12.08%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.87%</t>
+          <t>-23.64%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.23%</t>
+          <t>-12.97%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.64%</t>
+          <t>-22.40%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.01%</t>
+          <t>-21.77%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.59%</t>
+          <t>-10.32%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.27%</t>
+          <t>-21.03%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.11%</t>
+          <t>-14.85%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.55%</t>
+          <t>-24.31%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.56%</t>
+          <t>-23.33%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.32%</t>
+          <t>-23.08%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.59%</t>
+          <t>-17.34%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.21%</t>
+          <t>-16.96%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.10%</t>
+          <t>-27.88%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-17.80%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.94%</t>
+          <t>-26.71%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.34%</t>
+          <t>-26.12%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.56%</t>
+          <t>-15.30%</t>
         </is>
       </c>
     </row>
@@ -3215,112 +3215,112 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.57% (1.14%)</t>
+          <t>1.44% (1.01%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.52% (-1.27%)</t>
+          <t>-0.40% (-1.15%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.82% (1.66%)</t>
+          <t>1.68% (1.52%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.21% (1.91%)</t>
+          <t>2.03% (1.72%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.54% (1.31%)</t>
+          <t>1.47% (1.24%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.35% (-0.30%)</t>
+          <t>0.25% (-0.41%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.08% (-0.67%)</t>
+          <t>-0.13% (-0.72%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.03% (4.68%)</t>
+          <t>5.16% (4.80%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.18% (-0.71%)</t>
+          <t>-0.26% (-0.78%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.09% (1.99%)</t>
+          <t>1.93% (1.83%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.96% (0.93%)</t>
+          <t>1.01% (0.98%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.21% (-0.60%)</t>
+          <t>0.13% (-0.68%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.52% (2.08%)</t>
+          <t>2.32% (1.88%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.39% (-1.14%)</t>
+          <t>-0.37% (-1.12%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.78% (2.61%)</t>
+          <t>2.87% (2.70%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.60% (3.29%)</t>
+          <t>3.44% (3.13%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.84% (2.60%)</t>
+          <t>2.61% (2.38%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.67% (0.02%)</t>
+          <t>0.51% (-0.15%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.20% (-0.39%)</t>
+          <t>0.08% (-0.51%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.24% (3.88%)</t>
+          <t>4.34% (3.98%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.16% (-0.36%)</t>
+          <t>0.02% (-0.50%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.51% (1.41%)</t>
+          <t>1.61% (1.50%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.20% (-0.62%)</t>
+          <t>0.02% (-0.80%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/9/2026</t>
+          <t>As of 1/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.13%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>4.95%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.68%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.50%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.55%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.30%</t>
+          <t>8.16%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>10.87%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.45%</t>
+          <t>-8.33%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.09%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.80%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.22%</t>
+          <t>17.86%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.88%</t>
+          <t>-0.58%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.77%</t>
+          <t>-10.67%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.93%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>5.73%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.97%</t>
+          <t>7.64%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.66%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.38%</t>
+          <t>-6.22%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.35%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.30%</t>
+          <t>-4.08%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.04%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.76%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-3.03%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.38%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.02%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>13.60%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-3.18%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.69%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.68%</t>
+          <t>15.97%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.02%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>15.61%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.04%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>1.02%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.19%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.40%</t>
+          <t>15.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>0.04%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.40%</t>
+          <t>-12.32%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.24%</t>
+          <t>13.07%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.44%</t>
+          <t>-12.31%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.65%</t>
+          <t>12.31%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.85%</t>
+          <t>-9.70%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 30/9/2026</t>
+          <t>As of 1/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.80%</t>
+          <t>15.65%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.21%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>1.18%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.51%</t>
+          <t>-7.43%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>16.28%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.08%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.84%</t>
+          <t>6.68%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>10.87%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.20%</t>
+          <t>-7.05%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.04%</t>
+          <t>18.91%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>3.98%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.03%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.22%</t>
+          <t>17.86%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.48%</t>
+          <t>-3.18%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.06%</t>
+          <t>-8.97%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.63%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.25%</t>
+          <t>6.37%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.97%</t>
+          <t>7.64%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.51%</t>
+          <t>-5.40%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.08%</t>
+          <t>13.99%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>9.61%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.74%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.97%</t>
+          <t>-3.81%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>14.14%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.06%</t>
+          <t>10.26%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.67%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.40%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-2.82%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.45%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>2.14%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.34%</t>
+          <t>10.68%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-2.92%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.84%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.42%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.61%</t>
+          <t>13.95%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.27%</t>
+          <t>-1.12%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.75%</t>
+          <t>12.90%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.34%</t>
+          <t>13.69%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.13%</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>15.59%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.40%</t>
+          <t>15.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.82%</t>
+          <t>-2.53%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.39%</t>
+          <t>16.25%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.41%</t>
+          <t>1.50%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.65%</t>
+          <t>-2.36%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.55%</t>
+          <t>-10.46%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>15.86%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>2.70%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.40%</t>
+          <t>8.31%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.65%</t>
+          <t>12.31%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.51%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.53%</t>
+          <t>-8.45%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-02]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/1/2026 at 2:50 PM ET)</t>
+          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>196 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>105 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>287 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>259 days</t>
+          <t>258 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>14 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>197 days</t>
+          <t>196 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>106 days</t>
+          <t>105 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>288 days</t>
+          <t>287 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>259 days</t>
+          <t>258 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>15 days</t>
+          <t>14 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.86 / 5.73%</t>
+          <t>$48.01 / 6.06%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.71 / 0.30%</t>
+          <t>$57.91 / 0.65%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.01 / 9.80%</t>
+          <t>$56.19 / 10.16%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.64 / 8.16%</t>
+          <t>$62.80 / 8.44%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.62 / 8.32%</t>
+          <t>$56.81 / 8.68%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.29 / 2.41%</t>
+          <t>$61.51 / 2.77%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.22 / 2.25%</t>
+          <t>$61.45 / 2.64%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.63 / 10.99%</t>
+          <t>$53.76 / 11.26%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.43 / 3.35%</t>
+          <t>$57.66 / 3.77%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.21 / 13.07%</t>
+          <t>$60.38 / 13.39%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.14 / 13.09%</t>
+          <t>$54.32 / 13.47%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.19 / 0.19%</t>
+          <t>$57.38 / 0.53%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.60 / 4.81%</t>
+          <t>$42.70 / 5.06%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.13 / 0.28%</t>
+          <t>$42.26 / 0.58%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.82 / 8.31%</t>
+          <t>$40.91 / 8.55%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.04 / 6.68%</t>
+          <t>$45.15 / 6.94%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.12 / 7.12%</t>
+          <t>$46.21 / 7.33%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.58 / 2.14%</t>
+          <t>$44.71 / 2.44%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.99 / 2.03%</t>
+          <t>$42.11 / 2.34%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.24 / 8.92%</t>
+          <t>$45.32 / 9.11%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.95 / 3.06%</t>
+          <t>$44.08 / 3.38%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.88 / 10.74%</t>
+          <t>$42.96 / 10.95%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.74 / 10.82%</t>
+          <t>$42.81 / 11.00%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.17 / 0.30%</t>
+          <t>$42.29 / 0.58%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$764.38 / 7.64%</t>
+          <t>$768.98 / 8.28%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$764.38 / -0.18%</t>
+          <t>$768.98 / 0.43%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$764.38 / 12.31%</t>
+          <t>$768.98 / 12.99%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$764.38 / 10.87%</t>
+          <t>$768.98 / 11.54%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$764.38 / 10.51%</t>
+          <t>$768.98 / 11.18%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$764.38 / 2.84%</t>
+          <t>$768.98 / 3.46%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$764.38 / 2.36%</t>
+          <t>$768.98 / 2.98%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$764.38 / 17.86%</t>
+          <t>$768.98 / 18.56%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$764.38 / 3.41%</t>
+          <t>$768.98 / 4.03%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$764.38 / 15.98%</t>
+          <t>$768.98 / 16.68%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$764.38 / 15.05%</t>
+          <t>$768.98 / 15.74%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$764.38 / 0.35%</t>
+          <t>$768.98 / 0.96%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$764.38 / 7.64%</t>
+          <t>$768.98 / 8.28%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$764.38 / -0.18%</t>
+          <t>$769.02 / 0.43%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$764.38 / 12.31%</t>
+          <t>$769.02 / 12.99%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$764.38 / 10.87%</t>
+          <t>$768.98 / 11.54%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$764.38 / 10.51%</t>
+          <t>$768.98 / 11.18%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$764.38 / 2.84%</t>
+          <t>$769.02 / 3.46%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$764.38 / 2.36%</t>
+          <t>$768.98 / 2.98%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$764.38 / 17.86%</t>
+          <t>$768.98 / 18.56%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$764.38 / 3.41%</t>
+          <t>$768.98 / 4.03%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$764.38 / 15.98%</t>
+          <t>$769.02 / 16.69%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$764.38 / 15.05%</t>
+          <t>$769.02 / 15.75%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$764.38 / 0.35%</t>
+          <t>$769.02 / 0.96%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.55% (8.12%)</t>
+          <t>8.21% (7.78%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.72% (15.97%)</t>
+          <t>16.32% (15.57%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.90% (3.74%)</t>
+          <t>3.56% (3.40%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.85% (5.55%)</t>
+          <t>5.58% (5.28%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.18% (4.95%)</t>
+          <t>4.83% (4.60%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.90% (13.25%)</t>
+          <t>13.49% (12.84%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.65% (13.06%)</t>
+          <t>13.22% (12.63%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>5.16% (4.80%)</t>
+          <t>4.90% (4.55%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.98% (12.46%)</t>
+          <t>12.52% (12.00%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.49% (2.39%)</t>
+          <t>2.20% (2.10%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.05% (1.02%)</t>
+          <t>0.71% (0.69%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.43% (15.61%)</t>
+          <t>16.03% (15.22%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.81% (6.37%)</t>
+          <t>6.56% (6.12%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.35% (12.60%)</t>
+          <t>12.99% (12.25%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.87% (2.70%)</t>
+          <t>2.64% (2.47%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.55% (4.24%)</t>
+          <t>4.29% (3.99%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.82% (3.59%)</t>
+          <t>3.62% (3.39%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.27% (10.61%)</t>
+          <t>10.94% (10.29%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.86% (10.26%)</t>
+          <t>10.52% (9.94%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.34% (3.98%)</t>
+          <t>4.15% (3.80%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.14% (9.61%)</t>
+          <t>9.80% (9.28%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.61% (1.50%)</t>
+          <t>1.42% (1.31%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.46% (0.43%)</t>
+          <t>0.29% (0.26%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.71% (12.90%)</t>
+          <t>13.40% (12.59%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>16.67%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>12.92%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.58%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.23%</t>
+          <t>12.55%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.56%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.95%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.01%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.18%</t>
+          <t>-3.76%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.36%</t>
+          <t>-2.95%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.53%</t>
+          <t>-3.11%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.69%</t>
+          <t>13.00%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.60% (10.17%)</t>
+          <t>10.80% (10.37%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.44% (8.69%)</t>
+          <t>9.64% (8.89%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.34% (10.17%)</t>
+          <t>10.51% (10.35%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.80% (10.50%)</t>
+          <t>11.05% (10.75%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.33% (10.10%)</t>
+          <t>10.51% (10.28%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.96% (9.31%)</t>
+          <t>10.13% (9.48%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.63% (9.04%)</t>
+          <t>9.79% (9.21%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.32% (12.97%)</t>
+          <t>13.56% (13.21%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.41% (8.89%)</t>
+          <t>9.54% (9.02%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.20% (10.09%)</t>
+          <t>10.41% (10.31%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.48% (9.45%)</t>
+          <t>9.65% (9.63%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.10% (9.28%)</t>
+          <t>10.29% (9.48%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.07% (15.63%)</t>
+          <t>16.31% (15.88%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.48% (13.73%)</t>
+          <t>14.69% (13.94%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.03% (15.86%)</t>
+          <t>16.28% (16.12%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.59% (16.28%)</t>
+          <t>16.82% (16.51%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.88% (15.65%)</t>
+          <t>16.16% (15.93%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.08% (14.42%)</t>
+          <t>15.29% (14.64%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.73% (14.14%)</t>
+          <t>14.93% (14.35%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.27% (18.91%)</t>
+          <t>19.54% (19.18%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.52% (13.99%)</t>
+          <t>14.71% (14.19%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.35% (16.25%)</t>
+          <t>16.63% (16.52%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.62% (15.59%)</t>
+          <t>15.92% (15.89%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.98% (14.17%)</t>
+          <t>15.22% (14.41%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.78% (-6.22%)</t>
+          <t>-6.08% (-6.51%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.40% (-1.15%)</t>
+          <t>-0.74% (-1.49%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.53% (-9.70%)</t>
+          <t>-9.83% (-9.99%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.02% (-8.33%)</t>
+          <t>-8.26% (-8.56%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.23% (-8.46%)</t>
+          <t>-8.54% (-8.77%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.52% (-3.18%)</t>
+          <t>-2.87% (-3.52%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.44% (-3.03%)</t>
+          <t>-2.81% (-3.39%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.31% (-10.67%)</t>
+          <t>-10.53% (-10.88%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.55% (-4.08%)</t>
+          <t>-3.95% (-4.47%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.21% (-12.31%)</t>
+          <t>-12.46% (-12.56%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.29% (-12.32%)</t>
+          <t>-12.59% (-12.61%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.22% (-1.04%)</t>
+          <t>-0.56% (-1.37%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-4.96% (-5.40%)</t>
+          <t>-5.19% (-5.62%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.37% (-1.12%)</t>
+          <t>-0.68% (-1.42%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.29% (-8.45%)</t>
+          <t>-8.49% (-8.65%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.74% (-7.05%)</t>
+          <t>-6.97% (-7.28%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.20% (-7.43%)</t>
+          <t>-7.39% (-7.61%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.26% (-2.92%)</t>
+          <t>-2.55% (-3.20%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.23% (-2.82%)</t>
+          <t>-2.52% (-3.11%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.61% (-8.97%)</t>
+          <t>-8.77% (-9.13%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.28% (-3.81%)</t>
+          <t>-3.58% (-4.10%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.36% (-10.46%)</t>
+          <t>-10.53% (-10.63%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.50% (-10.53%)</t>
+          <t>-10.65% (-10.67%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.31% (-1.13%)</t>
+          <t>-0.59% (-1.40%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.39%</t>
+          <t>-16.89%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.84%</t>
+          <t>-10.38%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.87%</t>
+          <t>-20.34%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.82%</t>
+          <t>-19.31%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.56%</t>
+          <t>-19.05%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.48%</t>
+          <t>-13.01%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.08%</t>
+          <t>-12.60%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.64%</t>
+          <t>-24.09%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.97%</t>
+          <t>-13.49%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.40%</t>
+          <t>-22.87%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.77%</t>
+          <t>-22.24%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.32%</t>
+          <t>-10.85%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.03%</t>
+          <t>-21.50%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.85%</t>
+          <t>-15.36%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.31%</t>
+          <t>-24.77%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.33%</t>
+          <t>-23.79%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.08%</t>
+          <t>-23.54%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.34%</t>
+          <t>-17.84%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.96%</t>
+          <t>-17.46%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.88%</t>
+          <t>-28.31%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.80%</t>
+          <t>-18.29%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.71%</t>
+          <t>-27.15%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.12%</t>
+          <t>-26.56%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.30%</t>
+          <t>-15.81%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.44% (1.01%)</t>
+          <t>1.73% (1.30%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.40% (-1.15%)</t>
+          <t>-0.32% (-1.07%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.68% (1.52%)</t>
+          <t>1.96% (1.80%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.03% (1.72%)</t>
+          <t>2.38% (2.08%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.47% (1.24%)</t>
+          <t>1.74% (1.52%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.25% (-0.41%)</t>
+          <t>0.49% (-0.16%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.13% (-0.72%)</t>
+          <t>0.09% (-0.49%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5.16% (4.80%)</t>
+          <t>4.90% (4.55%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.78%)</t>
+          <t>-0.06% (-0.58%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.93% (1.83%)</t>
+          <t>2.20% (2.10%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.01% (0.98%)</t>
+          <t>0.71% (0.69%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.13% (-0.68%)</t>
+          <t>0.39% (-0.42%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.32% (1.88%)</t>
+          <t>2.70% (2.26%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.37% (-1.12%)</t>
+          <t>-0.25% (-1.00%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.87% (2.70%)</t>
+          <t>2.64% (2.47%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.44% (3.13%)</t>
+          <t>3.81% (3.51%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.61% (2.38%)</t>
+          <t>3.03% (2.80%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.51% (-0.15%)</t>
+          <t>0.83% (0.17%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.08% (-0.51%)</t>
+          <t>0.39% (-0.20%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.34% (3.98%)</t>
+          <t>4.15% (3.80%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.02% (-0.50%)</t>
+          <t>0.32% (-0.20%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.61% (1.50%)</t>
+          <t>1.42% (1.31%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.46% (0.43%)</t>
+          <t>0.29% (0.26%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.02% (-0.80%)</t>
+          <t>0.35% (-0.46%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 1/10/2026</t>
+          <t>As of 2/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.95%</t>
+          <t>4.60%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.68%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.77%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.55%</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.16%</t>
+          <t>8.44%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.87%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.33%</t>
+          <t>-8.56%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.80%</t>
+          <t>4.55%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.99%</t>
+          <t>11.26%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.86%</t>
+          <t>18.56%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.58%</t>
+          <t>-1.18%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.67%</t>
+          <t>-10.88%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>10.37%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>7.78%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.73%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.64%</t>
+          <t>8.28%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>6.35%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.22%</t>
+          <t>-6.51%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.23%</t>
+          <t>12.55%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.08%</t>
+          <t>-4.47%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.04%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>12.63%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.64%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.03%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>12.84%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.77%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.60%</t>
+          <t>12.92%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.18%</t>
+          <t>-3.52%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.69%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.97%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>16.67%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.49%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.61%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.19%</t>
+          <t>0.53%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.04%</t>
+          <t>-1.37%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.09%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.05%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.04%</t>
+          <t>-0.56%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.32%</t>
+          <t>-12.61%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.07%</t>
+          <t>13.39%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.68%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.31%</t>
+          <t>-12.56%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.40%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.31%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.70%</t>
+          <t>-9.99%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 1/10/2026</t>
+          <t>As of 2/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.65%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.39%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>7.33%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.43%</t>
+          <t>-7.61%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.28%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.24%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.68%</t>
+          <t>6.94%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.87%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.05%</t>
+          <t>-7.28%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.91%</t>
+          <t>19.18%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.98%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.86%</t>
+          <t>18.56%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.18%</t>
+          <t>-3.76%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-8.97%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.63%</t>
+          <t>15.88%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.37%</t>
+          <t>6.12%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.64%</t>
+          <t>8.28%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.40%</t>
+          <t>-5.62%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.99%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.61%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-4.10%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.14%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.26%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>2.34%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.82%</t>
+          <t>-3.11%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>14.64%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.14%</t>
+          <t>2.44%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.68%</t>
+          <t>10.01%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.92%</t>
+          <t>-3.20%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.94%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.58%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.95%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-1.42%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>14.41%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.90%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.58%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.69%</t>
+          <t>13.00%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.13%</t>
+          <t>-1.40%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.59%</t>
+          <t>15.89%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.05%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.53%</t>
+          <t>-3.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.53%</t>
+          <t>-10.67%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.25%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.95%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.69%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.36%</t>
+          <t>-2.95%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.46%</t>
+          <t>-10.63%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.86%</t>
+          <t>16.12%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.70%</t>
+          <t>2.47%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.31%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.31%</t>
+          <t>12.99%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.45%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-05]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:30 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/2/2026 at 2:31 PM ET)</t>
+          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>196 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>322 days</t>
+          <t>319 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>77 days</t>
+          <t>74 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>140 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>105 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>287 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>258 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>168 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>49 days</t>
+          <t>46 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>14 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>347 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>196 days</t>
+          <t>193 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>322 days</t>
+          <t>319 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>77 days</t>
+          <t>74 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>140 days</t>
+          <t>137 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>105 days</t>
+          <t>102 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>287 days</t>
+          <t>284 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>258 days</t>
+          <t>255 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>168 days</t>
+          <t>165 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>228 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>49 days</t>
+          <t>46 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>14 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>350 days</t>
+          <t>347 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.01 / 6.06%</t>
+          <t>$48.19 / 6.44%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.91 / 0.65%</t>
+          <t>$58.19 / 1.14%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.19 / 10.16%</t>
+          <t>$56.40 / 10.56%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.80 / 8.44%</t>
+          <t>$63.06 / 8.88%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.81 / 8.68%</t>
+          <t>$57.01 / 9.07%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.51 / 2.77%</t>
+          <t>$61.76 / 3.19%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.45 / 2.64%</t>
+          <t>$61.70 / 3.05%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.76 / 11.26%</t>
+          <t>$53.89 / 11.53%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.66 / 3.77%</t>
+          <t>$57.94 / 4.28%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.38 / 13.39%</t>
+          <t>$60.59 / 13.79%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.32 / 13.47%</t>
+          <t>$54.49 / 13.83%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.38 / 0.53%</t>
+          <t>$57.65 / 1.00%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.70 / 5.06%</t>
+          <t>$42.81 / 5.33%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.26 / 0.58%</t>
+          <t>$42.39 / 0.91%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.91 / 8.55%</t>
+          <t>$41.01 / 8.82%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.15 / 6.94%</t>
+          <t>$45.27 / 7.21%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.21 / 7.33%</t>
+          <t>$46.35 / 7.66%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.71 / 2.44%</t>
+          <t>$44.86 / 2.78%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.11 / 2.34%</t>
+          <t>$42.26 / 2.69%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.32 / 9.11%</t>
+          <t>$45.41 / 9.33%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.08 / 3.38%</t>
+          <t>$44.24 / 3.74%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.96 / 10.95%</t>
+          <t>$43.05 / 11.18%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.81 / 11.00%</t>
+          <t>$42.88 / 11.17%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.29 / 0.58%</t>
+          <t>$42.44 / 0.95%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$768.98 / 8.28%</t>
+          <t>$774.93 / 9.12%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$768.98 / 0.43%</t>
+          <t>$774.93 / 1.20%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$768.98 / 12.99%</t>
+          <t>$774.93 / 13.86%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$768.98 / 11.54%</t>
+          <t>$774.93 / 12.40%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$768.98 / 11.18%</t>
+          <t>$774.93 / 12.04%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$768.98 / 3.46%</t>
+          <t>$774.93 / 4.26%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$768.98 / 2.98%</t>
+          <t>$774.93 / 3.77%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$768.98 / 18.56%</t>
+          <t>$774.93 / 19.48%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$768.98 / 4.03%</t>
+          <t>$774.93 / 4.84%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$768.98 / 16.68%</t>
+          <t>$774.93 / 17.59%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$768.98 / 15.74%</t>
+          <t>$774.93 / 16.64%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$768.98 / 0.96%</t>
+          <t>$774.93 / 1.74%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$768.98 / 8.28%</t>
+          <t>$774.93 / 9.12%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$769.02 / 0.43%</t>
+          <t>$774.93 / 1.20%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$769.02 / 12.99%</t>
+          <t>$774.93 / 13.86%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$768.98 / 11.54%</t>
+          <t>$774.93 / 12.40%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$768.98 / 11.18%</t>
+          <t>$774.93 / 12.04%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$769.02 / 3.46%</t>
+          <t>$774.93 / 4.26%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$768.98 / 2.98%</t>
+          <t>$774.93 / 3.77%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$768.98 / 18.56%</t>
+          <t>$774.93 / 19.48%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$768.98 / 4.03%</t>
+          <t>$774.93 / 4.84%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$769.02 / 16.69%</t>
+          <t>$774.93 / 17.59%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$769.02 / 15.75%</t>
+          <t>$774.93 / 16.64%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$769.02 / 0.96%</t>
+          <t>$774.93 / 1.74%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.21% (7.78%)</t>
+          <t>7.81% (7.39%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.32% (15.57%)</t>
+          <t>15.75% (15.01%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.56% (3.40%)</t>
+          <t>3.18% (3.02%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.58% (5.28%)</t>
+          <t>5.15% (4.85%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.83% (4.60%)</t>
+          <t>4.44% (4.22%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.49% (12.84%)</t>
+          <t>13.03% (12.39%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.22% (12.63%)</t>
+          <t>12.75% (12.18%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.90% (4.55%)</t>
+          <t>4.64% (4.30%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.52% (12.00%)</t>
+          <t>11.97% (11.46%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.20% (2.10%)</t>
+          <t>1.84% (1.74%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.71% (0.69%)</t>
+          <t>0.38% (0.36%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.03% (15.22%)</t>
+          <t>15.48% (14.68%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.56% (6.12%)</t>
+          <t>6.28% (5.85%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.99% (12.25%)</t>
+          <t>12.63% (11.89%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.64% (2.47%)</t>
+          <t>2.38% (2.22%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.29% (3.99%)</t>
+          <t>4.02% (3.73%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.62% (3.39%)</t>
+          <t>3.29% (3.07%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.94% (10.29%)</t>
+          <t>10.56% (9.92%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.52% (9.94%)</t>
+          <t>10.14% (9.56%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.15% (3.80%)</t>
+          <t>3.94% (3.59%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.80% (9.28%)</t>
+          <t>9.41% (8.89%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.42% (1.31%)</t>
+          <t>1.20% (1.10%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.29% (0.26%)</t>
+          <t>0.13% (0.11%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.40% (12.59%)</t>
+          <t>12.98% (12.18%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>0.78%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.92%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.94%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.55%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-1.33%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>2.95%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>-0.31%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.76%</t>
+          <t>-4.50%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.95%</t>
+          <t>-3.68%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-3.85%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.14%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.80% (10.37%)</t>
+          <t>11.09% (10.67%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.64% (8.89%)</t>
+          <t>9.84% (9.11%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.51% (10.35%)</t>
+          <t>10.79% (10.64%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.05% (10.75%)</t>
+          <t>11.29% (11.00%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.51% (10.28%)</t>
+          <t>10.79% (10.57%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.13% (9.48%)</t>
+          <t>10.40% (9.76%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.79% (9.21%)</t>
+          <t>10.06% (9.49%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.56% (13.21%)</t>
+          <t>13.92% (13.58%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.54% (9.02%)</t>
+          <t>9.73% (9.22%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.41% (10.31%)</t>
+          <t>10.69% (10.60%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.65% (9.63%)</t>
+          <t>9.97% (9.94%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.29% (9.48%)</t>
+          <t>10.50% (9.70%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.31% (15.88%)</t>
+          <t>16.67% (16.24%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.69% (13.94%)</t>
+          <t>15.01% (14.27%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.28% (16.12%)</t>
+          <t>16.63% (16.47%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.82% (16.51%)</t>
+          <t>17.16% (16.86%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.16% (15.93%)</t>
+          <t>16.45% (16.23%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.29% (14.64%)</t>
+          <t>15.58% (14.94%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.93% (14.35%)</t>
+          <t>15.23% (14.65%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.54% (19.18%)</t>
+          <t>19.90% (19.55%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.71% (14.19%)</t>
+          <t>14.99% (14.48%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.63% (16.52%)</t>
+          <t>16.99% (16.89%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.92% (15.89%)</t>
+          <t>16.34% (16.31%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.22% (14.41%)</t>
+          <t>15.49% (14.69%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.08% (-6.51%)</t>
+          <t>-6.43% (-6.85%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.74% (-1.49%)</t>
+          <t>-1.23% (-1.96%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.83% (-9.99%)</t>
+          <t>-10.16% (-10.32%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.26% (-8.56%)</t>
+          <t>-8.64% (-8.93%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.54% (-8.77%)</t>
+          <t>-8.88% (-9.10%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.87% (-3.52%)</t>
+          <t>-3.27% (-3.91%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.81% (-3.39%)</t>
+          <t>-3.21% (-3.79%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.53% (-10.88%)</t>
+          <t>-10.75% (-11.10%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.95% (-4.47%)</t>
+          <t>-4.42% (-4.93%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.46% (-12.56%)</t>
+          <t>-12.77% (-12.86%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.59% (-12.61%)</t>
+          <t>-12.87% (-12.90%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.56% (-1.37%)</t>
+          <t>-1.03% (-1.83%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.19% (-5.62%)</t>
+          <t>-5.44% (-5.86%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.68% (-1.42%)</t>
+          <t>-1.00% (-1.74%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.49% (-8.65%)</t>
+          <t>-8.72% (-8.88%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.97% (-7.28%)</t>
+          <t>-7.22% (-7.51%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.39% (-7.61%)</t>
+          <t>-7.68% (-7.90%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.55% (-3.20%)</t>
+          <t>-2.88% (-3.53%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.52% (-3.11%)</t>
+          <t>-2.86% (-3.44%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.77% (-9.13%)</t>
+          <t>-8.96% (-9.31%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.58% (-4.10%)</t>
+          <t>-3.93% (-4.44%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.53% (-10.63%)</t>
+          <t>-10.72% (-10.82%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.65% (-10.67%)</t>
+          <t>-10.79% (-10.81%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.59% (-1.40%)</t>
+          <t>-0.96% (-1.76%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.89%</t>
+          <t>-17.52%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.38%</t>
+          <t>-11.07%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.34%</t>
+          <t>-20.96%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.31%</t>
+          <t>-19.93%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.05%</t>
+          <t>-19.67%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.01%</t>
+          <t>-13.67%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.60%</t>
+          <t>-13.27%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.09%</t>
+          <t>-24.68%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.49%</t>
+          <t>-14.15%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.87%</t>
+          <t>-23.46%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.24%</t>
+          <t>-22.84%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.85%</t>
+          <t>-11.54%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.50%</t>
+          <t>-22.10%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.36%</t>
+          <t>-16.01%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.77%</t>
+          <t>-25.35%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.79%</t>
+          <t>-24.37%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.54%</t>
+          <t>-24.13%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.84%</t>
+          <t>-18.47%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.46%</t>
+          <t>-18.09%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.31%</t>
+          <t>-28.86%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.29%</t>
+          <t>-18.92%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.15%</t>
+          <t>-27.71%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.56%</t>
+          <t>-27.12%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.81%</t>
+          <t>-16.45%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.73% (1.30%)</t>
+          <t>2.14% (1.72%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.32% (-1.07%)</t>
+          <t>-0.04% (-0.77%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.96% (1.80%)</t>
+          <t>2.37% (2.22%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.38% (2.08%)</t>
+          <t>2.75% (2.46%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.74% (1.52%)</t>
+          <t>2.16% (1.94%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.49% (-0.16%)</t>
+          <t>0.85% (0.21%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.09% (-0.49%)</t>
+          <t>0.45% (-0.12%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.90% (4.55%)</t>
+          <t>4.64% (4.30%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.58%)</t>
+          <t>0.22% (-0.29%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.20% (2.10%)</t>
+          <t>1.84% (1.74%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.71% (0.69%)</t>
+          <t>0.38% (0.36%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.39% (-0.42%)</t>
+          <t>0.69% (-0.11%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.70% (2.26%)</t>
+          <t>3.22% (2.80%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.25% (-1.00%)</t>
+          <t>0.19% (-0.55%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.64% (2.47%)</t>
+          <t>2.38% (2.22%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.81% (3.51%)</t>
+          <t>4.02% (3.73%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.03% (2.80%)</t>
+          <t>3.29% (3.07%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.83% (0.17%)</t>
+          <t>1.25% (0.61%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.39% (-0.20%)</t>
+          <t>0.81% (0.23%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.15% (3.80%)</t>
+          <t>3.94% (3.59%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.32% (-0.20%)</t>
+          <t>0.73% (0.22%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.42% (1.31%)</t>
+          <t>1.20% (1.10%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.29% (0.26%)</t>
+          <t>0.13% (0.11%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.35% (-0.46%)</t>
+          <t>0.74% (-0.06%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 2/10/2026</t>
+          <t>As of 5/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.60%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.68%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.77%</t>
+          <t>-9.10%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>4.85%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.44%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.56%</t>
+          <t>-8.93%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>13.58%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.55%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>11.53%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.56%</t>
+          <t>19.48%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.94%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.88%</t>
+          <t>-11.10%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.78%</t>
+          <t>7.39%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.44%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.28%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.35%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.51%</t>
+          <t>-6.85%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>9.22%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.55%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.47%</t>
+          <t>-4.93%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.63%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.64%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.39%</t>
+          <t>-3.79%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.76%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.84%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.77%</t>
+          <t>3.19%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>4.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.92%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-3.91%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>15.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>1.14%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>1.20%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.49%</t>
+          <t>-1.96%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.53%</t>
+          <t>1.00%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-1.83%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.47%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-1.33%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.61%</t>
+          <t>-12.90%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.39%</t>
+          <t>13.79%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.68%</t>
+          <t>17.59%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.56%</t>
+          <t>-12.86%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.40%</t>
+          <t>3.02%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>13.86%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>0.78%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.99%</t>
+          <t>-10.32%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 2/10/2026</t>
+          <t>As of 5/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>16.23%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.39%</t>
+          <t>3.07%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.33%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>-0.20%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.61%</t>
+          <t>-7.90%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.86%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.94%</t>
+          <t>7.21%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>-0.31%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-7.51%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.18%</t>
+          <t>19.55%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.80%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.56%</t>
+          <t>19.48%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.76%</t>
+          <t>-4.50%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.31%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.88%</t>
+          <t>16.24%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>5.85%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>5.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.28%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>2.95%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.62%</t>
+          <t>-5.86%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>14.48%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>8.58%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.10%</t>
+          <t>-4.44%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>14.65%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.34%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-3.44%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.64%</t>
+          <t>14.94%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>9.92%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.44%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>4.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.20%</t>
+          <t>-3.53%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.94%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>11.89%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.58%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>1.20%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.42%</t>
+          <t>-1.74%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.41%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.59%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.58%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.74%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.14%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.76%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.89%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.17%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-3.85%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.67%</t>
+          <t>-10.81%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.95%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.69%</t>
+          <t>17.59%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.95%</t>
+          <t>-3.68%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.63%</t>
+          <t>-10.82%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.12%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.99%</t>
+          <t>13.86%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.88%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-06]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/5/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>319 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>347 days</t>
+          <t>346 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>193 days</t>
+          <t>192 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>319 days</t>
+          <t>318 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>74 days</t>
+          <t>73 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>137 days</t>
+          <t>136 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>102 days</t>
+          <t>101 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>284 days</t>
+          <t>283 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>255 days</t>
+          <t>254 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>165 days</t>
+          <t>164 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>228 days</t>
+          <t>227 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>46 days</t>
+          <t>45 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>347 days</t>
+          <t>346 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.19 / 6.44%</t>
+          <t>$48.37 / 6.84%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.19 / 1.14%</t>
+          <t>$58.45 / 1.60%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.40 / 10.56%</t>
+          <t>$56.54 / 10.84%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.06 / 8.88%</t>
+          <t>$63.23 / 9.17%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.01 / 9.07%</t>
+          <t>$57.19 / 9.41%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.76 / 3.19%</t>
+          <t>$62.02 / 3.63%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.70 / 3.05%</t>
+          <t>$62.01 / 3.56%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.89 / 11.53%</t>
+          <t>$54.00 / 11.76%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.94 / 4.28%</t>
+          <t>$58.19 / 4.73%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.59 / 13.79%</t>
+          <t>$60.74 / 14.08%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.49 / 13.83%</t>
+          <t>$54.57 / 14.00%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.65 / 1.00%</t>
+          <t>$57.89 / 1.42%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.81 / 5.33%</t>
+          <t>$42.95 / 5.66%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.39 / 0.91%</t>
+          <t>$42.57 / 1.32%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.01 / 8.82%</t>
+          <t>$41.11 / 9.07%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.27 / 7.21%</t>
+          <t>$45.37 / 7.45%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.35 / 7.66%</t>
+          <t>$46.45 / 7.90%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.86 / 2.78%</t>
+          <t>$45.00 / 3.10%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.26 / 2.69%</t>
+          <t>$42.41 / 3.05%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.41 / 9.33%</t>
+          <t>$45.45 / 9.44%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.24 / 3.74%</t>
+          <t>$44.41 / 4.14%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.05 / 11.18%</t>
+          <t>$43.11 / 11.34%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.88 / 11.17%</t>
+          <t>$42.89 / 11.21%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.44 / 0.95%</t>
+          <t>$42.57 / 1.26%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$774.93 / 9.12%</t>
+          <t>$780.02 / 9.84%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$774.93 / 1.20%</t>
+          <t>$780.02 / 1.87%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$774.93 / 13.86%</t>
+          <t>$780.02 / 14.61%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$774.93 / 12.40%</t>
+          <t>$780.02 / 13.14%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$774.93 / 12.04%</t>
+          <t>$780.02 / 12.77%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$774.93 / 4.26%</t>
+          <t>$780.02 / 4.94%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$774.93 / 3.77%</t>
+          <t>$780.02 / 4.46%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$774.93 / 19.48%</t>
+          <t>$780.02 / 20.27%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$774.93 / 4.84%</t>
+          <t>$780.02 / 5.53%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$774.93 / 17.59%</t>
+          <t>$780.02 / 18.36%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$774.93 / 16.64%</t>
+          <t>$780.02 / 17.40%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$774.93 / 1.74%</t>
+          <t>$780.02 / 2.41%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$774.93 / 9.12%</t>
+          <t>$780.02 / 9.84%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$774.93 / 1.20%</t>
+          <t>$780.02 / 1.87%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$774.93 / 13.86%</t>
+          <t>$780.02 / 14.61%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$774.93 / 12.40%</t>
+          <t>$780.02 / 13.14%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$774.93 / 12.04%</t>
+          <t>$780.02 / 12.77%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$774.93 / 4.26%</t>
+          <t>$780.02 / 4.94%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$774.93 / 3.77%</t>
+          <t>$780.02 / 4.46%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$774.93 / 19.48%</t>
+          <t>$780.02 / 20.27%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$774.93 / 4.84%</t>
+          <t>$780.02 / 5.53%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$774.93 / 17.59%</t>
+          <t>$780.02 / 18.36%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$774.93 / 16.64%</t>
+          <t>$780.02 / 17.40%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$774.93 / 1.74%</t>
+          <t>$780.02 / 2.41%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.81% (7.39%)</t>
+          <t>7.41% (6.99%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.75% (15.01%)</t>
+          <t>15.22% (14.49%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.18% (3.02%)</t>
+          <t>2.92% (2.77%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.15% (4.85%)</t>
+          <t>4.86% (4.57%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.44% (4.22%)</t>
+          <t>4.12% (3.91%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.03% (12.39%)</t>
+          <t>12.54% (11.91%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.75% (12.18%)</t>
+          <t>12.20% (11.62%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.64% (4.30%)</t>
+          <t>4.43% (4.09%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.97% (11.46%)</t>
+          <t>11.48% (10.98%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.84% (1.74%)</t>
+          <t>1.58% (1.49%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.38% (0.36%)</t>
+          <t>0.24% (0.21%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.48% (14.68%)</t>
+          <t>15.00% (14.21%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.28% (5.85%)</t>
+          <t>5.94% (5.52%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.63% (11.89%)</t>
+          <t>12.16% (11.43%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.38% (2.22%)</t>
+          <t>2.14% (1.99%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.02% (3.73%)</t>
+          <t>3.79% (3.50%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.29% (3.07%)</t>
+          <t>3.06% (2.84%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.56% (9.92%)</t>
+          <t>10.22% (9.58%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.14% (9.56%)</t>
+          <t>9.75% (9.17%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.94% (3.59%)</t>
+          <t>3.84% (3.49%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.41% (8.89%)</t>
+          <t>8.98% (8.48%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.20% (1.10%)</t>
+          <t>1.05% (0.96%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.13% (0.11%)</t>
+          <t>0.10% (0.08%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.98% (12.18%)</t>
+          <t>12.63% (11.84%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>15.02%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.78%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>1.65%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.94%</t>
+          <t>-2.57%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.47%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.69%</t>
+          <t>13.94%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-2.20%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.31%</t>
+          <t>-0.96%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.50%</t>
+          <t>-5.12%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-4.48%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.14%</t>
+          <t>11.41%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.09% (10.67%)</t>
+          <t>11.28% (10.86%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.84% (9.11%)</t>
+          <t>9.97% (9.24%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.79% (10.64%)</t>
+          <t>11.08% (10.93%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.29% (11.00%)</t>
+          <t>11.57% (11.28%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.79% (10.57%)</t>
+          <t>11.04% (10.82%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.40% (9.76%)</t>
+          <t>10.55% (9.91%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.06% (9.49%)</t>
+          <t>10.15% (9.58%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.92% (13.58%)</t>
+          <t>14.23% (13.89%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.73% (9.22%)</t>
+          <t>9.88% (9.37%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.69% (10.60%)</t>
+          <t>10.97% (10.88%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.97% (9.94%)</t>
+          <t>10.34% (10.32%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.50% (9.70%)</t>
+          <t>10.67% (9.87%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.67% (16.24%)</t>
+          <t>16.88% (16.45%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.01% (14.27%)</t>
+          <t>15.15% (14.42%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.63% (16.47%)</t>
+          <t>16.90% (16.74%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.16% (16.86%)</t>
+          <t>17.44% (17.15%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.45% (16.23%)</t>
+          <t>16.74% (16.52%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.58% (14.94%)</t>
+          <t>15.81% (15.17%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.23% (14.65%)</t>
+          <t>15.42% (14.84%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.90% (19.55%)</t>
+          <t>20.27% (19.92%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.99% (14.48%)</t>
+          <t>15.15% (14.64%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.99% (16.89%)</t>
+          <t>17.33% (17.24%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.34% (16.31%)</t>
+          <t>16.78% (16.76%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.49% (14.69%)</t>
+          <t>15.73% (14.94%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.43% (-6.85%)</t>
+          <t>-6.78% (-7.20%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.23% (-1.96%)</t>
+          <t>-1.68% (-2.41%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.16% (-10.32%)</t>
+          <t>-10.39% (-10.54%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.64% (-8.93%)</t>
+          <t>-8.89% (-9.18%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.88% (-9.10%)</t>
+          <t>-9.16% (-9.38%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.27% (-3.91%)</t>
+          <t>-3.69% (-4.32%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.79%)</t>
+          <t>-3.69% (-4.26%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.75% (-11.10%)</t>
+          <t>-10.94% (-11.28%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.42% (-4.93%)</t>
+          <t>-4.83% (-5.34%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.77% (-12.86%)</t>
+          <t>-12.99% (-13.08%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.87% (-12.90%)</t>
+          <t>-13.00% (-13.02%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.03% (-1.83%)</t>
+          <t>-1.45% (-2.24%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.44% (-5.86%)</t>
+          <t>-5.74% (-6.16%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.00% (-1.74%)</t>
+          <t>-1.41% (-2.14%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.72% (-8.88%)</t>
+          <t>-8.93% (-9.09%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.22% (-7.51%)</t>
+          <t>-7.42% (-7.72%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.68% (-7.90%)</t>
+          <t>-7.88% (-8.10%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.88% (-3.53%)</t>
+          <t>-3.19% (-3.83%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.86% (-3.44%)</t>
+          <t>-3.21% (-3.78%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.96% (-9.31%)</t>
+          <t>-9.05% (-9.40%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.93% (-4.44%)</t>
+          <t>-4.30% (-4.80%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.72% (-10.82%)</t>
+          <t>-10.85% (-10.94%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.79% (-10.81%)</t>
+          <t>-10.82% (-10.84%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.96% (-1.76%)</t>
+          <t>-1.26% (-2.06%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.52%</t>
+          <t>-18.06%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-11.07%</t>
+          <t>-11.65%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.96%</t>
+          <t>-21.47%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.93%</t>
+          <t>-20.45%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.67%</t>
+          <t>-20.20%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.67%</t>
+          <t>-14.24%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.27%</t>
+          <t>-13.84%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.68%</t>
+          <t>-25.17%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.15%</t>
+          <t>-14.71%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.46%</t>
+          <t>-23.96%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.84%</t>
+          <t>-23.34%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.54%</t>
+          <t>-12.11%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.10%</t>
+          <t>-22.61%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.01%</t>
+          <t>-16.56%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.35%</t>
+          <t>-25.83%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.37%</t>
+          <t>-24.87%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.13%</t>
+          <t>-24.63%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.47%</t>
+          <t>-19.00%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.09%</t>
+          <t>-18.62%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.86%</t>
+          <t>-29.32%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.92%</t>
+          <t>-19.45%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.71%</t>
+          <t>-28.18%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.12%</t>
+          <t>-27.60%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.45%</t>
+          <t>-17.00%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.14% (1.72%)</t>
+          <t>2.43% (2.01%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.77%)</t>
+          <t>0.16% (-0.57%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.37% (2.22%)</t>
+          <t>2.79% (2.64%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.75% (2.46%)</t>
+          <t>3.15% (2.86%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.16% (1.94%)</t>
+          <t>2.52% (2.30%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.85% (0.21%)</t>
+          <t>1.08% (0.44%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.45% (-0.12%)</t>
+          <t>0.61% (0.04%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.64% (4.30%)</t>
+          <t>4.43% (4.09%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.22% (-0.29%)</t>
+          <t>0.44% (-0.06%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.84% (1.74%)</t>
+          <t>1.58% (1.49%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.38% (0.36%)</t>
+          <t>0.24% (0.21%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.69% (-0.11%)</t>
+          <t>0.93% (0.13%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.22% (2.80%)</t>
+          <t>3.57% (3.15%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.19% (-0.55%)</t>
+          <t>0.43% (-0.30%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.38% (2.22%)</t>
+          <t>2.14% (1.99%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.02% (3.73%)</t>
+          <t>3.79% (3.50%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.29% (3.07%)</t>
+          <t>3.06% (2.84%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.25% (0.61%)</t>
+          <t>1.60% (0.96%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.81% (0.23%)</t>
+          <t>1.11% (0.54%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.94% (3.59%)</t>
+          <t>3.84% (3.49%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.73% (0.22%)</t>
+          <t>1.01% (0.50%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.20% (1.10%)</t>
+          <t>1.05% (0.96%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.13% (0.11%)</t>
+          <t>0.10% (0.08%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.74% (-0.06%)</t>
+          <t>1.09% (0.30%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 5/10/2026</t>
+          <t>As of 6/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>10.82%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.04%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.10%</t>
+          <t>-9.38%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.28%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.85%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>13.14%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>1.65%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.93%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.58%</t>
+          <t>13.89%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.53%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.48%</t>
+          <t>20.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.94%</t>
+          <t>-2.57%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.10%</t>
+          <t>-11.28%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.39%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.44%</t>
+          <t>6.84%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.85%</t>
+          <t>-7.20%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.22%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>4.73%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.93%</t>
+          <t>-5.34%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.21%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.79%</t>
+          <t>-4.26%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.76%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.19%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.26%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.91%</t>
+          <t>-4.32%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.01%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.14%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.20%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>15.02%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.96%</t>
+          <t>-2.41%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.69%</t>
+          <t>13.94%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.83%</t>
+          <t>-2.24%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.36%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>17.40%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.90%</t>
+          <t>-13.02%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>1.49%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.79%</t>
+          <t>14.08%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.59%</t>
+          <t>18.36%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.47%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.86%</t>
+          <t>-13.08%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.93%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>2.77%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.84%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.86%</t>
+          <t>14.61%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.78%</t>
+          <t>0.12%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.32%</t>
+          <t>-10.54%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 5/10/2026</t>
+          <t>As of 6/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.07%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>7.90%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.04%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.90%</t>
+          <t>-8.10%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.86%</t>
+          <t>17.15%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.21%</t>
+          <t>7.45%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>13.14%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.31%</t>
+          <t>-0.96%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.51%</t>
+          <t>-7.72%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.55%</t>
+          <t>19.92%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.48%</t>
+          <t>20.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.50%</t>
+          <t>-5.12%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.31%</t>
+          <t>-9.40%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>16.45%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.85%</t>
+          <t>5.52%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.33%</t>
+          <t>5.66%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>2.28%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.86%</t>
+          <t>-6.16%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.48%</t>
+          <t>14.64%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>4.14%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.58%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-4.80%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.65%</t>
+          <t>14.84%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>8.52%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-3.78%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.94%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.92%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.26%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-3.83%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.89%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>1.32%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.20%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>11.67%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.74%</t>
+          <t>-2.14%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.69%</t>
+          <t>14.94%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.18%</t>
+          <t>11.84%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>1.26%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.74%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.14%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.76%</t>
+          <t>-2.06%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.31%</t>
+          <t>16.76%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.17%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>17.40%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-4.48%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.81%</t>
+          <t>-10.84%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.59%</t>
+          <t>18.36%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.82%</t>
+          <t>-10.94%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.74%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>1.99%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.86%</t>
+          <t>14.61%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-2.20%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.88%</t>
+          <t>-9.09%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-07]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/6/2026 at 2:54 PM ET)</t>
+          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>192 days</t>
+          <t>191 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>318 days</t>
+          <t>317 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>73 days</t>
+          <t>72 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>136 days</t>
+          <t>135 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>101 days</t>
+          <t>100 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>283 days</t>
+          <t>282 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>254 days</t>
+          <t>253 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>164 days</t>
+          <t>163 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>227 days</t>
+          <t>226 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>45 days</t>
+          <t>44 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>346 days</t>
+          <t>345 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.37 / 6.84%</t>
+          <t>$48.31 / 6.72%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.45 / 1.60%</t>
+          <t>$58.34 / 1.40%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.54 / 10.84%</t>
+          <t>$56.47 / 10.71%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.23 / 9.17%</t>
+          <t>$63.15 / 9.03%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.19 / 9.41%</t>
+          <t>$57.14 / 9.32%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$62.02 / 3.63%</t>
+          <t>$61.94 / 3.50%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$62.01 / 3.56%</t>
+          <t>$61.89 / 3.36%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$54.00 / 11.76%</t>
+          <t>$53.94 / 11.64%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$58.19 / 4.73%</t>
+          <t>$58.10 / 4.56%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.74 / 14.08%</t>
+          <t>$60.68 / 13.97%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.57 / 14.00%</t>
+          <t>$54.57 / 13.99%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.89 / 1.42%</t>
+          <t>$57.79 / 1.25%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.95 / 5.66%</t>
+          <t>$42.90 / 5.54%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.57 / 1.32%</t>
+          <t>$42.50 / 1.17%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.11 / 9.07%</t>
+          <t>$41.09 / 9.01%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.37 / 7.45%</t>
+          <t>$45.33 / 7.37%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.45 / 7.90%</t>
+          <t>$46.40 / 7.78%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$45.00 / 3.10%</t>
+          <t>$44.95 / 2.98%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.41 / 3.05%</t>
+          <t>$42.36 / 2.94%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.45 / 9.44%</t>
+          <t>$45.44 / 9.40%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.41 / 4.14%</t>
+          <t>$44.33 / 3.97%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.11 / 11.34%</t>
+          <t>$43.10 / 11.30%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.89 / 11.21%</t>
+          <t>$42.88 / 11.19%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.57 / 1.26%</t>
+          <t>$42.52 / 1.14%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$780.02 / 9.84%</t>
+          <t>$777.02 / 9.42%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$780.02 / 1.87%</t>
+          <t>$777.00 / 1.47%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$780.02 / 14.61%</t>
+          <t>$777.00 / 14.16%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$780.02 / 13.14%</t>
+          <t>$777.02 / 12.70%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$780.02 / 12.77%</t>
+          <t>$777.02 / 12.34%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$780.02 / 4.94%</t>
+          <t>$777.00 / 4.53%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$780.02 / 4.46%</t>
+          <t>$777.00 / 4.05%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$780.02 / 20.27%</t>
+          <t>$777.02 / 19.81%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$780.02 / 5.53%</t>
+          <t>$777.02 / 5.12%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$780.02 / 18.36%</t>
+          <t>$777.00 / 17.90%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$780.02 / 17.40%</t>
+          <t>$777.00 / 16.95%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$780.02 / 2.41%</t>
+          <t>$777.00 / 2.01%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$780.02 / 9.84%</t>
+          <t>$777.00 / 9.41%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$780.02 / 1.87%</t>
+          <t>$777.00 / 1.47%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$780.02 / 14.61%</t>
+          <t>$777.00 / 14.16%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$780.02 / 13.14%</t>
+          <t>$777.00 / 12.70%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$780.02 / 12.77%</t>
+          <t>$777.00 / 12.34%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$780.02 / 4.94%</t>
+          <t>$777.00 / 4.53%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$780.02 / 4.46%</t>
+          <t>$777.00 / 4.05%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$780.02 / 20.27%</t>
+          <t>$777.00 / 19.80%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$780.02 / 5.53%</t>
+          <t>$777.00 / 5.12%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$780.02 / 18.36%</t>
+          <t>$777.00 / 17.90%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$780.02 / 17.40%</t>
+          <t>$777.00 / 16.95%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$780.02 / 2.41%</t>
+          <t>$777.00 / 2.01%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.41% (6.99%)</t>
+          <t>7.53% (7.11%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.22% (14.49%)</t>
+          <t>15.45% (14.72%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.92% (2.77%)</t>
+          <t>3.04% (2.88%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.86% (4.57%)</t>
+          <t>4.99% (4.70%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.12% (3.91%)</t>
+          <t>4.20% (3.99%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.54% (11.91%)</t>
+          <t>12.68% (12.05%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.20% (11.62%)</t>
+          <t>12.41% (11.84%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.43% (4.09%)</t>
+          <t>4.53% (4.19%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.48% (10.98%)</t>
+          <t>11.66% (11.16%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.58% (1.49%)</t>
+          <t>1.68% (1.59%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.24% (0.21%)</t>
+          <t>0.24% (0.22%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.00% (14.21%)</t>
+          <t>15.20% (14.40%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>5.94% (5.52%)</t>
+          <t>6.06% (5.64%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.16% (11.43%)</t>
+          <t>12.33% (11.60%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.14% (1.99%)</t>
+          <t>2.19% (2.04%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.79% (3.50%)</t>
+          <t>3.87% (3.58%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.06% (2.84%)</t>
+          <t>3.17% (2.95%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.22% (9.58%)</t>
+          <t>10.35% (9.71%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.75% (9.17%)</t>
+          <t>9.86% (9.29%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.84% (3.49%)</t>
+          <t>3.87% (3.52%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>8.98% (8.48%)</t>
+          <t>9.17% (8.66%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.05% (0.96%)</t>
+          <t>1.09% (1.00%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.10% (0.08%)</t>
+          <t>0.12% (0.10%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.63% (11.84%)</t>
+          <t>12.76% (11.97%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>5.25%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.02%</t>
+          <t>15.47%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.65%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.95%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>11.75%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.92%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.57%</t>
+          <t>-2.20%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.39%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.47%</t>
+          <t>-1.09%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.97%</t>
+          <t>-1.59%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>13.94%</t>
+          <t>14.38%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>2.68%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-2.20%</t>
+          <t>-1.82%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-5.12%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-3.94%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.48%</t>
+          <t>-4.11%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.84%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.28% (10.86%)</t>
+          <t>11.07% (10.65%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.97% (9.24%)</t>
+          <t>9.82% (9.09%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>11.08% (10.93%)</t>
+          <t>10.88% (10.73%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.57% (11.28%)</t>
+          <t>11.37% (11.08%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.04% (10.82%)</t>
+          <t>10.80% (10.58%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.55% (9.91%)</t>
+          <t>10.34% (9.70%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.15% (9.58%)</t>
+          <t>10.00% (9.43%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.23% (13.89%)</t>
+          <t>14.03% (13.69%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.88% (9.37%)</t>
+          <t>9.70% (9.20%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.97% (10.88%)</t>
+          <t>10.76% (10.67%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.34% (10.32%)</t>
+          <t>10.05% (10.03%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.67% (9.87%)</t>
+          <t>10.50% (9.70%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.88% (16.45%)</t>
+          <t>16.68% (16.26%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.15% (14.42%)</t>
+          <t>14.97% (14.24%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.90% (16.74%)</t>
+          <t>16.65% (16.50%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.44% (17.15%)</t>
+          <t>17.22% (16.93%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.74% (16.52%)</t>
+          <t>16.55% (16.33%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.81% (15.17%)</t>
+          <t>15.61% (14.97%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.42% (14.84%)</t>
+          <t>15.20% (14.63%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.27% (19.92%)</t>
+          <t>20.03% (19.68%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.15% (14.64%)</t>
+          <t>15.00% (14.49%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.33% (17.24%)</t>
+          <t>17.08% (16.99%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.78% (16.76%)</t>
+          <t>16.51% (16.50%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.73% (14.94%)</t>
+          <t>15.52% (14.73%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.78% (-7.20%)</t>
+          <t>-6.68% (-7.09%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.68% (-2.41%)</t>
+          <t>-1.49% (-2.21%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.39% (-10.54%)</t>
+          <t>-10.29% (-10.44%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.89% (-9.18%)</t>
+          <t>-8.77% (-9.06%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.16% (-9.38%)</t>
+          <t>-9.09% (-9.30%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.69% (-4.32%)</t>
+          <t>-3.57% (-4.20%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.69% (-4.26%)</t>
+          <t>-3.50% (-4.07%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.94% (-11.28%)</t>
+          <t>-10.85% (-11.19%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.83% (-5.34%)</t>
+          <t>-4.68% (-5.18%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.99% (-13.08%)</t>
+          <t>-12.91% (-13.00%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.00% (-13.02%)</t>
+          <t>-13.00% (-13.01%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.45% (-2.24%)</t>
+          <t>-1.28% (-2.07%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.74% (-6.16%)</t>
+          <t>-5.63% (-6.05%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.41% (-2.14%)</t>
+          <t>-1.26% (-1.99%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.93% (-9.09%)</t>
+          <t>-8.89% (-9.04%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.42% (-7.72%)</t>
+          <t>-7.35% (-7.65%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.88% (-8.10%)</t>
+          <t>-7.79% (-8.00%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.19% (-3.83%)</t>
+          <t>-3.07% (-3.71%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.78%)</t>
+          <t>-3.11% (-3.68%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.05% (-9.40%)</t>
+          <t>-9.02% (-9.37%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.30% (-4.80%)</t>
+          <t>-4.14% (-4.64%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.85% (-10.94%)</t>
+          <t>-10.82% (-10.91%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.82% (-10.84%)</t>
+          <t>-10.80% (-10.82%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.26% (-2.06%)</t>
+          <t>-1.15% (-1.94%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-18.06%</t>
+          <t>-17.75%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-11.65%</t>
+          <t>-11.31%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.47%</t>
+          <t>-21.17%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.45%</t>
+          <t>-20.14%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-20.20%</t>
+          <t>-19.89%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-14.24%</t>
+          <t>-13.90%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.84%</t>
+          <t>-13.50%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-25.17%</t>
+          <t>-24.88%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.71%</t>
+          <t>-14.38%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.96%</t>
+          <t>-23.66%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.34%</t>
+          <t>-23.04%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-12.11%</t>
+          <t>-11.77%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.61%</t>
+          <t>-22.31%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.56%</t>
+          <t>-16.23%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.83%</t>
+          <t>-25.54%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.87%</t>
+          <t>-24.58%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.63%</t>
+          <t>-24.33%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-19.00%</t>
+          <t>-18.68%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.62%</t>
+          <t>-18.31%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.32%</t>
+          <t>-29.05%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.45%</t>
+          <t>-19.14%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-28.18%</t>
+          <t>-27.90%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.60%</t>
+          <t>-27.32%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-17.00%</t>
+          <t>-16.67%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.43% (2.01%)</t>
+          <t>2.15% (1.73%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.16% (-0.57%)</t>
+          <t>-0.03% (-0.76%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.79% (2.64%)</t>
+          <t>2.51% (2.36%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.15% (2.86%)</t>
+          <t>2.88% (2.59%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.52% (2.30%)</t>
+          <t>2.20% (1.99%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.08% (0.44%)</t>
+          <t>0.81% (0.18%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.61% (0.04%)</t>
+          <t>0.42% (-0.15%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.43% (4.09%)</t>
+          <t>4.53% (4.19%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.44% (-0.06%)</t>
+          <t>0.22% (-0.29%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.58% (1.49%)</t>
+          <t>1.68% (1.59%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.24% (0.21%)</t>
+          <t>0.24% (0.22%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.93% (0.13%)</t>
+          <t>0.71% (-0.09%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.57% (3.15%)</t>
+          <t>3.29% (2.87%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.43% (-0.30%)</t>
+          <t>0.19% (-0.54%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.14% (1.99%)</t>
+          <t>2.19% (2.04%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.79% (3.50%)</t>
+          <t>3.87% (3.58%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.06% (2.84%)</t>
+          <t>3.17% (2.95%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.60% (0.96%)</t>
+          <t>1.33% (0.69%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.11% (0.54%)</t>
+          <t>0.83% (0.25%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.84% (3.49%)</t>
+          <t>3.87% (3.52%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>1.01% (0.50%)</t>
+          <t>0.78% (0.28%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.05% (0.96%)</t>
+          <t>1.09% (1.00%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.10% (0.08%)</t>
+          <t>0.12% (0.10%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>1.09% (0.30%)</t>
+          <t>0.82% (0.02%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/10/2026</t>
+          <t>As of 7/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.82%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>1.95%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.38%</t>
+          <t>-9.30%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.28%</t>
+          <t>11.08%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.03%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.14%</t>
+          <t>12.70%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.65%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.06%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.89%</t>
+          <t>13.69%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.27%</t>
+          <t>19.81%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.57%</t>
+          <t>-2.20%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.28%</t>
+          <t>-11.19%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>10.65%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>7.11%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.84%</t>
+          <t>6.72%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.84%</t>
+          <t>5.25%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.20%</t>
+          <t>-7.09%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.20%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>11.16%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.73%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.12%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.39%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-5.34%</t>
+          <t>-5.18%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.84%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.36%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.92%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>-4.07%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.91%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>11.75%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.20%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>14.72%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.47%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.02%</t>
+          <t>15.47%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.41%</t>
+          <t>-2.21%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>14.40%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.42%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.94%</t>
+          <t>14.38%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.24%</t>
+          <t>-2.07%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.03%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>13.99%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.40%</t>
+          <t>16.95%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.97%</t>
+          <t>-1.59%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.02%</t>
+          <t>-13.01%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.08%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.36%</t>
+          <t>17.90%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.47%</t>
+          <t>-1.09%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.08%</t>
+          <t>-13.00%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.77%</t>
+          <t>2.88%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.84%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.61%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.54%</t>
+          <t>-10.44%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 6/10/2026</t>
+          <t>As of 7/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>16.33%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>2.95%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.90%</t>
+          <t>7.78%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.10%</t>
+          <t>-8.00%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.15%</t>
+          <t>16.93%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.45%</t>
+          <t>7.37%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.14%</t>
+          <t>12.70%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.72%</t>
+          <t>-7.65%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.92%</t>
+          <t>19.68%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.27%</t>
+          <t>19.80%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-5.12%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.40%</t>
+          <t>-9.37%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.45%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.52%</t>
+          <t>5.64%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>5.54%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>2.68%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.16%</t>
+          <t>-6.05%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.64%</t>
+          <t>14.49%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.66%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.14%</t>
+          <t>3.97%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.12%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7.87%</t>
+          <t>8.29%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.80%</t>
+          <t>-4.64%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.84%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>4.05%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.52%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.78%</t>
+          <t>-3.68%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.17%</t>
+          <t>14.97%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.71%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.83%</t>
+          <t>-3.71%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.32%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.47%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>11.67%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.14%</t>
+          <t>-1.99%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.94%</t>
+          <t>14.73%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>11.97%</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.14%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2.01%</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>11.84%</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1.26%</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2.41%</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>11.41%</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.06%</t>
+          <t>-1.94%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.76%</t>
+          <t>16.50%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.40%</t>
+          <t>16.95%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.48%</t>
+          <t>-4.11%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.84%</t>
+          <t>-10.82%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.00%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.34%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.36%</t>
+          <t>17.90%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-3.94%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.94%</t>
+          <t>-10.91%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.74%</t>
+          <t>16.50%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.99%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.01%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.61%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-2.20%</t>
+          <t>-1.82%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.09%</t>
+          <t>-9.04%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-08]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/7/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>191 days</t>
+          <t>190 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>317 days</t>
+          <t>316 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>72 days</t>
+          <t>71 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>135 days</t>
+          <t>134 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>100 days</t>
+          <t>99 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>282 days</t>
+          <t>281 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>253 days</t>
+          <t>252 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>163 days</t>
+          <t>162 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>226 days</t>
+          <t>225 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>44 days</t>
+          <t>43 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>8 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>345 days</t>
+          <t>344 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.31 / 6.72%</t>
+          <t>$48.19 / 6.44%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.34 / 1.40%</t>
+          <t>$58.16 / 1.09%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.47 / 10.71%</t>
+          <t>$56.39 / 10.54%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.15 / 9.03%</t>
+          <t>$63.01 / 8.80%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.14 / 9.32%</t>
+          <t>$57.03 / 9.10%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.94 / 3.50%</t>
+          <t>$61.75 / 3.17%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.89 / 3.36%</t>
+          <t>$61.72 / 3.08%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.94 / 11.64%</t>
+          <t>$53.89 / 11.53%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$58.10 / 4.56%</t>
+          <t>$57.89 / 4.19%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.68 / 13.97%</t>
+          <t>$60.58 / 13.77%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.57 / 13.99%</t>
+          <t>$54.53 / 13.91%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.79 / 1.25%</t>
+          <t>$57.63 / 0.96%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.90 / 5.54%</t>
+          <t>$42.83 / 5.37%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.50 / 1.17%</t>
+          <t>$42.40 / 0.93%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.09 / 9.01%</t>
+          <t>$41.02 / 8.83%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.33 / 7.37%</t>
+          <t>$45.26 / 7.19%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.40 / 7.78%</t>
+          <t>$46.34 / 7.63%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.95 / 2.98%</t>
+          <t>$44.85 / 2.75%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.36 / 2.94%</t>
+          <t>$42.26 / 2.70%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.44 / 9.40%</t>
+          <t>$45.41 / 9.33%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.33 / 3.97%</t>
+          <t>$44.24 / 3.74%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.10 / 11.30%</t>
+          <t>$43.06 / 11.19%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.88 / 11.19%</t>
+          <t>$42.89 / 11.21%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.52 / 1.14%</t>
+          <t>$42.42 / 0.90%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$777.02 / 9.42%</t>
+          <t>$772.96 / 8.85%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$777.00 / 1.47%</t>
+          <t>$772.96 / 0.94%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$777.00 / 14.16%</t>
+          <t>$772.96 / 13.57%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$777.02 / 12.70%</t>
+          <t>$772.96 / 12.12%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$777.02 / 12.34%</t>
+          <t>$772.96 / 11.75%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$777.00 / 4.53%</t>
+          <t>$772.96 / 3.99%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$777.00 / 4.05%</t>
+          <t>$772.96 / 3.51%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$777.02 / 19.81%</t>
+          <t>$772.96 / 19.18%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$777.02 / 5.12%</t>
+          <t>$772.96 / 4.57%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$777.00 / 17.90%</t>
+          <t>$772.96 / 17.29%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$777.00 / 16.95%</t>
+          <t>$772.96 / 16.34%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$777.00 / 2.01%</t>
+          <t>$772.96 / 1.48%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$777.00 / 9.41%</t>
+          <t>$772.96 / 8.85%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$777.00 / 1.47%</t>
+          <t>$772.96 / 0.94%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$777.00 / 14.16%</t>
+          <t>$772.96 / 13.57%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$777.00 / 12.70%</t>
+          <t>$772.96 / 12.12%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$777.00 / 12.34%</t>
+          <t>$772.96 / 11.75%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$777.00 / 4.53%</t>
+          <t>$772.96 / 3.99%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$777.00 / 4.05%</t>
+          <t>$772.96 / 3.51%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$777.00 / 19.80%</t>
+          <t>$772.96 / 19.18%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$777.00 / 5.12%</t>
+          <t>$772.96 / 4.57%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$777.00 / 17.90%</t>
+          <t>$772.96 / 17.29%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$777.00 / 16.95%</t>
+          <t>$772.96 / 16.34%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$777.00 / 2.01%</t>
+          <t>$772.96 / 1.48%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.53% (7.11%)</t>
+          <t>7.81% (7.39%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.45% (14.72%)</t>
+          <t>15.79% (15.06%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.04% (2.88%)</t>
+          <t>3.19% (3.04%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.99% (4.70%)</t>
+          <t>5.22% (4.93%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.20% (3.99%)</t>
+          <t>4.41% (4.20%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.68% (12.05%)</t>
+          <t>13.04% (12.40%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.41% (11.84%)</t>
+          <t>12.72% (12.15%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.53% (4.19%)</t>
+          <t>4.64% (4.30%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.66% (11.16%)</t>
+          <t>12.06% (11.55%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.68% (1.59%)</t>
+          <t>1.85% (1.76%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.24% (0.22%)</t>
+          <t>0.30% (0.29%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.20% (14.40%)</t>
+          <t>15.52% (14.73%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.06% (5.64%)</t>
+          <t>6.23% (5.82%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.33% (11.60%)</t>
+          <t>12.59% (11.86%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.19% (2.04%)</t>
+          <t>2.36% (2.21%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.87% (3.58%)</t>
+          <t>4.04% (3.75%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.17% (2.95%)</t>
+          <t>3.31% (3.10%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.35% (9.71%)</t>
+          <t>10.59% (9.96%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.86% (9.29%)</t>
+          <t>10.12% (9.55%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.87% (3.52%)</t>
+          <t>3.93% (3.59%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.17% (8.66%)</t>
+          <t>9.40% (8.89%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.09% (1.00%)</t>
+          <t>1.18% (1.09%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.12% (0.10%)</t>
+          <t>0.09% (0.08%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.76% (11.97%)</t>
+          <t>13.03% (12.23%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.25%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.47%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.95%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.75%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.92%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.20%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.39%</t>
+          <t>11.97%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.07%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.38%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.82%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>0.05%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-4.26%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.86%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.94%</t>
+          <t>-3.44%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.11%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>12.43%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.07% (10.65%)</t>
+          <t>10.88% (10.46%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.82% (9.09%)</t>
+          <t>9.65% (8.92%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.88% (10.73%)</t>
+          <t>10.60% (10.45%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.37% (11.08%)</t>
+          <t>11.15% (10.86%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.80% (10.58%)</t>
+          <t>10.56% (10.35%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.34% (9.70%)</t>
+          <t>10.19% (9.56%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.00% (9.43%)</t>
+          <t>9.81% (9.24%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.03% (13.69%)</t>
+          <t>13.72% (13.39%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.70% (9.20%)</t>
+          <t>9.59% (9.09%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.76% (10.67%)</t>
+          <t>10.51% (10.42%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.05% (10.03%)</t>
+          <t>9.70% (9.68%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.50% (9.70%)</t>
+          <t>10.31% (9.52%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.68% (16.26%)</t>
+          <t>16.43% (16.01%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.97% (14.24%)</t>
+          <t>14.76% (14.03%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.65% (16.50%)</t>
+          <t>16.42% (16.27%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.22% (16.93%)</t>
+          <t>16.98% (16.69%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.55% (16.33%)</t>
+          <t>16.28% (16.06%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.61% (14.97%)</t>
+          <t>15.40% (14.76%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.20% (14.63%)</t>
+          <t>15.00% (14.43%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.03% (19.68%)</t>
+          <t>19.71% (19.37%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.00% (14.49%)</t>
+          <t>14.78% (14.28%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.08% (16.99%)</t>
+          <t>16.79% (16.70%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.51% (16.50%)</t>
+          <t>16.11% (16.10%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.52% (14.73%)</t>
+          <t>15.32% (14.53%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.68% (-7.09%)</t>
+          <t>-6.44% (-6.85%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.49% (-2.21%)</t>
+          <t>-1.19% (-1.92%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.29% (-10.44%)</t>
+          <t>-10.15% (-10.30%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.77% (-9.06%)</t>
+          <t>-8.58% (-8.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.09% (-9.30%)</t>
+          <t>-8.91% (-9.12%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.57% (-4.20%)</t>
+          <t>-3.26% (-3.90%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.50% (-4.07%)</t>
+          <t>-3.24% (-3.81%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.85% (-11.19%)</t>
+          <t>-10.76% (-11.10%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.68% (-5.18%)</t>
+          <t>-4.34% (-4.85%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.91% (-13.00%)</t>
+          <t>-12.76% (-12.85%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.00% (-13.01%)</t>
+          <t>-12.94% (-12.96%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.28% (-2.07%)</t>
+          <t>-1.00% (-1.79%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.63% (-6.05%)</t>
+          <t>-5.48% (-5.90%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.26% (-1.99%)</t>
+          <t>-1.03% (-1.76%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.89% (-9.04%)</t>
+          <t>-8.74% (-8.89%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.35% (-7.65%)</t>
+          <t>-7.20% (-7.49%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.79% (-8.00%)</t>
+          <t>-7.66% (-7.87%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.07% (-3.71%)</t>
+          <t>-2.86% (-3.49%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.11% (-3.68%)</t>
+          <t>-2.88% (-3.45%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.02% (-9.37%)</t>
+          <t>-8.96% (-9.31%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.14% (-4.64%)</t>
+          <t>-3.93% (-4.44%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.82% (-10.91%)</t>
+          <t>-10.74% (-10.83%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.80% (-10.82%)</t>
+          <t>-10.82% (-10.84%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.15% (-1.94%)</t>
+          <t>-0.92% (-1.71%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.75%</t>
+          <t>-17.31%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>-10.84%</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-20.75%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-19.72%</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-19.47%</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-13.45%</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-13.05%</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-24.48%</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>-13.93%</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-23.26%</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-22.64%</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>-11.31%</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>-21.17%</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>-20.14%</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>-19.89%</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>-13.90%</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>-13.50%</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>-24.88%</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>-14.38%</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>-23.66%</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>-23.04%</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>-11.77%</t>
-        </is>
-      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.31%</t>
+          <t>-21.90%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.23%</t>
+          <t>-15.79%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.54%</t>
+          <t>-25.15%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.58%</t>
+          <t>-24.18%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.33%</t>
+          <t>-23.94%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.68%</t>
+          <t>-18.26%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.31%</t>
+          <t>-17.88%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.05%</t>
+          <t>-28.68%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.14%</t>
+          <t>-18.71%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.90%</t>
+          <t>-27.52%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.32%</t>
+          <t>-26.94%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.67%</t>
+          <t>-16.24%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.15% (1.73%)</t>
+          <t>1.87% (1.46%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.03% (-0.76%)</t>
+          <t>-0.26% (-0.99%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.51% (2.36%)</t>
+          <t>2.12% (1.97%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.88% (2.59%)</t>
+          <t>2.56% (2.27%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.20% (1.99%)</t>
+          <t>1.86% (1.65%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.81% (0.18%)</t>
+          <t>0.60% (-0.03%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.42% (-0.15%)</t>
+          <t>0.17% (-0.40%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.53% (4.19%)</t>
+          <t>4.64% (4.30%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.22% (-0.29%)</t>
+          <t>0.04% (-0.46%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.68% (1.59%)</t>
+          <t>1.85% (1.76%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.24% (0.22%)</t>
+          <t>0.30% (0.29%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.71% (-0.09%)</t>
+          <t>0.47% (-0.33%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.29% (2.87%)</t>
+          <t>2.92% (2.50%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.19% (-0.54%)</t>
+          <t>-0.10% (-0.83%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.19% (2.04%)</t>
+          <t>2.36% (2.21%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.87% (3.58%)</t>
+          <t>4.04% (3.75%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.17% (2.95%)</t>
+          <t>3.26% (3.04%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.33% (0.69%)</t>
+          <t>1.02% (0.39%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.83% (0.25%)</t>
+          <t>0.54% (-0.04%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.87% (3.52%)</t>
+          <t>3.93% (3.59%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.78% (0.28%)</t>
+          <t>0.47% (-0.04%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.09% (1.00%)</t>
+          <t>1.18% (1.09%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.12% (0.10%)</t>
+          <t>0.09% (0.08%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.82% (0.02%)</t>
+          <t>0.53% (-0.27%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/10/2026</t>
+          <t>As of 8/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>11.75%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.95%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.30%</t>
+          <t>-9.12%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.08%</t>
+          <t>10.86%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.03%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.70%</t>
+          <t>12.12%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.06%</t>
+          <t>-8.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.69%</t>
+          <t>13.39%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>11.53%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.81%</t>
+          <t>19.18%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.20%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.19%</t>
+          <t>-11.10%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.65%</t>
+          <t>10.46%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.11%</t>
+          <t>7.39%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.72%</t>
+          <t>6.44%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.25%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.09%</t>
+          <t>-6.85%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.20%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.16%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.12%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.39%</t>
+          <t>11.97%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-5.18%</t>
+          <t>-4.85%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>9.24%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.36%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.92%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.07%</t>
+          <t>-3.81%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>12.40%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.75%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.20%</t>
+          <t>-3.90%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14.72%</t>
+          <t>15.06%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.40%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.47%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>-1.92%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.52%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.40%</t>
+          <t>14.73%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>0.96%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.38%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-1.79%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.03%</t>
+          <t>9.68%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.99%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.95%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.07%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.01%</t>
+          <t>-12.96%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.59%</t>
+          <t>1.76%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.90%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.00%</t>
+          <t>-12.85%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.88%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.54%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>13.57%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.44%</t>
+          <t>-10.30%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 7/10/2026</t>
+          <t>As of 8/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.33%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.95%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.78%</t>
+          <t>7.63%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>11.75%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>0.05%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.00%</t>
+          <t>-7.87%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.93%</t>
+          <t>16.69%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.37%</t>
+          <t>7.19%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.70%</t>
+          <t>12.12%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.65%</t>
+          <t>-7.49%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.68%</t>
+          <t>19.37%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.80%</t>
+          <t>19.18%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-4.26%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.37%</t>
+          <t>-9.31%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.01%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.64%</t>
+          <t>5.82%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.54%</t>
+          <t>5.37%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.05%</t>
+          <t>-5.90%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.49%</t>
+          <t>14.28%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.66%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.97%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.12%</t>
+          <t>4.57%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.29%</t>
+          <t>8.86%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.64%</t>
+          <t>-4.44%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>14.43%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.70%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-3.45%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.97%</t>
+          <t>14.76%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.71%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>3.99%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.71%</t>
+          <t>-3.49%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>14.03%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.86%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-1.76%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.73%</t>
+          <t>14.53%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11.97%</t>
+          <t>12.23%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.14%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>1.48%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.94%</t>
+          <t>-1.71%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>16.10%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.95%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.11%</t>
+          <t>-3.61%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.82%</t>
+          <t>-10.84%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>11.19%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.90%</t>
+          <t>17.29%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.94%</t>
+          <t>-3.44%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.91%</t>
+          <t>-10.83%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.21%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.01%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>13.57%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.82%</t>
+          <t>-1.31%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-8.89%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-09]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/8/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>251 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>190 days</t>
+          <t>189 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>316 days</t>
+          <t>315 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>71 days</t>
+          <t>70 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>134 days</t>
+          <t>133 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>99 days</t>
+          <t>98 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>281 days</t>
+          <t>280 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>252 days</t>
+          <t>251 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>162 days</t>
+          <t>161 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>225 days</t>
+          <t>224 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>43 days</t>
+          <t>42 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>8 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>344 days</t>
+          <t>343 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.19 / 6.44%</t>
+          <t>$48.39 / 6.89%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.16 / 1.09%</t>
+          <t>$58.46 / 1.62%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.39 / 10.54%</t>
+          <t>$56.61 / 10.98%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.01 / 8.80%</t>
+          <t>$63.25 / 9.21%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.03 / 9.10%</t>
+          <t>$57.27 / 9.56%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.75 / 3.17%</t>
+          <t>$62.06 / 3.70%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.72 / 3.08%</t>
+          <t>$62.02 / 3.59%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.89 / 11.53%</t>
+          <t>$54.03 / 11.82%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.89 / 4.19%</t>
+          <t>$58.20 / 4.74%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.58 / 13.77%</t>
+          <t>$60.80 / 14.18%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.53 / 13.91%</t>
+          <t>$54.64 / 14.13%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.63 / 0.96%</t>
+          <t>$57.91 / 1.45%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.83 / 5.37%</t>
+          <t>$42.97 / 5.71%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.40 / 0.93%</t>
+          <t>$42.55 / 1.28%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.02 / 8.83%</t>
+          <t>$41.13 / 9.12%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.26 / 7.19%</t>
+          <t>$45.37 / 7.45%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.34 / 7.63%</t>
+          <t>$46.49 / 7.99%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.85 / 2.75%</t>
+          <t>$45.01 / 3.11%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.26 / 2.70%</t>
+          <t>$42.43 / 3.11%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.41 / 9.33%</t>
+          <t>$45.47 / 9.49%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.24 / 3.74%</t>
+          <t>$44.41 / 4.15%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.06 / 11.19%</t>
+          <t>$43.15 / 11.44%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.89 / 11.21%</t>
+          <t>$42.92 / 11.29%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.42 / 0.90%</t>
+          <t>$42.60 / 1.32%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$772.96 / 8.85%</t>
+          <t>$779.39 / 9.75%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$772.96 / 0.94%</t>
+          <t>$779.39 / 1.79%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$772.96 / 13.57%</t>
+          <t>$779.39 / 14.52%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$772.96 / 12.12%</t>
+          <t>$779.39 / 13.05%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$772.96 / 11.75%</t>
+          <t>$779.39 / 12.68%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$772.96 / 3.99%</t>
+          <t>$779.39 / 4.86%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$772.96 / 3.51%</t>
+          <t>$779.39 / 4.37%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$772.96 / 19.18%</t>
+          <t>$779.39 / 20.17%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$772.96 / 4.57%</t>
+          <t>$779.39 / 5.44%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$772.96 / 17.29%</t>
+          <t>$779.39 / 18.26%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$772.96 / 16.34%</t>
+          <t>$779.39 / 17.31%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$772.96 / 1.48%</t>
+          <t>$779.39 / 2.32%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$772.96 / 8.85%</t>
+          <t>$779.39 / 9.75%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$772.96 / 0.94%</t>
+          <t>$779.39 / 1.79%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$772.96 / 13.57%</t>
+          <t>$779.39 / 14.52%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$772.96 / 12.12%</t>
+          <t>$779.39 / 13.05%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$772.96 / 11.75%</t>
+          <t>$779.39 / 12.68%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$772.96 / 3.99%</t>
+          <t>$779.39 / 4.86%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$772.96 / 3.51%</t>
+          <t>$779.39 / 4.37%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$772.96 / 19.18%</t>
+          <t>$779.39 / 20.17%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$772.96 / 4.57%</t>
+          <t>$779.39 / 5.44%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$772.96 / 17.29%</t>
+          <t>$779.39 / 18.26%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$772.96 / 16.34%</t>
+          <t>$779.39 / 17.31%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$772.96 / 1.48%</t>
+          <t>$779.39 / 2.32%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.81% (7.39%)</t>
+          <t>7.36% (6.95%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.79% (15.06%)</t>
+          <t>15.19% (14.47%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.19% (3.04%)</t>
+          <t>2.78% (2.63%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.22% (4.93%)</t>
+          <t>4.81% (4.53%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.41% (4.20%)</t>
+          <t>3.97% (3.76%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.04% (12.40%)</t>
+          <t>12.46% (11.83%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.72% (12.15%)</t>
+          <t>12.16% (11.60%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.64% (4.30%)</t>
+          <t>4.36% (4.03%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.06% (11.55%)</t>
+          <t>11.46% (10.96%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.85% (1.76%)</t>
+          <t>1.48% (1.39%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.30% (0.29%)</t>
+          <t>0.11% (0.10%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.52% (14.73%)</t>
+          <t>14.96% (14.18%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.23% (5.82%)</t>
+          <t>5.89% (5.47%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.59% (11.86%)</t>
+          <t>12.21% (11.48%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.36% (2.21%)</t>
+          <t>2.09% (1.94%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.04% (3.75%)</t>
+          <t>3.79% (3.50%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.31% (3.10%)</t>
+          <t>2.97% (2.76%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.59% (9.96%)</t>
+          <t>10.20% (9.56%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.12% (9.55%)</t>
+          <t>9.68% (9.11%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.93% (3.59%)</t>
+          <t>3.78% (3.44%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.40% (8.89%)</t>
+          <t>8.96% (8.46%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.18% (1.09%)</t>
+          <t>0.95% (0.87%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.09% (0.08%)</t>
+          <t>0.02% (0.01%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.03% (12.23%)</t>
+          <t>12.56% (11.77%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.80%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-2.50%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.97%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-1.89%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>14.03%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-2.12%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.88%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>-5.05%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.86%</t>
+          <t>7.96%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-4.24%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-4.40%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>11.50%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.88% (10.46%)</t>
+          <t>11.17% (10.76%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.65% (8.92%)</t>
+          <t>9.88% (9.15%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.60% (10.45%)</t>
+          <t>10.90% (10.75%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.15% (10.86%)</t>
+          <t>11.46% (11.18%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.56% (10.35%)</t>
+          <t>10.84% (10.63%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.19% (9.56%)</t>
+          <t>10.41% (9.78%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.81% (9.24%)</t>
+          <t>10.05% (9.49%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.72% (13.39%)</t>
+          <t>14.11% (13.78%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.59% (9.09%)</t>
+          <t>9.79% (9.29%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.51% (10.42%)</t>
+          <t>10.82% (10.74%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.70% (9.68%)</t>
+          <t>10.17% (10.15%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.31% (9.52%)</t>
+          <t>10.57% (9.78%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.43% (16.01%)</t>
+          <t>16.76% (16.35%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.76% (14.03%)</t>
+          <t>15.12% (14.39%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.42% (16.27%)</t>
+          <t>16.79% (16.64%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.98% (16.69%)</t>
+          <t>17.38% (17.09%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.28% (16.06%)</t>
+          <t>16.60% (16.38%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.40% (14.76%)</t>
+          <t>15.73% (15.10%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.00% (14.43%)</t>
+          <t>15.29% (14.72%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.71% (19.37%)</t>
+          <t>20.17% (19.83%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.78% (14.28%)</t>
+          <t>15.07% (14.57%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.79% (16.70%)</t>
+          <t>17.19% (17.10%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.11% (16.10%)</t>
+          <t>16.65% (16.64%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.32% (14.53%)</t>
+          <t>15.60% (14.81%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.44% (-6.85%)</t>
+          <t>-6.82% (-7.24%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.19% (-1.92%)</t>
+          <t>-1.70% (-2.42%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.15% (-10.30%)</t>
+          <t>-10.51% (-10.66%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.58% (-8.87%)</t>
+          <t>-8.93% (-9.21%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.91% (-9.12%)</t>
+          <t>-9.29% (-9.50%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.26% (-3.90%)</t>
+          <t>-3.76% (-4.39%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.24% (-3.81%)</t>
+          <t>-3.72% (-4.28%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.76% (-11.10%)</t>
+          <t>-10.99% (-11.33%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.34% (-4.85%)</t>
+          <t>-4.86% (-5.35%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.76% (-12.85%)</t>
+          <t>-13.08% (-13.16%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.94% (-12.96%)</t>
+          <t>-13.11% (-13.13%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.00% (-1.79%)</t>
+          <t>-1.48% (-2.27%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.48% (-5.90%)</t>
+          <t>-5.79% (-6.20%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.03% (-1.76%)</t>
+          <t>-1.37% (-2.09%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.74% (-8.89%)</t>
+          <t>-8.98% (-9.13%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.20% (-7.49%)</t>
+          <t>-7.43% (-7.72%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.66% (-7.87%)</t>
+          <t>-7.97% (-8.18%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.86% (-3.49%)</t>
+          <t>-3.21% (-3.84%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.88% (-3.45%)</t>
+          <t>-3.27% (-3.84%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.96% (-9.31%)</t>
+          <t>-9.09% (-9.44%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.93% (-4.44%)</t>
+          <t>-4.31% (-4.81%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.74% (-10.83%)</t>
+          <t>-10.94% (-11.02%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.82% (-10.84%)</t>
+          <t>-10.89% (-10.90%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.92% (-1.71%)</t>
+          <t>-1.33% (-2.12%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.31%</t>
+          <t>-18.00%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.84%</t>
+          <t>-11.58%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.75%</t>
+          <t>-21.41%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.72%</t>
+          <t>-20.39%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.47%</t>
+          <t>-20.13%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.45%</t>
+          <t>-14.17%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.05%</t>
+          <t>-13.77%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.48%</t>
+          <t>-25.11%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.93%</t>
+          <t>-14.64%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.26%</t>
+          <t>-23.90%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.64%</t>
+          <t>-23.28%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.31%</t>
+          <t>-12.04%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.90%</t>
+          <t>-22.55%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.79%</t>
+          <t>-16.49%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.15%</t>
+          <t>-25.77%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.18%</t>
+          <t>-24.81%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.94%</t>
+          <t>-24.57%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.26%</t>
+          <t>-18.93%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.88%</t>
+          <t>-18.56%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.68%</t>
+          <t>-29.27%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.71%</t>
+          <t>-19.38%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.52%</t>
+          <t>-28.12%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.94%</t>
+          <t>-27.54%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.24%</t>
+          <t>-16.93%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.87% (1.46%)</t>
+          <t>2.30% (1.89%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.99%)</t>
+          <t>0.06% (-0.67%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.12% (1.97%)</t>
+          <t>2.57% (2.42%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.56% (2.27%)</t>
+          <t>3.02% (2.74%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.86% (1.65%)</t>
+          <t>2.28% (2.08%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.60% (-0.03%)</t>
+          <t>0.93% (0.30%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.17% (-0.40%)</t>
+          <t>0.50% (-0.06%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.64% (4.30%)</t>
+          <t>4.36% (4.03%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.04% (-0.46%)</t>
+          <t>0.34% (-0.16%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.85% (1.76%)</t>
+          <t>1.48% (1.39%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.30% (0.29%)</t>
+          <t>0.11% (0.10%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.47% (-0.33%)</t>
+          <t>0.81% (0.02%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.92% (2.50%)</t>
+          <t>3.44% (3.02%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.10% (-0.83%)</t>
+          <t>0.39% (-0.33%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.36% (2.21%)</t>
+          <t>2.09% (1.94%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>4.04% (3.75%)</t>
+          <t>3.79% (3.50%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.26% (3.04%)</t>
+          <t>2.97% (2.76%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.02% (0.39%)</t>
+          <t>1.50% (0.87%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.54% (-0.04%)</t>
+          <t>0.97% (0.40%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.93% (3.59%)</t>
+          <t>3.78% (3.44%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.47% (-0.04%)</t>
+          <t>0.91% (0.41%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.18% (1.09%)</t>
+          <t>0.95% (0.87%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.09% (0.08%)</t>
+          <t>0.02% (0.01%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.53% (-0.27%)</t>
+          <t>0.95% (0.16%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 8/10/2026</t>
+          <t>As of 9/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.63%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>3.76%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.75%</t>
+          <t>12.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.12%</t>
+          <t>-9.50%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.86%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.12%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.87%</t>
+          <t>-9.21%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.39%</t>
+          <t>13.78%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.30%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.53%</t>
+          <t>11.82%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.18%</t>
+          <t>20.17%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-2.50%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.10%</t>
+          <t>-11.33%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.46%</t>
+          <t>10.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.39%</t>
+          <t>6.95%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.44%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.80%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.85%</t>
+          <t>-7.24%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.74%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.97%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.85%</t>
+          <t>-5.35%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.24%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.15%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.51%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-4.28%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.40%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.90%</t>
+          <t>-4.39%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.06%</t>
+          <t>14.47%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>1.79%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>15.11%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.92%</t>
+          <t>-2.42%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.52%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.73%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.96%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>14.03%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-2.27%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.68%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-1.89%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-12.96%</t>
+          <t>-13.13%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.74%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.76%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>18.26%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.85%</t>
+          <t>-13.16%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.45%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.54%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>14.52%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.30%</t>
+          <t>-10.66%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 8/10/2026</t>
+          <t>As of 9/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>16.38%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>2.76%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.63%</t>
+          <t>7.99%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.75%</t>
+          <t>12.68%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.87%</t>
+          <t>-8.18%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.69%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.19%</t>
+          <t>7.45%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.12%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.88%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.49%</t>
+          <t>-7.72%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.37%</t>
+          <t>19.83%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.44%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.18%</t>
+          <t>20.17%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>-5.05%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.31%</t>
+          <t>-9.44%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.01%</t>
+          <t>16.35%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.82%</t>
+          <t>5.47%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.37%</t>
+          <t>5.71%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.90%</t>
+          <t>-6.20%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.28%</t>
+          <t>14.57%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.46%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.57%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.86%</t>
+          <t>7.96%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-4.81%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.43%</t>
+          <t>14.72%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.70%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.51%</t>
+          <t>4.37%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.45%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.76%</t>
+          <t>15.10%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.49%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.03%</t>
+          <t>14.39%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.86%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>1.79%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.76%</t>
+          <t>-2.09%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.53%</t>
+          <t>14.81%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.32%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.48%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>11.50%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.71%</t>
+          <t>-2.12%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.10%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>17.31%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-4.40%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.84%</t>
+          <t>-10.90%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.70%</t>
+          <t>17.10%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>0.87%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.19%</t>
+          <t>11.44%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.29%</t>
+          <t>18.26%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.44%</t>
+          <t>-4.24%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.83%</t>
+          <t>-11.02%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>16.64%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>1.94%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.57%</t>
+          <t>14.52%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-2.12%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.89%</t>
+          <t>-9.13%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-12]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/9/2026 at 2:51 PM ET)</t>
+          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>312 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>251 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>189 days</t>
+          <t>186 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>315 days</t>
+          <t>312 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>70 days</t>
+          <t>67 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>133 days</t>
+          <t>130 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>98 days</t>
+          <t>95 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>280 days</t>
+          <t>277 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>251 days</t>
+          <t>248 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>161 days</t>
+          <t>158 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>224 days</t>
+          <t>221 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>42 days</t>
+          <t>39 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>7 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>343 days</t>
+          <t>340 days</t>
         </is>
       </c>
     </row>
@@ -2326,62 +2326,62 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.39 / 6.89%</t>
+          <t>$48.37 / 6.84%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.46 / 1.62%</t>
+          <t>$58.43 / 1.55%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.61 / 10.98%</t>
+          <t>$56.62 / 10.99%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.25 / 9.21%</t>
+          <t>$63.24 / 9.19%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.27 / 9.56%</t>
+          <t>$57.26 / 9.54%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$62.06 / 3.70%</t>
+          <t>$62.00 / 3.60%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$62.02 / 3.59%</t>
+          <t>$61.99 / 3.53%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$54.03 / 11.82%</t>
+          <t>$54.03 / 11.83%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$58.20 / 4.74%</t>
+          <t>$58.17 / 4.68%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.80 / 14.18%</t>
+          <t>$60.82 / 14.22%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.64 / 14.13%</t>
+          <t>$54.66 / 14.19%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.91 / 1.45%</t>
+          <t>$57.86 / 1.36%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2391,57 +2391,57 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.55 / 1.28%</t>
+          <t>$42.54 / 1.25%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.13 / 9.12%</t>
+          <t>$41.14 / 9.15%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.37 / 7.45%</t>
+          <t>$45.39 / 7.50%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.49 / 7.99%</t>
+          <t>$46.49 / 7.98%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$45.01 / 3.11%</t>
+          <t>$45.00 / 3.09%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.43 / 3.11%</t>
+          <t>$42.42 / 3.09%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.47 / 9.49%</t>
+          <t>$45.50 / 9.55%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.41 / 4.15%</t>
+          <t>$44.41 / 4.14%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.15 / 11.44%</t>
+          <t>$43.17 / 11.48%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.92 / 11.29%</t>
+          <t>$42.94 / 11.33%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.60 / 1.32%</t>
+          <t>$42.59 / 1.29%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$779.39 / 9.75%</t>
+          <t>$778.05 / 9.56%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$779.39 / 1.79%</t>
+          <t>$778.05 / 1.61%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$779.39 / 14.52%</t>
+          <t>$778.05 / 14.32%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$779.39 / 13.05%</t>
+          <t>$778.05 / 12.85%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$779.39 / 12.68%</t>
+          <t>$778.05 / 12.49%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$779.39 / 4.86%</t>
+          <t>$778.05 / 4.68%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$779.39 / 4.37%</t>
+          <t>$778.05 / 4.19%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$779.39 / 20.17%</t>
+          <t>$778.05 / 19.96%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$779.39 / 5.44%</t>
+          <t>$778.05 / 5.26%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$779.39 / 18.26%</t>
+          <t>$778.05 / 18.06%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$779.39 / 17.31%</t>
+          <t>$778.05 / 17.11%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$779.39 / 2.32%</t>
+          <t>$778.05 / 2.15%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$779.39 / 9.75%</t>
+          <t>$778.05 / 9.56%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$779.39 / 1.79%</t>
+          <t>$778.05 / 1.61%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$779.39 / 14.52%</t>
+          <t>$778.05 / 14.32%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$779.39 / 13.05%</t>
+          <t>$778.05 / 12.85%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$779.39 / 12.68%</t>
+          <t>$778.05 / 12.49%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$779.39 / 4.86%</t>
+          <t>$778.05 / 4.68%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$779.39 / 4.37%</t>
+          <t>$778.05 / 4.19%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$779.39 / 20.17%</t>
+          <t>$778.05 / 19.96%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$779.39 / 5.44%</t>
+          <t>$778.05 / 5.26%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$779.39 / 18.26%</t>
+          <t>$778.05 / 18.06%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$779.39 / 17.31%</t>
+          <t>$778.05 / 17.11%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$779.39 / 2.32%</t>
+          <t>$778.05 / 2.15%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.36% (6.95%)</t>
+          <t>7.40% (6.99%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.19% (14.47%)</t>
+          <t>15.26% (14.54%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.78% (2.63%)</t>
+          <t>2.76% (2.62%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.81% (4.53%)</t>
+          <t>4.83% (4.56%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.97% (3.76%)</t>
+          <t>3.98% (3.78%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.46% (11.83%)</t>
+          <t>12.56% (11.94%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.16% (11.60%)</t>
+          <t>12.22% (11.66%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.36% (4.03%)</t>
+          <t>4.35% (4.02%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.46% (10.96%)</t>
+          <t>11.52% (11.03%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.48% (1.39%)</t>
+          <t>1.44% (1.36%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.11% (0.10%)</t>
+          <t>0.06% (0.05%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>14.96% (14.18%)</t>
+          <t>15.06% (14.27%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>5.89% (5.47%)</t>
+          <t>5.88% (5.47%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.21% (11.48%)</t>
+          <t>12.23% (11.51%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.09% (1.94%)</t>
+          <t>2.06% (1.91%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.79% (3.50%)</t>
+          <t>3.73% (3.45%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2.97% (2.76%)</t>
+          <t>2.97% (2.77%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.20% (9.56%)</t>
+          <t>10.21% (9.59%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.68% (9.11%)</t>
+          <t>9.69% (9.13%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.78% (3.44%)</t>
+          <t>3.72% (3.38%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>8.96% (8.46%)</t>
+          <t>8.97% (8.48%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.95% (0.87%)</t>
+          <t>0.91% (0.83%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.02% (0.01%)</t>
+          <t>-0.02% (-0.03%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.56% (11.77%)</t>
+          <t>12.58% (11.80%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>5.11%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.38%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.73%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.81%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.50%</t>
+          <t>-2.33%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>11.24%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-1.22%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.89%</t>
+          <t>-1.72%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.03%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-1.96%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.88%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.60%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-5.05%</t>
+          <t>-4.89%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>7.96%</t>
+          <t>8.14%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
+          <t>-4.07%</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
           <t>-4.24%</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>-4.40%</t>
-        </is>
-      </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>11.69%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.17% (10.76%)</t>
+          <t>11.06% (10.66%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.88% (9.15%)</t>
+          <t>9.78% (9.06%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.90% (10.75%)</t>
+          <t>10.75% (10.61%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.46% (11.18%)</t>
+          <t>11.34% (11.06%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.84% (10.63%)</t>
+          <t>10.71% (10.51%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.41% (9.78%)</t>
+          <t>10.35% (9.73%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>10.05% (9.49%)</t>
+          <t>9.95% (9.39%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>14.11% (13.78%)</t>
+          <t>13.97% (13.64%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.79% (9.29%)</t>
+          <t>9.69% (9.20%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.82% (10.74%)</t>
+          <t>10.66% (10.58%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.17% (10.15%)</t>
+          <t>9.99% (9.98%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.57% (9.78%)</t>
+          <t>10.49% (9.71%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.76% (16.35%)</t>
+          <t>16.62% (16.21%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>15.12% (14.39%)</t>
+          <t>14.99% (14.27%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.79% (16.64%)</t>
+          <t>16.63% (16.49%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.38% (17.09%)</t>
+          <t>17.20% (16.92%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.60% (16.38%)</t>
+          <t>16.47% (16.26%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.73% (15.10%)</t>
+          <t>15.60% (14.98%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.29% (14.72%)</t>
+          <t>15.16% (14.60%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.17% (19.83%)</t>
+          <t>19.99% (19.66%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.07% (14.57%)</t>
+          <t>14.94% (14.44%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.19% (17.10%)</t>
+          <t>17.03% (16.95%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.65% (16.64%)</t>
+          <t>16.49% (16.48%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.60% (14.81%)</t>
+          <t>15.48% (14.69%)</t>
         </is>
       </c>
     </row>
@@ -2961,62 +2961,62 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.82% (-7.24%)</t>
+          <t>-6.79% (-7.20%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.70% (-2.42%)</t>
+          <t>-1.65% (-2.37%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.51% (-10.66%)</t>
+          <t>-10.53% (-10.67%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.93% (-9.21%)</t>
+          <t>-8.91% (-9.19%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.29% (-9.50%)</t>
+          <t>-9.28% (-9.49%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.76% (-4.39%)</t>
+          <t>-3.67% (-4.29%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.72% (-4.28%)</t>
+          <t>-3.67% (-4.23%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.99% (-11.33%)</t>
+          <t>-11.01% (-11.34%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.86% (-5.35%)</t>
+          <t>-4.81% (-5.30%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.08% (-13.16%)</t>
+          <t>-13.11% (-13.19%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.11% (-13.13%)</t>
+          <t>-13.16% (-13.17%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.48% (-2.27%)</t>
+          <t>-1.40% (-2.18%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -3026,57 +3026,57 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.37% (-2.09%)</t>
+          <t>-1.35% (-2.07%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.98% (-9.13%)</t>
+          <t>-9.01% (-9.15%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.43% (-7.72%)</t>
+          <t>-7.48% (-7.76%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.97% (-8.18%)</t>
+          <t>-7.97% (-8.17%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.84%)</t>
+          <t>-3.19% (-3.82%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.27% (-3.84%)</t>
+          <t>-3.26% (-3.82%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.09% (-9.44%)</t>
+          <t>-9.15% (-9.49%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.31% (-4.81%)</t>
+          <t>-4.31% (-4.80%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.94% (-11.02%)</t>
+          <t>-10.97% (-11.05%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.89% (-10.90%)</t>
+          <t>-10.93% (-10.93%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.33% (-2.12%)</t>
+          <t>-1.31% (-2.09%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-18.00%</t>
+          <t>-17.85%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-11.58%</t>
+          <t>-11.43%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.41%</t>
+          <t>-21.27%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.39%</t>
+          <t>-20.25%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-20.13%</t>
+          <t>-19.99%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-14.17%</t>
+          <t>-14.02%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.77%</t>
+          <t>-13.62%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-25.11%</t>
+          <t>-24.98%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.64%</t>
+          <t>-14.50%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.90%</t>
+          <t>-23.77%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.28%</t>
+          <t>-23.15%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-12.04%</t>
+          <t>-11.89%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.55%</t>
+          <t>-22.42%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.49%</t>
+          <t>-16.34%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.77%</t>
+          <t>-25.64%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.81%</t>
+          <t>-24.68%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.57%</t>
+          <t>-24.44%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.93%</t>
+          <t>-18.79%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.56%</t>
+          <t>-18.42%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.27%</t>
+          <t>-29.14%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.38%</t>
+          <t>-19.25%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-28.12%</t>
+          <t>-28.00%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.54%</t>
+          <t>-27.41%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.93%</t>
+          <t>-16.79%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.30% (1.89%)</t>
+          <t>2.16% (1.75%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.06% (-0.67%)</t>
+          <t>-0.06% (-0.78%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.57% (2.42%)</t>
+          <t>2.37% (2.23%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.02% (2.74%)</t>
+          <t>2.86% (2.58%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.28% (2.08%)</t>
+          <t>2.12% (1.92%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.93% (0.30%)</t>
+          <t>0.84% (0.22%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.50% (-0.06%)</t>
+          <t>0.38% (-0.18%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.36% (4.03%)</t>
+          <t>4.35% (4.02%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.34% (-0.16%)</t>
+          <t>0.22% (-0.27%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.48% (1.39%)</t>
+          <t>1.44% (1.36%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.11% (0.10%)</t>
+          <t>0.06% (0.05%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.81% (0.02%)</t>
+          <t>0.72% (-0.06%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.44% (3.02%)</t>
+          <t>3.25% (2.84%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.39% (-0.33%)</t>
+          <t>0.23% (-0.48%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.09% (1.94%)</t>
+          <t>2.06% (1.91%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.79% (3.50%)</t>
+          <t>3.73% (3.45%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.97% (2.76%)</t>
+          <t>2.97% (2.77%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.50% (0.87%)</t>
+          <t>1.34% (0.72%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.97% (0.40%)</t>
+          <t>0.81% (0.25%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.78% (3.44%)</t>
+          <t>3.72% (3.38%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.91% (0.41%)</t>
+          <t>0.74% (0.24%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.95% (0.87%)</t>
+          <t>0.91% (0.83%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.02% (0.01%)</t>
+          <t>-0.02% (-0.03%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.95% (0.16%)</t>
+          <t>0.79% (0.01%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 9/10/2026</t>
+          <t>As of 12/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.63%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.68%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.81%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.50%</t>
+          <t>-9.49%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.06%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>12.85%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.73%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.21%</t>
+          <t>-9.19%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.78%</t>
+          <t>13.64%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.17%</t>
+          <t>19.96%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.50%</t>
+          <t>-2.33%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.33%</t>
+          <t>-11.34%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.76%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.95%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>6.84%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>5.11%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.24%</t>
+          <t>-7.20%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.20%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.03%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.74%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>11.24%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-5.35%</t>
+          <t>-5.30%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.28%</t>
+          <t>-4.23%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.94%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>3.60%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.39%</t>
+          <t>-4.29%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>9.06%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14.47%</t>
+          <t>14.54%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.11%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.42%</t>
+          <t>-2.37%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>9.71%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.15%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.03%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.27%</t>
+          <t>-2.18%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>0.05%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>17.11%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.89%</t>
+          <t>-1.72%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.13%</t>
+          <t>-13.17%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.74%</t>
+          <t>10.58%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.26%</t>
+          <t>18.06%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-1.22%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.16%</t>
+          <t>-13.19%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.61%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.98%</t>
+          <t>10.99%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.52%</t>
+          <t>14.32%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.38%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.66%</t>
+          <t>-10.67%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 9/10/2026</t>
+          <t>As of 12/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.38%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.76%</t>
+          <t>2.77%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.99%</t>
+          <t>7.98%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.68%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.60%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.18%</t>
+          <t>-8.17%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>16.92%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.45%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>12.85%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.88%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.72%</t>
+          <t>-7.76%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.83%</t>
+          <t>19.66%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.44%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.49%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.17%</t>
+          <t>19.96%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-5.05%</t>
+          <t>-4.89%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.44%</t>
+          <t>-9.49%</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.35%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4051,12 +4051,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.57%</t>
+          <t>14.44%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.46%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>4.14%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.26%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7.96%</t>
+          <t>8.14%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.81%</t>
+          <t>-4.80%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.72%</t>
+          <t>14.60%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.37%</t>
+          <t>4.19%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-3.82%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.10%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-3.82%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.39%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.51%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>1.61%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-2.07%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.81%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>11.80%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.32%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.15%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>11.69%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-2.09%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>16.48%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>17.11%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.40%</t>
+          <t>-4.24%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.90%</t>
+          <t>-10.93%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17.10%</t>
+          <t>16.95%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>0.83%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.44%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.26%</t>
+          <t>18.06%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-4.07%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.02%</t>
+          <t>-11.05%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.64%</t>
+          <t>16.49%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.94%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.52%</t>
+          <t>14.32%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-1.96%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.13%</t>
+          <t>-9.15%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-13]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/12/2026 at 4:00 PM ET)</t>
+          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>312 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>186 days</t>
+          <t>185 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>312 days</t>
+          <t>311 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>67 days</t>
+          <t>66 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>130 days</t>
+          <t>129 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>95 days</t>
+          <t>94 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>277 days</t>
+          <t>276 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>248 days</t>
+          <t>247 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>158 days</t>
+          <t>157 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>221 days</t>
+          <t>220 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>39 days</t>
+          <t>38 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>340 days</t>
+          <t>339 days</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.37 / 6.84%</t>
+          <t>$48.39 / 6.89%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2336,27 +2336,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.62 / 10.99%</t>
+          <t>$56.60 / 10.95%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.24 / 9.19%</t>
+          <t>$63.25 / 9.21%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.26 / 9.54%</t>
+          <t>$57.23 / 9.50%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$62.00 / 3.60%</t>
+          <t>$62.03 / 3.65%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.99 / 3.53%</t>
+          <t>$62.00 / 3.55%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2366,22 +2366,22 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$58.17 / 4.68%</t>
+          <t>$58.18 / 4.71%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.82 / 14.22%</t>
+          <t>$60.81 / 14.21%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.66 / 14.19%</t>
+          <t>$54.69 / 14.24%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.86 / 1.36%</t>
+          <t>$57.88 / 1.40%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2391,42 +2391,42 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.54 / 1.25%</t>
+          <t>$42.55 / 1.29%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.14 / 9.15%</t>
+          <t>$41.15 / 9.17%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.39 / 7.50%</t>
+          <t>$45.38 / 7.48%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.49 / 7.98%</t>
+          <t>$46.51 / 8.03%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$45.00 / 3.09%</t>
+          <t>$45.01 / 3.11%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.42 / 3.09%</t>
+          <t>$42.42 / 3.08%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.50 / 9.55%</t>
+          <t>$45.48 / 9.51%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.41 / 4.14%</t>
+          <t>$44.39 / 4.09%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.59 / 1.29%</t>
+          <t>$42.57 / 1.24%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$778.05 / 9.56%</t>
+          <t>$778.23 / 9.59%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$778.05 / 1.61%</t>
+          <t>$778.23 / 1.63%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$778.05 / 14.32%</t>
+          <t>$778.23 / 14.35%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$778.05 / 12.85%</t>
+          <t>$778.23 / 12.88%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$778.05 / 12.49%</t>
+          <t>$778.23 / 12.52%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$778.05 / 4.68%</t>
+          <t>$778.23 / 4.70%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$778.05 / 4.19%</t>
+          <t>$778.23 / 4.22%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$778.05 / 19.96%</t>
+          <t>$778.23 / 19.99%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$778.05 / 5.26%</t>
+          <t>$778.23 / 5.28%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$778.05 / 18.06%</t>
+          <t>$778.23 / 18.09%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$778.05 / 17.11%</t>
+          <t>$778.23 / 17.13%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$778.05 / 2.15%</t>
+          <t>$778.23 / 2.17%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$778.05 / 9.56%</t>
+          <t>$778.23 / 9.59%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$778.05 / 1.61%</t>
+          <t>$778.23 / 1.63%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$778.05 / 14.32%</t>
+          <t>$778.23 / 14.35%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$778.05 / 12.85%</t>
+          <t>$778.23 / 12.88%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$778.05 / 12.49%</t>
+          <t>$778.23 / 12.52%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$778.05 / 4.68%</t>
+          <t>$778.23 / 4.70%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$778.05 / 4.19%</t>
+          <t>$778.23 / 4.22%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$778.05 / 19.96%</t>
+          <t>$778.23 / 19.99%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$778.05 / 5.26%</t>
+          <t>$778.23 / 5.28%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$778.05 / 18.06%</t>
+          <t>$778.23 / 18.09%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$778.05 / 17.11%</t>
+          <t>$778.23 / 17.13%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$778.05 / 2.15%</t>
+          <t>$778.23 / 2.17%</t>
         </is>
       </c>
     </row>
@@ -2580,37 +2580,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.40% (6.99%)</t>
+          <t>7.35% (6.95%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.26% (14.54%)</t>
+          <t>15.25% (14.54%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.76% (2.62%)</t>
+          <t>2.80% (2.66%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.83% (4.56%)</t>
+          <t>4.81% (4.53%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.98% (3.78%)</t>
+          <t>4.02% (3.82%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.56% (11.94%)</t>
+          <t>12.51% (11.89%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.22% (11.66%)</t>
+          <t>12.20% (11.64%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2620,22 +2620,22 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.52% (11.03%)</t>
+          <t>11.49% (11.00%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.44% (1.36%)</t>
+          <t>1.45% (1.37%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.06% (0.05%)</t>
+          <t>0.01% (0.00%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.06% (14.27%)</t>
+          <t>15.01% (14.23%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2645,42 +2645,42 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.23% (11.51%)</t>
+          <t>12.19% (11.47%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.06% (1.91%)</t>
+          <t>2.03% (1.89%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.73% (3.45%)</t>
+          <t>3.74% (3.46%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2.97% (2.77%)</t>
+          <t>2.93% (2.72%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.21% (9.59%)</t>
+          <t>10.19% (9.56%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.69% (9.13%)</t>
+          <t>9.70% (9.15%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.72% (3.38%)</t>
+          <t>3.75% (3.42%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>8.97% (8.48%)</t>
+          <t>9.02% (8.53%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.58% (11.80%)</t>
+          <t>12.63% (11.85%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.11%</t>
+          <t>5.08%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.29%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.38%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.81%</t>
+          <t>1.79%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.33%</t>
+          <t>-2.35%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.24%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.22%</t>
+          <t>-1.24%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.72%</t>
+          <t>-1.74%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>14.20%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.92%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.96%</t>
+          <t>-1.98%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.60%</t>
+          <t>-0.62%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.74%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.89%</t>
+          <t>-4.91%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.14%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-4.07%</t>
+          <t>-4.09%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-4.26%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>11.66%</t>
         </is>
       </c>
     </row>
@@ -2834,72 +2834,72 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.06% (10.66%)</t>
+          <t>11.04% (10.64%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.78% (9.06%)</t>
+          <t>9.79% (9.08%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.75% (10.61%)</t>
+          <t>10.79% (10.66%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.34% (11.06%)</t>
+          <t>11.33% (11.06%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.71% (10.51%)</t>
+          <t>10.77% (10.57%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.35% (9.73%)</t>
+          <t>10.32% (9.70%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.95% (9.39%)</t>
+          <t>9.95% (9.40%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.97% (13.64%)</t>
+          <t>13.99% (13.66%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.69% (9.20%)</t>
+          <t>9.68% (9.20%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.66% (10.58%)</t>
+          <t>10.68% (10.60%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.99% (9.98%)</t>
+          <t>9.97% (9.96%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.49% (9.71%)</t>
+          <t>10.48% (9.70%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.62% (16.21%)</t>
+          <t>16.64% (16.23%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.99% (14.27%)</t>
+          <t>14.97% (14.26%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.20% (16.92%)</t>
+          <t>17.23% (16.95%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.47% (16.26%)</t>
+          <t>16.44% (16.24%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2924,32 +2924,32 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.16% (14.60%)</t>
+          <t>15.19% (14.63%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.99% (19.66%)</t>
+          <t>20.04% (19.70%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.94% (14.44%)</t>
+          <t>15.00% (14.50%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.03% (16.95%)</t>
+          <t>17.04% (16.96%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.49% (16.48%)</t>
+          <t>16.50% (16.50%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.48% (14.69%)</t>
+          <t>15.54% (14.76%)</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.79% (-7.20%)</t>
+          <t>-6.83% (-7.24%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2971,27 +2971,27 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.53% (-10.67%)</t>
+          <t>-10.50% (-10.64%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.91% (-9.19%)</t>
+          <t>-8.94% (-9.21%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.28% (-9.49%)</t>
+          <t>-9.25% (-9.45%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.67% (-4.29%)</t>
+          <t>-3.72% (-4.34%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.67% (-4.23%)</t>
+          <t>-3.69% (-4.24%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3001,67 +3001,67 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.81% (-5.30%)</t>
+          <t>-4.83% (-5.32%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.11% (-13.19%)</t>
+          <t>-13.11% (-13.18%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.16% (-13.17%)</t>
+          <t>-13.20% (-13.21%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.40% (-2.18%)</t>
+          <t>-1.44% (-2.22%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.79% (-6.20%)</t>
+          <t>-5.80% (-6.20%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.35% (-2.07%)</t>
+          <t>-1.39% (-2.11%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-9.01% (-9.15%)</t>
+          <t>-9.04% (-9.18%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.48% (-7.76%)</t>
+          <t>-7.47% (-7.75%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.97% (-8.17%)</t>
+          <t>-8.01% (-8.21%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.19% (-3.82%)</t>
+          <t>-3.21% (-3.84%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.26% (-3.82%)</t>
+          <t>-3.25% (-3.80%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.15% (-9.49%)</t>
+          <t>-9.12% (-9.46%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.31% (-4.80%)</t>
+          <t>-4.27% (-4.76%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.31% (-2.09%)</t>
+          <t>-1.27% (-2.05%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.85%</t>
+          <t>-17.87%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-11.43%</t>
+          <t>-11.45%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.27%</t>
+          <t>-21.29%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.25%</t>
+          <t>-20.27%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.99%</t>
+          <t>-20.01%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-14.02%</t>
+          <t>-14.04%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.62%</t>
+          <t>-13.64%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.98%</t>
+          <t>-25.00%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.50%</t>
+          <t>-14.52%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.77%</t>
+          <t>-23.78%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.15%</t>
+          <t>-23.17%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.89%</t>
+          <t>-11.91%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.42%</t>
+          <t>-22.43%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.34%</t>
+          <t>-16.36%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.64%</t>
+          <t>-25.66%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.68%</t>
+          <t>-24.70%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.44%</t>
+          <t>-24.45%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.79%</t>
+          <t>-18.81%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.42%</t>
+          <t>-18.44%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.14%</t>
+          <t>-29.16%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.25%</t>
+          <t>-19.26%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-28.00%</t>
+          <t>-28.02%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.41%</t>
+          <t>-27.43%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.79%</t>
+          <t>-16.81%</t>
         </is>
       </c>
     </row>
@@ -3215,17 +3215,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.16% (1.75%)</t>
+          <t>2.14% (1.73%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.78%)</t>
+          <t>-0.04% (-0.76%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.37% (2.23%)</t>
+          <t>2.43% (2.29%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -3235,17 +3235,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.12% (1.92%)</t>
+          <t>2.18% (1.98%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.84% (0.22%)</t>
+          <t>0.81% (0.19%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.38% (-0.18%)</t>
+          <t>0.38% (-0.17%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -3255,47 +3255,47 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.22% (-0.27%)</t>
+          <t>0.21% (-0.28%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.44% (1.36%)</t>
+          <t>1.45% (1.37%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.06% (0.05%)</t>
+          <t>0.01% (0.00%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.72% (-0.06%)</t>
+          <t>0.70% (-0.07%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.25% (2.84%)</t>
+          <t>3.27% (2.86%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.23% (-0.48%)</t>
+          <t>0.22% (-0.49%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.06% (1.91%)</t>
+          <t>2.03% (1.89%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.73% (3.45%)</t>
+          <t>3.74% (3.46%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.97% (2.77%)</t>
+          <t>2.93% (2.72%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -3305,17 +3305,17 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.81% (0.25%)</t>
+          <t>0.84% (0.28%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.72% (3.38%)</t>
+          <t>3.75% (3.42%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.74% (0.24%)</t>
+          <t>0.80% (0.31%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.79% (0.01%)</t>
+          <t>0.86% (0.08%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 12/10/2026</t>
+          <t>As of 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.81%</t>
+          <t>1.79%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.49%</t>
+          <t>-9.45%</t>
         </is>
       </c>
     </row>
@@ -3452,27 +3452,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.53%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.85%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.19%</t>
+          <t>-9.21%</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.64%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3499,12 +3499,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.96%</t>
+          <t>19.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.33%</t>
+          <t>-2.35%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.64%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>6.95%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.84%</t>
+          <t>6.89%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.11%</t>
+          <t>5.08%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.20%</t>
+          <t>-7.24%</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3563,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.03%</t>
+          <t>11.00%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.24%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-5.30%</t>
+          <t>-5.32%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>11.64%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.53%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.23%</t>
+          <t>-4.24%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.94%</t>
+          <t>11.89%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.60%</t>
+          <t>3.65%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.29%</t>
+          <t>-4.34%</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.06%</t>
+          <t>9.08%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.29%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.71%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.36%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>14.20%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.18%</t>
+          <t>-2.22%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.11%</t>
+          <t>17.13%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.72%</t>
+          <t>-1.74%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.17%</t>
+          <t>-13.21%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.58%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.36%</t>
+          <t>1.37%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.06%</t>
+          <t>18.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.22%</t>
+          <t>-1.24%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.19%</t>
+          <t>-13.18%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.61%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.66%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.99%</t>
+          <t>10.95%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.32%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.38%</t>
+          <t>0.35%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.67%</t>
+          <t>-10.64%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 12/10/2026</t>
+          <t>As of 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.24%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.77%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.98%</t>
+          <t>8.03%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.60%</t>
+          <t>-0.62%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.17%</t>
+          <t>-8.21%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.92%</t>
+          <t>16.95%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>3.46%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>7.48%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.85%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.73%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.76%</t>
+          <t>-7.75%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.66%</t>
+          <t>19.70%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.42%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.96%</t>
+          <t>19.99%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.89%</t>
+          <t>-4.91%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.49%</t>
+          <t>-9.46%</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>16.23%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4051,12 +4051,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>9.59%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>2.51%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.44%</t>
+          <t>14.50%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.53%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.14%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.26%</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.14%</t>
+          <t>8.12%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.80%</t>
+          <t>-4.76%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.60%</t>
+          <t>14.63%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.09%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.19%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.82%</t>
+          <t>-3.80%</t>
         </is>
       </c>
     </row>
@@ -4152,27 +4152,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>9.56%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.09%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.74%</t>
+          <t>8.71%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.82%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.26%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.51%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.61%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.92%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.11%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.69%</t>
+          <t>14.76%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11.80%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11.69%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-2.05%</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.48%</t>
+          <t>16.50%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.11%</t>
+          <t>17.13%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-4.26%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.95%</t>
+          <t>16.96%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4310,12 +4310,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.06%</t>
+          <t>18.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-4.07%</t>
+          <t>-4.09%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4337,27 +4337,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.32%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.96%</t>
+          <t>-1.98%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.15%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-14]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/13/2026 at 3:43 PM ET)</t>
+          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>185 days</t>
+          <t>184 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>311 days</t>
+          <t>310 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>66 days</t>
+          <t>65 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>129 days</t>
+          <t>128 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>94 days</t>
+          <t>93 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>276 days</t>
+          <t>275 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>247 days</t>
+          <t>246 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>157 days</t>
+          <t>156 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>220 days</t>
+          <t>219 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>38 days</t>
+          <t>37 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>339 days</t>
+          <t>338 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.39 / 6.89%</t>
+          <t>$48.05 / 6.14%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.43 / 1.55%</t>
+          <t>$57.91 / 0.66%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.60 / 10.95%</t>
+          <t>$56.32 / 10.41%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.25 / 9.21%</t>
+          <t>$62.88 / 8.57%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.23 / 9.50%</t>
+          <t>$56.91 / 8.88%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$62.03 / 3.65%</t>
+          <t>$61.50 / 2.77%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$62.00 / 3.55%</t>
+          <t>$61.50 / 2.72%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$54.03 / 11.83%</t>
+          <t>$53.85 / 11.45%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$58.18 / 4.71%</t>
+          <t>$57.65 / 3.75%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.81 / 14.21%</t>
+          <t>$60.51 / 13.65%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.69 / 14.24%</t>
+          <t>$54.56 / 13.97%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.88 / 1.40%</t>
+          <t>$57.40 / 0.57%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.97 / 5.71%</t>
+          <t>$42.75 / 5.18%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.55 / 1.29%</t>
+          <t>$42.26 / 0.58%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.15 / 9.17%</t>
+          <t>$40.98 / 8.72%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.38 / 7.48%</t>
+          <t>$45.22 / 7.10%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.51 / 8.03%</t>
+          <t>$46.31 / 7.56%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$45.01 / 3.11%</t>
+          <t>$44.73 / 2.48%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.42 / 3.08%</t>
+          <t>$42.14 / 2.41%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.48 / 9.51%</t>
+          <t>$45.34 / 9.17%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.39 / 4.09%</t>
+          <t>$44.12 / 3.47%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.17 / 11.48%</t>
+          <t>$43.06 / 11.21%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.94 / 11.33%</t>
+          <t>$42.92 / 11.29%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.57 / 1.24%</t>
+          <t>$42.30 / 0.60%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$778.23 / 9.59%</t>
+          <t>$767.55 / 8.08%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$778.23 / 1.63%</t>
+          <t>$767.55 / 0.24%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$778.23 / 14.35%</t>
+          <t>$767.55 / 12.78%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$778.23 / 12.88%</t>
+          <t>$767.55 / 11.33%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$778.23 / 12.52%</t>
+          <t>$767.55 / 10.97%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$778.23 / 4.70%</t>
+          <t>$767.55 / 3.26%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$778.23 / 4.22%</t>
+          <t>$767.55 / 2.79%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$778.23 / 19.99%</t>
+          <t>$767.55 / 18.34%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$778.23 / 5.28%</t>
+          <t>$767.55 / 3.84%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$778.23 / 18.09%</t>
+          <t>$767.55 / 16.47%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$778.23 / 17.13%</t>
+          <t>$767.55 / 15.53%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$778.23 / 2.17%</t>
+          <t>$767.55 / 0.77%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$778.23 / 9.59%</t>
+          <t>$767.55 / 8.08%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$778.23 / 1.63%</t>
+          <t>$767.55 / 0.24%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$778.23 / 14.35%</t>
+          <t>$767.55 / 12.78%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$778.23 / 12.88%</t>
+          <t>$767.55 / 11.33%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$778.23 / 12.52%</t>
+          <t>$767.55 / 10.97%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$778.23 / 4.70%</t>
+          <t>$767.55 / 3.26%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$778.23 / 4.22%</t>
+          <t>$767.55 / 2.79%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$778.23 / 19.99%</t>
+          <t>$767.55 / 18.34%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$778.23 / 5.28%</t>
+          <t>$767.55 / 3.84%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$778.23 / 18.09%</t>
+          <t>$767.55 / 16.47%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$778.23 / 17.13%</t>
+          <t>$767.55 / 15.53%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$778.23 / 2.17%</t>
+          <t>$767.55 / 0.77%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.35% (6.95%)</t>
+          <t>8.11% (7.70%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.25% (14.54%)</t>
+          <t>16.28% (15.56%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.80% (2.66%)</t>
+          <t>3.30% (3.17%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.81% (4.53%)</t>
+          <t>5.43% (5.15%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.02% (3.82%)</t>
+          <t>4.61% (4.41%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.51% (11.89%)</t>
+          <t>13.47% (12.85%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.20% (11.64%)</t>
+          <t>13.10% (12.54%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.35% (4.02%)</t>
+          <t>4.70% (4.38%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.49% (11.00%)</t>
+          <t>12.51% (12.02%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.45% (1.37%)</t>
+          <t>1.95% (1.87%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.01% (0.00%)</t>
+          <t>0.25% (0.24%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.01% (14.23%)</t>
+          <t>15.96% (15.18%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>5.88% (5.47%)</t>
+          <t>6.41% (6.00%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.19% (11.47%)</t>
+          <t>12.97% (12.25%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.03% (1.89%)</t>
+          <t>2.45% (2.31%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.74% (3.46%)</t>
+          <t>4.11% (3.83%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2.93% (2.72%)</t>
+          <t>3.37% (3.17%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.19% (9.56%)</t>
+          <t>10.86% (10.24%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.70% (9.15%)</t>
+          <t>10.42% (9.86%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.75% (3.42%)</t>
+          <t>4.07% (3.74%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.02% (8.53%)</t>
+          <t>9.67% (9.18%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.91% (0.83%)</t>
+          <t>1.15% (1.08%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>-0.02% (-0.03%)</t>
+          <t>0.01% (0.01%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.63% (11.85%)</t>
+          <t>13.35% (12.56%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.08%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.29%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-2.35%</t>
+          <t>-0.99%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-1.74%</t>
+          <t>-0.38%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.20%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>3.94%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>11.92%</t>
+          <t>13.48%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.62%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.91%</t>
+          <t>-3.58%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>-2.93%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>13.22%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11.04% (10.64%)</t>
+          <t>10.55% (10.15%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.79% (9.08%)</t>
+          <t>9.43% (8.72%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.79% (10.66%)</t>
+          <t>10.14% (10.00%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>11.33% (11.06%)</t>
+          <t>10.76% (10.49%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.77% (10.57%)</t>
+          <t>10.16% (9.96%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.32% (9.70%)</t>
+          <t>9.95% (9.33%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.95% (9.40%)</t>
+          <t>9.52% (8.97%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.99% (13.66%)</t>
+          <t>13.25% (12.92%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.68% (9.20%)</t>
+          <t>9.37% (8.88%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.68% (10.60%)</t>
+          <t>10.05% (9.97%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.97% (9.96%)</t>
+          <t>9.10% (9.10%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.48% (9.70%)</t>
+          <t>10.06% (9.28%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.64% (16.23%)</t>
+          <t>16.03% (15.62%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.97% (14.26%)</t>
+          <t>14.50% (13.78%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.63% (16.49%)</t>
+          <t>15.97% (15.83%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>17.23% (16.95%)</t>
+          <t>16.50% (16.23%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.44% (16.24%)</t>
+          <t>15.79% (15.59%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.60% (14.98%)</t>
+          <t>15.06% (14.44%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>15.19% (14.63%)</t>
+          <t>14.68% (14.12%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>20.04% (19.70%)</t>
+          <t>19.33% (19.00%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>15.00% (14.50%)</t>
+          <t>14.44% (13.95%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>17.04% (16.96%)</t>
+          <t>16.25% (16.18%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>16.50% (16.50%)</t>
+          <t>15.52% (15.52%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.54% (14.76%)</t>
+          <t>15.01% (14.23%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.83% (-7.24%)</t>
+          <t>-6.18% (-6.58%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.65% (-2.37%)</t>
+          <t>-0.78% (-1.50%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.50% (-10.64%)</t>
+          <t>-10.06% (-10.19%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.94% (-9.21%)</t>
+          <t>-8.40% (-8.67%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.25% (-9.45%)</t>
+          <t>-8.74% (-8.94%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.72% (-4.34%)</t>
+          <t>-2.89% (-3.52%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.69% (-4.24%)</t>
+          <t>-2.92% (-3.47%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-11.01% (-11.34%)</t>
+          <t>-10.70% (-11.03%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.83% (-5.32%)</t>
+          <t>-3.96% (-4.45%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.11% (-13.18%)</t>
+          <t>-12.68% (-12.75%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.20% (-13.21%)</t>
+          <t>-12.99% (-13.00%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.44% (-2.22%)</t>
+          <t>-0.62% (-1.41%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.80% (-6.20%)</t>
+          <t>-5.32% (-5.73%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.39% (-2.11%)</t>
+          <t>-0.70% (-1.42%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-9.04% (-9.18%)</t>
+          <t>-8.66% (-8.80%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.47% (-7.75%)</t>
+          <t>-7.14% (-7.42%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-8.01% (-8.21%)</t>
+          <t>-7.61% (-7.81%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.84%)</t>
+          <t>-2.62% (-3.25%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.25% (-3.80%)</t>
+          <t>-2.62% (-3.18%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.12% (-9.46%)</t>
+          <t>-8.84% (-9.18%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.27% (-4.76%)</t>
+          <t>-3.70% (-4.19%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.97% (-11.05%)</t>
+          <t>-10.76% (-10.84%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.93% (-10.93%)</t>
+          <t>-10.90% (-10.90%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.27% (-2.05%)</t>
+          <t>-0.64% (-1.42%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.87%</t>
+          <t>-16.73%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-11.45%</t>
+          <t>-10.21%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-21.29%</t>
+          <t>-20.20%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-20.27%</t>
+          <t>-19.16%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-20.01%</t>
+          <t>-18.90%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-14.04%</t>
+          <t>-12.84%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.64%</t>
+          <t>-12.44%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-25.00%</t>
+          <t>-23.95%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.52%</t>
+          <t>-13.33%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.78%</t>
+          <t>-22.72%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-23.17%</t>
+          <t>-22.10%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.91%</t>
+          <t>-10.69%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-22.43%</t>
+          <t>-21.35%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-16.36%</t>
+          <t>-15.20%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.66%</t>
+          <t>-24.63%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.70%</t>
+          <t>-23.65%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.45%</t>
+          <t>-23.40%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.81%</t>
+          <t>-17.68%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-18.44%</t>
+          <t>-17.30%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-29.16%</t>
+          <t>-28.17%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-19.26%</t>
+          <t>-18.14%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-28.02%</t>
+          <t>-27.01%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-27.43%</t>
+          <t>-26.42%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.81%</t>
+          <t>-15.65%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.14% (1.73%)</t>
+          <t>1.44% (1.04%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.76%)</t>
+          <t>-0.54% (-1.26%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.43% (2.29%)</t>
+          <t>1.52% (1.38%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.86% (2.58%)</t>
+          <t>2.04% (1.77%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2.18% (1.98%)</t>
+          <t>1.34% (1.14%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.81% (0.19%)</t>
+          <t>0.28% (-0.34%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.38% (-0.17%)</t>
+          <t>-0.20% (-0.76%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.35% (4.02%)</t>
+          <t>4.70% (4.38%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.21% (-0.28%)</t>
+          <t>-0.26% (-0.75%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.45% (1.37%)</t>
+          <t>1.81% (1.74%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.01% (0.00%)</t>
+          <t>0.25% (0.24%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.70% (-0.07%)</t>
+          <t>0.14% (-0.64%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>3.27% (2.86%)</t>
+          <t>2.36% (1.95%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.22% (-0.49%)</t>
+          <t>-0.47% (-1.19%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.03% (1.89%)</t>
+          <t>2.45% (2.31%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.74% (3.46%)</t>
+          <t>3.43% (3.15%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.93% (2.72%)</t>
+          <t>2.58% (2.38%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1.34% (0.72%)</t>
+          <t>0.56% (-0.07%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.84% (0.28%)</t>
+          <t>0.10% (-0.46%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.75% (3.42%)</t>
+          <t>4.07% (3.74%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.80% (0.31%)</t>
+          <t>0.01% (-0.48%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.91% (0.83%)</t>
+          <t>1.15% (1.08%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.03%)</t>
+          <t>0.01% (0.01%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.86% (0.08%)</t>
+          <t>0.11% (-0.68%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/10/2026</t>
+          <t>As of 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.57%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.45%</t>
+          <t>-8.94%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.06%</t>
+          <t>10.49%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.53%</t>
+          <t>5.15%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.21%</t>
+          <t>-8.67%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>12.92%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>4.38%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.45%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.99%</t>
+          <t>18.34%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.35%</t>
+          <t>-0.99%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.34%</t>
+          <t>-11.03%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.64%</t>
+          <t>10.15%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.95%</t>
+          <t>7.70%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>6.14%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.08%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.24%</t>
+          <t>-6.58%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.20%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>12.02%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.71%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-5.32%</t>
+          <t>-4.45%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11.64%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.74%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.24%</t>
+          <t>-3.47%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11.89%</t>
+          <t>12.85%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.65%</t>
+          <t>2.77%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-3.52%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.08%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14.54%</t>
+          <t>15.56%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>0.66%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.29%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.37%</t>
+          <t>-1.50%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>15.18%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.40%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.20%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.22%</t>
+          <t>-1.41%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.13%</t>
+          <t>15.53%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1.74%</t>
+          <t>-0.38%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.21%</t>
+          <t>-13.00%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>9.97%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.37%</t>
+          <t>1.87%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>13.65%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.09%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.18%</t>
+          <t>-12.75%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.95%</t>
+          <t>10.41%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.35%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.64%</t>
+          <t>-10.19%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 13/10/2026</t>
+          <t>As of 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>15.59%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.03%</t>
+          <t>7.56%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.62%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.21%</t>
+          <t>-7.81%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.95%</t>
+          <t>16.23%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>3.83%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.48%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.75%</t>
+          <t>-7.42%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.70%</t>
+          <t>19.00%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.42%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.99%</t>
+          <t>18.34%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.91%</t>
+          <t>-3.58%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.46%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.47%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.71%</t>
+          <t>5.18%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9.59%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2.51%</t>
+          <t>3.94%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.20%</t>
+          <t>-5.73%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.50%</t>
+          <t>13.95%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.53%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.12%</t>
+          <t>9.62%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.76%</t>
+          <t>-4.19%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.63%</t>
+          <t>14.12%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>9.86%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.22%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.80%</t>
+          <t>-3.18%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>14.44%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.56%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8.71%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>13.78%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>0.58%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>11.92%</t>
+          <t>13.48%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-1.42%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.76%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11.85%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>0.60%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>13.22%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-2.05%</t>
+          <t>-1.42%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>15.52%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>0.01%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.13%</t>
+          <t>15.53%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>-2.93%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.93%</t>
+          <t>-10.90%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.96%</t>
+          <t>16.18%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.21%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>18.09%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.05%</t>
+          <t>-10.84%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.49%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>2.31%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>8.72%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-8.80%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-15]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/14/2026 at 1:57 PM ET)</t>
+          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>184 days</t>
+          <t>183 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>310 days</t>
+          <t>309 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>65 days</t>
+          <t>64 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>128 days</t>
+          <t>127 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>93 days</t>
+          <t>92 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>275 days</t>
+          <t>274 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>246 days</t>
+          <t>245 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>156 days</t>
+          <t>155 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>219 days</t>
+          <t>218 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>37 days</t>
+          <t>36 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>1 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>338 days</t>
+          <t>337 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.05 / 6.14%</t>
+          <t>$48.15 / 6.37%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.91 / 0.66%</t>
+          <t>$58.08 / 0.95%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.32 / 10.41%</t>
+          <t>$56.38 / 10.52%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.88 / 8.57%</t>
+          <t>$63.01 / 8.80%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.91 / 8.88%</t>
+          <t>$57.04 / 9.12%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.50 / 2.77%</t>
+          <t>$61.67 / 3.05%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.50 / 2.72%</t>
+          <t>$61.60 / 2.89%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.85 / 11.45%</t>
+          <t>$53.89 / 11.54%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.65 / 3.75%</t>
+          <t>$57.81 / 4.04%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.51 / 13.65%</t>
+          <t>$60.64 / 13.89%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.56 / 13.97%</t>
+          <t>$54.66 / 14.19%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.40 / 0.57%</t>
+          <t>$57.54 / 0.81%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.75 / 5.18%</t>
+          <t>$42.80 / 5.31%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.26 / 0.58%</t>
+          <t>$42.35 / 0.80%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.98 / 8.72%</t>
+          <t>$41.04 / 8.90%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.22 / 7.10%</t>
+          <t>$45.28 / 7.24%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.31 / 7.56%</t>
+          <t>$46.36 / 7.69%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.73 / 2.48%</t>
+          <t>$44.79 / 2.62%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.14 / 2.41%</t>
+          <t>$42.23 / 2.61%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.34 / 9.17%</t>
+          <t>$45.42 / 9.37%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.12 / 3.47%</t>
+          <t>$44.20 / 3.66%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.06 / 11.21%</t>
+          <t>$43.10 / 11.30%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.92 / 11.29%</t>
+          <t>$42.93 / 11.32%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.30 / 0.60%</t>
+          <t>$42.39 / 0.82%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$767.55 / 8.08%</t>
+          <t>$771.01 / 8.57%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$767.55 / 0.24%</t>
+          <t>$771.01 / 0.69%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$767.55 / 12.78%</t>
+          <t>$771.01 / 13.29%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$767.55 / 11.33%</t>
+          <t>$771.01 / 11.83%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$767.55 / 10.97%</t>
+          <t>$771.01 / 11.47%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$767.55 / 3.26%</t>
+          <t>$771.01 / 3.73%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$767.55 / 2.79%</t>
+          <t>$771.01 / 3.25%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$767.55 / 18.34%</t>
+          <t>$771.01 / 18.88%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$767.55 / 3.84%</t>
+          <t>$771.01 / 4.31%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$767.55 / 16.47%</t>
+          <t>$771.01 / 16.99%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$767.55 / 15.53%</t>
+          <t>$771.01 / 16.05%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$767.55 / 0.77%</t>
+          <t>$771.01 / 1.22%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$767.55 / 8.08%</t>
+          <t>$771.01 / 8.57%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$767.55 / 0.24%</t>
+          <t>$771.01 / 0.69%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$767.55 / 12.78%</t>
+          <t>$771.01 / 13.29%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$767.55 / 11.33%</t>
+          <t>$771.01 / 11.83%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$767.55 / 10.97%</t>
+          <t>$771.01 / 11.47%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$767.55 / 3.26%</t>
+          <t>$771.01 / 3.73%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$767.55 / 2.79%</t>
+          <t>$771.01 / 3.25%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$767.55 / 18.34%</t>
+          <t>$771.01 / 18.88%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$767.55 / 3.84%</t>
+          <t>$771.01 / 4.31%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$767.55 / 16.47%</t>
+          <t>$771.01 / 16.99%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$767.55 / 15.53%</t>
+          <t>$771.01 / 16.05%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$767.55 / 0.77%</t>
+          <t>$771.01 / 1.22%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.11% (7.70%)</t>
+          <t>7.87% (7.47%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.28% (15.56%)</t>
+          <t>15.93% (15.22%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.30% (3.17%)</t>
+          <t>3.19% (3.06%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.43% (5.15%)</t>
+          <t>5.20% (4.93%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.61% (4.41%)</t>
+          <t>4.38% (4.18%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.47% (12.85%)</t>
+          <t>13.16% (12.54%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.10% (12.54%)</t>
+          <t>12.91% (12.36%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.70% (4.38%)</t>
+          <t>4.61% (4.29%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.51% (12.02%)</t>
+          <t>12.20% (11.71%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.95% (1.87%)</t>
+          <t>1.73% (1.65%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.25% (0.24%)</t>
+          <t>0.05% (0.05%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.96% (15.18%)</t>
+          <t>15.68% (14.90%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.41% (6.00%)</t>
+          <t>6.28% (5.88%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.97% (12.25%)</t>
+          <t>12.72% (12.01%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.45% (2.31%)</t>
+          <t>2.29% (2.15%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.11% (3.83%)</t>
+          <t>3.98% (3.70%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.37% (3.17%)</t>
+          <t>3.24% (3.04%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.86% (10.24%)</t>
+          <t>10.71% (10.09%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.42% (9.86%)</t>
+          <t>10.19% (9.64%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.07% (3.74%)</t>
+          <t>3.89% (3.56%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.67% (9.18%)</t>
+          <t>9.47% (8.98%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.15% (1.08%)</t>
+          <t>1.07% (1.00%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.01% (0.01%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.35% (12.56%)</t>
+          <t>13.10% (12.33%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>15.27%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.48%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>-1.06%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.58%</t>
+          <t>-4.02%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-3.20%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-2.93%</t>
+          <t>-3.36%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>12.71%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.55% (10.15%)</t>
+          <t>10.72% (10.32%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.43% (8.72%)</t>
+          <t>9.54% (8.83%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.14% (10.00%)</t>
+          <t>10.40% (10.27%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.76% (10.49%)</t>
+          <t>10.93% (10.66%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.16% (9.96%)</t>
+          <t>10.32% (10.13%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.95% (9.33%)</t>
+          <t>10.07% (9.45%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.52% (8.97%)</t>
+          <t>9.76% (9.20%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.25% (12.92%)</t>
+          <t>13.51% (13.19%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.37% (8.88%)</t>
+          <t>9.49% (9.00%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.05% (9.97%)</t>
+          <t>10.20% (10.13%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.10% (9.10%)</t>
+          <t>9.28% (9.28%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.06% (9.28%)</t>
+          <t>10.22% (9.44%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.03% (15.62%)</t>
+          <t>16.27% (15.87%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.50% (13.78%)</t>
+          <t>14.66% (13.95%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.97% (15.83%)</t>
+          <t>16.16% (16.02%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.50% (16.23%)</t>
+          <t>16.73% (16.46%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.79% (15.59%)</t>
+          <t>16.02% (15.82%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.06% (14.44%)</t>
+          <t>15.30% (14.68%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.68% (14.12%)</t>
+          <t>14.86% (14.30%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.33% (19.00%)</t>
+          <t>19.49% (19.16%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.44% (13.95%)</t>
+          <t>14.64% (14.15%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.25% (16.18%)</t>
+          <t>16.51% (16.43%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.52% (15.52%)</t>
+          <t>15.83% (15.83%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.01% (14.23%)</t>
+          <t>15.17% (14.40%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.18% (-6.58%)</t>
+          <t>-6.38% (-6.78%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.78% (-1.50%)</t>
+          <t>-1.07% (-1.79%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.06% (-10.19%)</t>
+          <t>-10.15% (-10.29%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.40% (-8.67%)</t>
+          <t>-8.59% (-8.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.74% (-8.94%)</t>
+          <t>-8.94% (-9.14%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.89% (-3.52%)</t>
+          <t>-3.16% (-3.78%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.92% (-3.47%)</t>
+          <t>-3.08% (-3.63%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.70% (-11.03%)</t>
+          <t>-10.78% (-11.11%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.96% (-4.45%)</t>
+          <t>-4.23% (-4.72%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.68% (-12.75%)</t>
+          <t>-12.87% (-12.94%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-12.99% (-13.00%)</t>
+          <t>-13.16% (-13.17%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.62% (-1.41%)</t>
+          <t>-0.87% (-1.65%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.32% (-5.73%)</t>
+          <t>-5.44% (-5.84%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.70% (-1.42%)</t>
+          <t>-0.92% (-1.63%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.66% (-8.80%)</t>
+          <t>-8.81% (-8.94%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.14% (-7.42%)</t>
+          <t>-7.26% (-7.53%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.61% (-7.81%)</t>
+          <t>-7.72% (-7.92%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.62% (-3.25%)</t>
+          <t>-2.75% (-3.38%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.62% (-3.18%)</t>
+          <t>-2.82% (-3.37%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.84% (-9.18%)</t>
+          <t>-9.01% (-9.34%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.70% (-4.19%)</t>
+          <t>-3.87% (-4.36%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.76% (-10.84%)</t>
+          <t>-10.83% (-10.91%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.90% (-10.90%)</t>
+          <t>-10.92% (-10.92%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.64% (-1.42%)</t>
+          <t>-0.85% (-1.63%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.73%</t>
+          <t>-17.10%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.21%</t>
+          <t>-10.62%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.20%</t>
+          <t>-20.55%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.16%</t>
+          <t>-19.52%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.90%</t>
+          <t>-19.26%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.84%</t>
+          <t>-13.24%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.44%</t>
+          <t>-12.83%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.95%</t>
+          <t>-24.29%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.33%</t>
+          <t>-13.72%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.72%</t>
+          <t>-23.07%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.10%</t>
+          <t>-22.45%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.69%</t>
+          <t>-11.09%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.35%</t>
+          <t>-21.71%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.20%</t>
+          <t>-15.58%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.63%</t>
+          <t>-24.97%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.65%</t>
+          <t>-23.99%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.40%</t>
+          <t>-23.75%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.68%</t>
+          <t>-18.05%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.30%</t>
+          <t>-17.67%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.17%</t>
+          <t>-28.50%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.14%</t>
+          <t>-18.51%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.01%</t>
+          <t>-27.34%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.42%</t>
+          <t>-26.75%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.65%</t>
+          <t>-16.03%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.44% (1.04%)</t>
+          <t>1.68% (1.28%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.54% (-1.26%)</t>
+          <t>-0.39% (-1.10%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.52% (1.38%)</t>
+          <t>1.87% (1.73%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.04% (1.77%)</t>
+          <t>2.28% (2.01%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.34% (1.14%)</t>
+          <t>1.57% (1.38%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.28% (-0.34%)</t>
+          <t>0.46% (-0.16%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.20% (-0.76%)</t>
+          <t>0.08% (-0.47%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.70% (4.38%)</t>
+          <t>4.61% (4.29%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.75%)</t>
+          <t>-0.09% (-0.58%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.81% (1.74%)</t>
+          <t>1.73% (1.65%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.25% (0.24%)</t>
+          <t>0.05% (0.05%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.14% (-0.64%)</t>
+          <t>0.35% (-0.43%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.36% (1.95%)</t>
+          <t>2.70% (2.30%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.47% (-1.19%)</t>
+          <t>-0.23% (-0.95%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.45% (2.31%)</t>
+          <t>2.29% (2.15%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.43% (3.15%)</t>
+          <t>3.77% (3.50%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.58% (2.38%)</t>
+          <t>2.93% (2.73%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.56% (-0.07%)</t>
+          <t>0.88% (0.26%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.10% (-0.46%)</t>
+          <t>0.35% (-0.21%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.07% (3.74%)</t>
+          <t>3.89% (3.56%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.01% (-0.48%)</t>
+          <t>0.28% (-0.21%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.15% (1.08%)</t>
+          <t>1.07% (1.00%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.01% (0.01%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.11% (-0.68%)</t>
+          <t>0.34% (-0.44%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/10/2026</t>
+          <t>As of 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>10.13%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>4.18%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>2.74%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.94%</t>
+          <t>-9.14%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.49%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.15%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.67%</t>
+          <t>-8.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.92%</t>
+          <t>13.19%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.38%</t>
+          <t>4.29%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.45%</t>
+          <t>11.54%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.34%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.03%</t>
+          <t>-11.11%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.15%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.70%</t>
+          <t>7.47%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.14%</t>
+          <t>6.37%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.58%</t>
+          <t>-6.78%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.02%</t>
+          <t>11.71%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.45%</t>
+          <t>-4.72%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>9.20%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>12.36%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>2.89%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.79%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.78%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.63%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.45%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.85%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.77%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-3.78%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.56%</t>
+          <t>15.22%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>16.37%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.50%</t>
+          <t>-1.79%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.18%</t>
+          <t>14.90%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.57%</t>
+          <t>0.81%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>15.27%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-1.65%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.05%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.53%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.00%</t>
+          <t>-13.17%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.97%</t>
+          <t>10.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.87%</t>
+          <t>1.65%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.65%</t>
+          <t>13.89%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.75%</t>
+          <t>-12.94%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>10.27%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.41%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.19%</t>
+          <t>-10.29%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 14/10/2026</t>
+          <t>As of 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.59%</t>
+          <t>15.82%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>3.04%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.56%</t>
+          <t>7.69%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.81%</t>
+          <t>-7.92%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.83%</t>
+          <t>3.70%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>7.24%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.42%</t>
+          <t>-7.53%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.00%</t>
+          <t>19.16%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.56%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.34%</t>
+          <t>18.88%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.58%</t>
+          <t>-4.02%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.34%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.18%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>8.57%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.73%</t>
+          <t>-5.84%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.95%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.62%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.19%</t>
+          <t>-4.36%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.12%</t>
+          <t>14.30%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.86%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.41%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.79%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>9.78%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.18%</t>
+          <t>-3.37%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.44%</t>
+          <t>14.68%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.09%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-3.38%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.78%</t>
+          <t>13.95%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.58%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.48%</t>
+          <t>12.97%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.42%</t>
+          <t>-1.63%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>14.40%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.42%</t>
+          <t>-1.63%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.52%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.01%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.53%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.93%</t>
+          <t>-3.36%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.90%</t>
+          <t>-10.92%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.18%</t>
+          <t>16.43%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>1.00%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.21%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-3.20%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.84%</t>
+          <t>-10.91%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>16.02%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.15%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.72%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>-1.06%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.80%</t>
+          <t>-8.94%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-16]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/15/2026 at 1:39 PM ET)</t>
+          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>244 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>183 days</t>
+          <t>182 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>309 days</t>
+          <t>308 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>64 days</t>
+          <t>63 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>127 days</t>
+          <t>126 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>92 days</t>
+          <t>91 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>274 days</t>
+          <t>273 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>245 days</t>
+          <t>244 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>155 days</t>
+          <t>154 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>218 days</t>
+          <t>217 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>36 days</t>
+          <t>35 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>1 days</t>
+          <t>0 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>337 days</t>
+          <t>336 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.15 / 6.37%</t>
+          <t>$47.87 / 5.75%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.08 / 0.95%</t>
+          <t>$57.70 / 0.29%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.38 / 10.52%</t>
+          <t>$56.08 / 9.94%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.01 / 8.80%</t>
+          <t>$62.67 / 8.21%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.04 / 9.12%</t>
+          <t>$56.71 / 8.49%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.67 / 3.05%</t>
+          <t>$61.27 / 2.37%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.60 / 2.89%</t>
+          <t>$61.20 / 2.22%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.89 / 11.54%</t>
+          <t>$53.73 / 11.20%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.81 / 4.04%</t>
+          <t>$57.43 / 3.35%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.64 / 13.89%</t>
+          <t>$60.34 / 13.32%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.66 / 14.19%</t>
+          <t>$54.61 / 14.08%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.54 / 0.81%</t>
+          <t>$57.18 / 0.17%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.80 / 5.31%</t>
+          <t>$42.63 / 4.89%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.35 / 0.80%</t>
+          <t>$42.14 / 0.31%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.04 / 8.90%</t>
+          <t>$40.88 / 8.47%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.28 / 7.24%</t>
+          <t>$45.10 / 6.82%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.36 / 7.69%</t>
+          <t>$46.17 / 7.25%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.79 / 2.62%</t>
+          <t>$44.62 / 2.22%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.23 / 2.61%</t>
+          <t>$42.02 / 2.10%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.42 / 9.37%</t>
+          <t>$45.30 / 9.07%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.20 / 3.66%</t>
+          <t>$43.96 / 3.10%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.10 / 11.30%</t>
+          <t>$42.97 / 10.96%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.93 / 11.32%</t>
+          <t>$42.99 / 11.47%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.39 / 0.82%</t>
+          <t>$42.18 / 0.32%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$771.01 / 8.57%</t>
+          <t>$763.43 / 7.50%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$771.01 / 0.69%</t>
+          <t>$763.43 / -0.30%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$771.01 / 13.29%</t>
+          <t>$763.43 / 12.17%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$771.01 / 11.83%</t>
+          <t>$763.43 / 10.73%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$771.01 / 11.47%</t>
+          <t>$763.43 / 10.38%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$771.01 / 3.73%</t>
+          <t>$763.43 / 2.71%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$771.01 / 3.25%</t>
+          <t>$763.43 / 2.23%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$771.01 / 18.88%</t>
+          <t>$763.43 / 17.71%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$771.01 / 4.31%</t>
+          <t>$763.43 / 3.28%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$771.01 / 16.99%</t>
+          <t>$763.43 / 15.84%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$771.01 / 16.05%</t>
+          <t>$763.43 / 14.91%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$771.01 / 1.22%</t>
+          <t>$763.43 / 0.23%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$771.01 / 8.57%</t>
+          <t>$763.43 / 7.50%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$771.01 / 0.69%</t>
+          <t>$764.07 / -0.22%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$771.01 / 13.29%</t>
+          <t>$764.07 / 12.27%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$771.01 / 11.83%</t>
+          <t>$763.43 / 10.73%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$771.01 / 11.47%</t>
+          <t>$763.43 / 10.38%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$771.01 / 3.73%</t>
+          <t>$764.07 / 2.80%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$771.01 / 3.25%</t>
+          <t>$764.07 / 2.32%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$771.01 / 18.88%</t>
+          <t>$763.43 / 17.71%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$771.01 / 4.31%</t>
+          <t>$763.43 / 3.28%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$771.01 / 16.99%</t>
+          <t>$764.07 / 15.94%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$771.01 / 16.05%</t>
+          <t>$764.07 / 15.00%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$771.01 / 1.22%</t>
+          <t>$764.07 / 0.31%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.87% (7.47%)</t>
+          <t>8.50% (8.10%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.93% (15.22%)</t>
+          <t>16.70% (15.98%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.19% (3.06%)</t>
+          <t>3.73% (3.60%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.20% (4.93%)</t>
+          <t>5.77% (5.50%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.38% (4.18%)</t>
+          <t>4.98% (4.79%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.16% (12.54%)</t>
+          <t>13.91% (13.28%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.91% (12.36%)</t>
+          <t>13.65% (13.09%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.61% (4.29%)</t>
+          <t>4.93% (4.61%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.20% (11.71%)</t>
+          <t>12.95% (12.46%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.73% (1.65%)</t>
+          <t>2.24% (2.17%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.05% (0.05%)</t>
+          <t>0.14% (0.14%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.68% (14.90%)</t>
+          <t>16.41% (15.63%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.28% (5.88%)</t>
+          <t>6.70% (6.30%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.72% (12.01%)</t>
+          <t>13.27% (12.56%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.29% (2.15%)</t>
+          <t>2.68% (2.55%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.98% (3.70%)</t>
+          <t>4.38% (4.11%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.24% (3.04%)</t>
+          <t>3.67% (3.47%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.71% (10.09%)</t>
+          <t>11.14% (10.52%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.19% (9.64%)</t>
+          <t>10.74% (10.19%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.89% (3.56%)</t>
+          <t>4.17% (3.84%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.47% (8.98%)</t>
+          <t>10.06% (9.57%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.07% (1.00%)</t>
+          <t>1.37% (1.30%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>-0.02% (-0.02%)</t>
+          <t>-0.16% (-0.16%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.10% (12.33%)</t>
+          <t>13.66% (12.88%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>17.52%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.86%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>3.76%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.74%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.46%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>13.37%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.27%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-0.16%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.02%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.20%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>-3.36%</t>
+          <t>-2.49%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>13.73%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.72% (10.32%)</t>
+          <t>10.44% (10.04%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.54% (8.83%)</t>
+          <t>9.31% (8.59%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.40% (10.27%)</t>
+          <t>10.08% (9.95%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.93% (10.66%)</t>
+          <t>10.62% (10.35%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.32% (10.13%)</t>
+          <t>10.05% (9.85%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.07% (9.45%)</t>
+          <t>9.85% (9.23%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.76% (9.20%)</t>
+          <t>9.52% (8.97%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.51% (13.19%)</t>
+          <t>13.03% (12.71%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.49% (9.00%)</t>
+          <t>9.27% (8.78%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.20% (10.13%)</t>
+          <t>9.88% (9.81%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.28% (9.28%)</t>
+          <t>8.59% (8.59%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.22% (9.44%)</t>
+          <t>9.97% (9.19%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.27% (15.87%)</t>
+          <t>15.87% (15.46%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.66% (13.95%)</t>
+          <t>14.38% (13.66%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.16% (16.02%)</t>
+          <t>15.83% (15.70%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.73% (16.46%)</t>
+          <t>16.33% (16.06%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.02% (15.82%)</t>
+          <t>15.64% (15.44%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.30% (14.68%)</t>
+          <t>14.93% (14.31%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.86% (14.30%)</t>
+          <t>14.59% (14.04%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.49% (19.16%)</t>
+          <t>19.03% (18.70%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.64% (14.15%)</t>
+          <t>14.35% (13.86%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.51% (16.43%)</t>
+          <t>16.12% (16.04%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.83% (15.83%)</t>
+          <t>15.04% (15.04%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.17% (14.40%)</t>
+          <t>14.90% (14.12%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.38% (-6.78%)</t>
+          <t>-5.84% (-6.24%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.07% (-1.79%)</t>
+          <t>-0.42% (-1.14%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.15% (-10.29%)</t>
+          <t>-9.68% (-9.82%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.59% (-8.87%)</t>
+          <t>-8.10% (-8.37%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.94% (-9.14%)</t>
+          <t>-8.41% (-8.61%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.16% (-3.78%)</t>
+          <t>-2.52% (-3.15%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.08% (-3.63%)</t>
+          <t>-2.44% (-3.00%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.78% (-11.11%)</t>
+          <t>-10.51% (-10.83%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.23% (-4.72%)</t>
+          <t>-3.59% (-4.08%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.87% (-12.94%)</t>
+          <t>-12.43% (-12.50%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.16% (-13.17%)</t>
+          <t>-13.09% (-13.09%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.87% (-1.65%)</t>
+          <t>-0.24% (-1.02%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.44% (-5.84%)</t>
+          <t>-5.06% (-5.47%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.92% (-1.63%)</t>
+          <t>-0.44% (-1.15%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.81% (-8.94%)</t>
+          <t>-8.45% (-8.59%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.26% (-7.53%)</t>
+          <t>-6.90% (-7.18%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.72% (-7.92%)</t>
+          <t>-7.35% (-7.54%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.75% (-3.38%)</t>
+          <t>-2.38% (-3.00%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.82% (-3.37%)</t>
+          <t>-2.33% (-2.89%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.01% (-9.34%)</t>
+          <t>-8.76% (-9.09%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.87% (-4.36%)</t>
+          <t>-3.35% (-3.84%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.83% (-10.91%)</t>
+          <t>-10.57% (-10.64%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-10.92% (-10.92%)</t>
+          <t>-11.05% (-11.05%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.85% (-1.63%)</t>
+          <t>-0.36% (-1.14%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.10%</t>
+          <t>-16.28%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.62%</t>
+          <t>-9.73%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.55%</t>
+          <t>-19.77%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.52%</t>
+          <t>-18.72%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.26%</t>
+          <t>-18.46%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.24%</t>
+          <t>-12.37%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.83%</t>
+          <t>-11.97%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.29%</t>
+          <t>-23.54%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.72%</t>
+          <t>-12.86%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.07%</t>
+          <t>-22.31%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-22.45%</t>
+          <t>-21.68%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.09%</t>
+          <t>-10.20%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.71%</t>
+          <t>-20.93%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.58%</t>
+          <t>-14.81%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.97%</t>
+          <t>-24.28%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.99%</t>
+          <t>-23.24%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.75%</t>
+          <t>-22.99%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-17.31%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.67%</t>
+          <t>-16.93%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.50%</t>
+          <t>-27.79%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.51%</t>
+          <t>-17.70%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.34%</t>
+          <t>-26.68%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.75%</t>
+          <t>-26.09%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.03%</t>
+          <t>-15.26%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.68% (1.28%)</t>
+          <t>1.26% (0.86%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.39% (-1.10%)</t>
+          <t>-0.42% (-1.14%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.87% (1.73%)</t>
+          <t>1.39% (1.25%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.28% (2.01%)</t>
+          <t>1.82% (1.55%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.57% (1.38%)</t>
+          <t>1.15% (0.96%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.46% (-0.16%)</t>
+          <t>0.12% (-0.50%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.08% (-0.47%)</t>
+          <t>-0.26% (-0.81%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.61% (4.29%)</t>
+          <t>4.93% (4.61%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.58%)</t>
+          <t>-0.41% (-0.90%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.73% (1.65%)</t>
+          <t>1.55% (1.48%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.05% (0.05%)</t>
+          <t>-0.02% (-0.02%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.35% (-0.43%)</t>
+          <t>-0.01% (-0.79%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.70% (2.30%)</t>
+          <t>2.09% (1.69%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.23% (-0.95%)</t>
+          <t>-0.44% (-1.15%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.29% (2.15%)</t>
+          <t>2.68% (2.55%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.77% (3.50%)</t>
+          <t>3.14% (2.87%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.93% (2.73%)</t>
+          <t>2.32% (2.13%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.88% (0.26%)</t>
+          <t>0.36% (-0.27%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.35% (-0.21%)</t>
+          <t>-0.06% (-0.62%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.89% (3.56%)</t>
+          <t>4.17% (3.84%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.28% (-0.21%)</t>
+          <t>-0.17% (-0.66%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.07% (1.00%)</t>
+          <t>1.37% (1.30%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.02%)</t>
+          <t>-0.16% (-0.16%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.34% (-0.44%)</t>
+          <t>-0.07% (-0.85%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/10/2026</t>
+          <t>As of 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.13%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.18%</t>
+          <t>4.79%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>8.49%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>10.38%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.74%</t>
+          <t>3.76%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.14%</t>
+          <t>-8.61%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.21%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.84%</t>
+          <t>3.86%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.87%</t>
+          <t>-8.37%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.19%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.29%</t>
+          <t>4.61%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>17.71%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.46%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.11%</t>
+          <t>-10.83%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.47%</t>
+          <t>8.10%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.37%</t>
+          <t>5.75%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.78%</t>
+          <t>-6.24%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.71%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>3.35%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>13.37%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.72%</t>
+          <t>-4.08%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.20%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>13.09%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.89%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.78%</t>
+          <t>13.91%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.63%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.45%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.54%</t>
+          <t>13.28%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.05%</t>
+          <t>2.37%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>13.74%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.78%</t>
+          <t>-3.15%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.22%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.37%</t>
+          <t>17.52%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.90%</t>
+          <t>15.63%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.23%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.27%</t>
+          <t>16.41%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.65%</t>
+          <t>-1.02%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>8.59%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>14.08%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>14.91%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.17%</t>
+          <t>-13.09%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.13%</t>
+          <t>9.81%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.65%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.89%</t>
+          <t>13.32%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.94%</t>
+          <t>-12.50%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.27%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>3.60%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.17%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.29%</t>
+          <t>-9.82%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 15/10/2026</t>
+          <t>As of 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.82%</t>
+          <t>15.44%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.04%</t>
+          <t>3.47%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.69%</t>
+          <t>7.25%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>10.38%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.92%</t>
+          <t>-7.54%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>16.06%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>4.11%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.24%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.53%</t>
+          <t>-7.18%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.16%</t>
+          <t>18.70%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.56%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.88%</t>
+          <t>17.71%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.02%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.34%</t>
+          <t>-9.09%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>15.46%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>6.30%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>4.89%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.57%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.84%</t>
+          <t>-5.47%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>13.86%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>9.57%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.28%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.36%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.30%</t>
+          <t>14.04%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>10.19%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.78%</t>
+          <t>10.78%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-2.89%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.31%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.09%</t>
+          <t>10.52%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.62%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.73%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>10.73%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.38%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.95%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>12.56%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-0.22%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.97%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.40%</t>
+          <t>14.12%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.63%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>15.04%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>-0.16%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-3.36%</t>
+          <t>-2.49%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-10.92%</t>
+          <t>-11.05%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.43%</t>
+          <t>16.04%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>10.96%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.99%</t>
+          <t>15.94%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.20%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.91%</t>
+          <t>-10.64%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.02%</t>
+          <t>15.70%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>12.27%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.06%</t>
+          <t>-0.16%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.94%</t>
+          <t>-8.59%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-19]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:27 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/16/2026 at 1:28 PM ET)</t>
+          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>10/20/2025 - 10/16/2026</t>
+          <t>10/19/2026 - 10/15/2027</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>10/20/2025 - 10/16/2026</t>
+          <t>10/19/2026 - 10/15/2027</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>15.09% (14.24%)</t>
+          <t>17.20% (16.35%)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>12.14% (11.30%)</t>
+          <t>14.05% (13.20%)</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>$47.87</t>
+          <t>$54.62</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>$38.57</t>
+          <t>$42.95</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>$54.69</t>
+          <t>$63.55</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>$42.92</t>
+          <t>$48.62</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>$664.39</t>
+          <t>$763.25</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>$664.39</t>
+          <t>$763.25</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>$764.65</t>
+          <t>$894.53</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>$745.07</t>
+          <t>$870.49</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.00% / $664.39</t>
+          <t>0.00% / $763.25</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>0.00% / $664.41</t>
+          <t>0.00% / $763.25</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>-10.00% / $597.95</t>
+          <t>-10.00% / $686.93</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>-15.00% / $564.75</t>
+          <t>-15.00% / $648.76</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>270 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>244 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>182 days</t>
+          <t>179 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>308 days</t>
+          <t>305 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>63 days</t>
+          <t>60 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>126 days</t>
+          <t>123 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>91 days</t>
+          <t>88 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>273 days</t>
+          <t>270 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>244 days</t>
+          <t>241 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>154 days</t>
+          <t>151 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>217 days</t>
+          <t>214 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>35 days</t>
+          <t>32 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>0 days</t>
+          <t>361 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>336 days</t>
+          <t>333 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.87 / 5.75%</t>
+          <t>$48.06 / 6.16%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.70 / 0.29%</t>
+          <t>$57.92 / 0.67%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.08 / 9.94%</t>
+          <t>$56.32 / 10.42%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.67 / 8.21%</t>
+          <t>$62.91 / 8.63%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.71 / 8.49%</t>
+          <t>$56.94 / 8.94%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.27 / 2.37%</t>
+          <t>$61.53 / 2.81%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.20 / 2.22%</t>
+          <t>$61.45 / 2.63%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.73 / 11.20%</t>
+          <t>$53.86 / 11.48%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.43 / 3.35%</t>
+          <t>$57.66 / 3.76%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.34 / 13.32%</t>
+          <t>$60.61 / 13.83%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.61 / 14.08%</t>
+          <t>$54.81 / 0.34%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.18 / 0.17%</t>
+          <t>$57.40 / 0.56%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.63 / 4.89%</t>
+          <t>$42.76 / 5.20%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.14 / 0.31%</t>
+          <t>$42.27 / 0.61%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.88 / 8.47%</t>
+          <t>$41.01 / 8.82%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.10 / 6.82%</t>
+          <t>$45.23 / 7.13%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.17 / 7.25%</t>
+          <t>$46.33 / 7.61%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.62 / 2.22%</t>
+          <t>$44.73 / 2.48%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.02 / 2.10%</t>
+          <t>$42.14 / 2.40%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.30 / 9.07%</t>
+          <t>$45.39 / 9.29%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.96 / 3.10%</t>
+          <t>$44.09 / 3.40%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$42.97 / 10.96%</t>
+          <t>$43.10 / 11.30%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.99 / 11.47%</t>
+          <t>$43.06 / 0.25%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.18 / 0.32%</t>
+          <t>$42.32 / 0.65%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$763.43 / 7.50%</t>
+          <t>$767.85 / 8.13%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$763.43 / -0.30%</t>
+          <t>$767.85 / 0.28%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$763.43 / 12.17%</t>
+          <t>$767.85 / 12.82%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$763.43 / 10.73%</t>
+          <t>$767.85 / 11.37%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$763.43 / 10.38%</t>
+          <t>$767.85 / 11.02%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$763.43 / 2.71%</t>
+          <t>$767.85 / 3.30%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$763.43 / 2.23%</t>
+          <t>$767.85 / 2.83%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$763.43 / 17.71%</t>
+          <t>$767.85 / 18.39%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$763.43 / 3.28%</t>
+          <t>$767.85 / 3.88%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$763.43 / 15.84%</t>
+          <t>$767.85 / 16.51%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$763.43 / 14.91%</t>
+          <t>$767.85 / 0.60%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$763.43 / 0.23%</t>
+          <t>$767.85 / 0.81%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$763.43 / 7.50%</t>
+          <t>$767.85 / 8.13%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$764.07 / -0.22%</t>
+          <t>$767.85 / 0.28%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$764.07 / 12.27%</t>
+          <t>$767.85 / 12.82%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$763.43 / 10.73%</t>
+          <t>$767.85 / 11.37%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$763.43 / 10.38%</t>
+          <t>$767.85 / 11.02%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$764.07 / 2.80%</t>
+          <t>$767.85 / 3.30%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$764.07 / 2.32%</t>
+          <t>$767.85 / 2.83%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$763.43 / 17.71%</t>
+          <t>$767.85 / 18.39%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$763.43 / 3.28%</t>
+          <t>$767.85 / 3.88%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$764.07 / 15.94%</t>
+          <t>$767.85 / 16.51%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$764.07 / 15.00%</t>
+          <t>$767.85 / 0.60%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$764.07 / 0.31%</t>
+          <t>$767.85 / 0.81%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.50% (8.10%)</t>
+          <t>8.07% (7.68%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.70% (15.98%)</t>
+          <t>16.26% (15.55%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.73% (3.60%)</t>
+          <t>3.29% (3.16%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.77% (5.50%)</t>
+          <t>5.36% (5.10%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.98% (4.79%)</t>
+          <t>4.54% (4.35%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.91% (13.28%)</t>
+          <t>13.42% (12.81%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.65% (13.09%)</t>
+          <t>13.19% (12.64%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.93% (4.61%)</t>
+          <t>4.66% (4.35%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.95% (12.46%)</t>
+          <t>12.49% (12.01%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.24% (2.17%)</t>
+          <t>1.77% (1.70%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.14% (0.14%)</t>
+          <t>16.79% (15.95%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.41% (15.63%)</t>
+          <t>15.96% (15.19%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.70% (6.30%)</t>
+          <t>6.38% (5.99%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.27% (12.56%)</t>
+          <t>12.93% (12.22%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.68% (2.55%)</t>
+          <t>2.35% (2.22%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.38% (4.11%)</t>
+          <t>4.07% (3.81%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.67% (3.47%)</t>
+          <t>3.31% (3.12%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.14% (10.52%)</t>
+          <t>10.85% (10.24%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.74% (10.19%)</t>
+          <t>10.42% (9.87%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.17% (3.84%)</t>
+          <t>3.95% (3.62%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.06% (9.57%)</t>
+          <t>9.73% (9.25%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.37% (1.30%)</t>
+          <t>1.06% (1.00%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>-0.16% (-0.16%)</t>
+          <t>13.76% (12.92%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.66% (12.88%)</t>
+          <t>13.28% (12.51%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.51%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.52%</t>
+          <t>16.84%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.86%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.74%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.46%</t>
+          <t>-1.03%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
+          <t>12.72%</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0.09%</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>16.50%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>15.74%</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>3.90%</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>13.44%</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-0.65%</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>0.61%</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>0.72%</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>10.18%</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>10.24%</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>-3.62%</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>9.58%</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>-2.80%</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
           <t>13.37%</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0.67%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>0.16%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>16.41%</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>4.50%</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>14.00%</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>-0.16%</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>1.19%</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>1.30%</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>10.73%</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>10.78%</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>-3.06%</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>10.22%</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>-2.32%</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>-2.49%</t>
-        </is>
-      </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.17%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.44% (10.04%)</t>
+          <t>10.56% (10.16%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.31% (8.59%)</t>
+          <t>9.45% (8.74%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.08% (9.95%)</t>
+          <t>10.15% (10.03%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.62% (10.35%)</t>
+          <t>10.73% (10.47%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.05% (9.85%)</t>
+          <t>10.13% (9.95%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.85% (9.23%)</t>
+          <t>9.94% (9.32%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.52% (8.97%)</t>
+          <t>9.63% (9.09%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.03% (12.71%)</t>
+          <t>13.24% (12.93%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.27% (8.78%)</t>
+          <t>9.38% (8.90%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.88% (9.81%)</t>
+          <t>9.92% (9.86%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>8.59% (8.59%)</t>
+          <t>10.19% (9.35%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.97% (9.19%)</t>
+          <t>10.10% (9.32%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.87% (15.46%)</t>
+          <t>16.04% (15.64%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.38% (13.66%)</t>
+          <t>14.49% (13.79%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.83% (15.70%)</t>
+          <t>15.91% (15.78%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.33% (16.06%)</t>
+          <t>16.50% (16.24%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.64% (15.44%)</t>
+          <t>15.77% (15.58%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.93% (14.31%)</t>
+          <t>15.08% (14.47%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.59% (14.04%)</t>
+          <t>14.72% (14.17%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.03% (18.70%)</t>
+          <t>19.25% (18.92%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.35% (13.86%)</t>
+          <t>14.53% (14.05%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.12% (16.04%)</t>
+          <t>16.20% (16.13%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.04% (15.04%)</t>
+          <t>15.26% (14.42%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.90% (14.12%)</t>
+          <t>14.98% (14.21%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.84% (-6.24%)</t>
+          <t>-6.21% (-6.60%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.42% (-1.14%)</t>
+          <t>-0.80% (-1.51%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.68% (-9.82%)</t>
+          <t>-10.07% (-10.20%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.10% (-8.37%)</t>
+          <t>-8.46% (-8.72%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.41% (-8.61%)</t>
+          <t>-8.80% (-8.99%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.52% (-3.15%)</t>
+          <t>-2.94% (-3.56%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.44% (-3.00%)</t>
+          <t>-2.84% (-3.39%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.51% (-10.83%)</t>
+          <t>-10.74% (-11.06%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.59% (-4.08%)</t>
+          <t>-3.98% (-4.46%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.43% (-12.50%)</t>
+          <t>-12.83% (-12.90%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-13.09% (-13.09%)</t>
+          <t>-0.35% (-1.19%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.24% (-1.02%)</t>
+          <t>-0.63% (-1.40%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.06% (-5.47%)</t>
+          <t>-5.35% (-5.74%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.44% (-1.15%)</t>
+          <t>-0.74% (-1.45%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.45% (-8.59%)</t>
+          <t>-8.75% (-8.88%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.90% (-7.18%)</t>
+          <t>-7.18% (-7.44%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.35% (-7.54%)</t>
+          <t>-7.66% (-7.85%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.38% (-3.00%)</t>
+          <t>-2.63% (-3.25%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.33% (-2.89%)</t>
+          <t>-2.62% (-3.17%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.76% (-9.09%)</t>
+          <t>-8.96% (-9.28%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.35% (-3.84%)</t>
+          <t>-3.64% (-4.12%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.57% (-10.64%)</t>
+          <t>-10.84% (-10.91%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-11.05% (-11.05%)</t>
+          <t>-0.25% (-1.09%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.36% (-1.14%)</t>
+          <t>-0.70% (-1.47%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.28%</t>
+          <t>-16.76%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.73%</t>
+          <t>-10.25%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.77%</t>
+          <t>-20.23%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.72%</t>
+          <t>-19.19%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.46%</t>
+          <t>-18.93%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.37%</t>
+          <t>-12.88%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.97%</t>
+          <t>-12.47%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.54%</t>
+          <t>-23.98%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.86%</t>
+          <t>-13.36%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.31%</t>
+          <t>-22.75%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-21.68%</t>
+          <t>-10.54%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.20%</t>
+          <t>-10.72%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.93%</t>
+          <t>-21.39%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.81%</t>
+          <t>-15.23%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.28%</t>
+          <t>-24.66%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.24%</t>
+          <t>-23.68%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.99%</t>
+          <t>-23.43%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.31%</t>
+          <t>-17.72%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.93%</t>
+          <t>-17.33%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.79%</t>
+          <t>-28.20%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.70%</t>
+          <t>-18.17%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.68%</t>
+          <t>-27.04%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-26.09%</t>
+          <t>-15.51%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.26%</t>
+          <t>-15.68%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.26% (0.86%)</t>
+          <t>1.45% (1.06%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.42% (-1.14%)</t>
+          <t>-0.52% (-1.23%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.39% (1.25%)</t>
+          <t>1.54% (1.41%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.82% (1.55%)</t>
+          <t>2.01% (1.75%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.15% (0.96%)</t>
+          <t>1.31% (1.13%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.12% (-0.50%)</t>
+          <t>0.27% (-0.34%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.26% (-0.81%)</t>
+          <t>-0.09% (-0.63%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.93% (4.61%)</t>
+          <t>4.66% (4.35%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.41% (-0.90%)</t>
+          <t>-0.24% (-0.72%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.55% (1.48%)</t>
+          <t>1.67% (1.61%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.02%)</t>
+          <t>0.25% (-0.59%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>-0.01% (-0.79%)</t>
+          <t>0.18% (-0.59%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.09% (1.69%)</t>
+          <t>2.38% (1.98%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.44% (-1.15%)</t>
+          <t>-0.47% (-1.17%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.68% (2.55%)</t>
+          <t>2.35% (2.22%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.14% (2.87%)</t>
+          <t>3.44% (3.17%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.32% (2.13%)</t>
+          <t>2.57% (2.38%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.36% (-0.27%)</t>
+          <t>0.59% (-0.03%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.62%)</t>
+          <t>0.14% (-0.41%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.17% (3.84%)</t>
+          <t>3.95% (3.62%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.17% (-0.66%)</t>
+          <t>0.11% (-0.37%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.37% (1.30%)</t>
+          <t>1.06% (1.00%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>-0.16% (-0.16%)</t>
+          <t>0.35% (-0.49%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.07% (-0.85%)</t>
+          <t>0.09% (-0.68%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/10/2026</t>
+          <t>As of 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.49%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.38%</t>
+          <t>11.02%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.61%</t>
+          <t>-8.99%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>5.10%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.21%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.86%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.37%</t>
+          <t>-8.72%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>12.93%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.61%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.20%</t>
+          <t>11.48%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.71%</t>
+          <t>18.39%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.46%</t>
+          <t>-1.03%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.83%</t>
+          <t>-11.06%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>10.16%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.10%</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.75%</t>
+          <t>6.16%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>6.51%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.24%</t>
+          <t>-6.60%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>8.90%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>3.76%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.37%</t>
+          <t>12.72%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.08%</t>
+          <t>-4.46%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.97%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.09%</t>
+          <t>12.64%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.83%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.91%</t>
+          <t>13.25%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.28%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.37%</t>
+          <t>2.81%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.74%</t>
+          <t>13.08%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.15%</t>
+          <t>-3.56%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.52%</t>
+          <t>16.84%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-1.51%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>9.32%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.63%</t>
+          <t>15.19%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.56%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.41%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.02%</t>
+          <t>-1.40%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.14%</t>
+          <t>15.95%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.08%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14.91%</t>
+          <t>0.60%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>16.50%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-13.09%</t>
+          <t>-1.19%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.81%</t>
+          <t>9.86%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.32%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.50%</t>
+          <t>-12.90%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>10.03%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.60%</t>
+          <t>3.16%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.94%</t>
+          <t>10.42%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.17%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.82%</t>
+          <t>-10.20%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 16/10/2026</t>
+          <t>As of 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.44%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.47%</t>
+          <t>3.12%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.25%</t>
+          <t>7.61%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.38%</t>
+          <t>11.02%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.30%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.54%</t>
+          <t>-7.85%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>16.24%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.11%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>7.13%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.19%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.18%</t>
+          <t>-7.44%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.70%</t>
+          <t>18.92%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>9.29%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.71%</t>
+          <t>18.39%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-3.62%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.09%</t>
+          <t>-9.28%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.46%</t>
+          <t>15.64%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.30%</t>
+          <t>5.99%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.89%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>3.90%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.47%</t>
+          <t>-5.74%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.86%</t>
+          <t>14.05%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.57%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>3.40%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.28%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-4.12%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.04%</t>
+          <t>14.17%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>9.87%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.83%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.78%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.89%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.31%</t>
+          <t>14.47%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>10.24%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>3.30%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.73%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>-3.25%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>13.79%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.56%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.45%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.12%</t>
+          <t>14.21%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>12.51%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.81%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.73%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-1.47%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.04%</t>
+          <t>14.42%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>12.92%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.47%</t>
+          <t>0.25%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>0.60%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-2.49%</t>
+          <t>13.37%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-11.05%</t>
+          <t>-1.09%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.04%</t>
+          <t>16.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.30%</t>
+          <t>1.00%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>11.30%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.94%</t>
+          <t>16.51%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-2.80%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.64%</t>
+          <t>-10.91%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.70%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.55%</t>
+          <t>2.22%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>8.82%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.27%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>-0.65%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.59%</t>
+          <t>-8.88%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-20]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:54 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:54 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/19/2026 at 3:17 PM ET)</t>
+          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>270 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>179 days</t>
+          <t>178 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>305 days</t>
+          <t>304 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>60 days</t>
+          <t>59 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>123 days</t>
+          <t>122 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>88 days</t>
+          <t>87 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>270 days</t>
+          <t>269 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>241 days</t>
+          <t>240 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>151 days</t>
+          <t>150 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>214 days</t>
+          <t>213 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>32 days</t>
+          <t>31 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>361 days</t>
+          <t>360 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>333 days</t>
+          <t>332 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.06 / 6.16%</t>
+          <t>$48.15 / 6.36%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.92 / 0.67%</t>
+          <t>$58.03 / 0.86%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.32 / 10.42%</t>
+          <t>$56.41 / 10.59%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.91 / 8.63%</t>
+          <t>$63.01 / 8.79%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.94 / 8.94%</t>
+          <t>$56.98 / 9.02%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.53 / 2.81%</t>
+          <t>$61.64 / 2.99%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.45 / 2.63%</t>
+          <t>$61.55 / 2.80%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.86 / 11.48%</t>
+          <t>$53.92 / 11.60%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.66 / 3.76%</t>
+          <t>$57.78 / 3.98%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.61 / 13.83%</t>
+          <t>$60.71 / 14.01%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.81 / 0.34%</t>
+          <t>$54.90 / 0.50%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.40 / 0.56%</t>
+          <t>$57.50 / 0.73%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.76 / 5.20%</t>
+          <t>$42.80 / 5.31%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.27 / 0.61%</t>
+          <t>$42.31 / 0.72%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.01 / 8.82%</t>
+          <t>$41.06 / 8.95%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.23 / 7.13%</t>
+          <t>$45.30 / 7.28%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.33 / 7.61%</t>
+          <t>$46.39 / 7.76%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.73 / 2.48%</t>
+          <t>$44.79 / 2.61%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.14 / 2.40%</t>
+          <t>$42.19 / 2.53%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.39 / 9.29%</t>
+          <t>$45.44 / 9.40%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.09 / 3.40%</t>
+          <t>$44.17 / 3.59%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.10 / 11.30%</t>
+          <t>$43.15 / 11.43%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.06 / 0.25%</t>
+          <t>$43.10 / 0.34%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.32 / 0.65%</t>
+          <t>$42.35 / 0.73%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$767.85 / 8.13%</t>
+          <t>$769.96 / 8.42%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.28%</t>
+          <t>$769.96 / 0.55%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$767.85 / 12.82%</t>
+          <t>$769.96 / 13.13%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$767.85 / 11.37%</t>
+          <t>$769.77 / 11.65%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$767.85 / 11.02%</t>
+          <t>$769.77 / 11.29%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$767.85 / 3.30%</t>
+          <t>$769.96 / 3.59%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$767.85 / 2.83%</t>
+          <t>$769.96 / 3.11%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$767.85 / 18.39%</t>
+          <t>$769.96 / 18.72%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$767.85 / 3.88%</t>
+          <t>$769.96 / 4.16%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$767.85 / 16.51%</t>
+          <t>$769.96 / 16.83%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.60%</t>
+          <t>$769.96 / 0.88%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.81%</t>
+          <t>$769.96 / 1.09%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$767.85 / 8.13%</t>
+          <t>$769.96 / 8.42%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.28%</t>
+          <t>$769.96 / 0.55%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$767.85 / 12.82%</t>
+          <t>$769.96 / 13.13%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$767.85 / 11.37%</t>
+          <t>$769.96 / 11.68%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$767.85 / 11.02%</t>
+          <t>$769.96 / 11.32%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$767.85 / 3.30%</t>
+          <t>$769.96 / 3.59%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$767.85 / 2.83%</t>
+          <t>$769.96 / 3.11%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$767.85 / 18.39%</t>
+          <t>$769.96 / 18.72%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$767.85 / 3.88%</t>
+          <t>$769.96 / 4.16%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$767.85 / 16.51%</t>
+          <t>$769.96 / 16.83%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.60%</t>
+          <t>$769.96 / 0.88%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$767.85 / 0.81%</t>
+          <t>$769.96 / 1.09%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.07% (7.68%)</t>
+          <t>7.87% (7.48%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.26% (15.55%)</t>
+          <t>16.03% (15.33%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.29% (3.16%)</t>
+          <t>3.12% (2.99%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.36% (5.10%)</t>
+          <t>5.20% (4.94%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.54% (4.35%)</t>
+          <t>4.47% (4.28%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.42% (12.81%)</t>
+          <t>13.21% (12.60%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.19% (12.64%)</t>
+          <t>13.00% (12.46%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.66% (4.35%)</t>
+          <t>4.54% (4.23%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.49% (12.01%)</t>
+          <t>12.25% (11.78%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.77% (1.70%)</t>
+          <t>1.61% (1.54%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.79% (15.95%)</t>
+          <t>16.61% (15.77%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.96% (15.19%)</t>
+          <t>15.76% (14.99%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.38% (5.99%)</t>
+          <t>6.27% (5.88%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.93% (12.22%)</t>
+          <t>12.81% (12.10%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.35% (2.22%)</t>
+          <t>2.23% (2.10%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.07% (3.81%)</t>
+          <t>3.92% (3.66%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.31% (3.12%)</t>
+          <t>3.17% (2.98%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.85% (10.24%)</t>
+          <t>10.71% (10.10%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.42% (9.87%)</t>
+          <t>10.27% (9.73%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.95% (3.62%)</t>
+          <t>3.84% (3.52%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.73% (9.25%)</t>
+          <t>9.53% (9.05%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.06% (1.00%)</t>
+          <t>0.94% (0.88%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.76% (12.92%)</t>
+          <t>13.65% (12.82%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.28% (12.51%)</t>
+          <t>13.19% (12.42%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.51%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.84%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.03%</t>
+          <t>-1.30%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.72%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.09%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>16.18%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.43%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.90%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.93%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.62%</t>
+          <t>-3.89%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.80%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>13.37%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>12.87%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.56% (10.16%)</t>
+          <t>10.61% (10.22%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.45% (8.74%)</t>
+          <t>9.50% (8.80%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.15% (10.03%)</t>
+          <t>10.23% (10.10%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.73% (10.47%)</t>
+          <t>10.79% (10.53%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.13% (9.95%)</t>
+          <t>10.27% (10.08%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.94% (9.32%)</t>
+          <t>10.00% (9.39%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.63% (9.09%)</t>
+          <t>9.71% (9.17%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.24% (12.93%)</t>
+          <t>13.35% (13.03%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.38% (8.90%)</t>
+          <t>9.42% (8.94%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.92% (9.86%)</t>
+          <t>10.00% (9.93%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.19% (9.35%)</t>
+          <t>10.28% (9.44%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.10% (9.32%)</t>
+          <t>10.16% (9.40%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.04% (15.64%)</t>
+          <t>16.15% (15.76%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.49% (13.79%)</t>
+          <t>14.62% (13.92%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.91% (15.78%)</t>
+          <t>16.00% (15.87%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.50% (16.24%)</t>
+          <t>16.58% (16.31%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.77% (15.58%)</t>
+          <t>15.85% (15.66%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.08% (14.47%)</t>
+          <t>15.19% (14.58%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.72% (14.17%)</t>
+          <t>14.81% (14.27%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.25% (18.92%)</t>
+          <t>19.35% (19.03%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.53% (14.05%)</t>
+          <t>14.58% (14.10%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.20% (16.13%)</t>
+          <t>16.29% (16.23%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.26% (14.42%)</t>
+          <t>15.39% (14.56%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.98% (14.21%)</t>
+          <t>15.13% (14.36%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.21% (-6.60%)</t>
+          <t>-6.38% (-6.77%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.80% (-1.51%)</t>
+          <t>-0.99% (-1.69%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.07% (-10.20%)</t>
+          <t>-10.22% (-10.34%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.46% (-8.72%)</t>
+          <t>-8.60% (-8.86%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.80% (-8.99%)</t>
+          <t>-8.86% (-9.05%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.94% (-3.56%)</t>
+          <t>-3.12% (-3.73%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.84% (-3.39%)</t>
+          <t>-3.00% (-3.54%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.74% (-11.06%)</t>
+          <t>-10.84% (-11.15%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.98% (-4.46%)</t>
+          <t>-4.18% (-4.66%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.83% (-12.90%)</t>
+          <t>-12.97% (-13.03%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.35% (-1.19%)</t>
+          <t>-0.51% (-1.34%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.63% (-1.40%)</t>
+          <t>-0.80% (-1.57%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.35% (-5.74%)</t>
+          <t>-5.45% (-5.84%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.74% (-1.45%)</t>
+          <t>-0.85% (-1.55%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.75% (-8.88%)</t>
+          <t>-8.86% (-8.99%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.18% (-7.44%)</t>
+          <t>-7.31% (-7.58%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.66% (-7.85%)</t>
+          <t>-7.80% (-7.98%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.63% (-3.25%)</t>
+          <t>-2.76% (-3.37%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.62% (-3.17%)</t>
+          <t>-2.75% (-3.29%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.96% (-9.28%)</t>
+          <t>-9.05% (-9.37%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.64% (-4.12%)</t>
+          <t>-3.82% (-4.30%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.84% (-10.91%)</t>
+          <t>-10.95% (-11.01%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.25% (-1.09%)</t>
+          <t>-0.35% (-1.18%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.70% (-1.47%)</t>
+          <t>-0.78% (-1.55%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.76%</t>
+          <t>-16.99%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.25%</t>
+          <t>-10.49%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.23%</t>
+          <t>-20.45%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.19%</t>
+          <t>-19.39%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.93%</t>
+          <t>-19.13%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.88%</t>
+          <t>-13.12%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.47%</t>
+          <t>-12.71%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.98%</t>
+          <t>-24.19%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.36%</t>
+          <t>-13.60%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.75%</t>
+          <t>-22.97%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.54%</t>
+          <t>-10.78%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.72%</t>
+          <t>-10.97%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.39%</t>
+          <t>-21.60%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.23%</t>
+          <t>-15.47%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.66%</t>
+          <t>-24.86%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.68%</t>
+          <t>-23.89%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.43%</t>
+          <t>-23.64%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.72%</t>
+          <t>-17.94%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.33%</t>
+          <t>-17.56%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.20%</t>
+          <t>-28.40%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.17%</t>
+          <t>-18.40%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.04%</t>
+          <t>-27.24%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-15.51%</t>
+          <t>-15.74%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.68%</t>
+          <t>-15.91%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.45% (1.06%)</t>
+          <t>1.54% (1.15%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.52% (-1.23%)</t>
+          <t>-0.44% (-1.14%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.54% (1.41%)</t>
+          <t>1.65% (1.53%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.01% (1.75%)</t>
+          <t>2.11% (1.85%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.31% (1.13%)</t>
+          <t>1.50% (1.31%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.27% (-0.34%)</t>
+          <t>0.36% (-0.24%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.63%)</t>
+          <t>0.02% (-0.52%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.66% (4.35%)</t>
+          <t>4.54% (4.23%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.24% (-0.72%)</t>
+          <t>-0.18% (-0.65%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.67% (1.61%)</t>
+          <t>1.61% (1.54%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.25% (-0.59%)</t>
+          <t>0.37% (-0.47%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.18% (-0.59%)</t>
+          <t>0.28% (-0.49%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.38% (1.98%)</t>
+          <t>2.55% (2.15%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.47% (-1.17%)</t>
+          <t>-0.30% (-1.00%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.35% (2.22%)</t>
+          <t>2.23% (2.10%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.44% (3.17%)</t>
+          <t>3.57% (3.31%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.57% (2.38%)</t>
+          <t>2.71% (2.52%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.59% (-0.03%)</t>
+          <t>0.74% (0.13%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.14% (-0.41%)</t>
+          <t>0.28% (-0.26%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.95% (3.62%)</t>
+          <t>3.84% (3.52%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.11% (-0.37%)</t>
+          <t>0.20% (-0.28%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.06% (1.00%)</t>
+          <t>0.94% (0.88%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.35% (-0.49%)</t>
+          <t>0.53% (-0.31%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.09% (-0.68%)</t>
+          <t>0.28% (-0.49%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 19/10/2026</t>
+          <t>As of 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.02%</t>
+          <t>11.29%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.17%</t>
+          <t>2.91%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.99%</t>
+          <t>-9.05%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>10.53%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.10%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.37%</t>
+          <t>11.65%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.72%</t>
+          <t>-8.86%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.93%</t>
+          <t>13.03%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>4.23%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.48%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.39%</t>
+          <t>18.72%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.03%</t>
+          <t>-1.30%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.06%</t>
+          <t>-11.15%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.16%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>7.48%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.16%</t>
+          <t>6.36%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.51%</t>
+          <t>6.21%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.60%</t>
+          <t>-6.77%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.90%</t>
+          <t>8.94%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.01%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.98%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.72%</t>
+          <t>12.41%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-4.66%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.64%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.83%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.25%</t>
+          <t>12.94%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.39%</t>
+          <t>-3.54%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.39%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.81%</t>
+          <t>2.99%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.08%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.56%</t>
+          <t>-3.73%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.74%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>15.33%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.84%</t>
+          <t>16.52%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-1.69%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.32%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.19%</t>
+          <t>14.99%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.56%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.74%</t>
+          <t>15.43%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.40%</t>
+          <t>-1.57%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.35%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.95%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>16.18%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-1.34%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.86%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.09%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.90%</t>
+          <t>-13.03%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.03%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.16%</t>
+          <t>2.99%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.42%</t>
+          <t>10.59%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>1.43%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.20%</t>
+          <t>-10.34%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 19/10/2026</t>
+          <t>As of 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>15.66%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.12%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.61%</t>
+          <t>7.76%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.02%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.85%</t>
+          <t>-7.98%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.13%</t>
+          <t>7.28%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.37%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.44%</t>
+          <t>-7.58%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.92%</t>
+          <t>19.03%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.52%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.29%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.39%</t>
+          <t>18.72%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.62%</t>
+          <t>-3.89%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.28%</t>
+          <t>-9.37%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.64%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.99%</t>
+          <t>5.88%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>5.31%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>8.42%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.90%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.74%</t>
+          <t>-5.84%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.05%</t>
+          <t>14.10%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.40%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.88%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.28%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.12%</t>
+          <t>-4.30%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.17%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.87%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.83%</t>
+          <t>3.11%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-3.29%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.47%</t>
+          <t>14.58%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.30%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.25%</t>
+          <t>-3.37%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.79%</t>
+          <t>13.92%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.22%</t>
+          <t>12.10%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.45%</t>
+          <t>-1.55%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.21%</t>
+          <t>14.36%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.51%</t>
+          <t>12.42%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.81%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>12.87%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.47%</t>
+          <t>-1.55%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.42%</t>
+          <t>14.56%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.92%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.25%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.37%</t>
+          <t>13.06%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-1.18%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.13%</t>
+          <t>16.23%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>0.88%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.30%</t>
+          <t>11.43%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.51%</t>
+          <t>16.83%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.80%</t>
+          <t>-3.06%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.91%</t>
+          <t>-11.01%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>2.10%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.82%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.65%</t>
+          <t>-0.93%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.88%</t>
+          <t>-8.99%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-21]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:54 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:54 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/20/2026 at 1:55 PM ET)</t>
+          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>178 days</t>
+          <t>177 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>304 days</t>
+          <t>303 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>59 days</t>
+          <t>58 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>122 days</t>
+          <t>121 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>87 days</t>
+          <t>86 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>269 days</t>
+          <t>268 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>240 days</t>
+          <t>239 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>150 days</t>
+          <t>149 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>213 days</t>
+          <t>212 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>31 days</t>
+          <t>30 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>360 days</t>
+          <t>359 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>332 days</t>
+          <t>331 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.15 / 6.36%</t>
+          <t>$48.28 / 6.64%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.03 / 0.86%</t>
+          <t>$58.23 / 1.22%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.41 / 10.59%</t>
+          <t>$56.56 / 10.89%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.01 / 8.79%</t>
+          <t>$63.17 / 9.07%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.98 / 9.02%</t>
+          <t>$57.19 / 9.41%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.64 / 2.99%</t>
+          <t>$61.83 / 3.32%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.55 / 2.80%</t>
+          <t>$61.76 / 3.15%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.92 / 11.60%</t>
+          <t>$54.01 / 11.78%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.78 / 3.98%</t>
+          <t>$57.97 / 4.32%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.71 / 14.01%</t>
+          <t>$60.82 / 14.23%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.90 / 0.50%</t>
+          <t>$55.09 / 0.86%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.50 / 0.73%</t>
+          <t>$57.70 / 1.09%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.80 / 5.31%</t>
+          <t>$42.91 / 5.56%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.31 / 0.72%</t>
+          <t>$42.44 / 1.01%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.06 / 8.95%</t>
+          <t>$41.14 / 9.16%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.30 / 7.28%</t>
+          <t>$45.35 / 7.40%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.39 / 7.76%</t>
+          <t>$46.46 / 7.92%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.79 / 2.61%</t>
+          <t>$44.91 / 2.89%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.19 / 2.53%</t>
+          <t>$42.31 / 2.81%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.44 / 9.40%</t>
+          <t>$45.50 / 9.55%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.17 / 3.59%</t>
+          <t>$44.29 / 3.87%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.15 / 11.43%</t>
+          <t>$43.20 / 11.56%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.10 / 0.34%</t>
+          <t>$43.23 / 0.64%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.35 / 0.73%</t>
+          <t>$42.46 / 0.99%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$769.96 / 8.42%</t>
+          <t>$773.70 / 8.95%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$769.96 / 0.55%</t>
+          <t>$773.70 / 1.04%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$769.96 / 13.13%</t>
+          <t>$773.70 / 13.68%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$769.77 / 11.65%</t>
+          <t>$773.70 / 12.22%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$769.77 / 11.29%</t>
+          <t>$773.70 / 11.86%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$769.96 / 3.59%</t>
+          <t>$773.70 / 4.09%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$769.96 / 3.11%</t>
+          <t>$773.70 / 3.61%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$769.96 / 18.72%</t>
+          <t>$773.70 / 19.29%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$769.96 / 4.16%</t>
+          <t>$773.70 / 4.67%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$769.96 / 16.83%</t>
+          <t>$773.70 / 17.40%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$769.96 / 0.88%</t>
+          <t>$773.70 / 1.37%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$769.96 / 1.09%</t>
+          <t>$773.70 / 1.58%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$769.96 / 8.42%</t>
+          <t>$773.58 / 8.93%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$769.96 / 0.55%</t>
+          <t>$773.58 / 1.03%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$769.96 / 13.13%</t>
+          <t>$773.58 / 13.66%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$769.96 / 11.68%</t>
+          <t>$773.70 / 12.22%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$769.96 / 11.32%</t>
+          <t>$773.70 / 11.86%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$769.96 / 3.59%</t>
+          <t>$773.58 / 4.08%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$769.96 / 3.11%</t>
+          <t>$773.58 / 3.59%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$769.96 / 18.72%</t>
+          <t>$773.58 / 19.27%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$769.96 / 4.16%</t>
+          <t>$773.58 / 4.66%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$769.96 / 16.83%</t>
+          <t>$773.58 / 17.38%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$769.96 / 0.88%</t>
+          <t>$773.58 / 1.35%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$769.96 / 1.09%</t>
+          <t>$773.58 / 1.56%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.87% (7.48%)</t>
+          <t>7.58% (7.19%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.03% (15.33%)</t>
+          <t>15.62% (14.93%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.12% (2.99%)</t>
+          <t>2.84% (2.72%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.20% (4.94%)</t>
+          <t>4.93% (4.67%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.47% (4.28%)</t>
+          <t>4.09% (3.91%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.21% (12.60%)</t>
+          <t>12.85% (12.25%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.00% (12.46%)</t>
+          <t>12.62% (12.08%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.54% (4.23%)</t>
+          <t>4.38% (4.07%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.25% (11.78%)</t>
+          <t>11.88% (11.41%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.61% (1.54%)</t>
+          <t>1.41% (1.35%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.61% (15.77%)</t>
+          <t>16.19% (15.36%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.76% (14.99%)</t>
+          <t>15.34% (14.58%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.27% (5.88%)</t>
+          <t>6.01% (5.62%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.81% (12.10%)</t>
+          <t>12.47% (11.77%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.23% (2.10%)</t>
+          <t>2.03% (1.90%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.92% (3.66%)</t>
+          <t>3.80% (3.54%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.17% (2.98%)</t>
+          <t>3.01% (2.82%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.71% (10.10%)</t>
+          <t>10.40% (9.80%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.27% (9.73%)</t>
+          <t>9.97% (9.43%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.84% (3.52%)</t>
+          <t>3.70% (3.38%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.53% (9.05%)</t>
+          <t>9.23% (8.76%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.94% (0.88%)</t>
+          <t>0.82% (0.76%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.65% (12.82%)</t>
+          <t>13.31% (12.48%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.19% (12.42%)</t>
+          <t>12.89% (12.13%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>15.96%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>12.23%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>11.86%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>16.18%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.43%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.93%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>-0.15%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.89%</t>
+          <t>-4.34%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-3.52%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.87%</t>
+          <t>12.34%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.61% (10.22%)</t>
+          <t>10.75% (10.37%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.50% (8.80%)</t>
+          <t>9.59% (8.89%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.23% (10.10%)</t>
+          <t>10.37% (10.25%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.79% (10.53%)</t>
+          <t>10.97% (10.71%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.27% (10.08%)</t>
+          <t>10.35% (10.17%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.00% (9.39%)</t>
+          <t>10.11% (9.51%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.71% (9.17%)</t>
+          <t>9.80% (9.26%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.35% (13.03%)</t>
+          <t>13.57% (13.26%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.42% (8.94%)</t>
+          <t>9.52% (9.05%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.00% (9.93%)</t>
+          <t>10.20% (10.14%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.28% (9.44%)</t>
+          <t>10.35% (9.52%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.16% (9.40%)</t>
+          <t>10.24% (9.48%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.15% (15.76%)</t>
+          <t>16.29% (15.90%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.62% (13.92%)</t>
+          <t>14.72% (14.02%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.00% (15.87%)</t>
+          <t>16.17% (16.05%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.58% (16.31%)</t>
+          <t>16.84% (16.58%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.85% (15.66%)</t>
+          <t>16.07% (15.89%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.19% (14.58%)</t>
+          <t>15.30% (14.69%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.81% (14.27%)</t>
+          <t>14.93% (14.39%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.35% (19.03%)</t>
+          <t>19.56% (19.25%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.58% (14.10%)</t>
+          <t>14.70% (14.22%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.29% (16.23%)</t>
+          <t>16.53% (16.47%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.39% (14.56%)</t>
+          <t>15.49% (14.65%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.13% (14.36%)</t>
+          <t>15.26% (14.50%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.38% (-6.77%)</t>
+          <t>-6.64% (-7.02%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.99% (-1.69%)</t>
+          <t>-1.34% (-2.04%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.22% (-10.34%)</t>
+          <t>-10.46% (-10.58%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.60% (-8.86%)</t>
+          <t>-8.83% (-9.09%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.86% (-9.05%)</t>
+          <t>-9.19% (-9.38%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.12% (-3.73%)</t>
+          <t>-3.43% (-4.03%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.00% (-3.54%)</t>
+          <t>-3.33% (-3.87%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.84% (-11.15%)</t>
+          <t>-10.98% (-11.29%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.18% (-4.66%)</t>
+          <t>-4.50% (-4.97%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.97% (-13.03%)</t>
+          <t>-13.14% (-13.20%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.51% (-1.34%)</t>
+          <t>-0.86% (-1.69%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.80% (-1.57%)</t>
+          <t>-1.16% (-1.92%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.45% (-5.84%)</t>
+          <t>-5.68% (-6.07%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.85% (-1.55%)</t>
+          <t>-1.14% (-1.84%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.86% (-8.99%)</t>
+          <t>-9.04% (-9.17%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.31% (-7.58%)</t>
+          <t>-7.42% (-7.68%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.80% (-7.98%)</t>
+          <t>-7.94% (-8.12%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.76% (-3.37%)</t>
+          <t>-3.03% (-3.63%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.75% (-3.29%)</t>
+          <t>-3.01% (-3.55%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.05% (-9.37%)</t>
+          <t>-9.17% (-9.49%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.82% (-4.30%)</t>
+          <t>-4.08% (-4.56%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.95% (-11.01%)</t>
+          <t>-11.05% (-11.12%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.35% (-1.18%)</t>
+          <t>-0.65% (-1.48%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.78% (-1.55%)</t>
+          <t>-1.04% (-1.80%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.99%</t>
+          <t>-17.39%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.49%</t>
+          <t>-10.93%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.45%</t>
+          <t>-20.83%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.39%</t>
+          <t>-19.80%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.13%</t>
+          <t>-19.54%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.12%</t>
+          <t>-13.54%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.71%</t>
+          <t>-13.14%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.19%</t>
+          <t>-24.56%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.60%</t>
+          <t>-14.02%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.97%</t>
+          <t>-23.34%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.78%</t>
+          <t>-11.21%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.97%</t>
+          <t>-11.40%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.60%</t>
+          <t>-21.97%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.47%</t>
+          <t>-15.86%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.86%</t>
+          <t>-25.22%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.89%</t>
+          <t>-24.25%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.64%</t>
+          <t>-24.01%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.94%</t>
+          <t>-18.33%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.56%</t>
+          <t>-17.95%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.40%</t>
+          <t>-28.73%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.40%</t>
+          <t>-18.78%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.24%</t>
+          <t>-27.58%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-15.74%</t>
+          <t>-16.14%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.91%</t>
+          <t>-16.31%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.54% (1.15%)</t>
+          <t>1.75% (1.37%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.44% (-1.14%)</t>
+          <t>-0.31% (-1.01%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.65% (1.53%)</t>
+          <t>1.88% (1.76%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.11% (1.85%)</t>
+          <t>2.37% (2.12%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.50% (1.31%)</t>
+          <t>1.65% (1.47%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.36% (-0.24%)</t>
+          <t>0.53% (-0.07%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.02% (-0.52%)</t>
+          <t>0.17% (-0.37%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.54% (4.23%)</t>
+          <t>4.38% (4.07%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.18% (-0.65%)</t>
+          <t>-0.02% (-0.49%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.61% (1.54%)</t>
+          <t>1.41% (1.35%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.37% (-0.47%)</t>
+          <t>0.50% (-0.33%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.28% (-0.49%)</t>
+          <t>0.40% (-0.36%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.55% (2.15%)</t>
+          <t>2.78% (2.39%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.30% (-1.00%)</t>
+          <t>-0.13% (-0.83%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.23% (2.10%)</t>
+          <t>2.03% (1.90%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.57% (3.31%)</t>
+          <t>3.80% (3.54%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.71% (2.52%)</t>
+          <t>3.01% (2.82%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.74% (0.13%)</t>
+          <t>0.93% (0.32%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.28% (-0.26%)</t>
+          <t>0.48% (-0.06%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.84% (3.52%)</t>
+          <t>3.70% (3.38%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.20% (-0.28%)</t>
+          <t>0.40% (-0.08%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.94% (0.88%)</t>
+          <t>0.82% (0.76%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.53% (-0.31%)</t>
+          <t>0.69% (-0.14%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.28% (-0.49%)</t>
+          <t>0.48% (-0.28%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 20/10/2026</t>
+          <t>As of 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>9.41%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.29%</t>
+          <t>11.86%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.91%</t>
+          <t>2.39%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.05%</t>
+          <t>-9.38%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.53%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.67%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>9.07%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.65%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.01%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.86%</t>
+          <t>-9.09%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.03%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.23%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.78%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.72%</t>
+          <t>19.29%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>-1.78%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.15%</t>
+          <t>-11.29%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.22%</t>
+          <t>10.37%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.48%</t>
+          <t>7.19%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.36%</t>
+          <t>6.64%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.42%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.21%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.77%</t>
+          <t>-7.02%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.94%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.98%</t>
+          <t>4.32%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.16%</t>
+          <t>4.67%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.41%</t>
+          <t>11.86%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.66%</t>
+          <t>-4.97%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.26%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.61%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.94%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.54%</t>
+          <t>-3.87%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.39%</t>
+          <t>9.51%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>12.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-4.03%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>8.89%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.33%</t>
+          <t>14.93%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.52%</t>
+          <t>15.96%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-2.04%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.48%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.99%</t>
+          <t>14.58%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.43%</t>
+          <t>14.87%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.57%</t>
+          <t>-1.92%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.52%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.36%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.37%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>16.18%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.34%</t>
+          <t>-1.69%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.14%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.54%</t>
+          <t>1.35%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>14.23%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.83%</t>
+          <t>17.40%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.03%</t>
+          <t>-13.20%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>10.25%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.59%</t>
+          <t>10.89%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.68%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.34%</t>
+          <t>-10.58%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 20/10/2026</t>
+          <t>As of 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.66%</t>
+          <t>15.89%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.76%</t>
+          <t>7.92%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>11.86%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.98%</t>
+          <t>-8.12%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.31%</t>
+          <t>16.58%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.28%</t>
+          <t>7.40%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>12.22%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>-0.15%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.58%</t>
+          <t>-7.68%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.03%</t>
+          <t>19.25%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.55%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.72%</t>
+          <t>19.27%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.89%</t>
+          <t>-4.34%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.37%</t>
+          <t>-9.49%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.90%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.88%</t>
+          <t>5.62%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.31%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.42%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.62%</t>
+          <t>3.13%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.84%</t>
+          <t>-6.07%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.10%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>8.76%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>3.87%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.16%</t>
+          <t>4.66%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.30%</t>
+          <t>-4.56%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.39%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.81%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.11%</t>
+          <t>3.59%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.55%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.58%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>2.89%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>4.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.37%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-3.63%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.92%</t>
+          <t>14.02%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.10%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.55%</t>
+          <t>-1.84%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.36%</t>
+          <t>14.50%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.42%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.99%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.87%</t>
+          <t>12.34%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.55%</t>
+          <t>-1.80%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.56%</t>
+          <t>14.65%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.48%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.35%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-1.48%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>16.47%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.43%</t>
+          <t>11.56%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.83%</t>
+          <t>17.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.06%</t>
+          <t>-3.52%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.01%</t>
+          <t>-11.12%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.87%</t>
+          <t>16.05%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.10%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>13.66%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.93%</t>
+          <t>-1.39%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.99%</t>
+          <t>-9.17%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-22]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:01 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/21/2026 at 2:02 PM ET)</t>
+          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>177 days</t>
+          <t>176 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>303 days</t>
+          <t>302 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>58 days</t>
+          <t>57 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>121 days</t>
+          <t>120 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>86 days</t>
+          <t>85 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>268 days</t>
+          <t>267 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>239 days</t>
+          <t>238 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>149 days</t>
+          <t>148 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>212 days</t>
+          <t>211 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>29 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>359 days</t>
+          <t>358 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>331 days</t>
+          <t>330 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.28 / 6.64%</t>
+          <t>$47.91 / 5.83%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.23 / 1.22%</t>
+          <t>$57.70 / 0.29%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.56 / 10.89%</t>
+          <t>$56.11 / 10.00%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.17 / 9.07%</t>
+          <t>$62.72 / 8.30%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.19 / 9.41%</t>
+          <t>$56.73 / 8.54%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.83 / 3.32%</t>
+          <t>$61.28 / 2.40%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.76 / 3.15%</t>
+          <t>$61.20 / 2.21%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$54.01 / 11.78%</t>
+          <t>$53.75 / 11.25%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.97 / 4.32%</t>
+          <t>$57.41 / 3.32%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.82 / 14.23%</t>
+          <t>$60.42 / 13.47%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$55.09 / 0.86%</t>
+          <t>$54.62 / 0.00%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.70 / 1.09%</t>
+          <t>$57.19 / 0.20%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.91 / 5.56%</t>
+          <t>$42.65 / 4.94%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.44 / 1.01%</t>
+          <t>$42.15 / 0.34%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.14 / 9.16%</t>
+          <t>$40.93 / 8.60%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.35 / 7.40%</t>
+          <t>$45.14 / 6.92%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.46 / 7.92%</t>
+          <t>$46.22 / 7.35%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.91 / 2.89%</t>
+          <t>$44.62 / 2.23%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.31 / 2.81%</t>
+          <t>$42.01 / 2.09%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.50 / 9.55%</t>
+          <t>$45.34 / 9.17%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.29 / 3.87%</t>
+          <t>$43.98 / 3.14%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.20 / 11.56%</t>
+          <t>$43.05 / 11.18%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.23 / 0.64%</t>
+          <t>$42.96 / 0.03%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.46 / 0.99%</t>
+          <t>$42.18 / 0.33%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$773.70 / 8.95%</t>
+          <t>$762.98 / 7.44%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$773.70 / 1.04%</t>
+          <t>$762.98 / -0.36%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$773.70 / 13.68%</t>
+          <t>$762.98 / 12.11%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$773.70 / 12.22%</t>
+          <t>$762.98 / 10.67%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$773.70 / 11.86%</t>
+          <t>$762.98 / 10.31%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$773.70 / 4.09%</t>
+          <t>$762.98 / 2.65%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$773.70 / 3.61%</t>
+          <t>$762.98 / 2.17%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$773.70 / 19.29%</t>
+          <t>$762.98 / 17.64%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$773.70 / 4.67%</t>
+          <t>$762.98 / 3.22%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$773.70 / 17.40%</t>
+          <t>$762.98 / 15.77%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$773.70 / 1.37%</t>
+          <t>$762.98 / -0.04%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$773.70 / 1.58%</t>
+          <t>$762.98 / 0.17%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$773.58 / 8.93%</t>
+          <t>$762.98 / 7.44%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$773.58 / 1.03%</t>
+          <t>$762.98 / -0.36%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$773.58 / 13.66%</t>
+          <t>$762.98 / 12.11%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$773.70 / 12.22%</t>
+          <t>$762.98 / 10.67%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$773.70 / 11.86%</t>
+          <t>$762.98 / 10.31%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.08%</t>
+          <t>$762.98 / 2.65%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$773.58 / 3.59%</t>
+          <t>$762.98 / 2.17%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$773.58 / 19.27%</t>
+          <t>$762.98 / 17.64%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$773.58 / 4.66%</t>
+          <t>$762.98 / 3.22%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$773.58 / 17.38%</t>
+          <t>$762.98 / 15.77%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$773.58 / 1.35%</t>
+          <t>$762.98 / -0.04%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$773.58 / 1.56%</t>
+          <t>$762.98 / 0.17%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.58% (7.19%)</t>
+          <t>8.41% (8.02%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.62% (14.93%)</t>
+          <t>16.68% (15.98%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.84% (2.72%)</t>
+          <t>3.67% (3.54%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.93% (4.67%)</t>
+          <t>5.67% (5.41%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.09% (3.91%)</t>
+          <t>4.92% (4.74%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.85% (12.25%)</t>
+          <t>13.86% (13.26%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.62% (12.08%)</t>
+          <t>13.64% (13.10%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.38% (4.07%)</t>
+          <t>4.87% (4.56%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>11.88% (11.41%)</t>
+          <t>12.96% (12.49%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.41% (1.35%)</t>
+          <t>2.09% (2.03%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.19% (15.36%)</t>
+          <t>17.19% (16.36%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.34% (14.58%)</t>
+          <t>16.37% (15.60%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.01% (5.62%)</t>
+          <t>6.64% (6.25%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.47% (11.77%)</t>
+          <t>13.23% (12.53%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.03% (1.90%)</t>
+          <t>2.55% (2.42%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.80% (3.54%)</t>
+          <t>4.27% (4.01%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.01% (2.82%)</t>
+          <t>3.55% (3.37%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.40% (9.80%)</t>
+          <t>11.12% (10.51%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.97% (9.43%)</t>
+          <t>10.74% (10.20%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.70% (3.38%)</t>
+          <t>4.05% (3.74%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.23% (8.76%)</t>
+          <t>10.00% (9.52%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.82% (0.76%)</t>
+          <t>1.16% (1.10%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.31% (12.48%)</t>
+          <t>14.01% (13.17%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.89% (12.13%)</t>
+          <t>13.64% (12.87%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.70%</t>
+          <t>7.18%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15.96%</t>
+          <t>17.59%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>3.92%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>13.81%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11.86%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>16.48%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>10.94%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-3.01%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-2.18%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>13.90%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.75% (10.37%)</t>
+          <t>10.31% (9.93%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.59% (8.89%)</t>
+          <t>9.24% (8.54%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.37% (10.25%)</t>
+          <t>9.97% (9.85%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.97% (10.71%)</t>
+          <t>10.49% (10.23%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.35% (10.17%)</t>
+          <t>9.95% (9.77%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.11% (9.51%)</t>
+          <t>9.76% (9.15%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.80% (9.26%)</t>
+          <t>9.47% (8.92%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.57% (13.26%)</t>
+          <t>12.93% (12.62%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.52% (9.05%)</t>
+          <t>9.23% (8.76%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10.20% (10.14%)</t>
+          <t>9.70% (9.65%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.35% (9.52%)</t>
+          <t>9.96% (9.12%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.24% (9.48%)</t>
+          <t>9.88% (9.11%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.29% (15.90%)</t>
+          <t>15.76% (15.37%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.72% (14.02%)</t>
+          <t>14.22% (13.52%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>16.17% (16.05%)</t>
+          <t>15.60% (15.48%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.84% (16.58%)</t>
+          <t>16.19% (15.93%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>16.07% (15.89%)</t>
+          <t>15.49% (15.31%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.30% (14.69%)</t>
+          <t>14.79% (14.18%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.93% (14.39%)</t>
+          <t>14.47% (13.93%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.56% (19.25%)</t>
+          <t>18.88% (18.57%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.70% (14.22%)</t>
+          <t>14.24% (13.77%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.53% (16.47%)</t>
+          <t>15.82% (15.76%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.49% (14.65%)</t>
+          <t>14.93% (14.10%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.26% (14.50%)</t>
+          <t>14.76% (13.99%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.64% (-7.02%)</t>
+          <t>-5.92% (-6.31%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.34% (-2.04%)</t>
+          <t>-0.44% (-1.14%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.46% (-10.58%)</t>
+          <t>-9.74% (-9.86%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.83% (-9.09%)</t>
+          <t>-8.19% (-8.45%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.19% (-9.38%)</t>
+          <t>-8.47% (-8.65%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.43% (-4.03%)</t>
+          <t>-2.56% (-3.17%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.33% (-3.87%)</t>
+          <t>-2.45% (-2.99%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.98% (-11.29%)</t>
+          <t>-10.56% (-10.87%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.50% (-4.97%)</t>
+          <t>-3.58% (-4.05%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.14% (-13.20%)</t>
+          <t>-12.56% (-12.62%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.86% (-1.69%)</t>
+          <t>-0.01% (-0.84%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.16% (-1.92%)</t>
+          <t>-0.28% (-1.04%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.68% (-6.07%)</t>
+          <t>-5.12% (-5.51%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.14% (-1.84%)</t>
+          <t>-0.48% (-1.18%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-9.04% (-9.17%)</t>
+          <t>-8.58% (-8.70%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.42% (-7.68%)</t>
+          <t>-7.00% (-7.26%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.94% (-8.12%)</t>
+          <t>-7.45% (-7.63%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-3.03% (-3.63%)</t>
+          <t>-2.40% (-3.01%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-3.01% (-3.55%)</t>
+          <t>-2.33% (-2.88%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.17% (-9.49%)</t>
+          <t>-8.86% (-9.18%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-4.08% (-4.56%)</t>
+          <t>-3.41% (-3.88%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-11.05% (-11.12%)</t>
+          <t>-10.76% (-10.82%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.65% (-1.48%)</t>
+          <t>-0.04% (-0.87%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.04% (-1.80%)</t>
+          <t>-0.39% (-1.15%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.39%</t>
+          <t>-16.23%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.93%</t>
+          <t>-9.68%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.83%</t>
+          <t>-19.72%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.80%</t>
+          <t>-18.68%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.54%</t>
+          <t>-18.41%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.54%</t>
+          <t>-12.32%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-13.14%</t>
+          <t>-11.92%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.56%</t>
+          <t>-23.50%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-14.02%</t>
+          <t>-12.81%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.34%</t>
+          <t>-22.26%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-11.21%</t>
+          <t>-9.97%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.40%</t>
+          <t>-10.15%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.97%</t>
+          <t>-20.88%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.86%</t>
+          <t>-14.69%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-25.22%</t>
+          <t>-24.18%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-24.25%</t>
+          <t>-23.19%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-24.01%</t>
+          <t>-22.94%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-18.33%</t>
+          <t>-17.19%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.95%</t>
+          <t>-16.81%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.73%</t>
+          <t>-27.74%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.78%</t>
+          <t>-17.65%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.58%</t>
+          <t>-26.58%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-16.14%</t>
+          <t>-14.97%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-16.31%</t>
+          <t>-15.14%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.75% (1.37%)</t>
+          <t>1.11% (0.72%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.31% (-1.01%)</t>
+          <t>-0.44% (-1.14%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.88% (1.76%)</t>
+          <t>1.26% (1.14%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.37% (2.12%)</t>
+          <t>1.66% (1.41%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.65% (1.47%)</t>
+          <t>1.03% (0.85%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.53% (-0.07%)</t>
+          <t>0.02% (-0.58%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.17% (-0.37%)</t>
+          <t>-0.32% (-0.86%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.38% (4.07%)</t>
+          <t>4.87% (4.56%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.02% (-0.49%)</t>
+          <t>-0.46% (-0.93%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.41% (1.35%)</t>
+          <t>1.34% (1.29%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.50% (-0.33%)</t>
+          <t>-0.01% (-0.84%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.40% (-0.36%)</t>
+          <t>-0.11% (-0.87%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.78% (2.39%)</t>
+          <t>1.97% (1.58%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.13% (-0.83%)</t>
+          <t>-0.48% (-1.18%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.03% (1.90%)</t>
+          <t>2.55% (2.42%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.80% (3.54%)</t>
+          <t>2.98% (2.72%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>3.01% (2.82%)</t>
+          <t>2.15% (1.97%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.93% (0.32%)</t>
+          <t>0.19% (-0.42%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.48% (-0.06%)</t>
+          <t>-0.21% (-0.75%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.70% (3.38%)</t>
+          <t>4.05% (3.74%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.40% (-0.08%)</t>
+          <t>-0.29% (-0.76%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.82% (0.76%)</t>
+          <t>1.16% (1.10%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.69% (-0.14%)</t>
+          <t>-0.04% (-0.87%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.48% (-0.28%)</t>
+          <t>-0.24% (-1.00%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/10/2026</t>
+          <t>As of 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.17%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.74%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.41%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.86%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.38%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.07%</t>
+          <t>8.30%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.22%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.48%</t>
+          <t>3.92%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.09%</t>
+          <t>-8.45%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>12.62%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.07%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.78%</t>
+          <t>11.25%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.29%</t>
+          <t>17.64%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.78%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.29%</t>
+          <t>-10.87%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.19%</t>
+          <t>8.02%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.64%</t>
+          <t>5.83%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.95%</t>
+          <t>7.44%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.70%</t>
+          <t>7.18%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-7.02%</t>
+          <t>-6.31%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>8.76%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.32%</t>
+          <t>3.32%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.86%</t>
+          <t>13.44%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.97%</t>
+          <t>-4.05%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>8.92%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.08%</t>
+          <t>13.10%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.15%</t>
+          <t>2.21%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.61%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>13.97%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.87%</t>
+          <t>-2.99%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.51%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.25%</t>
+          <t>13.26%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>2.40%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>13.81%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-4.03%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.89%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14.93%</t>
+          <t>15.98%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15.96%</t>
+          <t>17.59%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-1.14%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.48%</t>
+          <t>9.11%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.58%</t>
+          <t>15.60%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.87%</t>
+          <t>16.48%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.92%</t>
+          <t>-1.04%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.52%</t>
+          <t>9.12%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.36%</t>
+          <t>16.36%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.37%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.69%</t>
+          <t>-0.84%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10.14%</t>
+          <t>9.65%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.35%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.23%</t>
+          <t>13.47%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.40%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.20%</t>
+          <t>-12.62%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.89%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.68%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.58%</t>
+          <t>-9.86%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 21/10/2026</t>
+          <t>As of 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.89%</t>
+          <t>15.31%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>3.37%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.92%</t>
+          <t>7.35%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.86%</t>
+          <t>10.31%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.12%</t>
+          <t>-7.63%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.58%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>4.01%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.40%</t>
+          <t>6.92%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.22%</t>
+          <t>10.67%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.68%</t>
+          <t>-7.26%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.25%</t>
+          <t>18.57%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.55%</t>
+          <t>9.17%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.27%</t>
+          <t>17.64%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-3.01%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.49%</t>
+          <t>-9.18%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>15.37%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.62%</t>
+          <t>6.25%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.56%</t>
+          <t>4.94%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>7.44%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.13%</t>
+          <t>4.56%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.07%</t>
+          <t>-5.51%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.76%</t>
+          <t>9.52%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.87%</t>
+          <t>3.14%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.66%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.56%</t>
+          <t>-3.88%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.39%</t>
+          <t>13.93%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.81%</t>
+          <t>2.09%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.59%</t>
+          <t>2.17%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.42%</t>
+          <t>10.94%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.55%</t>
+          <t>-2.88%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.69%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.89%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.08%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.37%</t>
+          <t>10.88%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.63%</t>
+          <t>-3.01%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14.02%</t>
+          <t>13.52%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.77%</t>
+          <t>12.53%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.84%</t>
+          <t>-1.18%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.50%</t>
+          <t>13.99%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>12.87%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.99%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.56%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.34%</t>
+          <t>13.90%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.65%</t>
+          <t>14.10%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.48%</t>
+          <t>13.17%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.03%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.35%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>14.09%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.48%</t>
+          <t>-0.87%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.47%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.56%</t>
+          <t>11.18%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.38%</t>
+          <t>15.77%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.52%</t>
+          <t>-2.18%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.12%</t>
+          <t>-10.82%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16.05%</t>
+          <t>15.48%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.90%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.16%</t>
+          <t>8.60%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.66%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.39%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.17%</t>
+          <t>-8.70%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-23]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/22/2026 at 1:56 PM ET)</t>
+          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>237 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>176 days</t>
+          <t>175 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>302 days</t>
+          <t>301 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>57 days</t>
+          <t>56 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>120 days</t>
+          <t>119 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>85 days</t>
+          <t>84 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>267 days</t>
+          <t>266 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>238 days</t>
+          <t>237 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>148 days</t>
+          <t>147 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>211 days</t>
+          <t>210 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>29 days</t>
+          <t>28 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>358 days</t>
+          <t>357 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>330 days</t>
+          <t>329 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.91 / 5.83%</t>
+          <t>$47.80 / 5.58%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.70 / 0.29%</t>
+          <t>$57.56 / 0.05%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.11 / 10.00%</t>
+          <t>$56.01 / 9.80%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.72 / 8.30%</t>
+          <t>$62.61 / 8.10%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.73 / 8.54%</t>
+          <t>$56.62 / 8.32%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.28 / 2.40%</t>
+          <t>$61.16 / 2.19%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.20 / 2.21%</t>
+          <t>$61.06 / 1.99%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.75 / 11.25%</t>
+          <t>$53.69 / 11.13%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.41 / 3.32%</t>
+          <t>$57.29 / 3.10%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.42 / 13.47%</t>
+          <t>$60.33 / 13.31%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.62 / 0.00%</t>
+          <t>$54.50 / -0.23%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.19 / 0.20%</t>
+          <t>$57.07 / -0.02%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.65 / 4.94%</t>
+          <t>$42.61 / 4.83%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.15 / 0.34%</t>
+          <t>$42.07 / 0.13%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.93 / 8.60%</t>
+          <t>$40.87 / 8.43%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.14 / 6.92%</t>
+          <t>$45.09 / 6.79%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.22 / 7.35%</t>
+          <t>$46.16 / 7.22%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.62 / 2.23%</t>
+          <t>$44.54 / 2.05%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.01 / 2.09%</t>
+          <t>$41.93 / 1.90%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.34 / 9.17%</t>
+          <t>$45.31 / 9.10%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.98 / 3.14%</t>
+          <t>$43.92 / 2.99%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.05 / 11.18%</t>
+          <t>$43.03 / 11.12%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.96 / 0.03%</t>
+          <t>$42.87 / -0.18%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.18 / 0.33%</t>
+          <t>$42.12 / 0.19%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$762.98 / 7.44%</t>
+          <t>$760.38 / 7.07%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$762.98 / -0.36%</t>
+          <t>$760.38 / -0.70%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$762.98 / 12.11%</t>
+          <t>$760.38 / 11.72%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$762.98 / 10.67%</t>
+          <t>$760.38 / 10.29%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$762.98 / 10.31%</t>
+          <t>$760.38 / 9.93%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$762.98 / 2.65%</t>
+          <t>$760.38 / 2.30%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$762.98 / 2.17%</t>
+          <t>$760.38 / 1.83%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$762.98 / 17.64%</t>
+          <t>$760.38 / 17.24%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$762.98 / 3.22%</t>
+          <t>$760.38 / 2.87%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$762.98 / 15.77%</t>
+          <t>$760.38 / 15.38%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$762.98 / -0.04%</t>
+          <t>$760.38 / -0.38%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$762.98 / 0.17%</t>
+          <t>$760.38 / -0.17%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$762.98 / 7.44%</t>
+          <t>$760.38 / 7.07%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$762.98 / -0.36%</t>
+          <t>$760.38 / -0.70%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$762.98 / 12.11%</t>
+          <t>$760.38 / 11.72%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$762.98 / 10.67%</t>
+          <t>$760.38 / 10.29%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$762.98 / 10.31%</t>
+          <t>$760.38 / 9.93%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$762.98 / 2.65%</t>
+          <t>$760.38 / 2.30%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$762.98 / 2.17%</t>
+          <t>$760.38 / 1.83%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$762.98 / 17.64%</t>
+          <t>$760.38 / 17.24%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$762.98 / 3.22%</t>
+          <t>$760.38 / 2.87%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$762.98 / 15.77%</t>
+          <t>$760.38 / 15.38%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$762.98 / -0.04%</t>
+          <t>$760.38 / -0.38%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$762.98 / 0.17%</t>
+          <t>$760.38 / -0.17%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.41% (8.02%)</t>
+          <t>8.65% (8.27%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.68% (15.98%)</t>
+          <t>16.96% (16.26%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.67% (3.54%)</t>
+          <t>3.86% (3.74%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.67% (5.41%)</t>
+          <t>5.86% (5.61%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.92% (4.74%)</t>
+          <t>5.13% (4.95%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.86% (13.26%)</t>
+          <t>14.09% (13.49%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.64% (13.10%)</t>
+          <t>13.89% (13.35%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.87% (4.56%)</t>
+          <t>4.99% (4.68%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.96% (12.49%)</t>
+          <t>13.21% (12.73%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.09% (2.03%)</t>
+          <t>2.23% (2.18%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>17.19% (16.36%)</t>
+          <t>17.46% (16.62%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.37% (15.60%)</t>
+          <t>16.62% (15.86%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.64% (6.25%)</t>
+          <t>6.75% (6.36%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.23% (12.53%)</t>
+          <t>13.46% (12.76%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.55% (2.42%)</t>
+          <t>2.71% (2.59%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.27% (4.01%)</t>
+          <t>4.40% (4.14%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.55% (3.37%)</t>
+          <t>3.67% (3.49%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.12% (10.51%)</t>
+          <t>11.32% (10.71%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.74% (10.20%)</t>
+          <t>10.95% (10.41%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.05% (3.74%)</t>
+          <t>4.12% (3.81%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.00% (9.52%)</t>
+          <t>10.16% (9.69%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.16% (1.10%)</t>
+          <t>1.22% (1.16%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>14.01% (13.17%)</t>
+          <t>14.24% (13.41%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.64% (12.87%)</t>
+          <t>13.80% (13.03%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.18%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.59%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.92%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>4.18%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.81%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.36%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.82%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>17.64%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.48%</t>
+          <t>16.88%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.92%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.36%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>11.26%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.94%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.01%</t>
+          <t>-2.67%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.18%</t>
+          <t>-1.84%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.48%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.31% (9.93%)</t>
+          <t>10.24% (9.85%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.24% (8.54%)</t>
+          <t>9.17% (8.47%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.97% (9.85%)</t>
+          <t>9.87% (9.75%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.49% (10.23%)</t>
+          <t>10.38% (10.12%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>9.95% (9.77%)</t>
+          <t>9.85% (9.67%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.76% (9.15%)</t>
+          <t>9.66% (9.05%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.47% (8.92%)</t>
+          <t>9.38% (8.84%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.93% (12.62%)</t>
+          <t>12.77% (12.46%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.23% (8.76%)</t>
+          <t>9.14% (8.67%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.70% (9.65%)</t>
+          <t>9.56% (9.50%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.96% (9.12%)</t>
+          <t>9.88% (9.04%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.88% (9.11%)</t>
+          <t>9.78% (9.02%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.76% (15.37%)</t>
+          <t>15.59% (15.20%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.22% (13.52%)</t>
+          <t>14.12% (13.42%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.60% (15.48%)</t>
+          <t>15.48% (15.36%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.19% (15.93%)</t>
+          <t>16.04% (15.78%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.49% (15.31%)</t>
+          <t>15.34% (15.15%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.79% (14.18%)</t>
+          <t>14.68% (14.07%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.47% (13.93%)</t>
+          <t>14.37% (13.83%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.88% (18.57%)</t>
+          <t>18.69% (18.38%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.24% (13.77%)</t>
+          <t>14.10% (13.63%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.82% (15.76%)</t>
+          <t>15.62% (15.56%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>14.93% (14.10%)</t>
+          <t>14.85% (14.01%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.76% (13.99%)</t>
+          <t>14.61% (13.84%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.92% (-6.31%)</t>
+          <t>-5.70% (-6.09%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.44% (-1.14%)</t>
+          <t>-0.20% (-0.90%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.74% (-9.86%)</t>
+          <t>-9.58% (-9.70%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.19% (-8.45%)</t>
+          <t>-8.02% (-8.28%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.47% (-8.65%)</t>
+          <t>-8.28% (-8.46%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.56% (-3.17%)</t>
+          <t>-2.37% (-2.97%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.45% (-2.99%)</t>
+          <t>-2.24% (-2.78%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.56% (-10.87%)</t>
+          <t>-10.47% (-10.77%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.58% (-4.05%)</t>
+          <t>-3.37% (-3.84%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.56% (-12.62%)</t>
+          <t>-12.44% (-12.49%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.01% (-0.84%)</t>
+          <t>0.00% (-0.62%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.28% (-1.04%)</t>
+          <t>-0.06% (-0.83%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.12% (-5.51%)</t>
+          <t>-5.02% (-5.41%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.48% (-1.18%)</t>
+          <t>-0.28% (-0.98%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.58% (-8.70%)</t>
+          <t>-8.43% (-8.55%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.00% (-7.26%)</t>
+          <t>-6.89% (-7.15%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.45% (-7.63%)</t>
+          <t>-7.34% (-7.52%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.40% (-3.01%)</t>
+          <t>-2.23% (-2.83%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.33% (-2.88%)</t>
+          <t>-2.15% (-2.69%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.86% (-9.18%)</t>
+          <t>-8.80% (-9.12%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.41% (-3.88%)</t>
+          <t>-3.27% (-3.74%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.76% (-10.82%)</t>
+          <t>-10.71% (-10.76%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.04% (-0.87%)</t>
+          <t>0.00% (-0.66%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.39% (-1.15%)</t>
+          <t>-0.25% (-1.01%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.23%</t>
+          <t>-15.95%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.68%</t>
+          <t>-9.37%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.72%</t>
+          <t>-19.44%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.68%</t>
+          <t>-18.40%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.41%</t>
+          <t>-18.13%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.32%</t>
+          <t>-12.02%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.92%</t>
+          <t>-11.61%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.50%</t>
+          <t>-23.23%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.81%</t>
+          <t>-12.51%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.26%</t>
+          <t>-22.00%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-9.97%</t>
+          <t>-9.66%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.15%</t>
+          <t>-9.84%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.88%</t>
+          <t>-20.61%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.69%</t>
+          <t>-14.40%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.18%</t>
+          <t>-23.92%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.19%</t>
+          <t>-22.93%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.94%</t>
+          <t>-22.68%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.19%</t>
+          <t>-16.91%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.81%</t>
+          <t>-16.52%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.74%</t>
+          <t>-27.50%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.65%</t>
+          <t>-17.37%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.58%</t>
+          <t>-26.33%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-14.97%</t>
+          <t>-14.68%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.14%</t>
+          <t>-14.85%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.11% (0.72%)</t>
+          <t>0.99% (0.61%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.44% (-1.14%)</t>
+          <t>-0.20% (-0.90%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.26% (1.14%)</t>
+          <t>1.10% (0.98%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.66% (1.41%)</t>
+          <t>1.50% (1.24%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.03% (0.85%)</t>
+          <t>0.89% (0.71%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>-0.12% (-0.72%)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-0.45% (-0.99%)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>4.99% (4.68%)</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>-0.59% (-1.06%)</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>1.14% (1.08%)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0.22% (-0.62%)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>-0.06% (-0.83%)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>1.72% (1.34%)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>-0.28% (-0.98%)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2.37% (2.25%)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>2.75% (2.49%)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1.92% (1.74%)</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
           <t>0.02% (-0.58%)</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>-0.32% (-0.86%)</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>4.87% (4.56%)</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>-0.46% (-0.93%)</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>1.34% (1.29%)</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>-0.01% (-0.84%)</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>-0.11% (-0.87%)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>1.97% (1.58%)</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>-0.48% (-1.18%)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>2.55% (2.42%)</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>2.98% (2.72%)</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>2.15% (1.97%)</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>0.19% (-0.42%)</t>
-        </is>
-      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.21% (-0.75%)</t>
+          <t>-0.36% (-0.90%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.05% (3.74%)</t>
+          <t>4.12% (3.81%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.29% (-0.76%)</t>
+          <t>-0.48% (-0.96%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.16% (1.10%)</t>
+          <t>1.22% (1.16%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.87%)</t>
+          <t>0.17% (-0.66%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.24% (-1.00%)</t>
+          <t>-0.25% (-1.01%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/10/2026</t>
+          <t>As of 23/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.67%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.74%</t>
+          <t>4.95%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.32%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>4.18%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.46%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>10.12%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.61%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.30%</t>
+          <t>8.10%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.92%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.45%</t>
+          <t>-8.28%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.62%</t>
+          <t>12.46%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.68%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.25%</t>
+          <t>11.13%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.64%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.87%</t>
+          <t>-10.77%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.02%</t>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.83%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.44%</t>
+          <t>7.07%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.18%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.31%</t>
+          <t>-6.09%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.76%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.73%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.32%</t>
+          <t>3.10%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.22%</t>
+          <t>2.87%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.44%</t>
+          <t>13.82%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.05%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.92%</t>
+          <t>8.84%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.10%</t>
+          <t>13.35%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>1.99%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>1.83%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.97%</t>
+          <t>14.36%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.99%</t>
+          <t>-2.78%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.26%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.40%</t>
+          <t>2.19%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.81%</t>
+          <t>14.19%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-2.97%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.47%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>16.26%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>0.05%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.59%</t>
+          <t>17.99%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.14%</t>
+          <t>-0.90%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.11%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.60%</t>
+          <t>15.86%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.48%</t>
+          <t>16.88%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.04%</t>
+          <t>-0.83%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.12%</t>
+          <t>9.04%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16.36%</t>
+          <t>16.62%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-0.23%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>-0.38%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>17.64%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.84%</t>
+          <t>-0.62%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.65%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.47%</t>
+          <t>13.31%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.62%</t>
+          <t>-12.49%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>9.75%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>9.80%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>11.72%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.36%</t>
+          <t>2.71%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.86%</t>
+          <t>-9.70%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 22/10/2026</t>
+          <t>As of 23/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.15%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.37%</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.35%</t>
+          <t>7.22%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.31%</t>
+          <t>9.93%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.36%</t>
+          <t>1.71%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.63%</t>
+          <t>-7.52%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>15.78%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.01%</t>
+          <t>4.14%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.92%</t>
+          <t>6.79%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.67%</t>
+          <t>10.29%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>1.60%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.26%</t>
+          <t>-7.15%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.57%</t>
+          <t>18.38%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.81%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.17%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.64%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.01%</t>
+          <t>-2.67%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.18%</t>
+          <t>-9.12%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.37%</t>
+          <t>15.20%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.25%</t>
+          <t>6.36%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>4.83%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.44%</t>
+          <t>7.07%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.56%</t>
+          <t>4.92%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.51%</t>
+          <t>-5.41%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>13.63%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.52%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.14%</t>
+          <t>2.99%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.22%</t>
+          <t>2.87%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.66%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.88%</t>
+          <t>-3.74%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.93%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.41%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.09%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.17%</t>
+          <t>1.83%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.94%</t>
+          <t>11.32%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-2.69%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>14.07%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.23%</t>
+          <t>2.05%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.88%</t>
+          <t>11.26%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.01%</t>
+          <t>-2.83%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.52%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.53%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.18%</t>
+          <t>-0.98%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13.99%</t>
+          <t>13.84%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.87%</t>
+          <t>13.03%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.90%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.01%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.10%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13.17%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.03%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>-0.38%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>14.09%</t>
+          <t>14.48%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.87%</t>
+          <t>-0.66%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.56%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.18%</t>
+          <t>11.12%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.38%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.18%</t>
+          <t>-1.84%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.82%</t>
+          <t>-10.76%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.48%</t>
+          <t>15.36%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>2.59%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.60%</t>
+          <t>8.43%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.11%</t>
+          <t>11.72%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.70%</t>
+          <t>-8.55%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-26]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/23/2026 at 1:45 PM ET)</t>
+          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>263 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>237 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>326 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>175 days</t>
+          <t>172 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>301 days</t>
+          <t>298 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>56 days</t>
+          <t>53 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>119 days</t>
+          <t>116 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>84 days</t>
+          <t>81 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>266 days</t>
+          <t>263 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>237 days</t>
+          <t>234 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>147 days</t>
+          <t>144 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>210 days</t>
+          <t>207 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>28 days</t>
+          <t>25 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>357 days</t>
+          <t>354 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>329 days</t>
+          <t>326 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$47.80 / 5.58%</t>
+          <t>$48.00 / 6.03%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.56 / 0.05%</t>
+          <t>$57.83 / 0.51%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.01 / 9.80%</t>
+          <t>$56.25 / 10.28%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.61 / 8.10%</t>
+          <t>$62.86 / 8.54%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.62 / 8.32%</t>
+          <t>$56.84 / 8.75%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.16 / 2.19%</t>
+          <t>$61.42 / 2.63%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.06 / 1.99%</t>
+          <t>$61.35 / 2.47%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.69 / 11.13%</t>
+          <t>$53.83 / 11.40%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.29 / 3.10%</t>
+          <t>$57.56 / 3.58%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.33 / 13.31%</t>
+          <t>$60.61 / 13.83%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.50 / -0.23%</t>
+          <t>$54.75 / 0.22%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.07 / -0.02%</t>
+          <t>$57.32 / 0.42%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.61 / 4.83%</t>
+          <t>$42.76 / 5.20%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.07 / 0.13%</t>
+          <t>$42.21 / 0.48%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$40.87 / 8.43%</t>
+          <t>$41.00 / 8.79%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.09 / 6.79%</t>
+          <t>$45.22 / 7.10%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.16 / 7.22%</t>
+          <t>$46.29 / 7.53%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.54 / 2.05%</t>
+          <t>$44.69 / 2.38%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$41.93 / 1.90%</t>
+          <t>$42.11 / 2.32%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.31 / 9.10%</t>
+          <t>$45.41 / 9.34%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$43.92 / 2.99%</t>
+          <t>$44.06 / 3.33%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.03 / 11.12%</t>
+          <t>$43.14 / 11.41%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$42.87 / -0.18%</t>
+          <t>$43.01 / 0.14%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.12 / 0.19%</t>
+          <t>$42.26 / 0.51%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$760.38 / 7.07%</t>
+          <t>$765.60 / 7.81%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.70%</t>
+          <t>$765.60 / -0.02%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$760.38 / 11.72%</t>
+          <t>$765.60 / 12.49%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$760.38 / 10.29%</t>
+          <t>$765.72 / 11.06%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$760.38 / 9.93%</t>
+          <t>$765.72 / 10.71%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$760.38 / 2.30%</t>
+          <t>$765.60 / 3.00%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$760.38 / 1.83%</t>
+          <t>$765.60 / 2.53%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$760.38 / 17.24%</t>
+          <t>$765.72 / 18.06%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$760.38 / 2.87%</t>
+          <t>$765.60 / 3.58%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$760.38 / 15.38%</t>
+          <t>$765.60 / 16.17%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.38%</t>
+          <t>$765.60 / 0.31%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.17%</t>
+          <t>$765.60 / 0.51%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$760.38 / 7.07%</t>
+          <t>$765.60 / 7.81%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.70%</t>
+          <t>$765.60 / -0.02%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$760.38 / 11.72%</t>
+          <t>$765.60 / 12.49%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$760.38 / 10.29%</t>
+          <t>$765.60 / 11.05%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$760.38 / 9.93%</t>
+          <t>$765.60 / 10.69%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$760.38 / 2.30%</t>
+          <t>$765.60 / 3.00%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$760.38 / 1.83%</t>
+          <t>$765.60 / 2.53%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$760.38 / 17.24%</t>
+          <t>$765.60 / 18.04%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$760.38 / 2.87%</t>
+          <t>$765.60 / 3.58%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$760.38 / 15.38%</t>
+          <t>$765.60 / 16.17%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.38%</t>
+          <t>$765.60 / 0.31%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$760.38 / -0.17%</t>
+          <t>$765.60 / 0.51%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.65% (8.27%)</t>
+          <t>8.19% (7.82%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.96% (16.26%)</t>
+          <t>16.42% (15.73%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.86% (3.74%)</t>
+          <t>3.40% (3.29%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.86% (5.61%)</t>
+          <t>5.43% (5.18%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5.13% (4.95%)</t>
+          <t>4.71% (4.54%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.09% (13.49%)</t>
+          <t>13.59% (13.00%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.89% (13.35%)</t>
+          <t>13.35% (12.82%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.99% (4.68%)</t>
+          <t>4.72% (4.41%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13.21% (12.73%)</t>
+          <t>12.67% (12.20%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.23% (2.18%)</t>
+          <t>1.75% (1.70%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>17.46% (16.62%)</t>
+          <t>16.91% (16.09%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.62% (15.86%)</t>
+          <t>16.11% (15.35%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.75% (6.36%)</t>
+          <t>6.37% (5.99%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.46% (12.76%)</t>
+          <t>13.06% (12.37%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.71% (2.59%)</t>
+          <t>2.36% (2.25%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.40% (4.14%)</t>
+          <t>4.08% (3.83%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.67% (3.49%)</t>
+          <t>3.37% (3.20%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>11.32% (10.71%)</t>
+          <t>10.95% (10.35%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.95% (10.41%)</t>
+          <t>10.48% (9.95%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>4.12% (3.81%)</t>
+          <t>3.88% (3.58%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>10.16% (9.69%)</t>
+          <t>9.79% (9.33%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>1.22% (1.16%)</t>
+          <t>0.94% (0.89%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>14.24% (13.41%)</t>
+          <t>13.87% (13.04%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.80% (13.03%)</t>
+          <t>13.43% (12.67%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7.55%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>17.19%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4.18%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.36%</t>
+          <t>13.58%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.82%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>17.64%</t>
+          <t>16.84%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.88%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.92%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-3.34%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-1.84%</t>
+          <t>-2.51%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>14.48%</t>
+          <t>13.70%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>13.51%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.24% (9.85%)</t>
+          <t>10.41% (10.04%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.17% (8.47%)</t>
+          <t>9.32% (8.63%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.87% (9.75%)</t>
+          <t>10.02% (9.90%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.38% (10.12%)</t>
+          <t>10.57% (10.32%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>9.85% (9.67%)</t>
+          <t>10.05% (9.88%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.66% (9.05%)</t>
+          <t>9.83% (9.23%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.38% (8.84%)</t>
+          <t>9.51% (8.98%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>12.77% (12.46%)</t>
+          <t>13.07% (12.77%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.14% (8.67%)</t>
+          <t>9.28% (8.81%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.56% (9.50%)</t>
+          <t>9.68% (9.63%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>9.88% (9.04%)</t>
+          <t>10.03% (9.21%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.78% (9.02%)</t>
+          <t>9.96% (9.20%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.59% (15.20%)</t>
+          <t>15.79% (15.41%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.12% (13.42%)</t>
+          <t>14.36% (13.67%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.48% (15.36%)</t>
+          <t>15.69% (15.58%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.04% (15.78%)</t>
+          <t>16.28% (16.03%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.34% (15.15%)</t>
+          <t>15.60% (15.42%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.68% (14.07%)</t>
+          <t>14.92% (14.32%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.37% (13.83%)</t>
+          <t>14.53% (13.99%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.69% (18.38%)</t>
+          <t>18.98% (18.67%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.10% (13.63%)</t>
+          <t>14.34% (13.87%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.62% (15.56%)</t>
+          <t>15.88% (15.83%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>14.85% (14.01%)</t>
+          <t>15.10% (14.27%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.61% (13.84%)</t>
+          <t>14.86% (14.11%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-5.70% (-6.09%)</t>
+          <t>-6.10% (-6.48%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.20% (-0.90%)</t>
+          <t>-0.66% (-1.35%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.58% (-9.70%)</t>
+          <t>-9.98% (-10.09%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.02% (-8.28%)</t>
+          <t>-8.40% (-8.65%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.28% (-8.46%)</t>
+          <t>-8.65% (-8.83%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.37% (-2.97%)</t>
+          <t>-2.79% (-3.39%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.24% (-2.78%)</t>
+          <t>-2.71% (-3.24%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.47% (-10.77%)</t>
+          <t>-10.70% (-11.00%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.37% (-3.84%)</t>
+          <t>-3.83% (-4.29%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.44% (-12.49%)</t>
+          <t>-12.85% (-12.90%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.00% (-0.62%)</t>
+          <t>-0.25% (-1.07%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.06% (-0.83%)</t>
+          <t>-0.50% (-1.26%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.02% (-5.41%)</t>
+          <t>-5.36% (-5.74%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.28% (-0.98%)</t>
+          <t>-0.63% (-1.32%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.43% (-8.55%)</t>
+          <t>-8.74% (-8.86%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-6.89% (-7.15%)</t>
+          <t>-7.17% (-7.42%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.34% (-7.52%)</t>
+          <t>-7.61% (-7.78%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.23% (-2.83%)</t>
+          <t>-2.55% (-3.15%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.15% (-2.69%)</t>
+          <t>-2.56% (-3.10%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-8.80% (-9.12%)</t>
+          <t>-9.01% (-9.32%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.27% (-3.74%)</t>
+          <t>-3.59% (-4.06%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.71% (-10.76%)</t>
+          <t>-10.95% (-11.00%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>0.00% (-0.66%)</t>
+          <t>-0.16% (-0.99%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.25% (-1.01%)</t>
+          <t>-0.57% (-1.33%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-15.95%</t>
+          <t>-16.52%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.37%</t>
+          <t>-9.99%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.44%</t>
+          <t>-19.99%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.40%</t>
+          <t>-18.97%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.13%</t>
+          <t>-18.70%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.02%</t>
+          <t>-12.62%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-11.61%</t>
+          <t>-12.22%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.23%</t>
+          <t>-23.77%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-12.51%</t>
+          <t>-13.11%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.00%</t>
+          <t>-22.53%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-9.66%</t>
+          <t>-10.28%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-9.84%</t>
+          <t>-10.46%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-20.61%</t>
+          <t>-21.15%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.40%</t>
+          <t>-14.98%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-23.92%</t>
+          <t>-24.44%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-22.93%</t>
+          <t>-23.45%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-22.68%</t>
+          <t>-23.21%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-16.91%</t>
+          <t>-17.47%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-16.52%</t>
+          <t>-17.09%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.50%</t>
+          <t>-27.99%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.37%</t>
+          <t>-17.93%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.33%</t>
+          <t>-26.83%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-14.68%</t>
+          <t>-15.26%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-14.85%</t>
+          <t>-15.43%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.99% (0.61%)</t>
+          <t>1.26% (0.88%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.20% (-0.90%)</t>
+          <t>-0.66% (-1.35%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.10% (0.98%)</t>
+          <t>1.35% (1.24%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.50% (1.24%)</t>
+          <t>1.79% (1.55%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.89% (0.71%)</t>
+          <t>1.19% (1.02%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.12% (-0.72%)</t>
+          <t>0.13% (-0.47%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.45% (-0.99%)</t>
+          <t>-0.24% (-0.77%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.99% (4.68%)</t>
+          <t>4.72% (4.41%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.59% (-1.06%)</t>
+          <t>-0.38% (-0.84%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.14% (1.08%)</t>
+          <t>1.36% (1.31%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.22% (-0.62%)</t>
+          <t>0.06% (-0.76%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.83%)</t>
+          <t>0.01% (-0.75%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.72% (1.34%)</t>
+          <t>2.06% (1.68%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.28% (-0.98%)</t>
+          <t>-0.63% (-1.32%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.37% (2.25%)</t>
+          <t>2.36% (2.25%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2.75% (2.49%)</t>
+          <t>3.14% (2.89%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.92% (1.74%)</t>
+          <t>2.33% (2.15%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.02% (-0.58%)</t>
+          <t>0.38% (-0.22%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.36% (-0.90%)</t>
+          <t>-0.10% (-0.63%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>4.12% (3.81%)</t>
+          <t>3.88% (3.58%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.48% (-0.96%)</t>
+          <t>-0.13% (-0.60%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1.22% (1.16%)</t>
+          <t>0.94% (0.89%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.17% (-0.66%)</t>
+          <t>0.14% (-0.68%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.25% (-1.01%)</t>
+          <t>-0.08% (-0.84%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/10/2026</t>
+          <t>As of 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>9.88%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.95%</t>
+          <t>4.54%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.32%</t>
+          <t>8.75%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4.18%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.46%</t>
+          <t>-8.83%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.12%</t>
+          <t>10.32%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.61%</t>
+          <t>5.18%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.10%</t>
+          <t>8.54%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>11.06%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>3.55%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.28%</t>
+          <t>-8.65%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.46%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.68%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.13%</t>
+          <t>11.40%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>18.06%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-10.77%</t>
+          <t>-11.00%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8.27%</t>
+          <t>7.82%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.58%</t>
+          <t>6.03%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.07%</t>
+          <t>7.81%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.55%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.09%</t>
+          <t>-6.48%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.67%</t>
+          <t>8.81%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.73%</t>
+          <t>12.20%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.87%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.82%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-4.29%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.84%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13.35%</t>
+          <t>12.82%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.99%</t>
+          <t>2.47%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.83%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14.36%</t>
+          <t>13.58%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.78%</t>
+          <t>-3.24%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>9.23%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>13.00%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.19%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.19%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.97%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.47%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>15.73%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.99%</t>
+          <t>17.19%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.90%</t>
+          <t>-1.35%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>9.20%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.86%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.88%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-1.26%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.04%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16.62%</t>
+          <t>16.09%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-0.23%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>17.64%</t>
+          <t>16.84%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.62%</t>
+          <t>-1.07%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.31%</t>
+          <t>13.83%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.38%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.08%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.49%</t>
+          <t>-12.90%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.75%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.74%</t>
+          <t>3.29%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.80%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.72%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.71%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.70%</t>
+          <t>-10.09%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 23/10/2026</t>
+          <t>As of 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.15%</t>
+          <t>15.42%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.20%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.22%</t>
+          <t>7.53%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.93%</t>
+          <t>10.69%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.52%</t>
+          <t>-7.78%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.78%</t>
+          <t>16.03%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.14%</t>
+          <t>3.83%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.79%</t>
+          <t>7.10%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10.29%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>0.91%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.15%</t>
+          <t>-7.42%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.38%</t>
+          <t>18.67%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.81%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>9.34%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>18.04%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-3.34%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.12%</t>
+          <t>-9.32%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.20%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.36%</t>
+          <t>5.99%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.83%</t>
+          <t>5.20%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.07%</t>
+          <t>7.81%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.92%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.41%</t>
+          <t>-5.74%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.63%</t>
+          <t>13.87%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>9.33%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.99%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.87%</t>
+          <t>3.58%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10.66%</t>
+          <t>9.90%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-4.06%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>13.99%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10.41%</t>
+          <t>9.95%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.90%</t>
+          <t>2.32%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.83%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11.32%</t>
+          <t>10.56%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-2.69%</t>
+          <t>-3.10%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.07%</t>
+          <t>14.32%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>10.35%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.05%</t>
+          <t>2.38%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.30%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-2.83%</t>
+          <t>-3.15%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>13.67%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>12.37%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>0.48%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>13.77%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-1.32%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13.84%</t>
+          <t>14.11%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13.03%</t>
+          <t>12.67%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.19%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>0.51%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>13.51%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.01%</t>
+          <t>-1.33%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-0.18%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-0.38%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>14.48%</t>
+          <t>13.70%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-0.99%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.56%</t>
+          <t>15.83%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.16%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.12%</t>
+          <t>11.41%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15.38%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-1.84%</t>
+          <t>-2.51%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-10.76%</t>
+          <t>-11.00%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.36%</t>
+          <t>15.58%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.59%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.43%</t>
+          <t>8.79%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11.72%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.32%</t>
+          <t>-0.36%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.55%</t>
+          <t>-8.86%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-27]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:21 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/26/2026 at 3:22 PM ET)</t>
+          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>172 days</t>
+          <t>171 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>298 days</t>
+          <t>297 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>53 days</t>
+          <t>52 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>116 days</t>
+          <t>115 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>81 days</t>
+          <t>80 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>263 days</t>
+          <t>262 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>234 days</t>
+          <t>233 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>144 days</t>
+          <t>143 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>207 days</t>
+          <t>206 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>354 days</t>
+          <t>353 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>326 days</t>
+          <t>325 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.00 / 6.03%</t>
+          <t>$48.14 / 6.33%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$57.83 / 0.51%</t>
+          <t>$58.02 / 0.84%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.25 / 10.28%</t>
+          <t>$56.42 / 10.60%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$62.86 / 8.54%</t>
+          <t>$63.01 / 8.80%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.84 / 8.75%</t>
+          <t>$57.02 / 9.09%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.42 / 2.63%</t>
+          <t>$61.62 / 2.97%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.35 / 2.47%</t>
+          <t>$61.56 / 2.82%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.83 / 11.40%</t>
+          <t>$53.94 / 11.63%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.56 / 3.58%</t>
+          <t>$57.75 / 3.93%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.61 / 13.83%</t>
+          <t>$60.78 / 14.15%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.75 / 0.22%</t>
+          <t>$54.91 / 0.52%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.32 / 0.42%</t>
+          <t>$57.51 / 0.76%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.76 / 5.20%</t>
+          <t>$42.84 / 5.39%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.21 / 0.48%</t>
+          <t>$42.33 / 0.76%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.00 / 8.79%</t>
+          <t>$41.09 / 9.03%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.22 / 7.10%</t>
+          <t>$45.31 / 7.31%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.29 / 7.53%</t>
+          <t>$46.41 / 7.79%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.69 / 2.38%</t>
+          <t>$44.81 / 2.65%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.11 / 2.32%</t>
+          <t>$42.20 / 2.55%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.41 / 9.34%</t>
+          <t>$45.48 / 9.50%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.06 / 3.33%</t>
+          <t>$44.19 / 3.64%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.14 / 11.41%</t>
+          <t>$43.20 / 11.56%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.01 / 0.14%</t>
+          <t>$43.13 / 0.42%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.26 / 0.51%</t>
+          <t>$42.38 / 0.79%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$765.60 / 7.81%</t>
+          <t>$769.39 / 8.34%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$765.60 / -0.02%</t>
+          <t>$769.39 / 0.48%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$765.60 / 12.49%</t>
+          <t>$769.39 / 13.05%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$765.72 / 11.06%</t>
+          <t>$769.39 / 11.60%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$765.72 / 10.71%</t>
+          <t>$769.39 / 11.24%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$765.60 / 3.00%</t>
+          <t>$769.39 / 3.51%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$765.60 / 2.53%</t>
+          <t>$769.39 / 3.03%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$765.72 / 18.06%</t>
+          <t>$769.39 / 18.63%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$765.60 / 3.58%</t>
+          <t>$769.39 / 4.09%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$765.60 / 16.17%</t>
+          <t>$769.39 / 16.75%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$765.60 / 0.31%</t>
+          <t>$769.39 / 0.80%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$765.60 / 0.51%</t>
+          <t>$769.39 / 1.01%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$765.60 / 7.81%</t>
+          <t>$769.39 / 8.34%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$765.60 / -0.02%</t>
+          <t>$769.39 / 0.48%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$765.60 / 12.49%</t>
+          <t>$769.39 / 13.05%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$765.60 / 11.05%</t>
+          <t>$769.39 / 11.60%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$765.60 / 10.69%</t>
+          <t>$769.39 / 11.24%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$765.60 / 3.00%</t>
+          <t>$769.39 / 3.51%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$765.60 / 2.53%</t>
+          <t>$769.39 / 3.03%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$765.60 / 18.04%</t>
+          <t>$769.39 / 18.63%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$765.60 / 3.58%</t>
+          <t>$769.39 / 4.09%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$765.60 / 16.17%</t>
+          <t>$769.39 / 16.75%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$765.60 / 0.31%</t>
+          <t>$769.39 / 0.80%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$765.60 / 0.51%</t>
+          <t>$769.39 / 1.01%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8.19% (7.82%)</t>
+          <t>7.88% (7.50%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.42% (15.73%)</t>
+          <t>16.04% (15.35%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.40% (3.29%)</t>
+          <t>3.09% (2.98%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.43% (5.18%)</t>
+          <t>5.18% (4.93%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.71% (4.54%)</t>
+          <t>4.38% (4.21%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.59% (13.00%)</t>
+          <t>13.22% (12.63%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.35% (12.82%)</t>
+          <t>12.96% (12.43%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.72% (4.41%)</t>
+          <t>4.50% (4.20%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.67% (12.20%)</t>
+          <t>12.30% (11.83%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.75% (1.70%)</t>
+          <t>1.47% (1.42%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.91% (16.09%)</t>
+          <t>16.57% (15.75%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>16.11% (15.35%)</t>
+          <t>15.71% (14.96%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.37% (5.99%)</t>
+          <t>6.17% (5.79%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>13.06% (12.37%)</t>
+          <t>12.74% (12.05%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.36% (2.25%)</t>
+          <t>2.14% (2.03%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>4.08% (3.83%)</t>
+          <t>3.88% (3.63%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.37% (3.20%)</t>
+          <t>3.12% (2.94%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.95% (10.35%)</t>
+          <t>10.65% (10.05%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.48% (9.95%)</t>
+          <t>10.23% (9.70%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.88% (3.58%)</t>
+          <t>3.73% (3.43%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.79% (9.33%)</t>
+          <t>9.47% (9.00%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.94% (0.89%)</t>
+          <t>0.81% (0.76%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.87% (13.04%)</t>
+          <t>13.55% (12.73%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.43% (12.67%)</t>
+          <t>13.10% (12.35%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.19%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>12.86%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.58%</t>
+          <t>13.02%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-1.23%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>16.84%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.34%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>9.36%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.51%</t>
+          <t>-2.99%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>13.70%</t>
+          <t>13.14%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>12.95%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.41% (10.04%)</t>
+          <t>10.55% (10.18%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.32% (8.63%)</t>
+          <t>9.44% (8.75%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.02% (9.90%)</t>
+          <t>10.14% (10.04%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.57% (10.32%)</t>
+          <t>10.73% (10.49%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.05% (9.88%)</t>
+          <t>10.15% (9.98%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.83% (9.23%)</t>
+          <t>9.94% (9.35%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.51% (8.98%)</t>
+          <t>9.61% (9.08%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.07% (12.77%)</t>
+          <t>13.25% (12.95%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.28% (8.81%)</t>
+          <t>9.39% (8.93%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.68% (9.63%)</t>
+          <t>9.82% (9.77%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.03% (9.21%)</t>
+          <t>10.18% (9.36%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.96% (9.20%)</t>
+          <t>10.06% (9.31%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.79% (15.41%)</t>
+          <t>16.00% (15.62%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.36% (13.67%)</t>
+          <t>14.49% (13.81%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.69% (15.58%)</t>
+          <t>15.86% (15.75%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.28% (16.03%)</t>
+          <t>16.48% (16.23%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.60% (15.42%)</t>
+          <t>15.74% (15.57%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.92% (14.32%)</t>
+          <t>15.07% (14.47%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.53% (13.99%)</t>
+          <t>14.71% (14.18%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.98% (18.67%)</t>
+          <t>19.20% (18.90%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.34% (13.87%)</t>
+          <t>14.46% (14.00%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.88% (15.83%)</t>
+          <t>16.12% (16.07%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.10% (14.27%)</t>
+          <t>15.23% (14.41%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.86% (14.11%)</t>
+          <t>14.99% (14.24%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.10% (-6.48%)</t>
+          <t>-6.38% (-6.75%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.66% (-1.35%)</t>
+          <t>-0.99% (-1.68%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-9.98% (-10.09%)</t>
+          <t>-10.24% (-10.35%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.40% (-8.65%)</t>
+          <t>-8.62% (-8.87%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.65% (-8.83%)</t>
+          <t>-8.94% (-9.11%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.79% (-3.39%)</t>
+          <t>-3.11% (-3.70%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.71% (-3.24%)</t>
+          <t>-3.04% (-3.57%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.70% (-11.00%)</t>
+          <t>-10.88% (-11.18%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.83% (-4.29%)</t>
+          <t>-4.15% (-4.61%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-12.85% (-12.90%)</t>
+          <t>-13.09% (-13.14%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.25% (-1.07%)</t>
+          <t>-0.54% (-1.36%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.50% (-1.26%)</t>
+          <t>-0.84% (-1.59%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.36% (-5.74%)</t>
+          <t>-5.54% (-5.92%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.63% (-1.32%)</t>
+          <t>-0.91% (-1.60%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.74% (-8.86%)</t>
+          <t>-8.94% (-9.05%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.17% (-7.42%)</t>
+          <t>-7.35% (-7.60%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.61% (-7.78%)</t>
+          <t>-7.84% (-8.01%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.55% (-3.15%)</t>
+          <t>-2.81% (-3.41%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.56% (-3.10%)</t>
+          <t>-2.79% (-3.31%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.01% (-9.32%)</t>
+          <t>-9.14% (-9.45%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.59% (-4.06%)</t>
+          <t>-3.88% (-4.34%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-10.95% (-11.00%)</t>
+          <t>-11.07% (-11.12%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.16% (-0.99%)</t>
+          <t>-0.45% (-1.26%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.57% (-1.33%)</t>
+          <t>-0.86% (-1.61%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.52%</t>
+          <t>-16.93%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-9.99%</t>
+          <t>-10.43%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-19.99%</t>
+          <t>-20.39%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-18.97%</t>
+          <t>-19.35%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.70%</t>
+          <t>-19.09%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.62%</t>
+          <t>-13.05%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.22%</t>
+          <t>-12.65%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.77%</t>
+          <t>-24.13%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.11%</t>
+          <t>-13.53%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.53%</t>
+          <t>-22.91%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.28%</t>
+          <t>-10.72%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.46%</t>
+          <t>-10.90%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.15%</t>
+          <t>-21.54%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-14.98%</t>
+          <t>-15.40%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.44%</t>
+          <t>-24.81%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.45%</t>
+          <t>-23.83%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-23.58%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.47%</t>
+          <t>-17.88%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.09%</t>
+          <t>-17.50%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-27.99%</t>
+          <t>-28.35%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-17.93%</t>
+          <t>-18.34%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-26.83%</t>
+          <t>-27.19%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-15.26%</t>
+          <t>-15.68%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.43%</t>
+          <t>-15.85%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.26% (0.88%)</t>
+          <t>1.47% (1.09%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.66% (-1.35%)</t>
+          <t>-0.51% (-1.20%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.35% (1.24%)</t>
+          <t>1.55% (1.44%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.79% (1.55%)</t>
+          <t>2.04% (1.79%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.19% (1.02%)</t>
+          <t>1.36% (1.19%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.13% (-0.47%)</t>
+          <t>0.30% (-0.29%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.24% (-0.77%)</t>
+          <t>-0.09% (-0.62%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.72% (4.41%)</t>
+          <t>4.50% (4.20%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.38% (-0.84%)</t>
+          <t>-0.21% (-0.68%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.36% (1.31%)</t>
+          <t>1.47% (1.42%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.06% (-0.76%)</t>
+          <t>0.26% (-0.56%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.01% (-0.75%)</t>
+          <t>0.16% (-0.59%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.06% (1.68%)</t>
+          <t>2.37% (2.00%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.63% (-1.32%)</t>
+          <t>-0.44% (-1.12%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.36% (2.25%)</t>
+          <t>2.14% (2.03%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.14% (2.89%)</t>
+          <t>3.46% (3.21%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.33% (2.15%)</t>
+          <t>2.58% (2.41%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.38% (-0.22%)</t>
+          <t>0.60% (0.01%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.10% (-0.63%)</t>
+          <t>0.17% (-0.36%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.88% (3.58%)</t>
+          <t>3.73% (3.43%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.13% (-0.60%)</t>
+          <t>0.06% (-0.40%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.94% (0.89%)</t>
+          <t>0.81% (0.76%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.14% (-0.68%)</t>
+          <t>0.36% (-0.46%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.08% (-0.84%)</t>
+          <t>0.13% (-0.62%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 26/10/2026</t>
+          <t>As of 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.88%</t>
+          <t>9.98%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.54%</t>
+          <t>4.21%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8.75%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>11.24%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>2.96%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.83%</t>
+          <t>-9.11%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.32%</t>
+          <t>10.49%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.18%</t>
+          <t>4.93%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.54%</t>
+          <t>8.80%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.06%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.06%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.65%</t>
+          <t>-8.87%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>12.95%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>4.20%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.40%</t>
+          <t>11.63%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.06%</t>
+          <t>18.63%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.76%</t>
+          <t>-1.23%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.00%</t>
+          <t>-11.18%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>10.18%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.82%</t>
+          <t>7.50%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.03%</t>
+          <t>6.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.81%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.82%</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.48%</t>
+          <t>-6.75%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.81%</t>
+          <t>8.93%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.20%</t>
+          <t>11.83%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.93%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>12.49%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.29%</t>
+          <t>-4.61%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.98%</t>
+          <t>9.08%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.82%</t>
+          <t>12.43%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.47%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.58%</t>
+          <t>13.02%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.24%</t>
+          <t>-3.57%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.23%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13.00%</t>
+          <t>12.63%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>12.86%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.39%</t>
+          <t>-3.70%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.63%</t>
+          <t>8.75%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.73%</t>
+          <t>15.35%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.48%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17.19%</t>
+          <t>16.61%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.68%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.20%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>14.96%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>15.51%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.59%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>9.36%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16.09%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>16.84%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-1.36%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>9.77%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.83%</t>
+          <t>14.15%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-12.90%</t>
+          <t>-13.14%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3.29%</t>
+          <t>2.98%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>10.60%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2.01%</t>
+          <t>1.51%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.09%</t>
+          <t>-10.35%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 26/10/2026</t>
+          <t>As of 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.42%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.20%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.53%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.69%</t>
+          <t>11.24%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-7.78%</t>
+          <t>-8.01%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.03%</t>
+          <t>16.23%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.83%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.10%</t>
+          <t>7.31%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>11.60%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.42%</t>
+          <t>-7.60%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>18.90%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>3.43%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.34%</t>
+          <t>9.50%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.04%</t>
+          <t>18.63%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.34%</t>
+          <t>-3.81%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.32%</t>
+          <t>-9.45%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.41%</t>
+          <t>15.62%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.99%</t>
+          <t>5.79%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.20%</t>
+          <t>5.39%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.81%</t>
+          <t>8.34%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>3.69%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.74%</t>
+          <t>-5.92%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.87%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.33%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>3.64%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.58%</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.90%</t>
+          <t>9.36%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.06%</t>
+          <t>-4.34%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13.99%</t>
+          <t>14.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.95%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>3.03%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.56%</t>
+          <t>10.02%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.10%</t>
+          <t>-3.31%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.32%</t>
+          <t>14.47%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.35%</t>
+          <t>10.05%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.38%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.51%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.51%</t>
+          <t>9.96%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.15%</t>
+          <t>-3.41%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.67%</t>
+          <t>13.81%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.37%</t>
+          <t>12.05%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>0.48%</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>-0.02%</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.77%</t>
+          <t>13.21%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.32%</t>
+          <t>-1.60%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.11%</t>
+          <t>14.24%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.67%</t>
+          <t>12.35%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.79%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.51%</t>
+          <t>12.95%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>-1.61%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.41%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>12.73%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.14%</t>
+          <t>0.42%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.31%</t>
+          <t>0.80%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.70%</t>
+          <t>13.14%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-1.26%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.83%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>11.56%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.75%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.51%</t>
+          <t>-2.99%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.00%</t>
+          <t>-11.12%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.58%</t>
+          <t>15.75%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.79%</t>
+          <t>9.03%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>13.05%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.85%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-8.86%</t>
+          <t>-9.05%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-28]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/27/2026 at 2:46 PM ET)</t>
+          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>171 days</t>
+          <t>170 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>297 days</t>
+          <t>296 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>52 days</t>
+          <t>51 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>115 days</t>
+          <t>114 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>80 days</t>
+          <t>79 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>262 days</t>
+          <t>261 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>233 days</t>
+          <t>232 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>143 days</t>
+          <t>142 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>206 days</t>
+          <t>205 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>353 days</t>
+          <t>352 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>325 days</t>
+          <t>324 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.14 / 6.33%</t>
+          <t>$48.25 / 6.59%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.02 / 0.84%</t>
+          <t>$58.13 / 1.03%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.42 / 10.60%</t>
+          <t>$56.52 / 10.80%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.01 / 8.80%</t>
+          <t>$63.13 / 9.01%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.02 / 9.09%</t>
+          <t>$57.14 / 9.31%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.62 / 2.97%</t>
+          <t>$61.75 / 3.18%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.56 / 2.82%</t>
+          <t>$61.67 / 3.00%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.94 / 11.63%</t>
+          <t>$54.02 / 11.81%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.75 / 3.93%</t>
+          <t>$57.86 / 4.12%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.78 / 14.15%</t>
+          <t>$60.88 / 14.34%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.91 / 0.52%</t>
+          <t>$55.01 / 0.70%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.51 / 0.76%</t>
+          <t>$57.61 / 0.93%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.84 / 5.39%</t>
+          <t>$42.88 / 5.50%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.33 / 0.76%</t>
+          <t>$42.41 / 0.94%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.09 / 9.03%</t>
+          <t>$41.18 / 9.25%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.31 / 7.31%</t>
+          <t>$45.37 / 7.45%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.41 / 7.79%</t>
+          <t>$46.45 / 7.89%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.81 / 2.65%</t>
+          <t>$44.87 / 2.79%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.20 / 2.55%</t>
+          <t>$42.27 / 2.72%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.48 / 9.50%</t>
+          <t>$45.51 / 9.58%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.19 / 3.64%</t>
+          <t>$44.24 / 3.75%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.20 / 11.56%</t>
+          <t>$43.25 / 11.68%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.13 / 0.42%</t>
+          <t>$43.18 / 0.54%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.38 / 0.79%</t>
+          <t>$42.44 / 0.94%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$769.39 / 8.34%</t>
+          <t>$771.68 / 8.67%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$769.39 / 0.48%</t>
+          <t>$771.68 / 0.78%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$769.39 / 13.05%</t>
+          <t>$771.68 / 13.38%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$769.39 / 11.60%</t>
+          <t>$771.68 / 11.93%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$769.39 / 11.24%</t>
+          <t>$771.68 / 11.57%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$769.39 / 3.51%</t>
+          <t>$771.68 / 3.82%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$769.39 / 3.03%</t>
+          <t>$771.68 / 3.34%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$769.39 / 18.63%</t>
+          <t>$771.68 / 18.98%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$769.39 / 4.09%</t>
+          <t>$771.68 / 4.40%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$769.39 / 16.75%</t>
+          <t>$771.68 / 17.09%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$769.39 / 0.80%</t>
+          <t>$771.68 / 1.10%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$769.39 / 1.01%</t>
+          <t>$771.68 / 1.31%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$769.39 / 8.34%</t>
+          <t>$771.68 / 8.67%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$769.39 / 0.48%</t>
+          <t>$771.68 / 0.78%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$769.39 / 13.05%</t>
+          <t>$771.68 / 13.38%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$769.39 / 11.60%</t>
+          <t>$771.68 / 11.93%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$769.39 / 11.24%</t>
+          <t>$771.68 / 11.57%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$769.39 / 3.51%</t>
+          <t>$771.68 / 3.82%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$769.39 / 3.03%</t>
+          <t>$771.68 / 3.34%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$769.39 / 18.63%</t>
+          <t>$771.68 / 18.98%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$769.39 / 4.09%</t>
+          <t>$771.68 / 4.40%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$769.39 / 16.75%</t>
+          <t>$771.68 / 17.09%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$769.39 / 0.80%</t>
+          <t>$771.68 / 1.10%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$769.39 / 1.01%</t>
+          <t>$771.68 / 1.31%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.88% (7.50%)</t>
+          <t>7.62% (7.25%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.04% (15.35%)</t>
+          <t>15.81% (15.13%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.09% (2.98%)</t>
+          <t>2.91% (2.80%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.18% (4.93%)</t>
+          <t>4.97% (4.73%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.38% (4.21%)</t>
+          <t>4.16% (4.00%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.22% (12.63%)</t>
+          <t>12.98% (12.39%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.96% (12.43%)</t>
+          <t>12.76% (12.24%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.50% (4.20%)</t>
+          <t>4.33% (4.04%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.30% (11.83%)</t>
+          <t>12.08% (11.62%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.47% (1.42%)</t>
+          <t>1.30% (1.25%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.57% (15.75%)</t>
+          <t>16.36% (15.54%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.71% (14.96%)</t>
+          <t>15.51% (14.76%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.17% (5.79%)</t>
+          <t>6.05% (5.68%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.74% (12.05%)</t>
+          <t>12.53% (11.85%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.14% (2.03%)</t>
+          <t>1.92% (1.81%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.88% (3.63%)</t>
+          <t>3.74% (3.50%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.12% (2.94%)</t>
+          <t>3.03% (2.86%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.65% (10.05%)</t>
+          <t>10.50% (9.91%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.23% (9.70%)</t>
+          <t>10.05% (9.52%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.73% (3.43%)</t>
+          <t>3.65% (3.35%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.47% (9.00%)</t>
+          <t>9.34% (8.88%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.81% (0.76%)</t>
+          <t>0.69% (0.64%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.55% (12.73%)</t>
+          <t>13.41% (12.60%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.10% (12.35%)</t>
+          <t>12.94% (12.19%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>5.98%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>1.21%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.86%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.02%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.23%</t>
+          <t>-1.52%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.16%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-4.10%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>9.04%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.99%</t>
+          <t>-3.28%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>13.14%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.95%</t>
+          <t>12.61%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.55% (10.18%)</t>
+          <t>10.57% (10.20%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.44% (8.75%)</t>
+          <t>9.52% (8.83%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.14% (10.04%)</t>
+          <t>10.22% (10.11%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.73% (10.49%)</t>
+          <t>10.80% (10.55%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.15% (9.98%)</t>
+          <t>10.21% (10.04%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.94% (9.35%)</t>
+          <t>9.99% (9.40%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.61% (9.08%)</t>
+          <t>9.70% (9.18%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.25% (12.95%)</t>
+          <t>13.33% (13.04%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.39% (8.93%)</t>
+          <t>9.46% (9.00%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.82% (9.77%)</t>
+          <t>9.90% (9.85%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.18% (9.36%)</t>
+          <t>10.26% (9.44%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.06% (9.31%)</t>
+          <t>10.15% (9.40%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.00% (15.62%)</t>
+          <t>16.13% (15.76%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.49% (13.81%)</t>
+          <t>14.57% (13.88%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.86% (15.75%)</t>
+          <t>15.90% (15.79%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.48% (16.23%)</t>
+          <t>16.58% (16.34%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.74% (15.57%)</t>
+          <t>15.89% (15.72%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.07% (14.47%)</t>
+          <t>15.18% (14.59%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.71% (14.18%)</t>
+          <t>14.80% (14.27%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.20% (18.90%)</t>
+          <t>19.34% (19.04%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.46% (14.00%)</t>
+          <t>14.59% (14.13%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.12% (16.07%)</t>
+          <t>16.23% (16.19%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.23% (14.41%)</t>
+          <t>15.37% (14.55%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.99% (14.24%)</t>
+          <t>15.10% (14.35%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.38% (-6.75%)</t>
+          <t>-6.61% (-6.98%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.99% (-1.68%)</t>
+          <t>-1.18% (-1.86%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.24% (-10.35%)</t>
+          <t>-10.40% (-10.51%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.62% (-8.87%)</t>
+          <t>-8.80% (-9.04%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.94% (-9.11%)</t>
+          <t>-9.13% (-9.30%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.11% (-3.70%)</t>
+          <t>-3.32% (-3.91%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.04% (-3.57%)</t>
+          <t>-3.21% (-3.73%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.88% (-11.18%)</t>
+          <t>-11.02% (-11.32%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.15% (-4.61%)</t>
+          <t>-4.33% (-4.79%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.09% (-13.14%)</t>
+          <t>-13.24% (-13.28%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.54% (-1.36%)</t>
+          <t>-0.72% (-1.54%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.84% (-1.59%)</t>
+          <t>-1.02% (-1.77%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.54% (-5.92%)</t>
+          <t>-5.64% (-6.02%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.91% (-1.60%)</t>
+          <t>-1.09% (-1.77%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.94% (-9.05%)</t>
+          <t>-9.13% (-9.24%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.35% (-7.60%)</t>
+          <t>-7.47% (-7.72%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.84% (-8.01%)</t>
+          <t>-7.92% (-8.09%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.81% (-3.41%)</t>
+          <t>-2.95% (-3.54%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.79% (-3.31%)</t>
+          <t>-2.95% (-3.47%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.14% (-9.45%)</t>
+          <t>-9.21% (-9.52%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.88% (-4.34%)</t>
+          <t>-3.99% (-4.45%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-11.07% (-11.12%)</t>
+          <t>-11.17% (-11.22%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.45% (-1.26%)</t>
+          <t>-0.56% (-1.38%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.86% (-1.61%)</t>
+          <t>-1.00% (-1.75%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.93%</t>
+          <t>-17.18%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.43%</t>
+          <t>-10.69%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.39%</t>
+          <t>-20.62%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.35%</t>
+          <t>-19.59%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.09%</t>
+          <t>-19.33%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.05%</t>
+          <t>-13.31%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.65%</t>
+          <t>-12.91%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.13%</t>
+          <t>-24.36%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.53%</t>
+          <t>-13.79%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.91%</t>
+          <t>-23.14%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.72%</t>
+          <t>-10.98%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.90%</t>
+          <t>-11.16%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.54%</t>
+          <t>-21.78%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.40%</t>
+          <t>-15.65%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.81%</t>
+          <t>-25.03%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.83%</t>
+          <t>-24.06%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.58%</t>
+          <t>-23.81%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.88%</t>
+          <t>-18.12%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.50%</t>
+          <t>-17.74%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.35%</t>
+          <t>-28.56%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.34%</t>
+          <t>-18.58%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.19%</t>
+          <t>-27.40%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-15.68%</t>
+          <t>-15.93%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.85%</t>
+          <t>-16.10%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.47% (1.09%)</t>
+          <t>1.52% (1.15%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.51% (-1.20%)</t>
+          <t>-0.41% (-1.09%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.55% (1.44%)</t>
+          <t>1.68% (1.57%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.04% (1.79%)</t>
+          <t>2.15% (1.90%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.36% (1.19%)</t>
+          <t>1.46% (1.29%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.30% (-0.29%)</t>
+          <t>0.38% (-0.21%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.62%)</t>
+          <t>0.04% (-0.49%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.50% (4.20%)</t>
+          <t>4.33% (4.04%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.21% (-0.68%)</t>
+          <t>-0.11% (-0.57%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.47% (1.42%)</t>
+          <t>1.30% (1.25%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.26% (-0.56%)</t>
+          <t>0.37% (-0.44%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.16% (-0.59%)</t>
+          <t>0.28% (-0.47%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.37% (2.00%)</t>
+          <t>2.57% (2.19%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.44% (-1.12%)</t>
+          <t>-0.32% (-1.00%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.14% (2.03%)</t>
+          <t>1.92% (1.81%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.46% (3.21%)</t>
+          <t>3.63% (3.38%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.58% (2.41%)</t>
+          <t>2.80% (2.63%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.60% (0.01%)</t>
+          <t>0.77% (0.17%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.17% (-0.36%)</t>
+          <t>0.30% (-0.23%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.73% (3.43%)</t>
+          <t>3.65% (3.35%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.06% (-0.40%)</t>
+          <t>0.25% (-0.21%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.81% (0.76%)</t>
+          <t>0.69% (0.64%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.36% (-0.46%)</t>
+          <t>0.54% (-0.28%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.13% (-0.62%)</t>
+          <t>0.28% (-0.47%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 27/10/2026</t>
+          <t>As of 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.98%</t>
+          <t>10.04%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.21%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>9.31%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.24%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.96%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.11%</t>
+          <t>-9.30%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.49%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>4.73%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.80%</t>
+          <t>9.01%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.06%</t>
+          <t>2.75%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.87%</t>
+          <t>-9.04%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.95%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.20%</t>
+          <t>4.04%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.63%</t>
+          <t>11.81%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.63%</t>
+          <t>18.98%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.23%</t>
+          <t>-1.52%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.18%</t>
+          <t>-11.32%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.18%</t>
+          <t>10.20%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.50%</t>
+          <t>7.25%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.33%</t>
+          <t>6.59%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>5.98%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.75%</t>
+          <t>-6.98%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.93%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.83%</t>
+          <t>11.62%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.93%</t>
+          <t>4.12%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>4.40%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>12.16%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.61%</t>
+          <t>-4.79%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.08%</t>
+          <t>9.18%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.43%</t>
+          <t>12.24%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.02%</t>
+          <t>12.69%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.73%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.35%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.63%</t>
+          <t>12.39%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>3.18%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.51%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.86%</t>
+          <t>12.52%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.70%</t>
+          <t>-3.91%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.75%</t>
+          <t>8.83%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>15.13%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.84%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.48%</t>
+          <t>0.78%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.61%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.68%</t>
+          <t>-1.86%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.40%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.96%</t>
+          <t>14.76%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.51%</t>
+          <t>15.17%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.77%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.54%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>15.92%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.36%</t>
+          <t>-1.54%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.42%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.15%</t>
+          <t>14.34%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>-0.40%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.14%</t>
+          <t>-13.28%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.98%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.60%</t>
+          <t>10.80%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>1.21%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.35%</t>
+          <t>-10.51%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 27/10/2026</t>
+          <t>As of 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.57%</t>
+          <t>15.72%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>2.86%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>7.89%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.24%</t>
+          <t>11.57%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.52%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.01%</t>
+          <t>-8.09%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.23%</t>
+          <t>16.34%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.63%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.31%</t>
+          <t>7.45%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.60%</t>
+          <t>-7.72%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.90%</t>
+          <t>19.04%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.43%</t>
+          <t>3.35%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>9.58%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.63%</t>
+          <t>18.98%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.81%</t>
+          <t>-4.10%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.45%</t>
+          <t>-9.52%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>15.76%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.79%</t>
+          <t>5.68%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.39%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.92%</t>
+          <t>-6.02%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>14.13%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>4.40%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>9.04%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-4.45%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.18%</t>
+          <t>14.27%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.70%</t>
+          <t>9.52%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.55%</t>
+          <t>2.72%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.03%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.02%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.31%</t>
+          <t>-3.47%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.47%</t>
+          <t>14.59%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.05%</t>
+          <t>9.91%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.51%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.96%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-3.54%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.81%</t>
+          <t>13.88%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.05%</t>
+          <t>11.85%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.48%</t>
+          <t>0.78%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.21%</t>
+          <t>12.88%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-1.77%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.24%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.35%</t>
+          <t>12.19%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.79%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.31%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.95%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-1.75%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.41%</t>
+          <t>14.55%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.73%</t>
+          <t>12.60%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.42%</t>
+          <t>0.54%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.14%</t>
+          <t>12.81%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.26%</t>
+          <t>-1.38%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>16.19%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.56%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>17.09%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.99%</t>
+          <t>-3.28%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.12%</t>
+          <t>-11.22%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.75%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>1.81%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.03%</t>
+          <t>9.25%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.05%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-1.15%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.05%</t>
+          <t>-9.24%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-29]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/28/2026 at 2:55 PM ET)</t>
+          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>170 days</t>
+          <t>169 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>296 days</t>
+          <t>295 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>51 days</t>
+          <t>50 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>114 days</t>
+          <t>113 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>79 days</t>
+          <t>78 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>261 days</t>
+          <t>260 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>232 days</t>
+          <t>231 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>142 days</t>
+          <t>141 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>205 days</t>
+          <t>204 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>22 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>352 days</t>
+          <t>351 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>324 days</t>
+          <t>323 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.25 / 6.59%</t>
+          <t>$48.11 / 6.27%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.13 / 1.03%</t>
+          <t>$58.01 / 0.82%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.52 / 10.80%</t>
+          <t>$56.43 / 10.62%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.13 / 9.01%</t>
+          <t>$63.00 / 8.78%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$57.14 / 9.31%</t>
+          <t>$56.98 / 9.02%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.75 / 3.18%</t>
+          <t>$61.58 / 2.89%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.67 / 3.00%</t>
+          <t>$61.49 / 2.69%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$54.02 / 11.81%</t>
+          <t>$53.95 / 11.66%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.86 / 4.12%</t>
+          <t>$57.69 / 3.82%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.88 / 14.34%</t>
+          <t>$60.79 / 14.16%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$55.01 / 0.70%</t>
+          <t>$54.87 / 0.44%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.61 / 0.93%</t>
+          <t>$57.45 / 0.65%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.88 / 5.50%</t>
+          <t>$42.81 / 5.32%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.41 / 0.94%</t>
+          <t>$42.30 / 0.69%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.18 / 9.25%</t>
+          <t>$41.10 / 9.05%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.37 / 7.45%</t>
+          <t>$45.30 / 7.28%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.45 / 7.89%</t>
+          <t>$46.41 / 7.79%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.87 / 2.79%</t>
+          <t>$44.79 / 2.61%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.27 / 2.72%</t>
+          <t>$42.19 / 2.53%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.51 / 9.58%</t>
+          <t>$45.49 / 9.54%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.24 / 3.75%</t>
+          <t>$44.15 / 3.54%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.25 / 11.68%</t>
+          <t>$43.24 / 11.66%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.18 / 0.54%</t>
+          <t>$43.14 / 0.43%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.44 / 0.94%</t>
+          <t>$42.34 / 0.71%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$771.68 / 8.67%</t>
+          <t>$767.52 / 8.08%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$771.68 / 0.78%</t>
+          <t>$767.52 / 0.24%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$771.68 / 13.38%</t>
+          <t>$767.52 / 12.77%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$771.68 / 11.93%</t>
+          <t>$767.52 / 11.33%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$771.68 / 11.57%</t>
+          <t>$767.52 / 10.97%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$771.68 / 3.82%</t>
+          <t>$767.52 / 3.26%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$771.68 / 3.34%</t>
+          <t>$767.52 / 2.78%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$771.68 / 18.98%</t>
+          <t>$767.52 / 18.34%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$771.68 / 4.40%</t>
+          <t>$767.52 / 3.84%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$771.68 / 17.09%</t>
+          <t>$767.52 / 16.46%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$771.68 / 1.10%</t>
+          <t>$767.52 / 0.56%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$771.68 / 1.31%</t>
+          <t>$767.52 / 0.77%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$771.68 / 8.67%</t>
+          <t>$767.52 / 8.08%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$771.68 / 0.78%</t>
+          <t>$767.52 / 0.24%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$771.68 / 13.38%</t>
+          <t>$767.52 / 12.77%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$771.68 / 11.93%</t>
+          <t>$767.52 / 11.33%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$771.68 / 11.57%</t>
+          <t>$767.52 / 10.97%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$771.68 / 3.82%</t>
+          <t>$767.52 / 3.26%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$771.68 / 3.34%</t>
+          <t>$767.52 / 2.78%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$771.68 / 18.98%</t>
+          <t>$767.52 / 18.34%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$771.68 / 4.40%</t>
+          <t>$767.52 / 3.84%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$771.68 / 17.09%</t>
+          <t>$767.52 / 16.46%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$771.68 / 1.10%</t>
+          <t>$767.52 / 0.56%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$771.68 / 1.31%</t>
+          <t>$767.52 / 0.77%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.62% (7.25%)</t>
+          <t>7.94% (7.57%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.81% (15.13%)</t>
+          <t>16.05% (15.37%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.91% (2.80%)</t>
+          <t>3.07% (2.97%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.97% (4.73%)</t>
+          <t>5.19% (4.95%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.16% (4.00%)</t>
+          <t>4.45% (4.28%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.98% (12.39%)</t>
+          <t>13.30% (12.71%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>12.76% (12.24%)</t>
+          <t>13.09% (12.57%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.33% (4.04%)</t>
+          <t>4.47% (4.17%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.08% (11.62%)</t>
+          <t>12.41% (11.95%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.30% (1.25%)</t>
+          <t>1.46% (1.41%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.36% (15.54%)</t>
+          <t>16.65% (15.84%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.51% (14.76%)</t>
+          <t>15.83% (15.08%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.05% (5.68%)</t>
+          <t>6.24% (5.86%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.53% (11.85%)</t>
+          <t>12.81% (12.13%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>1.92% (1.81%)</t>
+          <t>2.11% (2.00%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.74% (3.50%)</t>
+          <t>3.90% (3.66%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.03% (2.86%)</t>
+          <t>3.11% (2.94%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.50% (9.91%)</t>
+          <t>10.69% (10.10%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.05% (9.52%)</t>
+          <t>10.25% (9.73%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.65% (3.35%)</t>
+          <t>3.70% (3.40%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.34% (8.88%)</t>
+          <t>9.56% (9.10%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.69% (0.64%)</t>
+          <t>0.71% (0.67%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.41% (12.60%)</t>
+          <t>13.53% (12.71%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>12.94% (12.19%)</t>
+          <t>13.19% (12.44%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>5.98%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>3.31%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-0.99%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.16%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.17%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.94%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-4.10%</t>
+          <t>-3.58%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.04%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>13.22%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.57% (10.20%)</t>
+          <t>10.40% (10.03%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.52% (8.83%)</t>
+          <t>9.23% (8.55%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.22% (10.11%)</t>
+          <t>9.93% (9.83%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.80% (10.55%)</t>
+          <t>10.55% (10.30%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.21% (10.04%)</t>
+          <t>10.01% (9.85%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.99% (9.40%)</t>
+          <t>9.80% (9.21%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.70% (9.18%)</t>
+          <t>9.51% (8.99%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.33% (13.04%)</t>
+          <t>13.04% (12.74%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.46% (9.00%)</t>
+          <t>9.27% (8.81%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.90% (9.85%)</t>
+          <t>9.62% (9.57%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.26% (9.44%)</t>
+          <t>10.03% (9.21%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10.15% (9.40%)</t>
+          <t>9.94% (9.19%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>16.13% (15.76%)</t>
+          <t>15.87% (15.50%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.57% (13.88%)</t>
+          <t>14.35% (13.67%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.90% (15.79%)</t>
+          <t>15.65% (15.55%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.58% (16.34%)</t>
+          <t>16.31% (16.07%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.89% (15.72%)</t>
+          <t>15.55% (15.39%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>15.18% (14.59%)</t>
+          <t>14.90% (14.31%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.80% (14.27%)</t>
+          <t>14.53% (14.01%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>19.34% (19.04%)</t>
+          <t>18.99% (18.69%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.59% (14.13%)</t>
+          <t>14.34% (13.88%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>16.23% (16.19%)</t>
+          <t>15.86% (15.81%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.37% (14.55%)</t>
+          <t>15.01% (14.20%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>15.10% (14.35%)</t>
+          <t>14.87% (14.12%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.61% (-6.98%)</t>
+          <t>-6.33% (-6.70%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-1.18% (-1.86%)</t>
+          <t>-0.98% (-1.66%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.40% (-10.51%)</t>
+          <t>-10.26% (-10.37%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.80% (-9.04%)</t>
+          <t>-8.61% (-8.85%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-9.13% (-9.30%)</t>
+          <t>-8.88% (-9.05%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.32% (-3.91%)</t>
+          <t>-3.04% (-3.63%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-3.21% (-3.73%)</t>
+          <t>-2.93% (-3.45%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-11.02% (-11.32%)</t>
+          <t>-10.91% (-11.20%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.33% (-4.79%)</t>
+          <t>-4.05% (-4.51%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.24% (-13.28%)</t>
+          <t>-13.10% (-13.15%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.72% (-1.54%)</t>
+          <t>-0.47% (-1.29%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-1.02% (-1.77%)</t>
+          <t>-0.74% (-1.49%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.64% (-6.02%)</t>
+          <t>-5.48% (-5.85%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-1.09% (-1.77%)</t>
+          <t>-0.84% (-1.53%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-9.13% (-9.24%)</t>
+          <t>-8.97% (-9.08%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.47% (-7.72%)</t>
+          <t>-7.33% (-7.58%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.92% (-8.09%)</t>
+          <t>-7.84% (-8.01%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.95% (-3.54%)</t>
+          <t>-2.78% (-3.37%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.95% (-3.47%)</t>
+          <t>-2.77% (-3.29%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.21% (-9.52%)</t>
+          <t>-9.18% (-9.48%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.99% (-4.45%)</t>
+          <t>-3.80% (-4.25%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-11.17% (-11.22%)</t>
+          <t>-11.15% (-11.20%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.56% (-1.38%)</t>
+          <t>-0.46% (-1.28%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-1.00% (-1.75%)</t>
+          <t>-0.78% (-1.53%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-17.18%</t>
+          <t>-16.73%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.69%</t>
+          <t>-10.21%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.62%</t>
+          <t>-20.19%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.59%</t>
+          <t>-19.16%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-19.33%</t>
+          <t>-18.90%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-13.31%</t>
+          <t>-12.84%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.91%</t>
+          <t>-12.44%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-24.36%</t>
+          <t>-23.95%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.79%</t>
+          <t>-13.32%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-23.14%</t>
+          <t>-22.72%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.98%</t>
+          <t>-10.50%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-11.16%</t>
+          <t>-10.68%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.78%</t>
+          <t>-21.35%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>-15.20%</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-24.62%</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-23.64%</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-23.40%</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>-17.68%</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>-17.30%</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>-28.17%</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>-18.14%</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>-27.01%</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>-15.47%</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
           <t>-15.65%</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-25.03%</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-24.06%</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-23.81%</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>-18.12%</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>-17.74%</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>-28.56%</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>-18.58%</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>-27.40%</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>-15.93%</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>-16.10%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.52% (1.15%)</t>
+          <t>1.28% (0.91%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.41% (-1.09%)</t>
+          <t>-0.74% (-1.43%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.68% (1.57%)</t>
+          <t>1.28% (1.18%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.15% (1.90%)</t>
+          <t>1.80% (1.56%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.46% (1.29%)</t>
+          <t>1.18% (1.01%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.38% (-0.21%)</t>
+          <t>0.12% (-0.47%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.04% (-0.49%)</t>
+          <t>-0.22% (-0.74%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.33% (4.04%)</t>
+          <t>4.47% (4.17%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.11% (-0.57%)</t>
+          <t>-0.36% (-0.82%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.30% (1.25%)</t>
+          <t>1.32% (1.27%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.37% (-0.44%)</t>
+          <t>0.08% (-0.73%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.28% (-0.47%)</t>
+          <t>0.02% (-0.73%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.57% (2.19%)</t>
+          <t>2.19% (1.82%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.32% (-1.00%)</t>
+          <t>-0.61% (-1.30%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>1.92% (1.81%)</t>
+          <t>2.11% (2.00%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.63% (3.38%)</t>
+          <t>3.22% (2.98%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.80% (2.63%)</t>
+          <t>2.33% (2.16%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.77% (0.17%)</t>
+          <t>0.40% (-0.19%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.30% (-0.23%)</t>
+          <t>-0.06% (-0.58%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.65% (3.35%)</t>
+          <t>3.70% (3.40%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.25% (-0.21%)</t>
+          <t>-0.09% (-0.55%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.69% (0.64%)</t>
+          <t>0.71% (0.67%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.54% (-0.28%)</t>
+          <t>0.10% (-0.72%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.28% (-0.47%)</t>
+          <t>-0.04% (-0.79%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/10/2026</t>
+          <t>As of 29/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.04%</t>
+          <t>9.85%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>4.28%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.31%</t>
+          <t>9.02%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>3.21%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.30%</t>
+          <t>-9.05%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.55%</t>
+          <t>10.30%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.73%</t>
+          <t>4.95%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.01%</t>
+          <t>8.78%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2.75%</t>
+          <t>3.31%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-9.04%</t>
+          <t>-8.85%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>12.74%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.04%</t>
+          <t>4.17%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.81%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.98%</t>
+          <t>18.34%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-0.99%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.32%</t>
+          <t>-11.20%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>10.03%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.25%</t>
+          <t>7.57%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.59%</t>
+          <t>6.27%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.67%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>5.98%</t>
+          <t>6.55%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.98%</t>
+          <t>-6.70%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.81%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.62%</t>
+          <t>11.95%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>3.82%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.40%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.16%</t>
+          <t>12.76%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.79%</t>
+          <t>-4.51%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9.18%</t>
+          <t>8.99%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.24%</t>
+          <t>12.57%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>2.69%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12.69%</t>
+          <t>13.30%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.73%</t>
+          <t>-3.45%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>2.89%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12.52%</t>
+          <t>13.13%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.91%</t>
+          <t>-3.63%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.83%</t>
+          <t>8.55%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.13%</t>
+          <t>15.37%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.78%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>16.89%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.86%</t>
+          <t>-1.66%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.40%</t>
+          <t>9.19%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14.76%</t>
+          <t>15.08%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.93%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.17%</t>
+          <t>15.79%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-1.49%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.44%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.54%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.70%</t>
+          <t>0.44%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>15.92%</t>
+          <t>16.55%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.54%</t>
+          <t>-1.29%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>9.57%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>1.41%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.34%</t>
+          <t>14.16%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.28%</t>
+          <t>-13.15%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>9.83%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.80%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.80%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.51%</t>
+          <t>-10.37%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 28/10/2026</t>
+          <t>As of 29/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.72%</t>
+          <t>15.39%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.89%</t>
+          <t>7.79%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11.57%</t>
+          <t>10.97%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.76%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.09%</t>
+          <t>-8.01%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.34%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.66%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.45%</t>
+          <t>7.28%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>11.33%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.65%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.72%</t>
+          <t>-7.58%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19.04%</t>
+          <t>18.69%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.35%</t>
+          <t>3.40%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>9.54%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.98%</t>
+          <t>18.34%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-4.10%</t>
+          <t>-3.58%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.52%</t>
+          <t>-9.48%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.76%</t>
+          <t>15.50%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.68%</t>
+          <t>5.86%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>5.32%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.67%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>3.94%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.02%</t>
+          <t>-5.85%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14.13%</t>
+          <t>13.88%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.88%</t>
+          <t>9.10%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.54%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.40%</t>
+          <t>3.84%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.04%</t>
+          <t>9.63%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.45%</t>
+          <t>-4.25%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.27%</t>
+          <t>14.01%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.52%</t>
+          <t>9.73%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>10.28%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.47%</t>
+          <t>-3.29%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.59%</t>
+          <t>14.31%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9.91%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.79%</t>
+          <t>2.61%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>3.26%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>10.23%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.54%</t>
+          <t>-3.37%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.88%</t>
+          <t>13.67%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11.85%</t>
+          <t>12.13%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>0.69%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.78%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>13.49%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-1.53%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>14.12%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.19%</t>
+          <t>12.44%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>0.71%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>0.77%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12.61%</t>
+          <t>13.22%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-1.53%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.55%</t>
+          <t>14.20%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.60%</t>
+          <t>12.71%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>12.81%</t>
+          <t>13.42%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.38%</t>
+          <t>-1.28%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16.19%</t>
+          <t>15.81%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>0.67%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>11.66%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>16.46%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-3.28%</t>
+          <t>-2.76%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.22%</t>
+          <t>-11.20%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>15.55%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.81%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.25%</t>
+          <t>9.05%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13.38%</t>
+          <t>12.77%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-0.61%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.24%</t>
+          <t>-9.08%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar reporte FT buffer [2026-10-30]
</commit_message>
<xml_diff>
--- a/FT buffer remaining cap.xlsx
+++ b/FT buffer remaining cap.xlsx
@@ -675,122 +675,122 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Current Values(as of 10/29/2026 at 3:03 PM ET)</t>
+          <t>Current Values(as of 10/30/2026 at 2:39 PM ET)</t>
         </is>
       </c>
     </row>
@@ -2199,122 +2199,122 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>230 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>169 days</t>
+          <t>168 days</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>295 days</t>
+          <t>294 days</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>50 days</t>
+          <t>49 days</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>113 days</t>
+          <t>112 days</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>78 days</t>
+          <t>77 days</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>260 days</t>
+          <t>259 days</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>231 days</t>
+          <t>230 days</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>141 days</t>
+          <t>140 days</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>204 days</t>
+          <t>203 days</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>22 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>351 days</t>
+          <t>350 days</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>323 days</t>
+          <t>322 days</t>
         </is>
       </c>
     </row>
@@ -2326,122 +2326,122 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$48.11 / 6.27%</t>
+          <t>$47.49 / 4.90%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$58.01 / 0.82%</t>
+          <t>$57.15 / -0.67%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$56.43 / 10.62%</t>
+          <t>$55.61 / 9.01%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$63.00 / 8.78%</t>
+          <t>$62.20 / 7.39%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>$56.98 / 9.02%</t>
+          <t>$56.22 / 7.55%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$61.58 / 2.89%</t>
+          <t>$60.70 / 1.42%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>$61.49 / 2.69%</t>
+          <t>$60.61 / 1.23%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$53.95 / 11.66%</t>
+          <t>$53.45 / 10.62%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$57.69 / 3.82%</t>
+          <t>$56.83 / 2.27%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$60.79 / 14.16%</t>
+          <t>$59.94 / 12.58%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>$54.87 / 0.44%</t>
+          <t>$54.09 / -0.97%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>$57.45 / 0.65%</t>
+          <t>$56.66 / -0.74%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>$42.81 / 5.32%</t>
+          <t>$42.41 / 4.33%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>$42.30 / 0.69%</t>
+          <t>$41.83 / -0.44%</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>$41.10 / 9.05%</t>
+          <t>$40.66 / 7.87%</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>$45.30 / 7.28%</t>
+          <t>$44.89 / 6.32%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>$46.41 / 7.79%</t>
+          <t>$45.92 / 6.67%</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>$44.79 / 2.61%</t>
+          <t>$44.28 / 1.44%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>$42.19 / 2.53%</t>
+          <t>$41.68 / 1.29%</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>$45.49 / 9.54%</t>
+          <t>$45.16 / 8.74%</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>$44.15 / 3.54%</t>
+          <t>$43.62 / 2.29%</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>$43.24 / 11.66%</t>
+          <t>$42.87 / 10.72%</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>$43.14 / 0.43%</t>
+          <t>$42.63 / -0.74%</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>$42.34 / 0.71%</t>
+          <t>$41.86 / -0.43%</t>
         </is>
       </c>
     </row>
@@ -2453,122 +2453,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>$767.52 / 8.08%</t>
+          <t>$751.33 / 5.80%</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.24%</t>
+          <t>$751.33 / -1.88%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>$767.52 / 12.77%</t>
+          <t>$751.33 / 10.39%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$767.52 / 11.33%</t>
+          <t>$751.33 / 8.98%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>$767.52 / 10.97%</t>
+          <t>$751.33 / 8.63%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>$767.52 / 3.26%</t>
+          <t>$751.33 / 1.08%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$767.52 / 2.78%</t>
+          <t>$751.33 / 0.61%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>$767.52 / 18.34%</t>
+          <t>$751.33 / 15.84%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$767.52 / 3.84%</t>
+          <t>$751.33 / 1.64%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$767.52 / 16.46%</t>
+          <t>$751.33 / 14.00%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.56%</t>
+          <t>$751.33 / -1.56%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.77%</t>
+          <t>$751.33 / -1.36%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>$767.52 / 8.08%</t>
+          <t>$751.33 / 5.80%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.24%</t>
+          <t>$751.33 / -1.88%</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>$767.52 / 12.77%</t>
+          <t>$751.33 / 10.39%</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>$767.52 / 11.33%</t>
+          <t>$751.33 / 8.98%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>$767.52 / 10.97%</t>
+          <t>$751.33 / 8.63%</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>$767.52 / 3.26%</t>
+          <t>$751.33 / 1.08%</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>$767.52 / 2.78%</t>
+          <t>$751.33 / 0.61%</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>$767.52 / 18.34%</t>
+          <t>$751.33 / 15.84%</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>$767.52 / 3.84%</t>
+          <t>$751.33 / 1.64%</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>$767.52 / 16.46%</t>
+          <t>$751.33 / 14.00%</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.56%</t>
+          <t>$751.33 / -1.56%</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>$767.52 / 0.77%</t>
+          <t>$751.33 / -1.36%</t>
         </is>
       </c>
     </row>
@@ -2580,122 +2580,122 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7.94% (7.57%)</t>
+          <t>9.35% (8.97%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16.05% (15.37%)</t>
+          <t>17.80% (17.11%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.07% (2.97%)</t>
+          <t>4.59% (4.48%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5.19% (4.95%)</t>
+          <t>6.55% (6.30%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4.45% (4.28%)</t>
+          <t>5.87% (5.70%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13.30% (12.71%)</t>
+          <t>14.94% (14.35%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>13.09% (12.57%)</t>
+          <t>14.73% (14.20%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4.47% (4.17%)</t>
+          <t>5.45% (5.16%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12.41% (11.95%)</t>
+          <t>14.11% (13.65%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.46% (1.41%)</t>
+          <t>2.88% (2.84%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>16.65% (15.84%)</t>
+          <t>18.32% (17.50%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>15.83% (15.08%)</t>
+          <t>17.45% (16.69%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>6.24% (5.86%)</t>
+          <t>7.24% (6.86%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>12.81% (12.13%)</t>
+          <t>14.09% (13.40%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.11% (2.00%)</t>
+          <t>3.22% (3.12%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>3.90% (3.66%)</t>
+          <t>4.84% (4.59%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>3.11% (2.94%)</t>
+          <t>4.20% (4.03%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>10.69% (10.10%)</t>
+          <t>11.97% (11.37%)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>10.25% (9.73%)</t>
+          <t>11.60% (11.07%)</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3.70% (3.40%)</t>
+          <t>4.45% (4.15%)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>9.56% (9.10%)</t>
+          <t>10.90% (10.44%)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.71% (0.67%)</t>
+          <t>1.57% (1.53%)</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>13.53% (12.71%)</t>
+          <t>14.87% (14.05%)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>13.19% (12.44%)</t>
+          <t>14.49% (13.73%)</t>
         </is>
       </c>
     </row>
@@ -2707,122 +2707,122 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>19.41%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3.31%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>15.20%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.14%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>19.06%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>18.29%</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>12.66%</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>-3.58%</t>
+          <t>-1.50%</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>15.86%</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>15.66%</t>
         </is>
       </c>
     </row>
@@ -2834,122 +2834,122 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10.40% (10.03%)</t>
+          <t>9.83% (9.46%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9.23% (8.55%)</t>
+          <t>8.79% (8.10%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.93% (9.83%)</t>
+          <t>9.53% (9.43%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10.55% (10.30%)</t>
+          <t>9.98% (9.74%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>10.01% (9.85%)</t>
+          <t>9.50% (9.34%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>9.80% (9.21%)</t>
+          <t>9.32% (8.73%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9.51% (8.99%)</t>
+          <t>9.03% (8.50%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>13.04% (12.74%)</t>
+          <t>12.24% (11.94%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9.27% (8.81%)</t>
+          <t>8.85% (8.39%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.62% (9.57%)</t>
+          <t>9.18% (9.13%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>10.03% (9.21%)</t>
+          <t>9.52% (8.70%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>9.94% (9.19%)</t>
+          <t>9.40% (8.65%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>15.87% (15.50%)</t>
+          <t>15.07% (14.69%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>14.35% (13.67%)</t>
+          <t>13.65% (12.96%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>15.65% (15.55%)</t>
+          <t>15.02% (14.92%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16.31% (16.07%)</t>
+          <t>15.50% (15.26%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>15.55% (15.39%)</t>
+          <t>14.87% (14.71%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>14.90% (14.31%)</t>
+          <t>14.25% (13.65%)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.53% (14.01%)</t>
+          <t>13.94% (13.41%)</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>18.99% (18.69%)</t>
+          <t>18.11% (17.81%)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.34% (13.88%)</t>
+          <t>13.76% (13.29%)</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>15.86% (15.81%)</t>
+          <t>15.04% (15.00%)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>15.01% (14.20%)</t>
+          <t>14.37% (13.55%)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>14.87% (14.12%)</t>
+          <t>14.18% (13.43%)</t>
         </is>
       </c>
     </row>
@@ -2961,122 +2961,122 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-6.33% (-6.70%)</t>
+          <t>-5.10% (-5.48%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.98% (-1.66%)</t>
+          <t>0.00% (-0.18%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-10.26% (-10.37%)</t>
+          <t>-8.94% (-9.05%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-8.61% (-8.85%)</t>
+          <t>-7.43% (-7.67%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-8.88% (-9.05%)</t>
+          <t>-7.64% (-7.81%)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-3.04% (-3.63%)</t>
+          <t>-1.64% (-2.24%)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-2.93% (-3.45%)</t>
+          <t>-1.52% (-2.05%)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-10.91% (-11.20%)</t>
+          <t>-10.07% (-10.37%)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-4.05% (-4.51%)</t>
+          <t>-2.60% (-3.06%)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>-13.10% (-13.15%)</t>
+          <t>-11.88% (-11.92%)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.47% (-1.29%)</t>
+          <t>0.00% (0.00%)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>-0.74% (-1.49%)</t>
+          <t>0.00% (-0.11%)</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>-5.48% (-5.85%)</t>
+          <t>-4.59% (-4.96%)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>-0.84% (-1.53%)</t>
+          <t>0.00% (-0.41%)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>-8.97% (-9.08%)</t>
+          <t>-7.98% (-8.08%)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-7.33% (-7.58%)</t>
+          <t>-6.50% (-6.74%)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-7.84% (-8.01%)</t>
+          <t>-6.87% (-7.04%)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>-2.78% (-3.37%)</t>
+          <t>-1.66% (-2.25%)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>-2.77% (-3.29%)</t>
+          <t>-1.58% (-2.11%)</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>-9.18% (-9.48%)</t>
+          <t>-8.52% (-8.82%)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>-3.80% (-4.25%)</t>
+          <t>-2.62% (-3.08%)</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-11.15% (-11.20%)</t>
+          <t>-10.40% (-10.44%)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>-0.46% (-1.28%)</t>
+          <t>0.00% (-0.11%)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>-0.78% (-1.53%)</t>
+          <t>0.00% (-0.40%)</t>
         </is>
       </c>
     </row>
@@ -3088,122 +3088,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-16.73%</t>
+          <t>-14.93%</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-10.21%</t>
+          <t>-8.28%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-20.19%</t>
+          <t>-18.47%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-19.16%</t>
+          <t>-17.41%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-18.90%</t>
+          <t>-17.15%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-12.84%</t>
+          <t>-10.96%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>-12.44%</t>
+          <t>-10.55%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-23.95%</t>
+          <t>-22.31%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-13.32%</t>
+          <t>-11.46%</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>-22.72%</t>
+          <t>-21.06%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-10.50%</t>
+          <t>-8.57%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>-10.68%</t>
+          <t>-8.76%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-21.35%</t>
+          <t>-19.66%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>-15.20%</t>
+          <t>-13.37%</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>-24.62%</t>
+          <t>-23.00%</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-23.64%</t>
+          <t>-22.00%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>-23.40%</t>
+          <t>-21.75%</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>-17.68%</t>
+          <t>-15.91%</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>-17.30%</t>
+          <t>-15.52%</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>-28.17%</t>
+          <t>-26.62%</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>-18.14%</t>
+          <t>-16.37%</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-27.01%</t>
+          <t>-25.44%</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>-15.47%</t>
+          <t>-13.65%</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>-15.65%</t>
+          <t>-13.83%</t>
         </is>
       </c>
     </row>
@@ -3215,122 +3215,122 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.28% (0.91%)</t>
+          <t>0.42% (0.05%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.74% (-1.43%)</t>
+          <t>0.51% (-0.18%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.28% (1.18%)</t>
+          <t>0.59% (0.49%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.80% (1.56%)</t>
+          <t>0.93% (0.69%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.18% (1.01%)</t>
+          <t>0.38% (0.21%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.12% (-0.47%)</t>
+          <t>-0.58% (-1.17%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.22% (-0.74%)</t>
+          <t>-0.91% (-1.44%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.47% (4.17%)</t>
+          <t>4.25% (3.96%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.36% (-0.82%)</t>
+          <t>-0.99% (-1.46%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.32% (1.27%)</t>
+          <t>0.56% (0.52%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.08% (-0.73%)</t>
+          <t>0.95% (0.13%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.02% (-0.73%)</t>
+          <t>0.65% (-0.11%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2.19% (1.82%)</t>
+          <t>0.97% (0.59%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>-0.61% (-1.30%)</t>
+          <t>0.28% (-0.41%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.11% (2.00%)</t>
+          <t>1.66% (1.55%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>3.22% (2.98%)</t>
+          <t>1.94% (1.70%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2.33% (2.16%)</t>
+          <t>1.21% (1.04%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.40% (-0.19%)</t>
+          <t>-0.59% (-1.19%)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>-0.06% (-0.58%)</t>
+          <t>-0.98% (-1.50%)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3.70% (3.40%)</t>
+          <t>4.45% (4.15%)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>-0.09% (-0.55%)</t>
+          <t>-1.01% (-1.47%)</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.71% (0.67%)</t>
+          <t>1.57% (1.53%)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.10% (-0.72%)</t>
+          <t>0.72% (-0.11%)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>-0.04% (-0.79%)</t>
+          <t>0.36% (-0.40%)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/10/2026</t>
+          <t>As of 30/10/2026</t>
         </is>
       </c>
     </row>
@@ -3410,32 +3410,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.85%</t>
+          <t>9.34%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.28%</t>
+          <t>5.70%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>7.55%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-9.05%</t>
+          <t>-7.81%</t>
         </is>
       </c>
     </row>
@@ -3447,32 +3447,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.30%</t>
+          <t>9.74%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.95%</t>
+          <t>6.30%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>7.39%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.31%</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-8.85%</t>
+          <t>-7.67%</t>
         </is>
       </c>
     </row>
@@ -3484,32 +3484,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.74%</t>
+          <t>11.94%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.17%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>10.62%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.34%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>1.15%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-11.20%</t>
+          <t>-10.37%</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.03%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.57%</t>
+          <t>8.97%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.27%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.55%</t>
+          <t>8.85%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-6.70%</t>
+          <t>-5.48%</t>
         </is>
       </c>
     </row>
@@ -3558,32 +3558,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.81%</t>
+          <t>8.39%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>13.65%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.82%</t>
+          <t>2.27%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.76%</t>
+          <t>15.20%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.51%</t>
+          <t>-3.06%</t>
         </is>
       </c>
     </row>
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.99%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.57%</t>
+          <t>14.20%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.69%</t>
+          <t>1.23%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>13.30%</t>
+          <t>15.74%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.45%</t>
+          <t>-2.05%</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>8.73%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>14.35%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.89%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>13.13%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.63%</t>
+          <t>-2.24%</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8.55%</t>
+          <t>8.10%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15.37%</t>
+          <t>17.11%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>-0.67%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>-1.88%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16.89%</t>
+          <t>19.41%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-0.18%</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9.19%</t>
+          <t>8.65%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15.08%</t>
+          <t>16.69%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>-1.36%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>15.79%</t>
+          <t>18.29%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.49%</t>
+          <t>-0.11%</t>
         </is>
       </c>
     </row>
@@ -3743,32 +3743,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9.21%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15.84%</t>
+          <t>17.50%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.44%</t>
+          <t>-0.97%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.56%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>19.06%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3780,32 +3780,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9.57%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.41%</t>
+          <t>2.84%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>12.58%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.14%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-13.15%</t>
+          <t>-11.92%</t>
         </is>
       </c>
     </row>
@@ -3817,32 +3817,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9.83%</t>
+          <t>9.43%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.97%</t>
+          <t>4.48%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.62%</t>
+          <t>9.01%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-10.37%</t>
+          <t>-9.05%</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>As of 29/10/2026</t>
+          <t>As of 30/10/2026</t>
         </is>
       </c>
     </row>
@@ -3925,32 +3925,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.39%</t>
+          <t>14.71%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.94%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.79%</t>
+          <t>6.67%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10.97%</t>
+          <t>8.63%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.76%</t>
+          <t>2.93%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-8.01%</t>
+          <t>-7.04%</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.07%</t>
+          <t>15.26%</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.66%</t>
+          <t>4.59%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.28%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11.33%</t>
+          <t>8.98%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-7.58%</t>
+          <t>-6.74%</t>
         </is>
       </c>
     </row>
@@ -3999,32 +3999,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18.69%</t>
+          <t>17.81%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.40%</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18.34%</t>
+          <t>15.84%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-3.58%</t>
+          <t>-1.50%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-9.48%</t>
+          <t>-8.82%</t>
         </is>
       </c>
     </row>
@@ -4036,32 +4036,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.50%</t>
+          <t>14.69%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.86%</t>
+          <t>6.86%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.32%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>5.80%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.94%</t>
+          <t>6.18%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-5.85%</t>
+          <t>-4.96%</t>
         </is>
       </c>
     </row>
@@ -4073,32 +4073,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.88%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9.10%</t>
+          <t>10.44%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>2.29%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3.84%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9.63%</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-4.25%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -4110,32 +4110,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9.73%</t>
+          <t>11.07%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>1.29%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>0.61%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.28%</t>
+          <t>12.66%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.11%</t>
         </is>
       </c>
     </row>
@@ -4147,32 +4147,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>14.31%</t>
+          <t>13.65%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.61%</t>
+          <t>1.44%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10.23%</t>
+          <t>12.61%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-3.37%</t>
+          <t>-2.25%</t>
         </is>
       </c>
     </row>
@@ -4184,32 +4184,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.67%</t>
+          <t>12.96%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12.13%</t>
+          <t>13.40%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>-1.88%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>13.49%</t>
+          <t>15.93%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-1.53%</t>
+          <t>-0.41%</t>
         </is>
       </c>
     </row>
@@ -4221,32 +4221,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14.12%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12.44%</t>
+          <t>13.73%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.71%</t>
+          <t>-0.43%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>-1.36%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13.22%</t>
+          <t>15.66%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-1.53%</t>
+          <t>-0.40%</t>
         </is>
       </c>
     </row>
@@ -4258,32 +4258,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.20%</t>
+          <t>13.55%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.71%</t>
+          <t>14.05%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>-0.74%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.56%</t>
+          <t>-1.56%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13.42%</t>
+          <t>15.86%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-1.28%</t>
+          <t>-0.11%</t>
         </is>
       </c>
     </row>
@@ -4295,32 +4295,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.81%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.66%</t>
+          <t>10.72%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16.46%</t>
+          <t>14.00%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-0.66%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-11.20%</t>
+          <t>-10.44%</t>
         </is>
       </c>
     </row>
@@ -4332,32 +4332,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>14.92%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>3.12%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.05%</t>
+          <t>7.87%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>10.39%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>1.53%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-9.08%</t>
+          <t>-8.08%</t>
         </is>
       </c>
     </row>

</xml_diff>